<commit_message>
Restructure balance sheet into grouped format (Equity & Liabilities / Assets) with historical data filled FY20-FY33; add CF cash roll for all years
</commit_message>
<xml_diff>
--- a/BHEL_Financial_Model.xlsx
+++ b/BHEL_Financial_Model.xlsx
@@ -194,7 +194,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="67">
+  <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -284,7 +284,11 @@
     <xf numFmtId="165" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="4" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
@@ -3013,7 +3017,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O25"/>
+  <dimension ref="A1:O26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -3774,6 +3778,27 @@
           <t>Opening cash &amp; bank</t>
         </is>
       </c>
+      <c r="B24" s="21" t="n">
+        <v>6353</v>
+      </c>
+      <c r="C24" s="21" t="n">
+        <v>6961</v>
+      </c>
+      <c r="D24" s="21" t="n">
+        <v>7084</v>
+      </c>
+      <c r="E24" s="21" t="n">
+        <v>6297</v>
+      </c>
+      <c r="F24" s="21" t="n">
+        <v>7126</v>
+      </c>
+      <c r="G24" s="21" t="n">
+        <v>7400</v>
+      </c>
+      <c r="H24" s="21" t="n">
+        <v>6004</v>
+      </c>
       <c r="I24" s="24">
         <f>'Working Capital Schedule'!H19</f>
         <v/>
@@ -3809,6 +3834,27 @@
           <t>Closing cash &amp; bank</t>
         </is>
       </c>
+      <c r="B25" s="39" t="n">
+        <v>6961</v>
+      </c>
+      <c r="C25" s="39" t="n">
+        <v>7084</v>
+      </c>
+      <c r="D25" s="39" t="n">
+        <v>6297</v>
+      </c>
+      <c r="E25" s="39" t="n">
+        <v>7126</v>
+      </c>
+      <c r="F25" s="39" t="n">
+        <v>7400</v>
+      </c>
+      <c r="G25" s="39" t="n">
+        <v>6004</v>
+      </c>
+      <c r="H25" s="39" t="n">
+        <v>7000</v>
+      </c>
       <c r="I25" s="37">
         <f>I24+I23</f>
         <v/>
@@ -3836,6 +3882,13 @@
       <c r="O25" s="37">
         <f>O24+O23</f>
         <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="27" t="inlineStr">
+        <is>
+          <t>FY20-26 operating/investing/financing shown at reported subtotal level; cash balances rolled from reported net cash flow (FY26 anchor estimated).</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -3849,7 +3902,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O42"/>
+  <dimension ref="A1:O64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -4947,59 +5000,59 @@
         </is>
       </c>
       <c r="B21" s="26">
-        <f>B20/'Assumptions'!C40</f>
+        <f>B20/'Assumptions'!C43</f>
         <v/>
       </c>
       <c r="C21" s="26">
-        <f>C20/'Assumptions'!C40</f>
+        <f>C20/'Assumptions'!C43</f>
         <v/>
       </c>
       <c r="D21" s="26">
-        <f>D20/'Assumptions'!C40</f>
+        <f>D20/'Assumptions'!C43</f>
         <v/>
       </c>
       <c r="E21" s="26">
-        <f>E20/'Assumptions'!C40</f>
+        <f>E20/'Assumptions'!C43</f>
         <v/>
       </c>
       <c r="F21" s="26">
-        <f>F20/'Assumptions'!C40</f>
+        <f>F20/'Assumptions'!C43</f>
         <v/>
       </c>
       <c r="G21" s="26">
-        <f>G20/'Assumptions'!C40</f>
+        <f>G20/'Assumptions'!C43</f>
         <v/>
       </c>
       <c r="H21" s="26">
-        <f>H20/'Assumptions'!C40</f>
+        <f>H20/'Assumptions'!C43</f>
         <v/>
       </c>
       <c r="I21" s="26">
-        <f>I20/'Assumptions'!C40</f>
+        <f>I20/'Assumptions'!C43</f>
         <v/>
       </c>
       <c r="J21" s="26">
-        <f>J20/'Assumptions'!C40</f>
+        <f>J20/'Assumptions'!C43</f>
         <v/>
       </c>
       <c r="K21" s="26">
-        <f>K20/'Assumptions'!C40</f>
+        <f>K20/'Assumptions'!C43</f>
         <v/>
       </c>
       <c r="L21" s="26">
-        <f>L20/'Assumptions'!C40</f>
+        <f>L20/'Assumptions'!C43</f>
         <v/>
       </c>
       <c r="M21" s="26">
-        <f>M20/'Assumptions'!C40</f>
+        <f>M20/'Assumptions'!C43</f>
         <v/>
       </c>
       <c r="N21" s="26">
-        <f>N20/'Assumptions'!C40</f>
+        <f>N20/'Assumptions'!C43</f>
         <v/>
       </c>
       <c r="O21" s="26">
-        <f>O20/'Assumptions'!C40</f>
+        <f>O20/'Assumptions'!C43</f>
         <v/>
       </c>
     </row>
@@ -5069,7 +5122,7 @@
     <row r="24">
       <c r="A24" s="11" t="inlineStr">
         <is>
-          <t>B.  BALANCE SHEET  (FY2026 reported, FY2027-33 forecast)</t>
+          <t>B.  BALANCE SHEET  (FY2020-FY2026 reported, FY2027-33 forecast)</t>
         </is>
       </c>
       <c r="B24" s="1" t="n"/>
@@ -5088,17 +5141,41 @@
       <c r="O24" s="1" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="39" t="inlineStr">
-        <is>
-          <t>FY20-25: see Historical Financial Statements</t>
-        </is>
-      </c>
-      <c r="B25" s="13" t="inlineStr"/>
-      <c r="C25" s="13" t="inlineStr"/>
-      <c r="D25" s="13" t="inlineStr"/>
-      <c r="E25" s="13" t="inlineStr"/>
-      <c r="F25" s="13" t="inlineStr"/>
-      <c r="G25" s="13" t="inlineStr"/>
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>Particulars</t>
+        </is>
+      </c>
+      <c r="B25" s="13" t="inlineStr">
+        <is>
+          <t>FY2020</t>
+        </is>
+      </c>
+      <c r="C25" s="13" t="inlineStr">
+        <is>
+          <t>FY2021</t>
+        </is>
+      </c>
+      <c r="D25" s="13" t="inlineStr">
+        <is>
+          <t>FY2022</t>
+        </is>
+      </c>
+      <c r="E25" s="13" t="inlineStr">
+        <is>
+          <t>FY2023</t>
+        </is>
+      </c>
+      <c r="F25" s="13" t="inlineStr">
+        <is>
+          <t>FY2024</t>
+        </is>
+      </c>
+      <c r="G25" s="13" t="inlineStr">
+        <is>
+          <t>FY2025</t>
+        </is>
+      </c>
       <c r="H25" s="13" t="inlineStr">
         <is>
           <t>FY2026</t>
@@ -5141,482 +5218,479 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="5" t="inlineStr">
-        <is>
-          <t>Net property, plant &amp; equipment</t>
-        </is>
-      </c>
-      <c r="H26" s="35">
-        <f>'Historical Financial Statements'!H28</f>
-        <v/>
-      </c>
-      <c r="I26" s="35">
-        <f>'Fixed Asset Schedule'!I10</f>
-        <v/>
-      </c>
-      <c r="J26" s="35">
-        <f>'Fixed Asset Schedule'!J10</f>
-        <v/>
-      </c>
-      <c r="K26" s="35">
-        <f>'Fixed Asset Schedule'!K10</f>
-        <v/>
-      </c>
-      <c r="L26" s="35">
-        <f>'Fixed Asset Schedule'!L10</f>
-        <v/>
-      </c>
-      <c r="M26" s="35">
-        <f>'Fixed Asset Schedule'!M10</f>
-        <v/>
-      </c>
-      <c r="N26" s="35">
-        <f>'Fixed Asset Schedule'!N10</f>
-        <v/>
-      </c>
-      <c r="O26" s="35">
-        <f>'Fixed Asset Schedule'!O10</f>
-        <v/>
-      </c>
+      <c r="A26" s="40" t="inlineStr">
+        <is>
+          <t>Equities &amp; Liabilities</t>
+        </is>
+      </c>
+      <c r="B26" s="41" t="n"/>
+      <c r="C26" s="41" t="n"/>
+      <c r="D26" s="41" t="n"/>
+      <c r="E26" s="41" t="n"/>
+      <c r="F26" s="41" t="n"/>
+      <c r="G26" s="41" t="n"/>
+      <c r="H26" s="41" t="n"/>
+      <c r="I26" s="41" t="n"/>
+      <c r="J26" s="41" t="n"/>
+      <c r="K26" s="41" t="n"/>
+      <c r="L26" s="41" t="n"/>
+      <c r="M26" s="41" t="n"/>
+      <c r="N26" s="41" t="n"/>
+      <c r="O26" s="41" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="5" t="inlineStr">
-        <is>
-          <t>Capital work-in-progress</t>
-        </is>
-      </c>
-      <c r="H27" s="35">
-        <f>'Historical Financial Statements'!H29</f>
-        <v/>
-      </c>
-      <c r="I27" s="35">
-        <f>'Assumptions'!I21</f>
-        <v/>
-      </c>
-      <c r="J27" s="35">
-        <f>'Assumptions'!J21</f>
-        <v/>
-      </c>
-      <c r="K27" s="35">
-        <f>'Assumptions'!K21</f>
-        <v/>
-      </c>
-      <c r="L27" s="35">
-        <f>'Assumptions'!L21</f>
-        <v/>
-      </c>
-      <c r="M27" s="35">
-        <f>'Assumptions'!M21</f>
-        <v/>
-      </c>
-      <c r="N27" s="35">
-        <f>'Assumptions'!N21</f>
-        <v/>
-      </c>
-      <c r="O27" s="35">
-        <f>'Assumptions'!O21</f>
-        <v/>
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Shareholders' Fund</t>
+        </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>Investments</t>
-        </is>
-      </c>
-      <c r="H28" s="35">
-        <f>'Historical Financial Statements'!H30</f>
-        <v/>
+          <t xml:space="preserve">   Share Capital</t>
+        </is>
+      </c>
+      <c r="B28" s="21" t="n">
+        <v>696</v>
+      </c>
+      <c r="C28" s="21" t="n">
+        <v>696</v>
+      </c>
+      <c r="D28" s="21" t="n">
+        <v>696</v>
+      </c>
+      <c r="E28" s="21" t="n">
+        <v>696</v>
+      </c>
+      <c r="F28" s="21" t="n">
+        <v>696</v>
+      </c>
+      <c r="G28" s="21" t="n">
+        <v>696</v>
+      </c>
+      <c r="H28" s="21" t="n">
+        <v>696</v>
       </c>
       <c r="I28" s="35">
-        <f>'Assumptions'!I22</f>
+        <f>'Equity Schedule'!I12</f>
         <v/>
       </c>
       <c r="J28" s="35">
-        <f>'Assumptions'!J22</f>
+        <f>'Equity Schedule'!J12</f>
         <v/>
       </c>
       <c r="K28" s="35">
-        <f>'Assumptions'!K22</f>
+        <f>'Equity Schedule'!K12</f>
         <v/>
       </c>
       <c r="L28" s="35">
-        <f>'Assumptions'!L22</f>
+        <f>'Equity Schedule'!L12</f>
         <v/>
       </c>
       <c r="M28" s="35">
-        <f>'Assumptions'!M22</f>
+        <f>'Equity Schedule'!M12</f>
         <v/>
       </c>
       <c r="N28" s="35">
-        <f>'Assumptions'!N22</f>
+        <f>'Equity Schedule'!N12</f>
         <v/>
       </c>
       <c r="O28" s="35">
-        <f>'Assumptions'!O22</f>
+        <f>'Equity Schedule'!O12</f>
         <v/>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Inventories</t>
-        </is>
-      </c>
-      <c r="H29" s="35">
-        <f>'Working Capital Schedule'!H9</f>
-        <v/>
+          <t xml:space="preserve">   Reserve &amp; Surplus</t>
+        </is>
+      </c>
+      <c r="B29" s="21" t="n">
+        <v>27964</v>
+      </c>
+      <c r="C29" s="21" t="n">
+        <v>25287</v>
+      </c>
+      <c r="D29" s="21" t="n">
+        <v>25810</v>
+      </c>
+      <c r="E29" s="21" t="n">
+        <v>23682</v>
+      </c>
+      <c r="F29" s="21" t="n">
+        <v>23742</v>
+      </c>
+      <c r="G29" s="21" t="n">
+        <v>24026</v>
+      </c>
+      <c r="H29" s="21" t="n">
+        <v>25450</v>
       </c>
       <c r="I29" s="35">
-        <f>'Working Capital Schedule'!I9</f>
+        <f>'Equity Schedule'!I10</f>
         <v/>
       </c>
       <c r="J29" s="35">
-        <f>'Working Capital Schedule'!J9</f>
+        <f>'Equity Schedule'!J10</f>
         <v/>
       </c>
       <c r="K29" s="35">
-        <f>'Working Capital Schedule'!K9</f>
+        <f>'Equity Schedule'!K10</f>
         <v/>
       </c>
       <c r="L29" s="35">
-        <f>'Working Capital Schedule'!L9</f>
+        <f>'Equity Schedule'!L10</f>
         <v/>
       </c>
       <c r="M29" s="35">
-        <f>'Working Capital Schedule'!M9</f>
+        <f>'Equity Schedule'!M10</f>
         <v/>
       </c>
       <c r="N29" s="35">
-        <f>'Working Capital Schedule'!N9</f>
+        <f>'Equity Schedule'!N10</f>
         <v/>
       </c>
       <c r="O29" s="35">
-        <f>'Working Capital Schedule'!O9</f>
+        <f>'Equity Schedule'!O10</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Trade receivables</t>
-        </is>
-      </c>
-      <c r="H30" s="35">
-        <f>'Working Capital Schedule'!H8</f>
-        <v/>
-      </c>
-      <c r="I30" s="35">
-        <f>'Working Capital Schedule'!I8</f>
-        <v/>
-      </c>
-      <c r="J30" s="35">
-        <f>'Working Capital Schedule'!J8</f>
-        <v/>
-      </c>
-      <c r="K30" s="35">
-        <f>'Working Capital Schedule'!K8</f>
-        <v/>
-      </c>
-      <c r="L30" s="35">
-        <f>'Working Capital Schedule'!L8</f>
-        <v/>
-      </c>
-      <c r="M30" s="35">
-        <f>'Working Capital Schedule'!M8</f>
-        <v/>
-      </c>
-      <c r="N30" s="35">
-        <f>'Working Capital Schedule'!N8</f>
-        <v/>
-      </c>
-      <c r="O30" s="35">
-        <f>'Working Capital Schedule'!O8</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Contract assets</t>
-        </is>
-      </c>
-      <c r="H31" s="35">
-        <f>'Working Capital Schedule'!H10</f>
-        <v/>
-      </c>
-      <c r="I31" s="35">
-        <f>'Working Capital Schedule'!I10</f>
-        <v/>
-      </c>
-      <c r="J31" s="35">
-        <f>'Working Capital Schedule'!J10</f>
-        <v/>
-      </c>
-      <c r="K31" s="35">
-        <f>'Working Capital Schedule'!K10</f>
-        <v/>
-      </c>
-      <c r="L31" s="35">
-        <f>'Working Capital Schedule'!L10</f>
-        <v/>
-      </c>
-      <c r="M31" s="35">
-        <f>'Working Capital Schedule'!M10</f>
-        <v/>
-      </c>
-      <c r="N31" s="35">
-        <f>'Working Capital Schedule'!N10</f>
-        <v/>
-      </c>
-      <c r="O31" s="35">
-        <f>'Working Capital Schedule'!O10</f>
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Total Shareholders' Fund</t>
+        </is>
+      </c>
+      <c r="B30" s="23">
+        <f>B28+B29</f>
+        <v/>
+      </c>
+      <c r="C30" s="23">
+        <f>C28+C29</f>
+        <v/>
+      </c>
+      <c r="D30" s="23">
+        <f>D28+D29</f>
+        <v/>
+      </c>
+      <c r="E30" s="23">
+        <f>E28+E29</f>
+        <v/>
+      </c>
+      <c r="F30" s="23">
+        <f>F28+F29</f>
+        <v/>
+      </c>
+      <c r="G30" s="23">
+        <f>G28+G29</f>
+        <v/>
+      </c>
+      <c r="H30" s="23">
+        <f>H28+H29</f>
+        <v/>
+      </c>
+      <c r="I30" s="23">
+        <f>I28+I29</f>
+        <v/>
+      </c>
+      <c r="J30" s="23">
+        <f>J28+J29</f>
+        <v/>
+      </c>
+      <c r="K30" s="23">
+        <f>K28+K29</f>
+        <v/>
+      </c>
+      <c r="L30" s="23">
+        <f>L28+L29</f>
+        <v/>
+      </c>
+      <c r="M30" s="23">
+        <f>M28+M29</f>
+        <v/>
+      </c>
+      <c r="N30" s="23">
+        <f>N28+N29</f>
+        <v/>
+      </c>
+      <c r="O30" s="23">
+        <f>O28+O29</f>
         <v/>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Cash &amp; bank balances</t>
-        </is>
-      </c>
-      <c r="H32" s="35">
-        <f>'Working Capital Schedule'!H19</f>
-        <v/>
-      </c>
-      <c r="I32" s="35">
-        <f>'Cash Flow Statement'!I25</f>
-        <v/>
-      </c>
-      <c r="J32" s="35">
-        <f>'Cash Flow Statement'!J25</f>
-        <v/>
-      </c>
-      <c r="K32" s="35">
-        <f>'Cash Flow Statement'!K25</f>
-        <v/>
-      </c>
-      <c r="L32" s="35">
-        <f>'Cash Flow Statement'!L25</f>
-        <v/>
-      </c>
-      <c r="M32" s="35">
-        <f>'Cash Flow Statement'!M25</f>
-        <v/>
-      </c>
-      <c r="N32" s="35">
-        <f>'Cash Flow Statement'!N25</f>
-        <v/>
-      </c>
-      <c r="O32" s="35">
-        <f>'Cash Flow Statement'!O25</f>
-        <v/>
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Liabilities</t>
+        </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Other current &amp; non-current assets</t>
-        </is>
-      </c>
-      <c r="H33" s="35">
-        <f>'Working Capital Schedule'!H11</f>
-        <v/>
-      </c>
-      <c r="I33" s="35">
-        <f>'Working Capital Schedule'!I11</f>
-        <v/>
-      </c>
-      <c r="J33" s="35">
-        <f>'Working Capital Schedule'!J11</f>
-        <v/>
-      </c>
-      <c r="K33" s="35">
-        <f>'Working Capital Schedule'!K11</f>
-        <v/>
-      </c>
-      <c r="L33" s="35">
-        <f>'Working Capital Schedule'!L11</f>
-        <v/>
-      </c>
-      <c r="M33" s="35">
-        <f>'Working Capital Schedule'!M11</f>
-        <v/>
-      </c>
-      <c r="N33" s="35">
-        <f>'Working Capital Schedule'!N11</f>
-        <v/>
-      </c>
-      <c r="O33" s="35">
-        <f>'Working Capital Schedule'!O11</f>
-        <v/>
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Non-Current Liabilities</t>
+        </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="4" t="inlineStr">
-        <is>
-          <t>TOTAL ASSETS</t>
-        </is>
-      </c>
-      <c r="H34" s="25">
-        <f>SUM(H26:H33)</f>
-        <v/>
-      </c>
-      <c r="I34" s="25">
-        <f>SUM(I26:I33)</f>
-        <v/>
-      </c>
-      <c r="J34" s="25">
-        <f>SUM(J26:J33)</f>
-        <v/>
-      </c>
-      <c r="K34" s="25">
-        <f>SUM(K26:K33)</f>
-        <v/>
-      </c>
-      <c r="L34" s="25">
-        <f>SUM(L26:L33)</f>
-        <v/>
-      </c>
-      <c r="M34" s="25">
-        <f>SUM(M26:M33)</f>
-        <v/>
-      </c>
-      <c r="N34" s="25">
-        <f>SUM(N26:N33)</f>
-        <v/>
-      </c>
-      <c r="O34" s="25">
-        <f>SUM(O26:O33)</f>
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   LT borrowings</t>
+        </is>
+      </c>
+      <c r="B34" s="21" t="n">
+        <v>1778</v>
+      </c>
+      <c r="C34" s="21" t="n">
+        <v>1733</v>
+      </c>
+      <c r="D34" s="21" t="n">
+        <v>1690</v>
+      </c>
+      <c r="E34" s="21" t="n">
+        <v>1909</v>
+      </c>
+      <c r="F34" s="21" t="n">
+        <v>3100</v>
+      </c>
+      <c r="G34" s="21" t="n">
+        <v>3155</v>
+      </c>
+      <c r="H34" s="21" t="n">
+        <v>2865</v>
+      </c>
+      <c r="I34" s="35">
+        <f>'Assumptions'!I28*'Debt Schedule'!I9</f>
+        <v/>
+      </c>
+      <c r="J34" s="35">
+        <f>'Assumptions'!J28*'Debt Schedule'!J9</f>
+        <v/>
+      </c>
+      <c r="K34" s="35">
+        <f>'Assumptions'!K28*'Debt Schedule'!K9</f>
+        <v/>
+      </c>
+      <c r="L34" s="35">
+        <f>'Assumptions'!L28*'Debt Schedule'!L9</f>
+        <v/>
+      </c>
+      <c r="M34" s="35">
+        <f>'Assumptions'!M28*'Debt Schedule'!M9</f>
+        <v/>
+      </c>
+      <c r="N34" s="35">
+        <f>'Assumptions'!N28*'Debt Schedule'!N9</f>
+        <v/>
+      </c>
+      <c r="O34" s="35">
+        <f>'Assumptions'!O28*'Debt Schedule'!O9</f>
         <v/>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>Equity share capital</t>
-        </is>
-      </c>
-      <c r="H35" s="35">
-        <f>'Historical Financial Statements'!H33</f>
-        <v/>
+          <t xml:space="preserve">   Other non current liabilities</t>
+        </is>
+      </c>
+      <c r="B35" s="21" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C35" s="21" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D35" s="21" t="n">
+        <v>5000</v>
+      </c>
+      <c r="E35" s="21" t="n">
+        <v>4000</v>
+      </c>
+      <c r="F35" s="21" t="n">
+        <v>4500</v>
+      </c>
+      <c r="G35" s="21" t="n">
+        <v>5500</v>
+      </c>
+      <c r="H35" s="21" t="n">
+        <v>6000</v>
       </c>
       <c r="I35" s="35">
-        <f>'Equity Schedule'!I12</f>
+        <f>'Assumptions'!I30</f>
         <v/>
       </c>
       <c r="J35" s="35">
-        <f>'Equity Schedule'!J12</f>
+        <f>'Assumptions'!J30</f>
         <v/>
       </c>
       <c r="K35" s="35">
-        <f>'Equity Schedule'!K12</f>
+        <f>'Assumptions'!K30</f>
         <v/>
       </c>
       <c r="L35" s="35">
-        <f>'Equity Schedule'!L12</f>
+        <f>'Assumptions'!L30</f>
         <v/>
       </c>
       <c r="M35" s="35">
-        <f>'Equity Schedule'!M12</f>
+        <f>'Assumptions'!M30</f>
         <v/>
       </c>
       <c r="N35" s="35">
-        <f>'Equity Schedule'!N12</f>
+        <f>'Assumptions'!N30</f>
         <v/>
       </c>
       <c r="O35" s="35">
-        <f>'Equity Schedule'!O12</f>
+        <f>'Assumptions'!O30</f>
         <v/>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="5" t="inlineStr">
-        <is>
-          <t>Other equity (reserves &amp; surplus)</t>
-        </is>
-      </c>
-      <c r="H36" s="35">
-        <f>'Historical Financial Statements'!H34</f>
-        <v/>
-      </c>
-      <c r="I36" s="35">
-        <f>'Equity Schedule'!I10</f>
-        <v/>
-      </c>
-      <c r="J36" s="35">
-        <f>'Equity Schedule'!J10</f>
-        <v/>
-      </c>
-      <c r="K36" s="35">
-        <f>'Equity Schedule'!K10</f>
-        <v/>
-      </c>
-      <c r="L36" s="35">
-        <f>'Equity Schedule'!L10</f>
-        <v/>
-      </c>
-      <c r="M36" s="35">
-        <f>'Equity Schedule'!M10</f>
-        <v/>
-      </c>
-      <c r="N36" s="35">
-        <f>'Equity Schedule'!N10</f>
-        <v/>
-      </c>
-      <c r="O36" s="35">
-        <f>'Equity Schedule'!O10</f>
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Total Non-Current Liabilities</t>
+        </is>
+      </c>
+      <c r="B36" s="22">
+        <f>B34+B35</f>
+        <v/>
+      </c>
+      <c r="C36" s="22">
+        <f>C34+C35</f>
+        <v/>
+      </c>
+      <c r="D36" s="22">
+        <f>D34+D35</f>
+        <v/>
+      </c>
+      <c r="E36" s="22">
+        <f>E34+E35</f>
+        <v/>
+      </c>
+      <c r="F36" s="22">
+        <f>F34+F35</f>
+        <v/>
+      </c>
+      <c r="G36" s="22">
+        <f>G34+G35</f>
+        <v/>
+      </c>
+      <c r="H36" s="22">
+        <f>H34+H35</f>
+        <v/>
+      </c>
+      <c r="I36" s="22">
+        <f>I34+I35</f>
+        <v/>
+      </c>
+      <c r="J36" s="22">
+        <f>J34+J35</f>
+        <v/>
+      </c>
+      <c r="K36" s="22">
+        <f>K34+K35</f>
+        <v/>
+      </c>
+      <c r="L36" s="22">
+        <f>L34+L35</f>
+        <v/>
+      </c>
+      <c r="M36" s="22">
+        <f>M34+M35</f>
+        <v/>
+      </c>
+      <c r="N36" s="22">
+        <f>N34+N35</f>
+        <v/>
+      </c>
+      <c r="O36" s="22">
+        <f>O34+O35</f>
         <v/>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>Borrowings (incl. leases)</t>
-        </is>
-      </c>
-      <c r="H37" s="35">
-        <f>'Historical Financial Statements'!H35</f>
-        <v/>
+          <t xml:space="preserve">   ST borrowings</t>
+        </is>
+      </c>
+      <c r="B37" s="21" t="n">
+        <v>3302</v>
+      </c>
+      <c r="C37" s="21" t="n">
+        <v>3218</v>
+      </c>
+      <c r="D37" s="21" t="n">
+        <v>3140</v>
+      </c>
+      <c r="E37" s="21" t="n">
+        <v>3545</v>
+      </c>
+      <c r="F37" s="21" t="n">
+        <v>5756</v>
+      </c>
+      <c r="G37" s="21" t="n">
+        <v>5860</v>
+      </c>
+      <c r="H37" s="21" t="n">
+        <v>5322</v>
       </c>
       <c r="I37" s="35">
-        <f>'Debt Schedule'!I9</f>
+        <f>'Debt Schedule'!I9-I34</f>
         <v/>
       </c>
       <c r="J37" s="35">
-        <f>'Debt Schedule'!J9</f>
+        <f>'Debt Schedule'!J9-J34</f>
         <v/>
       </c>
       <c r="K37" s="35">
-        <f>'Debt Schedule'!K9</f>
+        <f>'Debt Schedule'!K9-K34</f>
         <v/>
       </c>
       <c r="L37" s="35">
-        <f>'Debt Schedule'!L9</f>
+        <f>'Debt Schedule'!L9-L34</f>
         <v/>
       </c>
       <c r="M37" s="35">
-        <f>'Debt Schedule'!M9</f>
+        <f>'Debt Schedule'!M9-M34</f>
         <v/>
       </c>
       <c r="N37" s="35">
-        <f>'Debt Schedule'!N9</f>
+        <f>'Debt Schedule'!N9-N34</f>
         <v/>
       </c>
       <c r="O37" s="35">
-        <f>'Debt Schedule'!O9</f>
+        <f>'Debt Schedule'!O9-O34</f>
         <v/>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Trade payables</t>
-        </is>
-      </c>
-      <c r="H38" s="35">
-        <f>'Working Capital Schedule'!H13</f>
-        <v/>
+          <t xml:space="preserve">   Trade Payables</t>
+        </is>
+      </c>
+      <c r="B38" s="21" t="n">
+        <v>17750</v>
+      </c>
+      <c r="C38" s="21" t="n">
+        <v>15673</v>
+      </c>
+      <c r="D38" s="21" t="n">
+        <v>16248</v>
+      </c>
+      <c r="E38" s="21" t="n">
+        <v>21099</v>
+      </c>
+      <c r="F38" s="21" t="n">
+        <v>17147</v>
+      </c>
+      <c r="G38" s="21" t="n">
+        <v>19115</v>
+      </c>
+      <c r="H38" s="21" t="n">
+        <v>14386</v>
       </c>
       <c r="I38" s="35">
         <f>'Working Capital Schedule'!I13</f>
@@ -5650,157 +5724,1058 @@
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Contract liabilities / advances</t>
-        </is>
-      </c>
-      <c r="H39" s="35">
-        <f>'Working Capital Schedule'!H14</f>
-        <v/>
+          <t xml:space="preserve">   Other Current Liabilities (provisions, advances)</t>
+        </is>
+      </c>
+      <c r="B39" s="21" t="n">
+        <v>3800</v>
+      </c>
+      <c r="C39" s="21" t="n">
+        <v>4352</v>
+      </c>
+      <c r="D39" s="21" t="n">
+        <v>4406</v>
+      </c>
+      <c r="E39" s="21" t="n">
+        <v>2733</v>
+      </c>
+      <c r="F39" s="21" t="n">
+        <v>4842</v>
+      </c>
+      <c r="G39" s="21" t="n">
+        <v>10497</v>
+      </c>
+      <c r="H39" s="21" t="n">
+        <v>21466</v>
       </c>
       <c r="I39" s="35">
-        <f>'Working Capital Schedule'!I14</f>
+        <f>'Working Capital Schedule'!I14+'Working Capital Schedule'!I15-I35</f>
         <v/>
       </c>
       <c r="J39" s="35">
-        <f>'Working Capital Schedule'!J14</f>
+        <f>'Working Capital Schedule'!J14+'Working Capital Schedule'!J15-J35</f>
         <v/>
       </c>
       <c r="K39" s="35">
-        <f>'Working Capital Schedule'!K14</f>
+        <f>'Working Capital Schedule'!K14+'Working Capital Schedule'!K15-K35</f>
         <v/>
       </c>
       <c r="L39" s="35">
-        <f>'Working Capital Schedule'!L14</f>
+        <f>'Working Capital Schedule'!L14+'Working Capital Schedule'!L15-L35</f>
         <v/>
       </c>
       <c r="M39" s="35">
-        <f>'Working Capital Schedule'!M14</f>
+        <f>'Working Capital Schedule'!M14+'Working Capital Schedule'!M15-M35</f>
         <v/>
       </c>
       <c r="N39" s="35">
-        <f>'Working Capital Schedule'!N14</f>
+        <f>'Working Capital Schedule'!N14+'Working Capital Schedule'!N15-N35</f>
         <v/>
       </c>
       <c r="O39" s="35">
-        <f>'Working Capital Schedule'!O14</f>
+        <f>'Working Capital Schedule'!O14+'Working Capital Schedule'!O15-O35</f>
         <v/>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Provisions &amp; other liabilities</t>
-        </is>
-      </c>
-      <c r="H40" s="35">
-        <f>'Working Capital Schedule'!H15</f>
-        <v/>
-      </c>
-      <c r="I40" s="35">
-        <f>'Working Capital Schedule'!I15</f>
-        <v/>
-      </c>
-      <c r="J40" s="35">
-        <f>'Working Capital Schedule'!J15</f>
-        <v/>
-      </c>
-      <c r="K40" s="35">
-        <f>'Working Capital Schedule'!K15</f>
-        <v/>
-      </c>
-      <c r="L40" s="35">
-        <f>'Working Capital Schedule'!L15</f>
-        <v/>
-      </c>
-      <c r="M40" s="35">
-        <f>'Working Capital Schedule'!M15</f>
-        <v/>
-      </c>
-      <c r="N40" s="35">
-        <f>'Working Capital Schedule'!N15</f>
-        <v/>
-      </c>
-      <c r="O40" s="35">
-        <f>'Working Capital Schedule'!O15</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="4" t="inlineStr">
-        <is>
-          <t>TOTAL EQUITY &amp; LIABILITIES</t>
-        </is>
-      </c>
-      <c r="H41" s="25">
-        <f>SUM(H35:H40)</f>
-        <v/>
-      </c>
-      <c r="I41" s="25">
-        <f>SUM(I35:I40)</f>
-        <v/>
-      </c>
-      <c r="J41" s="25">
-        <f>SUM(J35:J40)</f>
-        <v/>
-      </c>
-      <c r="K41" s="25">
-        <f>SUM(K35:K40)</f>
-        <v/>
-      </c>
-      <c r="L41" s="25">
-        <f>SUM(L35:L40)</f>
-        <v/>
-      </c>
-      <c r="M41" s="25">
-        <f>SUM(M35:M40)</f>
-        <v/>
-      </c>
-      <c r="N41" s="25">
-        <f>SUM(N35:N40)</f>
-        <v/>
-      </c>
-      <c r="O41" s="25">
-        <f>SUM(O35:O40)</f>
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Total Liabilities</t>
+        </is>
+      </c>
+      <c r="B40" s="22">
+        <f>B36+B37+B38+B39</f>
+        <v/>
+      </c>
+      <c r="C40" s="22">
+        <f>C36+C37+C38+C39</f>
+        <v/>
+      </c>
+      <c r="D40" s="22">
+        <f>D36+D37+D38+D39</f>
+        <v/>
+      </c>
+      <c r="E40" s="22">
+        <f>E36+E37+E38+E39</f>
+        <v/>
+      </c>
+      <c r="F40" s="22">
+        <f>F36+F37+F38+F39</f>
+        <v/>
+      </c>
+      <c r="G40" s="22">
+        <f>G36+G37+G38+G39</f>
+        <v/>
+      </c>
+      <c r="H40" s="22">
+        <f>H36+H37+H38+H39</f>
+        <v/>
+      </c>
+      <c r="I40" s="22">
+        <f>I36+I37+I38+I39</f>
+        <v/>
+      </c>
+      <c r="J40" s="22">
+        <f>J36+J37+J38+J39</f>
+        <v/>
+      </c>
+      <c r="K40" s="22">
+        <f>K36+K37+K38+K39</f>
+        <v/>
+      </c>
+      <c r="L40" s="22">
+        <f>L36+L37+L38+L39</f>
+        <v/>
+      </c>
+      <c r="M40" s="22">
+        <f>M36+M37+M38+M39</f>
+        <v/>
+      </c>
+      <c r="N40" s="22">
+        <f>N36+N37+N38+N39</f>
+        <v/>
+      </c>
+      <c r="O40" s="22">
+        <f>O36+O37+O38+O39</f>
         <v/>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
+          <t>Total Equity &amp; Liabilities</t>
+        </is>
+      </c>
+      <c r="B42" s="25">
+        <f>B30+B40</f>
+        <v/>
+      </c>
+      <c r="C42" s="25">
+        <f>C30+C40</f>
+        <v/>
+      </c>
+      <c r="D42" s="25">
+        <f>D30+D40</f>
+        <v/>
+      </c>
+      <c r="E42" s="25">
+        <f>E30+E40</f>
+        <v/>
+      </c>
+      <c r="F42" s="25">
+        <f>F30+F40</f>
+        <v/>
+      </c>
+      <c r="G42" s="25">
+        <f>G30+G40</f>
+        <v/>
+      </c>
+      <c r="H42" s="25">
+        <f>H30+H40</f>
+        <v/>
+      </c>
+      <c r="I42" s="25">
+        <f>I30+I40</f>
+        <v/>
+      </c>
+      <c r="J42" s="25">
+        <f>J30+J40</f>
+        <v/>
+      </c>
+      <c r="K42" s="25">
+        <f>K30+K40</f>
+        <v/>
+      </c>
+      <c r="L42" s="25">
+        <f>L30+L40</f>
+        <v/>
+      </c>
+      <c r="M42" s="25">
+        <f>M30+M40</f>
+        <v/>
+      </c>
+      <c r="N42" s="25">
+        <f>N30+N40</f>
+        <v/>
+      </c>
+      <c r="O42" s="25">
+        <f>O30+O40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="40" t="inlineStr">
+        <is>
+          <t>Assets</t>
+        </is>
+      </c>
+      <c r="B44" s="41" t="n"/>
+      <c r="C44" s="41" t="n"/>
+      <c r="D44" s="41" t="n"/>
+      <c r="E44" s="41" t="n"/>
+      <c r="F44" s="41" t="n"/>
+      <c r="G44" s="41" t="n"/>
+      <c r="H44" s="41" t="n"/>
+      <c r="I44" s="41" t="n"/>
+      <c r="J44" s="41" t="n"/>
+      <c r="K44" s="41" t="n"/>
+      <c r="L44" s="41" t="n"/>
+      <c r="M44" s="41" t="n"/>
+      <c r="N44" s="41" t="n"/>
+      <c r="O44" s="41" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Non-Current Assets</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>Fixed Assets</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Property Plant &amp; Equip</t>
+        </is>
+      </c>
+      <c r="B47" s="21" t="n">
+        <v>2817</v>
+      </c>
+      <c r="C47" s="21" t="n">
+        <v>2491</v>
+      </c>
+      <c r="D47" s="21" t="n">
+        <v>2398</v>
+      </c>
+      <c r="E47" s="21" t="n">
+        <v>2476</v>
+      </c>
+      <c r="F47" s="21" t="n">
+        <v>2574</v>
+      </c>
+      <c r="G47" s="21" t="n">
+        <v>2947</v>
+      </c>
+      <c r="H47" s="21" t="n">
+        <v>3094</v>
+      </c>
+      <c r="I47" s="35">
+        <f>'Fixed Asset Schedule'!I10</f>
+        <v/>
+      </c>
+      <c r="J47" s="35">
+        <f>'Fixed Asset Schedule'!J10</f>
+        <v/>
+      </c>
+      <c r="K47" s="35">
+        <f>'Fixed Asset Schedule'!K10</f>
+        <v/>
+      </c>
+      <c r="L47" s="35">
+        <f>'Fixed Asset Schedule'!L10</f>
+        <v/>
+      </c>
+      <c r="M47" s="35">
+        <f>'Fixed Asset Schedule'!M10</f>
+        <v/>
+      </c>
+      <c r="N47" s="35">
+        <f>'Fixed Asset Schedule'!N10</f>
+        <v/>
+      </c>
+      <c r="O47" s="35">
+        <f>'Fixed Asset Schedule'!O10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Capital Work in Progress</t>
+        </is>
+      </c>
+      <c r="B48" s="21" t="n">
+        <v>314</v>
+      </c>
+      <c r="C48" s="21" t="n">
+        <v>420</v>
+      </c>
+      <c r="D48" s="21" t="n">
+        <v>431</v>
+      </c>
+      <c r="E48" s="21" t="n">
+        <v>354</v>
+      </c>
+      <c r="F48" s="21" t="n">
+        <v>308</v>
+      </c>
+      <c r="G48" s="21" t="n">
+        <v>195</v>
+      </c>
+      <c r="H48" s="21" t="n">
+        <v>399</v>
+      </c>
+      <c r="I48" s="35">
+        <f>'Assumptions'!I21</f>
+        <v/>
+      </c>
+      <c r="J48" s="35">
+        <f>'Assumptions'!J21</f>
+        <v/>
+      </c>
+      <c r="K48" s="35">
+        <f>'Assumptions'!K21</f>
+        <v/>
+      </c>
+      <c r="L48" s="35">
+        <f>'Assumptions'!L21</f>
+        <v/>
+      </c>
+      <c r="M48" s="35">
+        <f>'Assumptions'!M21</f>
+        <v/>
+      </c>
+      <c r="N48" s="35">
+        <f>'Assumptions'!N21</f>
+        <v/>
+      </c>
+      <c r="O48" s="35">
+        <f>'Assumptions'!O21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Investments</t>
+        </is>
+      </c>
+      <c r="B49" s="21" t="n">
+        <v>162</v>
+      </c>
+      <c r="C49" s="21" t="n">
+        <v>185</v>
+      </c>
+      <c r="D49" s="21" t="n">
+        <v>205</v>
+      </c>
+      <c r="E49" s="21" t="n">
+        <v>235</v>
+      </c>
+      <c r="F49" s="21" t="n">
+        <v>256</v>
+      </c>
+      <c r="G49" s="21" t="n">
+        <v>276</v>
+      </c>
+      <c r="H49" s="21" t="n">
+        <v>302</v>
+      </c>
+      <c r="I49" s="35">
+        <f>'Assumptions'!I22</f>
+        <v/>
+      </c>
+      <c r="J49" s="35">
+        <f>'Assumptions'!J22</f>
+        <v/>
+      </c>
+      <c r="K49" s="35">
+        <f>'Assumptions'!K22</f>
+        <v/>
+      </c>
+      <c r="L49" s="35">
+        <f>'Assumptions'!L22</f>
+        <v/>
+      </c>
+      <c r="M49" s="35">
+        <f>'Assumptions'!M22</f>
+        <v/>
+      </c>
+      <c r="N49" s="35">
+        <f>'Assumptions'!N22</f>
+        <v/>
+      </c>
+      <c r="O49" s="35">
+        <f>'Assumptions'!O22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Total Fixed Assets</t>
+        </is>
+      </c>
+      <c r="B50" s="22">
+        <f>SUM(B47:B49)</f>
+        <v/>
+      </c>
+      <c r="C50" s="22">
+        <f>SUM(C47:C49)</f>
+        <v/>
+      </c>
+      <c r="D50" s="22">
+        <f>SUM(D47:D49)</f>
+        <v/>
+      </c>
+      <c r="E50" s="22">
+        <f>SUM(E47:E49)</f>
+        <v/>
+      </c>
+      <c r="F50" s="22">
+        <f>SUM(F47:F49)</f>
+        <v/>
+      </c>
+      <c r="G50" s="22">
+        <f>SUM(G47:G49)</f>
+        <v/>
+      </c>
+      <c r="H50" s="22">
+        <f>SUM(H47:H49)</f>
+        <v/>
+      </c>
+      <c r="I50" s="22">
+        <f>SUM(I47:I49)</f>
+        <v/>
+      </c>
+      <c r="J50" s="22">
+        <f>SUM(J47:J49)</f>
+        <v/>
+      </c>
+      <c r="K50" s="22">
+        <f>SUM(K47:K49)</f>
+        <v/>
+      </c>
+      <c r="L50" s="22">
+        <f>SUM(L47:L49)</f>
+        <v/>
+      </c>
+      <c r="M50" s="22">
+        <f>SUM(M47:M49)</f>
+        <v/>
+      </c>
+      <c r="N50" s="22">
+        <f>SUM(N47:N49)</f>
+        <v/>
+      </c>
+      <c r="O50" s="22">
+        <f>SUM(O47:O49)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Other Non Current Assets</t>
+        </is>
+      </c>
+      <c r="B51" s="21" t="n">
+        <v>14000</v>
+      </c>
+      <c r="C51" s="21" t="n">
+        <v>13500</v>
+      </c>
+      <c r="D51" s="21" t="n">
+        <v>13000</v>
+      </c>
+      <c r="E51" s="21" t="n">
+        <v>13500</v>
+      </c>
+      <c r="F51" s="21" t="n">
+        <v>14000</v>
+      </c>
+      <c r="G51" s="21" t="n">
+        <v>14500</v>
+      </c>
+      <c r="H51" s="21" t="n">
+        <v>15000</v>
+      </c>
+      <c r="I51" s="35">
+        <f>'Assumptions'!I29</f>
+        <v/>
+      </c>
+      <c r="J51" s="35">
+        <f>'Assumptions'!J29</f>
+        <v/>
+      </c>
+      <c r="K51" s="35">
+        <f>'Assumptions'!K29</f>
+        <v/>
+      </c>
+      <c r="L51" s="35">
+        <f>'Assumptions'!L29</f>
+        <v/>
+      </c>
+      <c r="M51" s="35">
+        <f>'Assumptions'!M29</f>
+        <v/>
+      </c>
+      <c r="N51" s="35">
+        <f>'Assumptions'!N29</f>
+        <v/>
+      </c>
+      <c r="O51" s="35">
+        <f>'Assumptions'!O29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Total Non Current Assets</t>
+        </is>
+      </c>
+      <c r="B52" s="22">
+        <f>B50+B51</f>
+        <v/>
+      </c>
+      <c r="C52" s="22">
+        <f>C50+C51</f>
+        <v/>
+      </c>
+      <c r="D52" s="22">
+        <f>D50+D51</f>
+        <v/>
+      </c>
+      <c r="E52" s="22">
+        <f>E50+E51</f>
+        <v/>
+      </c>
+      <c r="F52" s="22">
+        <f>F50+F51</f>
+        <v/>
+      </c>
+      <c r="G52" s="22">
+        <f>G50+G51</f>
+        <v/>
+      </c>
+      <c r="H52" s="22">
+        <f>H50+H51</f>
+        <v/>
+      </c>
+      <c r="I52" s="22">
+        <f>I50+I51</f>
+        <v/>
+      </c>
+      <c r="J52" s="22">
+        <f>J50+J51</f>
+        <v/>
+      </c>
+      <c r="K52" s="22">
+        <f>K50+K51</f>
+        <v/>
+      </c>
+      <c r="L52" s="22">
+        <f>L50+L51</f>
+        <v/>
+      </c>
+      <c r="M52" s="22">
+        <f>M50+M51</f>
+        <v/>
+      </c>
+      <c r="N52" s="22">
+        <f>N50+N51</f>
+        <v/>
+      </c>
+      <c r="O52" s="22">
+        <f>O50+O51</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>Current Assets</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Accounts Receivables</t>
+        </is>
+      </c>
+      <c r="B55" s="21" t="n">
+        <v>7115</v>
+      </c>
+      <c r="C55" s="21" t="n">
+        <v>4030</v>
+      </c>
+      <c r="D55" s="21" t="n">
+        <v>3022</v>
+      </c>
+      <c r="E55" s="21" t="n">
+        <v>3137</v>
+      </c>
+      <c r="F55" s="21" t="n">
+        <v>4779</v>
+      </c>
+      <c r="G55" s="21" t="n">
+        <v>5901</v>
+      </c>
+      <c r="H55" s="21" t="n">
+        <v>6757</v>
+      </c>
+      <c r="I55" s="35">
+        <f>'Working Capital Schedule'!I8</f>
+        <v/>
+      </c>
+      <c r="J55" s="35">
+        <f>'Working Capital Schedule'!J8</f>
+        <v/>
+      </c>
+      <c r="K55" s="35">
+        <f>'Working Capital Schedule'!K8</f>
+        <v/>
+      </c>
+      <c r="L55" s="35">
+        <f>'Working Capital Schedule'!L8</f>
+        <v/>
+      </c>
+      <c r="M55" s="35">
+        <f>'Working Capital Schedule'!M8</f>
+        <v/>
+      </c>
+      <c r="N55" s="35">
+        <f>'Working Capital Schedule'!N8</f>
+        <v/>
+      </c>
+      <c r="O55" s="35">
+        <f>'Working Capital Schedule'!O8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Inventories</t>
+        </is>
+      </c>
+      <c r="B56" s="21" t="n">
+        <v>18994</v>
+      </c>
+      <c r="C56" s="21" t="n">
+        <v>18573</v>
+      </c>
+      <c r="D56" s="21" t="n">
+        <v>15301</v>
+      </c>
+      <c r="E56" s="21" t="n">
+        <v>15962</v>
+      </c>
+      <c r="F56" s="21" t="n">
+        <v>16069</v>
+      </c>
+      <c r="G56" s="21" t="n">
+        <v>21331</v>
+      </c>
+      <c r="H56" s="21" t="n">
+        <v>18260</v>
+      </c>
+      <c r="I56" s="35">
+        <f>'Working Capital Schedule'!I9</f>
+        <v/>
+      </c>
+      <c r="J56" s="35">
+        <f>'Working Capital Schedule'!J9</f>
+        <v/>
+      </c>
+      <c r="K56" s="35">
+        <f>'Working Capital Schedule'!K9</f>
+        <v/>
+      </c>
+      <c r="L56" s="35">
+        <f>'Working Capital Schedule'!L9</f>
+        <v/>
+      </c>
+      <c r="M56" s="35">
+        <f>'Working Capital Schedule'!M9</f>
+        <v/>
+      </c>
+      <c r="N56" s="35">
+        <f>'Working Capital Schedule'!N9</f>
+        <v/>
+      </c>
+      <c r="O56" s="35">
+        <f>'Working Capital Schedule'!O9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Other Current Assets</t>
+        </is>
+      </c>
+      <c r="B57" s="21" t="n">
+        <v>9927</v>
+      </c>
+      <c r="C57" s="21" t="n">
+        <v>9676</v>
+      </c>
+      <c r="D57" s="21" t="n">
+        <v>16336</v>
+      </c>
+      <c r="E57" s="21" t="n">
+        <v>14874</v>
+      </c>
+      <c r="F57" s="21" t="n">
+        <v>14397</v>
+      </c>
+      <c r="G57" s="21" t="n">
+        <v>17695</v>
+      </c>
+      <c r="H57" s="21" t="n">
+        <v>25373</v>
+      </c>
+      <c r="I57" s="35">
+        <f>'Working Capital Schedule'!I10+'Working Capital Schedule'!I11-I51</f>
+        <v/>
+      </c>
+      <c r="J57" s="35">
+        <f>'Working Capital Schedule'!J10+'Working Capital Schedule'!J11-J51</f>
+        <v/>
+      </c>
+      <c r="K57" s="35">
+        <f>'Working Capital Schedule'!K10+'Working Capital Schedule'!K11-K51</f>
+        <v/>
+      </c>
+      <c r="L57" s="35">
+        <f>'Working Capital Schedule'!L10+'Working Capital Schedule'!L11-L51</f>
+        <v/>
+      </c>
+      <c r="M57" s="35">
+        <f>'Working Capital Schedule'!M10+'Working Capital Schedule'!M11-M51</f>
+        <v/>
+      </c>
+      <c r="N57" s="35">
+        <f>'Working Capital Schedule'!N10+'Working Capital Schedule'!N11-N51</f>
+        <v/>
+      </c>
+      <c r="O57" s="35">
+        <f>'Working Capital Schedule'!O10+'Working Capital Schedule'!O11-O51</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Cash Balance (Incl. Bank and Current Invest)</t>
+        </is>
+      </c>
+      <c r="B58" s="21" t="n">
+        <v>6961</v>
+      </c>
+      <c r="C58" s="21" t="n">
+        <v>7084</v>
+      </c>
+      <c r="D58" s="21" t="n">
+        <v>6297</v>
+      </c>
+      <c r="E58" s="21" t="n">
+        <v>7126</v>
+      </c>
+      <c r="F58" s="21" t="n">
+        <v>7400</v>
+      </c>
+      <c r="G58" s="21" t="n">
+        <v>6004</v>
+      </c>
+      <c r="H58" s="21" t="n">
+        <v>7000</v>
+      </c>
+      <c r="I58" s="35">
+        <f>'Cash Flow Statement'!I25</f>
+        <v/>
+      </c>
+      <c r="J58" s="35">
+        <f>'Cash Flow Statement'!J25</f>
+        <v/>
+      </c>
+      <c r="K58" s="35">
+        <f>'Cash Flow Statement'!K25</f>
+        <v/>
+      </c>
+      <c r="L58" s="35">
+        <f>'Cash Flow Statement'!L25</f>
+        <v/>
+      </c>
+      <c r="M58" s="35">
+        <f>'Cash Flow Statement'!M25</f>
+        <v/>
+      </c>
+      <c r="N58" s="35">
+        <f>'Cash Flow Statement'!N25</f>
+        <v/>
+      </c>
+      <c r="O58" s="35">
+        <f>'Cash Flow Statement'!O25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="4" t="inlineStr">
+        <is>
+          <t>Total Current Assets</t>
+        </is>
+      </c>
+      <c r="B59" s="22">
+        <f>SUM(B55:B58)</f>
+        <v/>
+      </c>
+      <c r="C59" s="22">
+        <f>SUM(C55:C58)</f>
+        <v/>
+      </c>
+      <c r="D59" s="22">
+        <f>SUM(D55:D58)</f>
+        <v/>
+      </c>
+      <c r="E59" s="22">
+        <f>SUM(E55:E58)</f>
+        <v/>
+      </c>
+      <c r="F59" s="22">
+        <f>SUM(F55:F58)</f>
+        <v/>
+      </c>
+      <c r="G59" s="22">
+        <f>SUM(G55:G58)</f>
+        <v/>
+      </c>
+      <c r="H59" s="22">
+        <f>SUM(H55:H58)</f>
+        <v/>
+      </c>
+      <c r="I59" s="22">
+        <f>SUM(I55:I58)</f>
+        <v/>
+      </c>
+      <c r="J59" s="22">
+        <f>SUM(J55:J58)</f>
+        <v/>
+      </c>
+      <c r="K59" s="22">
+        <f>SUM(K55:K58)</f>
+        <v/>
+      </c>
+      <c r="L59" s="22">
+        <f>SUM(L55:L58)</f>
+        <v/>
+      </c>
+      <c r="M59" s="22">
+        <f>SUM(M55:M58)</f>
+        <v/>
+      </c>
+      <c r="N59" s="22">
+        <f>SUM(N55:N58)</f>
+        <v/>
+      </c>
+      <c r="O59" s="22">
+        <f>SUM(O55:O58)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="4" t="inlineStr">
+        <is>
+          <t>Total Assets</t>
+        </is>
+      </c>
+      <c r="B61" s="25">
+        <f>B52+B59</f>
+        <v/>
+      </c>
+      <c r="C61" s="25">
+        <f>C52+C59</f>
+        <v/>
+      </c>
+      <c r="D61" s="25">
+        <f>D52+D59</f>
+        <v/>
+      </c>
+      <c r="E61" s="25">
+        <f>E52+E59</f>
+        <v/>
+      </c>
+      <c r="F61" s="25">
+        <f>F52+F59</f>
+        <v/>
+      </c>
+      <c r="G61" s="25">
+        <f>G52+G59</f>
+        <v/>
+      </c>
+      <c r="H61" s="25">
+        <f>H52+H59</f>
+        <v/>
+      </c>
+      <c r="I61" s="25">
+        <f>I52+I59</f>
+        <v/>
+      </c>
+      <c r="J61" s="25">
+        <f>J52+J59</f>
+        <v/>
+      </c>
+      <c r="K61" s="25">
+        <f>K52+K59</f>
+        <v/>
+      </c>
+      <c r="L61" s="25">
+        <f>L52+L59</f>
+        <v/>
+      </c>
+      <c r="M61" s="25">
+        <f>M52+M59</f>
+        <v/>
+      </c>
+      <c r="N61" s="25">
+        <f>N52+N59</f>
+        <v/>
+      </c>
+      <c r="O61" s="25">
+        <f>O52+O59</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="4" t="inlineStr">
+        <is>
           <t>Balance check (TA - TE&amp;L)</t>
         </is>
       </c>
-      <c r="H42" s="24">
-        <f>H34-H41</f>
-        <v/>
-      </c>
-      <c r="I42" s="24">
-        <f>I34-I41</f>
-        <v/>
-      </c>
-      <c r="J42" s="24">
-        <f>J34-J41</f>
-        <v/>
-      </c>
-      <c r="K42" s="24">
-        <f>K34-K41</f>
-        <v/>
-      </c>
-      <c r="L42" s="24">
-        <f>L34-L41</f>
-        <v/>
-      </c>
-      <c r="M42" s="24">
-        <f>M34-M41</f>
-        <v/>
-      </c>
-      <c r="N42" s="24">
-        <f>N34-N41</f>
-        <v/>
-      </c>
-      <c r="O42" s="24">
-        <f>O34-O41</f>
-        <v/>
+      <c r="B62" s="24">
+        <f>B61-B42</f>
+        <v/>
+      </c>
+      <c r="C62" s="24">
+        <f>C61-C42</f>
+        <v/>
+      </c>
+      <c r="D62" s="24">
+        <f>D61-D42</f>
+        <v/>
+      </c>
+      <c r="E62" s="24">
+        <f>E61-E42</f>
+        <v/>
+      </c>
+      <c r="F62" s="24">
+        <f>F61-F42</f>
+        <v/>
+      </c>
+      <c r="G62" s="24">
+        <f>G61-G42</f>
+        <v/>
+      </c>
+      <c r="H62" s="24">
+        <f>H61-H42</f>
+        <v/>
+      </c>
+      <c r="I62" s="24">
+        <f>I61-I42</f>
+        <v/>
+      </c>
+      <c r="J62" s="24">
+        <f>J61-J42</f>
+        <v/>
+      </c>
+      <c r="K62" s="24">
+        <f>K61-K42</f>
+        <v/>
+      </c>
+      <c r="L62" s="24">
+        <f>L61-L42</f>
+        <v/>
+      </c>
+      <c r="M62" s="24">
+        <f>M61-M42</f>
+        <v/>
+      </c>
+      <c r="N62" s="24">
+        <f>N61-N42</f>
+        <v/>
+      </c>
+      <c r="O62" s="24">
+        <f>O61-O42</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="7" t="inlineStr">
+        <is>
+          <t>Memo: total borrowings (LT+ST)</t>
+        </is>
+      </c>
+      <c r="B63" s="24">
+        <f>B34+B37</f>
+        <v/>
+      </c>
+      <c r="C63" s="24">
+        <f>C34+C37</f>
+        <v/>
+      </c>
+      <c r="D63" s="24">
+        <f>D34+D37</f>
+        <v/>
+      </c>
+      <c r="E63" s="24">
+        <f>E34+E37</f>
+        <v/>
+      </c>
+      <c r="F63" s="24">
+        <f>F34+F37</f>
+        <v/>
+      </c>
+      <c r="G63" s="24">
+        <f>G34+G37</f>
+        <v/>
+      </c>
+      <c r="H63" s="24">
+        <f>H34+H37</f>
+        <v/>
+      </c>
+      <c r="I63" s="24">
+        <f>I34+I37</f>
+        <v/>
+      </c>
+      <c r="J63" s="24">
+        <f>J34+J37</f>
+        <v/>
+      </c>
+      <c r="K63" s="24">
+        <f>K34+K37</f>
+        <v/>
+      </c>
+      <c r="L63" s="24">
+        <f>L34+L37</f>
+        <v/>
+      </c>
+      <c r="M63" s="24">
+        <f>M34+M37</f>
+        <v/>
+      </c>
+      <c r="N63" s="24">
+        <f>N34+N37</f>
+        <v/>
+      </c>
+      <c r="O63" s="24">
+        <f>O34+O37</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="27" t="inlineStr">
+        <is>
+          <t>Historical balance-sheet sub-lines are analyst estimates anchored exactly to reported totals (debtor/inventory/payable days; cash rolled from reported net cash flow).</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -6319,35 +7294,35 @@
         <v/>
       </c>
       <c r="H13" s="28">
-        <f>'Forecast Financial Statements'!H20/((('Forecast Financial Statements'!H35+'Forecast Financial Statements'!H36)+('Historical Financial Statements'!G33+'Historical Financial Statements'!G34))/2)</f>
+        <f>'Forecast Financial Statements'!H20/((('Forecast Financial Statements'!H28+'Forecast Financial Statements'!H29)+('Historical Financial Statements'!G33+'Historical Financial Statements'!G34))/2)</f>
         <v/>
       </c>
       <c r="I13" s="28">
-        <f>'Forecast Financial Statements'!I20/((('Forecast Financial Statements'!I35+'Forecast Financial Statements'!I36)+('Forecast Financial Statements'!H35+'Forecast Financial Statements'!H36))/2)</f>
+        <f>'Forecast Financial Statements'!I20/((('Forecast Financial Statements'!I28+'Forecast Financial Statements'!I29)+('Forecast Financial Statements'!H28+'Forecast Financial Statements'!H29))/2)</f>
         <v/>
       </c>
       <c r="J13" s="28">
-        <f>'Forecast Financial Statements'!J20/((('Forecast Financial Statements'!J35+'Forecast Financial Statements'!J36)+('Forecast Financial Statements'!I35+'Forecast Financial Statements'!I36))/2)</f>
+        <f>'Forecast Financial Statements'!J20/((('Forecast Financial Statements'!J28+'Forecast Financial Statements'!J29)+('Forecast Financial Statements'!I28+'Forecast Financial Statements'!I29))/2)</f>
         <v/>
       </c>
       <c r="K13" s="28">
-        <f>'Forecast Financial Statements'!K20/((('Forecast Financial Statements'!K35+'Forecast Financial Statements'!K36)+('Forecast Financial Statements'!J35+'Forecast Financial Statements'!J36))/2)</f>
+        <f>'Forecast Financial Statements'!K20/((('Forecast Financial Statements'!K28+'Forecast Financial Statements'!K29)+('Forecast Financial Statements'!J28+'Forecast Financial Statements'!J29))/2)</f>
         <v/>
       </c>
       <c r="L13" s="28">
-        <f>'Forecast Financial Statements'!L20/((('Forecast Financial Statements'!L35+'Forecast Financial Statements'!L36)+('Forecast Financial Statements'!K35+'Forecast Financial Statements'!K36))/2)</f>
+        <f>'Forecast Financial Statements'!L20/((('Forecast Financial Statements'!L28+'Forecast Financial Statements'!L29)+('Forecast Financial Statements'!K28+'Forecast Financial Statements'!K29))/2)</f>
         <v/>
       </c>
       <c r="M13" s="28">
-        <f>'Forecast Financial Statements'!M20/((('Forecast Financial Statements'!M35+'Forecast Financial Statements'!M36)+('Forecast Financial Statements'!L35+'Forecast Financial Statements'!L36))/2)</f>
+        <f>'Forecast Financial Statements'!M20/((('Forecast Financial Statements'!M28+'Forecast Financial Statements'!M29)+('Forecast Financial Statements'!L28+'Forecast Financial Statements'!L29))/2)</f>
         <v/>
       </c>
       <c r="N13" s="28">
-        <f>'Forecast Financial Statements'!N20/((('Forecast Financial Statements'!N35+'Forecast Financial Statements'!N36)+('Forecast Financial Statements'!M35+'Forecast Financial Statements'!M36))/2)</f>
+        <f>'Forecast Financial Statements'!N20/((('Forecast Financial Statements'!N28+'Forecast Financial Statements'!N29)+('Forecast Financial Statements'!M28+'Forecast Financial Statements'!M29))/2)</f>
         <v/>
       </c>
       <c r="O13" s="28">
-        <f>'Forecast Financial Statements'!O20/((('Forecast Financial Statements'!O35+'Forecast Financial Statements'!O36)+('Forecast Financial Statements'!N35+'Forecast Financial Statements'!N36))/2)</f>
+        <f>'Forecast Financial Statements'!O20/((('Forecast Financial Statements'!O28+'Forecast Financial Statements'!O29)+('Forecast Financial Statements'!N28+'Forecast Financial Statements'!N29))/2)</f>
         <v/>
       </c>
     </row>
@@ -6382,35 +7357,35 @@
         <v/>
       </c>
       <c r="H14" s="28">
-        <f>'Forecast Financial Statements'!H14/(('Forecast Financial Statements'!H35+'Forecast Financial Statements'!H36)+'Forecast Financial Statements'!H37)</f>
+        <f>'Forecast Financial Statements'!H14/(('Forecast Financial Statements'!H28+'Forecast Financial Statements'!H29)+'Forecast Financial Statements'!H63)</f>
         <v/>
       </c>
       <c r="I14" s="28">
-        <f>'Forecast Financial Statements'!I14/(('Forecast Financial Statements'!I35+'Forecast Financial Statements'!I36)+'Forecast Financial Statements'!I37)</f>
+        <f>'Forecast Financial Statements'!I14/(('Forecast Financial Statements'!I28+'Forecast Financial Statements'!I29)+'Forecast Financial Statements'!I63)</f>
         <v/>
       </c>
       <c r="J14" s="28">
-        <f>'Forecast Financial Statements'!J14/(('Forecast Financial Statements'!J35+'Forecast Financial Statements'!J36)+'Forecast Financial Statements'!J37)</f>
+        <f>'Forecast Financial Statements'!J14/(('Forecast Financial Statements'!J28+'Forecast Financial Statements'!J29)+'Forecast Financial Statements'!J63)</f>
         <v/>
       </c>
       <c r="K14" s="28">
-        <f>'Forecast Financial Statements'!K14/(('Forecast Financial Statements'!K35+'Forecast Financial Statements'!K36)+'Forecast Financial Statements'!K37)</f>
+        <f>'Forecast Financial Statements'!K14/(('Forecast Financial Statements'!K28+'Forecast Financial Statements'!K29)+'Forecast Financial Statements'!K63)</f>
         <v/>
       </c>
       <c r="L14" s="28">
-        <f>'Forecast Financial Statements'!L14/(('Forecast Financial Statements'!L35+'Forecast Financial Statements'!L36)+'Forecast Financial Statements'!L37)</f>
+        <f>'Forecast Financial Statements'!L14/(('Forecast Financial Statements'!L28+'Forecast Financial Statements'!L29)+'Forecast Financial Statements'!L63)</f>
         <v/>
       </c>
       <c r="M14" s="28">
-        <f>'Forecast Financial Statements'!M14/(('Forecast Financial Statements'!M35+'Forecast Financial Statements'!M36)+'Forecast Financial Statements'!M37)</f>
+        <f>'Forecast Financial Statements'!M14/(('Forecast Financial Statements'!M28+'Forecast Financial Statements'!M29)+'Forecast Financial Statements'!M63)</f>
         <v/>
       </c>
       <c r="N14" s="28">
-        <f>'Forecast Financial Statements'!N14/(('Forecast Financial Statements'!N35+'Forecast Financial Statements'!N36)+'Forecast Financial Statements'!N37)</f>
+        <f>'Forecast Financial Statements'!N14/(('Forecast Financial Statements'!N28+'Forecast Financial Statements'!N29)+'Forecast Financial Statements'!N63)</f>
         <v/>
       </c>
       <c r="O14" s="28">
-        <f>'Forecast Financial Statements'!O14/(('Forecast Financial Statements'!O35+'Forecast Financial Statements'!O36)+'Forecast Financial Statements'!O37)</f>
+        <f>'Forecast Financial Statements'!O14/(('Forecast Financial Statements'!O28+'Forecast Financial Statements'!O29)+'Forecast Financial Statements'!O63)</f>
         <v/>
       </c>
     </row>
@@ -6445,35 +7420,35 @@
         <v/>
       </c>
       <c r="H15" s="28">
-        <f>'Forecast Financial Statements'!H20/'Forecast Financial Statements'!H34</f>
+        <f>'Forecast Financial Statements'!H20/'Forecast Financial Statements'!H61</f>
         <v/>
       </c>
       <c r="I15" s="28">
-        <f>'Forecast Financial Statements'!I20/'Forecast Financial Statements'!I34</f>
+        <f>'Forecast Financial Statements'!I20/'Forecast Financial Statements'!I61</f>
         <v/>
       </c>
       <c r="J15" s="28">
-        <f>'Forecast Financial Statements'!J20/'Forecast Financial Statements'!J34</f>
+        <f>'Forecast Financial Statements'!J20/'Forecast Financial Statements'!J61</f>
         <v/>
       </c>
       <c r="K15" s="28">
-        <f>'Forecast Financial Statements'!K20/'Forecast Financial Statements'!K34</f>
+        <f>'Forecast Financial Statements'!K20/'Forecast Financial Statements'!K61</f>
         <v/>
       </c>
       <c r="L15" s="28">
-        <f>'Forecast Financial Statements'!L20/'Forecast Financial Statements'!L34</f>
+        <f>'Forecast Financial Statements'!L20/'Forecast Financial Statements'!L61</f>
         <v/>
       </c>
       <c r="M15" s="28">
-        <f>'Forecast Financial Statements'!M20/'Forecast Financial Statements'!M34</f>
+        <f>'Forecast Financial Statements'!M20/'Forecast Financial Statements'!M61</f>
         <v/>
       </c>
       <c r="N15" s="28">
-        <f>'Forecast Financial Statements'!N20/'Forecast Financial Statements'!N34</f>
+        <f>'Forecast Financial Statements'!N20/'Forecast Financial Statements'!N61</f>
         <v/>
       </c>
       <c r="O15" s="28">
-        <f>'Forecast Financial Statements'!O20/'Forecast Financial Statements'!O34</f>
+        <f>'Forecast Financial Statements'!O20/'Forecast Financial Statements'!O61</f>
         <v/>
       </c>
     </row>
@@ -6508,35 +7483,35 @@
         <v/>
       </c>
       <c r="H16" s="29">
-        <f>'Forecast Financial Statements'!H5/'Forecast Financial Statements'!H34</f>
+        <f>'Forecast Financial Statements'!H5/'Forecast Financial Statements'!H61</f>
         <v/>
       </c>
       <c r="I16" s="29">
-        <f>'Forecast Financial Statements'!I5/'Forecast Financial Statements'!I34</f>
+        <f>'Forecast Financial Statements'!I5/'Forecast Financial Statements'!I61</f>
         <v/>
       </c>
       <c r="J16" s="29">
-        <f>'Forecast Financial Statements'!J5/'Forecast Financial Statements'!J34</f>
+        <f>'Forecast Financial Statements'!J5/'Forecast Financial Statements'!J61</f>
         <v/>
       </c>
       <c r="K16" s="29">
-        <f>'Forecast Financial Statements'!K5/'Forecast Financial Statements'!K34</f>
+        <f>'Forecast Financial Statements'!K5/'Forecast Financial Statements'!K61</f>
         <v/>
       </c>
       <c r="L16" s="29">
-        <f>'Forecast Financial Statements'!L5/'Forecast Financial Statements'!L34</f>
+        <f>'Forecast Financial Statements'!L5/'Forecast Financial Statements'!L61</f>
         <v/>
       </c>
       <c r="M16" s="29">
-        <f>'Forecast Financial Statements'!M5/'Forecast Financial Statements'!M34</f>
+        <f>'Forecast Financial Statements'!M5/'Forecast Financial Statements'!M61</f>
         <v/>
       </c>
       <c r="N16" s="29">
-        <f>'Forecast Financial Statements'!N5/'Forecast Financial Statements'!N34</f>
+        <f>'Forecast Financial Statements'!N5/'Forecast Financial Statements'!N61</f>
         <v/>
       </c>
       <c r="O16" s="29">
-        <f>'Forecast Financial Statements'!O5/'Forecast Financial Statements'!O34</f>
+        <f>'Forecast Financial Statements'!O5/'Forecast Financial Statements'!O61</f>
         <v/>
       </c>
     </row>
@@ -6592,35 +7567,35 @@
         <v/>
       </c>
       <c r="H19" s="29">
-        <f>'Forecast Financial Statements'!H37/('Forecast Financial Statements'!H35+'Forecast Financial Statements'!H36)</f>
+        <f>'Forecast Financial Statements'!H63/('Forecast Financial Statements'!H28+'Forecast Financial Statements'!H29)</f>
         <v/>
       </c>
       <c r="I19" s="29">
-        <f>'Forecast Financial Statements'!I37/('Forecast Financial Statements'!I35+'Forecast Financial Statements'!I36)</f>
+        <f>'Forecast Financial Statements'!I63/('Forecast Financial Statements'!I28+'Forecast Financial Statements'!I29)</f>
         <v/>
       </c>
       <c r="J19" s="29">
-        <f>'Forecast Financial Statements'!J37/('Forecast Financial Statements'!J35+'Forecast Financial Statements'!J36)</f>
+        <f>'Forecast Financial Statements'!J63/('Forecast Financial Statements'!J28+'Forecast Financial Statements'!J29)</f>
         <v/>
       </c>
       <c r="K19" s="29">
-        <f>'Forecast Financial Statements'!K37/('Forecast Financial Statements'!K35+'Forecast Financial Statements'!K36)</f>
+        <f>'Forecast Financial Statements'!K63/('Forecast Financial Statements'!K28+'Forecast Financial Statements'!K29)</f>
         <v/>
       </c>
       <c r="L19" s="29">
-        <f>'Forecast Financial Statements'!L37/('Forecast Financial Statements'!L35+'Forecast Financial Statements'!L36)</f>
+        <f>'Forecast Financial Statements'!L63/('Forecast Financial Statements'!L28+'Forecast Financial Statements'!L29)</f>
         <v/>
       </c>
       <c r="M19" s="29">
-        <f>'Forecast Financial Statements'!M37/('Forecast Financial Statements'!M35+'Forecast Financial Statements'!M36)</f>
+        <f>'Forecast Financial Statements'!M63/('Forecast Financial Statements'!M28+'Forecast Financial Statements'!M29)</f>
         <v/>
       </c>
       <c r="N19" s="29">
-        <f>'Forecast Financial Statements'!N37/('Forecast Financial Statements'!N35+'Forecast Financial Statements'!N36)</f>
+        <f>'Forecast Financial Statements'!N63/('Forecast Financial Statements'!N28+'Forecast Financial Statements'!N29)</f>
         <v/>
       </c>
       <c r="O19" s="29">
-        <f>'Forecast Financial Statements'!O37/('Forecast Financial Statements'!O35+'Forecast Financial Statements'!O36)</f>
+        <f>'Forecast Financial Statements'!O63/('Forecast Financial Statements'!O28+'Forecast Financial Statements'!O29)</f>
         <v/>
       </c>
     </row>
@@ -6694,35 +7669,35 @@
         </is>
       </c>
       <c r="H21" s="29">
-        <f>('Forecast Financial Statements'!H37-'Forecast Financial Statements'!H32)/'Forecast Financial Statements'!H12</f>
+        <f>('Forecast Financial Statements'!H63-'Forecast Financial Statements'!H58)/'Forecast Financial Statements'!H12</f>
         <v/>
       </c>
       <c r="I21" s="29">
-        <f>('Forecast Financial Statements'!I37-'Forecast Financial Statements'!I32)/'Forecast Financial Statements'!I12</f>
+        <f>('Forecast Financial Statements'!I63-'Forecast Financial Statements'!I58)/'Forecast Financial Statements'!I12</f>
         <v/>
       </c>
       <c r="J21" s="29">
-        <f>('Forecast Financial Statements'!J37-'Forecast Financial Statements'!J32)/'Forecast Financial Statements'!J12</f>
+        <f>('Forecast Financial Statements'!J63-'Forecast Financial Statements'!J58)/'Forecast Financial Statements'!J12</f>
         <v/>
       </c>
       <c r="K21" s="29">
-        <f>('Forecast Financial Statements'!K37-'Forecast Financial Statements'!K32)/'Forecast Financial Statements'!K12</f>
+        <f>('Forecast Financial Statements'!K63-'Forecast Financial Statements'!K58)/'Forecast Financial Statements'!K12</f>
         <v/>
       </c>
       <c r="L21" s="29">
-        <f>('Forecast Financial Statements'!L37-'Forecast Financial Statements'!L32)/'Forecast Financial Statements'!L12</f>
+        <f>('Forecast Financial Statements'!L63-'Forecast Financial Statements'!L58)/'Forecast Financial Statements'!L12</f>
         <v/>
       </c>
       <c r="M21" s="29">
-        <f>('Forecast Financial Statements'!M37-'Forecast Financial Statements'!M32)/'Forecast Financial Statements'!M12</f>
+        <f>('Forecast Financial Statements'!M63-'Forecast Financial Statements'!M58)/'Forecast Financial Statements'!M12</f>
         <v/>
       </c>
       <c r="N21" s="29">
-        <f>('Forecast Financial Statements'!N37-'Forecast Financial Statements'!N32)/'Forecast Financial Statements'!N12</f>
+        <f>('Forecast Financial Statements'!N63-'Forecast Financial Statements'!N58)/'Forecast Financial Statements'!N12</f>
         <v/>
       </c>
       <c r="O21" s="29">
-        <f>('Forecast Financial Statements'!O37-'Forecast Financial Statements'!O32)/'Forecast Financial Statements'!O12</f>
+        <f>('Forecast Financial Statements'!O63-'Forecast Financial Statements'!O58)/'Forecast Financial Statements'!O12</f>
         <v/>
       </c>
     </row>
@@ -6753,59 +7728,59 @@
           <t>EPS (INR)</t>
         </is>
       </c>
-      <c r="B24" s="40">
+      <c r="B24" s="42">
         <f>'Historical Financial Statements'!B21</f>
         <v/>
       </c>
-      <c r="C24" s="40">
+      <c r="C24" s="42">
         <f>'Historical Financial Statements'!C21</f>
         <v/>
       </c>
-      <c r="D24" s="40">
+      <c r="D24" s="42">
         <f>'Historical Financial Statements'!D21</f>
         <v/>
       </c>
-      <c r="E24" s="40">
+      <c r="E24" s="42">
         <f>'Historical Financial Statements'!E21</f>
         <v/>
       </c>
-      <c r="F24" s="40">
+      <c r="F24" s="42">
         <f>'Historical Financial Statements'!F21</f>
         <v/>
       </c>
-      <c r="G24" s="40">
+      <c r="G24" s="42">
         <f>'Historical Financial Statements'!G21</f>
         <v/>
       </c>
-      <c r="H24" s="40">
+      <c r="H24" s="42">
         <f>'Forecast Financial Statements'!H21</f>
         <v/>
       </c>
-      <c r="I24" s="40">
+      <c r="I24" s="42">
         <f>'Forecast Financial Statements'!I21</f>
         <v/>
       </c>
-      <c r="J24" s="40">
+      <c r="J24" s="42">
         <f>'Forecast Financial Statements'!J21</f>
         <v/>
       </c>
-      <c r="K24" s="40">
+      <c r="K24" s="42">
         <f>'Forecast Financial Statements'!K21</f>
         <v/>
       </c>
-      <c r="L24" s="40">
+      <c r="L24" s="42">
         <f>'Forecast Financial Statements'!L21</f>
         <v/>
       </c>
-      <c r="M24" s="40">
+      <c r="M24" s="42">
         <f>'Forecast Financial Statements'!M21</f>
         <v/>
       </c>
-      <c r="N24" s="40">
+      <c r="N24" s="42">
         <f>'Forecast Financial Statements'!N21</f>
         <v/>
       </c>
-      <c r="O24" s="40">
+      <c r="O24" s="42">
         <f>'Forecast Financial Statements'!O21</f>
         <v/>
       </c>
@@ -6816,60 +7791,60 @@
           <t>DPS (INR)</t>
         </is>
       </c>
-      <c r="B25" s="40">
-        <f>'Historical Financial Statements'!B22/'Assumptions'!C40</f>
-        <v/>
-      </c>
-      <c r="C25" s="40">
-        <f>'Historical Financial Statements'!C22/'Assumptions'!C40</f>
-        <v/>
-      </c>
-      <c r="D25" s="40">
-        <f>'Historical Financial Statements'!D22/'Assumptions'!C40</f>
-        <v/>
-      </c>
-      <c r="E25" s="40">
-        <f>'Historical Financial Statements'!E22/'Assumptions'!C40</f>
-        <v/>
-      </c>
-      <c r="F25" s="40">
-        <f>'Historical Financial Statements'!F22/'Assumptions'!C40</f>
-        <v/>
-      </c>
-      <c r="G25" s="40">
-        <f>'Historical Financial Statements'!G22/'Assumptions'!C40</f>
-        <v/>
-      </c>
-      <c r="H25" s="40">
-        <f>'Forecast Financial Statements'!H22/'Assumptions'!C40</f>
-        <v/>
-      </c>
-      <c r="I25" s="40">
-        <f>'Forecast Financial Statements'!I22/'Assumptions'!C40</f>
-        <v/>
-      </c>
-      <c r="J25" s="40">
-        <f>'Forecast Financial Statements'!J22/'Assumptions'!C40</f>
-        <v/>
-      </c>
-      <c r="K25" s="40">
-        <f>'Forecast Financial Statements'!K22/'Assumptions'!C40</f>
-        <v/>
-      </c>
-      <c r="L25" s="40">
-        <f>'Forecast Financial Statements'!L22/'Assumptions'!C40</f>
-        <v/>
-      </c>
-      <c r="M25" s="40">
-        <f>'Forecast Financial Statements'!M22/'Assumptions'!C40</f>
-        <v/>
-      </c>
-      <c r="N25" s="40">
-        <f>'Forecast Financial Statements'!N22/'Assumptions'!C40</f>
-        <v/>
-      </c>
-      <c r="O25" s="40">
-        <f>'Forecast Financial Statements'!O22/'Assumptions'!C40</f>
+      <c r="B25" s="42">
+        <f>'Historical Financial Statements'!B22/'Assumptions'!C43</f>
+        <v/>
+      </c>
+      <c r="C25" s="42">
+        <f>'Historical Financial Statements'!C22/'Assumptions'!C43</f>
+        <v/>
+      </c>
+      <c r="D25" s="42">
+        <f>'Historical Financial Statements'!D22/'Assumptions'!C43</f>
+        <v/>
+      </c>
+      <c r="E25" s="42">
+        <f>'Historical Financial Statements'!E22/'Assumptions'!C43</f>
+        <v/>
+      </c>
+      <c r="F25" s="42">
+        <f>'Historical Financial Statements'!F22/'Assumptions'!C43</f>
+        <v/>
+      </c>
+      <c r="G25" s="42">
+        <f>'Historical Financial Statements'!G22/'Assumptions'!C43</f>
+        <v/>
+      </c>
+      <c r="H25" s="42">
+        <f>'Forecast Financial Statements'!H22/'Assumptions'!C43</f>
+        <v/>
+      </c>
+      <c r="I25" s="42">
+        <f>'Forecast Financial Statements'!I22/'Assumptions'!C43</f>
+        <v/>
+      </c>
+      <c r="J25" s="42">
+        <f>'Forecast Financial Statements'!J22/'Assumptions'!C43</f>
+        <v/>
+      </c>
+      <c r="K25" s="42">
+        <f>'Forecast Financial Statements'!K22/'Assumptions'!C43</f>
+        <v/>
+      </c>
+      <c r="L25" s="42">
+        <f>'Forecast Financial Statements'!L22/'Assumptions'!C43</f>
+        <v/>
+      </c>
+      <c r="M25" s="42">
+        <f>'Forecast Financial Statements'!M22/'Assumptions'!C43</f>
+        <v/>
+      </c>
+      <c r="N25" s="42">
+        <f>'Forecast Financial Statements'!N22/'Assumptions'!C43</f>
+        <v/>
+      </c>
+      <c r="O25" s="42">
+        <f>'Forecast Financial Statements'!O22/'Assumptions'!C43</f>
         <v/>
       </c>
     </row>
@@ -6942,60 +7917,60 @@
           <t>Book value per share (INR)</t>
         </is>
       </c>
-      <c r="B27" s="40">
-        <f>('Historical Financial Statements'!B33+'Historical Financial Statements'!B34)/'Assumptions'!C40</f>
-        <v/>
-      </c>
-      <c r="C27" s="40">
-        <f>('Historical Financial Statements'!C33+'Historical Financial Statements'!C34)/'Assumptions'!C40</f>
-        <v/>
-      </c>
-      <c r="D27" s="40">
-        <f>('Historical Financial Statements'!D33+'Historical Financial Statements'!D34)/'Assumptions'!C40</f>
-        <v/>
-      </c>
-      <c r="E27" s="40">
-        <f>('Historical Financial Statements'!E33+'Historical Financial Statements'!E34)/'Assumptions'!C40</f>
-        <v/>
-      </c>
-      <c r="F27" s="40">
-        <f>('Historical Financial Statements'!F33+'Historical Financial Statements'!F34)/'Assumptions'!C40</f>
-        <v/>
-      </c>
-      <c r="G27" s="40">
-        <f>('Historical Financial Statements'!G33+'Historical Financial Statements'!G34)/'Assumptions'!C40</f>
-        <v/>
-      </c>
-      <c r="H27" s="40">
-        <f>('Forecast Financial Statements'!H35+'Forecast Financial Statements'!H36)/'Assumptions'!C40</f>
-        <v/>
-      </c>
-      <c r="I27" s="40">
-        <f>('Forecast Financial Statements'!I35+'Forecast Financial Statements'!I36)/'Assumptions'!C40</f>
-        <v/>
-      </c>
-      <c r="J27" s="40">
-        <f>('Forecast Financial Statements'!J35+'Forecast Financial Statements'!J36)/'Assumptions'!C40</f>
-        <v/>
-      </c>
-      <c r="K27" s="40">
-        <f>('Forecast Financial Statements'!K35+'Forecast Financial Statements'!K36)/'Assumptions'!C40</f>
-        <v/>
-      </c>
-      <c r="L27" s="40">
-        <f>('Forecast Financial Statements'!L35+'Forecast Financial Statements'!L36)/'Assumptions'!C40</f>
-        <v/>
-      </c>
-      <c r="M27" s="40">
-        <f>('Forecast Financial Statements'!M35+'Forecast Financial Statements'!M36)/'Assumptions'!C40</f>
-        <v/>
-      </c>
-      <c r="N27" s="40">
-        <f>('Forecast Financial Statements'!N35+'Forecast Financial Statements'!N36)/'Assumptions'!C40</f>
-        <v/>
-      </c>
-      <c r="O27" s="40">
-        <f>('Forecast Financial Statements'!O35+'Forecast Financial Statements'!O36)/'Assumptions'!C40</f>
+      <c r="B27" s="42">
+        <f>('Historical Financial Statements'!B33+'Historical Financial Statements'!B34)/'Assumptions'!C43</f>
+        <v/>
+      </c>
+      <c r="C27" s="42">
+        <f>('Historical Financial Statements'!C33+'Historical Financial Statements'!C34)/'Assumptions'!C43</f>
+        <v/>
+      </c>
+      <c r="D27" s="42">
+        <f>('Historical Financial Statements'!D33+'Historical Financial Statements'!D34)/'Assumptions'!C43</f>
+        <v/>
+      </c>
+      <c r="E27" s="42">
+        <f>('Historical Financial Statements'!E33+'Historical Financial Statements'!E34)/'Assumptions'!C43</f>
+        <v/>
+      </c>
+      <c r="F27" s="42">
+        <f>('Historical Financial Statements'!F33+'Historical Financial Statements'!F34)/'Assumptions'!C43</f>
+        <v/>
+      </c>
+      <c r="G27" s="42">
+        <f>('Historical Financial Statements'!G33+'Historical Financial Statements'!G34)/'Assumptions'!C43</f>
+        <v/>
+      </c>
+      <c r="H27" s="42">
+        <f>('Forecast Financial Statements'!H28+'Forecast Financial Statements'!H29)/'Assumptions'!C43</f>
+        <v/>
+      </c>
+      <c r="I27" s="42">
+        <f>('Forecast Financial Statements'!I28+'Forecast Financial Statements'!I29)/'Assumptions'!C43</f>
+        <v/>
+      </c>
+      <c r="J27" s="42">
+        <f>('Forecast Financial Statements'!J28+'Forecast Financial Statements'!J29)/'Assumptions'!C43</f>
+        <v/>
+      </c>
+      <c r="K27" s="42">
+        <f>('Forecast Financial Statements'!K28+'Forecast Financial Statements'!K29)/'Assumptions'!C43</f>
+        <v/>
+      </c>
+      <c r="L27" s="42">
+        <f>('Forecast Financial Statements'!L28+'Forecast Financial Statements'!L29)/'Assumptions'!C43</f>
+        <v/>
+      </c>
+      <c r="M27" s="42">
+        <f>('Forecast Financial Statements'!M28+'Forecast Financial Statements'!M29)/'Assumptions'!C43</f>
+        <v/>
+      </c>
+      <c r="N27" s="42">
+        <f>('Forecast Financial Statements'!N28+'Forecast Financial Statements'!N29)/'Assumptions'!C43</f>
+        <v/>
+      </c>
+      <c r="O27" s="42">
+        <f>('Forecast Financial Statements'!O28+'Forecast Financial Statements'!O29)/'Assumptions'!C43</f>
         <v/>
       </c>
     </row>
@@ -7026,36 +8001,36 @@
           <t>Receivable days</t>
         </is>
       </c>
-      <c r="H30" s="41">
-        <f>'Forecast Financial Statements'!H30/'Forecast Financial Statements'!H5*365</f>
-        <v/>
-      </c>
-      <c r="I30" s="41">
-        <f>'Forecast Financial Statements'!I30/'Forecast Financial Statements'!I5*365</f>
-        <v/>
-      </c>
-      <c r="J30" s="41">
-        <f>'Forecast Financial Statements'!J30/'Forecast Financial Statements'!J5*365</f>
-        <v/>
-      </c>
-      <c r="K30" s="41">
-        <f>'Forecast Financial Statements'!K30/'Forecast Financial Statements'!K5*365</f>
-        <v/>
-      </c>
-      <c r="L30" s="41">
-        <f>'Forecast Financial Statements'!L30/'Forecast Financial Statements'!L5*365</f>
-        <v/>
-      </c>
-      <c r="M30" s="41">
-        <f>'Forecast Financial Statements'!M30/'Forecast Financial Statements'!M5*365</f>
-        <v/>
-      </c>
-      <c r="N30" s="41">
-        <f>'Forecast Financial Statements'!N30/'Forecast Financial Statements'!N5*365</f>
-        <v/>
-      </c>
-      <c r="O30" s="41">
-        <f>'Forecast Financial Statements'!O30/'Forecast Financial Statements'!O5*365</f>
+      <c r="H30" s="43">
+        <f>'Forecast Financial Statements'!H55/'Forecast Financial Statements'!H5*365</f>
+        <v/>
+      </c>
+      <c r="I30" s="43">
+        <f>'Forecast Financial Statements'!I55/'Forecast Financial Statements'!I5*365</f>
+        <v/>
+      </c>
+      <c r="J30" s="43">
+        <f>'Forecast Financial Statements'!J55/'Forecast Financial Statements'!J5*365</f>
+        <v/>
+      </c>
+      <c r="K30" s="43">
+        <f>'Forecast Financial Statements'!K55/'Forecast Financial Statements'!K5*365</f>
+        <v/>
+      </c>
+      <c r="L30" s="43">
+        <f>'Forecast Financial Statements'!L55/'Forecast Financial Statements'!L5*365</f>
+        <v/>
+      </c>
+      <c r="M30" s="43">
+        <f>'Forecast Financial Statements'!M55/'Forecast Financial Statements'!M5*365</f>
+        <v/>
+      </c>
+      <c r="N30" s="43">
+        <f>'Forecast Financial Statements'!N55/'Forecast Financial Statements'!N5*365</f>
+        <v/>
+      </c>
+      <c r="O30" s="43">
+        <f>'Forecast Financial Statements'!O55/'Forecast Financial Statements'!O5*365</f>
         <v/>
       </c>
     </row>
@@ -7065,32 +8040,32 @@
           <t>Inventory days</t>
         </is>
       </c>
-      <c r="I31" s="41">
-        <f>'Forecast Financial Statements'!I29/'Cost Forecast'!I16*365</f>
-        <v/>
-      </c>
-      <c r="J31" s="41">
-        <f>'Forecast Financial Statements'!J29/'Cost Forecast'!J16*365</f>
-        <v/>
-      </c>
-      <c r="K31" s="41">
-        <f>'Forecast Financial Statements'!K29/'Cost Forecast'!K16*365</f>
-        <v/>
-      </c>
-      <c r="L31" s="41">
-        <f>'Forecast Financial Statements'!L29/'Cost Forecast'!L16*365</f>
-        <v/>
-      </c>
-      <c r="M31" s="41">
-        <f>'Forecast Financial Statements'!M29/'Cost Forecast'!M16*365</f>
-        <v/>
-      </c>
-      <c r="N31" s="41">
-        <f>'Forecast Financial Statements'!N29/'Cost Forecast'!N16*365</f>
-        <v/>
-      </c>
-      <c r="O31" s="41">
-        <f>'Forecast Financial Statements'!O29/'Cost Forecast'!O16*365</f>
+      <c r="I31" s="43">
+        <f>'Forecast Financial Statements'!I56/'Cost Forecast'!I16*365</f>
+        <v/>
+      </c>
+      <c r="J31" s="43">
+        <f>'Forecast Financial Statements'!J56/'Cost Forecast'!J16*365</f>
+        <v/>
+      </c>
+      <c r="K31" s="43">
+        <f>'Forecast Financial Statements'!K56/'Cost Forecast'!K16*365</f>
+        <v/>
+      </c>
+      <c r="L31" s="43">
+        <f>'Forecast Financial Statements'!L56/'Cost Forecast'!L16*365</f>
+        <v/>
+      </c>
+      <c r="M31" s="43">
+        <f>'Forecast Financial Statements'!M56/'Cost Forecast'!M16*365</f>
+        <v/>
+      </c>
+      <c r="N31" s="43">
+        <f>'Forecast Financial Statements'!N56/'Cost Forecast'!N16*365</f>
+        <v/>
+      </c>
+      <c r="O31" s="43">
+        <f>'Forecast Financial Statements'!O56/'Cost Forecast'!O16*365</f>
         <v/>
       </c>
     </row>
@@ -7100,31 +8075,31 @@
           <t>Payable days</t>
         </is>
       </c>
-      <c r="I32" s="41">
+      <c r="I32" s="43">
         <f>'Forecast Financial Statements'!I38/'Cost Forecast'!I16*365</f>
         <v/>
       </c>
-      <c r="J32" s="41">
+      <c r="J32" s="43">
         <f>'Forecast Financial Statements'!J38/'Cost Forecast'!J16*365</f>
         <v/>
       </c>
-      <c r="K32" s="41">
+      <c r="K32" s="43">
         <f>'Forecast Financial Statements'!K38/'Cost Forecast'!K16*365</f>
         <v/>
       </c>
-      <c r="L32" s="41">
+      <c r="L32" s="43">
         <f>'Forecast Financial Statements'!L38/'Cost Forecast'!L16*365</f>
         <v/>
       </c>
-      <c r="M32" s="41">
+      <c r="M32" s="43">
         <f>'Forecast Financial Statements'!M38/'Cost Forecast'!M16*365</f>
         <v/>
       </c>
-      <c r="N32" s="41">
+      <c r="N32" s="43">
         <f>'Forecast Financial Statements'!N38/'Cost Forecast'!N16*365</f>
         <v/>
       </c>
-      <c r="O32" s="41">
+      <c r="O32" s="43">
         <f>'Forecast Financial Statements'!O38/'Cost Forecast'!O16*365</f>
         <v/>
       </c>
@@ -7608,25 +8583,25 @@
           <t>Discount period (years)</t>
         </is>
       </c>
-      <c r="I13" s="42" t="n">
+      <c r="I13" s="44" t="n">
         <v>1</v>
       </c>
-      <c r="J13" s="42" t="n">
+      <c r="J13" s="44" t="n">
         <v>2</v>
       </c>
-      <c r="K13" s="42" t="n">
+      <c r="K13" s="44" t="n">
         <v>3</v>
       </c>
-      <c r="L13" s="42" t="n">
+      <c r="L13" s="44" t="n">
         <v>4</v>
       </c>
-      <c r="M13" s="42" t="n">
+      <c r="M13" s="44" t="n">
         <v>5</v>
       </c>
-      <c r="N13" s="42" t="n">
+      <c r="N13" s="44" t="n">
         <v>6</v>
       </c>
-      <c r="O13" s="42" t="n">
+      <c r="O13" s="44" t="n">
         <v>7</v>
       </c>
     </row>
@@ -7636,32 +8611,32 @@
           <t>Discount factor @ WACC</t>
         </is>
       </c>
-      <c r="I14" s="43">
-        <f>1/(1+'Assumptions'!C39)^I13</f>
-        <v/>
-      </c>
-      <c r="J14" s="43">
-        <f>1/(1+'Assumptions'!C39)^J13</f>
-        <v/>
-      </c>
-      <c r="K14" s="43">
-        <f>1/(1+'Assumptions'!C39)^K13</f>
-        <v/>
-      </c>
-      <c r="L14" s="43">
-        <f>1/(1+'Assumptions'!C39)^L13</f>
-        <v/>
-      </c>
-      <c r="M14" s="43">
-        <f>1/(1+'Assumptions'!C39)^M13</f>
-        <v/>
-      </c>
-      <c r="N14" s="43">
-        <f>1/(1+'Assumptions'!C39)^N13</f>
-        <v/>
-      </c>
-      <c r="O14" s="43">
-        <f>1/(1+'Assumptions'!C39)^O13</f>
+      <c r="I14" s="45">
+        <f>1/(1+'Assumptions'!C42)^I13</f>
+        <v/>
+      </c>
+      <c r="J14" s="45">
+        <f>1/(1+'Assumptions'!C42)^J13</f>
+        <v/>
+      </c>
+      <c r="K14" s="45">
+        <f>1/(1+'Assumptions'!C42)^K13</f>
+        <v/>
+      </c>
+      <c r="L14" s="45">
+        <f>1/(1+'Assumptions'!C42)^L13</f>
+        <v/>
+      </c>
+      <c r="M14" s="45">
+        <f>1/(1+'Assumptions'!C42)^M13</f>
+        <v/>
+      </c>
+      <c r="N14" s="45">
+        <f>1/(1+'Assumptions'!C42)^N13</f>
+        <v/>
+      </c>
+      <c r="O14" s="45">
+        <f>1/(1+'Assumptions'!C42)^O13</f>
         <v/>
       </c>
     </row>
@@ -7727,7 +8702,7 @@
           <t>Sum of PV of explicit FCFF (FY27-33)</t>
         </is>
       </c>
-      <c r="C18" s="44">
+      <c r="C18" s="46">
         <f>SUM(I15:O15)</f>
         <v/>
       </c>
@@ -7738,8 +8713,8 @@
           <t>WACC</t>
         </is>
       </c>
-      <c r="C19" s="45">
-        <f>'Assumptions'!C39</f>
+      <c r="C19" s="47">
+        <f>'Assumptions'!C42</f>
         <v/>
       </c>
     </row>
@@ -7749,8 +8724,8 @@
           <t>Terminal growth rate (g)</t>
         </is>
       </c>
-      <c r="C20" s="45">
-        <f>'Assumptions'!C37</f>
+      <c r="C20" s="47">
+        <f>'Assumptions'!C40</f>
         <v/>
       </c>
     </row>
@@ -7760,7 +8735,7 @@
           <t>Terminal value (Gordon growth)</t>
         </is>
       </c>
-      <c r="C21" s="44">
+      <c r="C21" s="46">
         <f>O12*(1+C20)/(C19-C20)</f>
         <v/>
       </c>
@@ -7771,7 +8746,7 @@
           <t>PV of terminal value</t>
         </is>
       </c>
-      <c r="C22" s="44">
+      <c r="C22" s="46">
         <f>C21*O14</f>
         <v/>
       </c>
@@ -7782,7 +8757,7 @@
           <t>Enterprise value (EV)</t>
         </is>
       </c>
-      <c r="C23" s="46">
+      <c r="C23" s="48">
         <f>C18+C22</f>
         <v/>
       </c>
@@ -7793,8 +8768,8 @@
           <t>Less: net debt (FY26 debt - cash)</t>
         </is>
       </c>
-      <c r="C24" s="47">
-        <f>-('Forecast Financial Statements'!H37-'Forecast Financial Statements'!H32)</f>
+      <c r="C24" s="49">
+        <f>-('Forecast Financial Statements'!H63-'Forecast Financial Statements'!H58)</f>
         <v/>
       </c>
     </row>
@@ -7804,7 +8779,7 @@
           <t>Equity value</t>
         </is>
       </c>
-      <c r="C25" s="46">
+      <c r="C25" s="48">
         <f>C23+C24</f>
         <v/>
       </c>
@@ -7815,8 +8790,8 @@
           <t>Shares outstanding (crore)</t>
         </is>
       </c>
-      <c r="C26" s="48">
-        <f>'Assumptions'!C40</f>
+      <c r="C26" s="50">
+        <f>'Assumptions'!C43</f>
         <v/>
       </c>
     </row>
@@ -7826,7 +8801,7 @@
           <t>Intrinsic value per share (INR)</t>
         </is>
       </c>
-      <c r="C27" s="49">
+      <c r="C27" s="51">
         <f>C25/C26</f>
         <v/>
       </c>
@@ -7837,8 +8812,8 @@
           <t>Current market price (INR)</t>
         </is>
       </c>
-      <c r="C28" s="50">
-        <f>'Assumptions'!C41</f>
+      <c r="C28" s="52">
+        <f>'Assumptions'!C44</f>
         <v/>
       </c>
     </row>
@@ -7963,19 +8938,19 @@
           <t>Siemens India</t>
         </is>
       </c>
-      <c r="B6" s="51" t="n">
+      <c r="B6" s="53" t="n">
         <v>5.5</v>
       </c>
-      <c r="C6" s="51" t="n">
+      <c r="C6" s="53" t="n">
         <v>42</v>
       </c>
-      <c r="D6" s="51" t="n">
+      <c r="D6" s="53" t="n">
         <v>60</v>
       </c>
-      <c r="E6" s="51" t="n">
+      <c r="E6" s="53" t="n">
         <v>9</v>
       </c>
-      <c r="F6" s="52" t="n">
+      <c r="F6" s="54" t="n">
         <v>0.4</v>
       </c>
     </row>
@@ -7985,19 +8960,19 @@
           <t>ABB India</t>
         </is>
       </c>
-      <c r="B7" s="51" t="n">
+      <c r="B7" s="53" t="n">
         <v>7</v>
       </c>
-      <c r="C7" s="51" t="n">
+      <c r="C7" s="53" t="n">
         <v>50</v>
       </c>
-      <c r="D7" s="51" t="n">
+      <c r="D7" s="53" t="n">
         <v>68</v>
       </c>
-      <c r="E7" s="51" t="n">
+      <c r="E7" s="53" t="n">
         <v>14</v>
       </c>
-      <c r="F7" s="52" t="n">
+      <c r="F7" s="54" t="n">
         <v>0.4</v>
       </c>
     </row>
@@ -8007,19 +8982,19 @@
           <t>CG Power &amp; Ind.</t>
         </is>
       </c>
-      <c r="B8" s="51" t="n">
+      <c r="B8" s="53" t="n">
         <v>6.5</v>
       </c>
-      <c r="C8" s="51" t="n">
+      <c r="C8" s="53" t="n">
         <v>45</v>
       </c>
-      <c r="D8" s="51" t="n">
+      <c r="D8" s="53" t="n">
         <v>62</v>
       </c>
-      <c r="E8" s="51" t="n">
+      <c r="E8" s="53" t="n">
         <v>18</v>
       </c>
-      <c r="F8" s="52" t="n">
+      <c r="F8" s="54" t="n">
         <v>0.2</v>
       </c>
     </row>
@@ -8029,19 +9004,19 @@
           <t>GE Vernova T&amp;D India</t>
         </is>
       </c>
-      <c r="B9" s="51" t="n">
+      <c r="B9" s="53" t="n">
         <v>8</v>
       </c>
-      <c r="C9" s="51" t="n">
+      <c r="C9" s="53" t="n">
         <v>48</v>
       </c>
-      <c r="D9" s="51" t="n">
+      <c r="D9" s="53" t="n">
         <v>65</v>
       </c>
-      <c r="E9" s="51" t="n">
+      <c r="E9" s="53" t="n">
         <v>20</v>
       </c>
-      <c r="F9" s="52" t="n">
+      <c r="F9" s="54" t="n">
         <v>0.1</v>
       </c>
     </row>
@@ -8051,19 +9026,19 @@
           <t>Thermax</t>
         </is>
       </c>
-      <c r="B10" s="51" t="n">
+      <c r="B10" s="53" t="n">
         <v>4</v>
       </c>
-      <c r="C10" s="51" t="n">
+      <c r="C10" s="53" t="n">
         <v>38</v>
       </c>
-      <c r="D10" s="51" t="n">
+      <c r="D10" s="53" t="n">
         <v>55</v>
       </c>
-      <c r="E10" s="51" t="n">
+      <c r="E10" s="53" t="n">
         <v>8</v>
       </c>
-      <c r="F10" s="52" t="n">
+      <c r="F10" s="54" t="n">
         <v>0.3</v>
       </c>
     </row>
@@ -8073,19 +9048,19 @@
           <t>Triveni Turbine</t>
         </is>
       </c>
-      <c r="B11" s="51" t="n">
+      <c r="B11" s="53" t="n">
         <v>7.5</v>
       </c>
-      <c r="C11" s="51" t="n">
+      <c r="C11" s="53" t="n">
         <v>40</v>
       </c>
-      <c r="D11" s="51" t="n">
+      <c r="D11" s="53" t="n">
         <v>52</v>
       </c>
-      <c r="E11" s="51" t="n">
+      <c r="E11" s="53" t="n">
         <v>16</v>
       </c>
-      <c r="F11" s="52" t="n">
+      <c r="F11" s="54" t="n">
         <v>0.5</v>
       </c>
     </row>
@@ -8095,19 +9070,19 @@
           <t>Larsen &amp; Toubro</t>
         </is>
       </c>
-      <c r="B12" s="51" t="n">
+      <c r="B12" s="53" t="n">
         <v>2</v>
       </c>
-      <c r="C12" s="51" t="n">
+      <c r="C12" s="53" t="n">
         <v>22</v>
       </c>
-      <c r="D12" s="51" t="n">
+      <c r="D12" s="53" t="n">
         <v>32</v>
       </c>
-      <c r="E12" s="51" t="n">
+      <c r="E12" s="53" t="n">
         <v>5</v>
       </c>
-      <c r="F12" s="52" t="n">
+      <c r="F12" s="54" t="n">
         <v>0.7</v>
       </c>
     </row>
@@ -8117,45 +9092,45 @@
           <t>Kalpataru Projects</t>
         </is>
       </c>
-      <c r="B13" s="51" t="n">
+      <c r="B13" s="53" t="n">
         <v>0.9</v>
       </c>
-      <c r="C13" s="51" t="n">
+      <c r="C13" s="53" t="n">
         <v>12</v>
       </c>
-      <c r="D13" s="51" t="n">
+      <c r="D13" s="53" t="n">
         <v>22</v>
       </c>
-      <c r="E13" s="51" t="n">
+      <c r="E13" s="53" t="n">
         <v>3</v>
       </c>
-      <c r="F13" s="52" t="n">
+      <c r="F13" s="54" t="n">
         <v>0.4</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="53" t="inlineStr">
+      <c r="A14" s="55" t="inlineStr">
         <is>
           <t>Median</t>
         </is>
       </c>
-      <c r="B14" s="54">
+      <c r="B14" s="56">
         <f>MEDIAN(B6:B13)</f>
         <v/>
       </c>
-      <c r="C14" s="54">
+      <c r="C14" s="56">
         <f>MEDIAN(C6:C13)</f>
         <v/>
       </c>
-      <c r="D14" s="54">
+      <c r="D14" s="56">
         <f>MEDIAN(D6:D13)</f>
         <v/>
       </c>
-      <c r="E14" s="54">
+      <c r="E14" s="56">
         <f>MEDIAN(E6:E13)</f>
         <v/>
       </c>
-      <c r="F14" s="55">
+      <c r="F14" s="57">
         <f>MEDIAN(F6:F13)</f>
         <v/>
       </c>
@@ -8178,7 +9153,7 @@
           <t>BHEL FY2027E revenue</t>
         </is>
       </c>
-      <c r="C17" s="47">
+      <c r="C17" s="49">
         <f>'Forecast Financial Statements'!I5</f>
         <v/>
       </c>
@@ -8189,7 +9164,7 @@
           <t>BHEL FY2027E EBITDA</t>
         </is>
       </c>
-      <c r="C18" s="47">
+      <c r="C18" s="49">
         <f>'Forecast Financial Statements'!I12</f>
         <v/>
       </c>
@@ -8200,7 +9175,7 @@
           <t>BHEL FY2027E EPS (INR)</t>
         </is>
       </c>
-      <c r="C19" s="50">
+      <c r="C19" s="52">
         <f>'Forecast Financial Statements'!I21</f>
         <v/>
       </c>
@@ -8211,8 +9186,8 @@
           <t>Net debt (FY26)</t>
         </is>
       </c>
-      <c r="C20" s="47">
-        <f>'Forecast Financial Statements'!H37-'Forecast Financial Statements'!H32</f>
+      <c r="C20" s="49">
+        <f>'Forecast Financial Statements'!H63-'Forecast Financial Statements'!H58</f>
         <v/>
       </c>
     </row>
@@ -8222,7 +9197,7 @@
           <t>Implied EV (EV/EBITDA method)</t>
         </is>
       </c>
-      <c r="C22" s="44">
+      <c r="C22" s="46">
         <f>C18*C14</f>
         <v/>
       </c>
@@ -8233,7 +9208,7 @@
           <t>Implied equity value (EV/EBITDA)</t>
         </is>
       </c>
-      <c r="C23" s="44">
+      <c r="C23" s="46">
         <f>C22-C20</f>
         <v/>
       </c>
@@ -8244,8 +9219,8 @@
           <t>Implied price - EV/EBITDA (INR)</t>
         </is>
       </c>
-      <c r="C24" s="49">
-        <f>C23/'Assumptions'!C40</f>
+      <c r="C24" s="51">
+        <f>C23/'Assumptions'!C43</f>
         <v/>
       </c>
     </row>
@@ -8255,7 +9230,7 @@
           <t>Implied price - P/E method (INR)</t>
         </is>
       </c>
-      <c r="C25" s="49">
+      <c r="C25" s="51">
         <f>C19*D14</f>
         <v/>
       </c>
@@ -8266,7 +9241,7 @@
           <t>Implied EV (EV/Revenue method)</t>
         </is>
       </c>
-      <c r="C26" s="44">
+      <c r="C26" s="46">
         <f>C17*B14</f>
         <v/>
       </c>
@@ -8277,8 +9252,8 @@
           <t>Implied price - EV/Revenue (INR)</t>
         </is>
       </c>
-      <c r="C27" s="49">
-        <f>(C26-C20)/'Assumptions'!C40</f>
+      <c r="C27" s="51">
+        <f>(C26-C20)/'Assumptions'!C43</f>
         <v/>
       </c>
     </row>
@@ -8288,7 +9263,7 @@
           <t>Average implied target price (INR)</t>
         </is>
       </c>
-      <c r="C29" s="56">
+      <c r="C29" s="58">
         <f>AVERAGE(C24,C25,C27)</f>
         <v/>
       </c>
@@ -8365,153 +9340,153 @@
           <t>WACC \ g</t>
         </is>
       </c>
-      <c r="C5" s="57">
-        <f>'Assumptions'!C37+-0.015</f>
-        <v/>
-      </c>
-      <c r="D5" s="57">
-        <f>'Assumptions'!C37+-0.0075</f>
-        <v/>
-      </c>
-      <c r="E5" s="57">
-        <f>'Assumptions'!C37+0.0</f>
-        <v/>
-      </c>
-      <c r="F5" s="57">
-        <f>'Assumptions'!C37+0.0075</f>
-        <v/>
-      </c>
-      <c r="G5" s="57">
-        <f>'Assumptions'!C37+0.015</f>
+      <c r="C5" s="59">
+        <f>'Assumptions'!C40+-0.015</f>
+        <v/>
+      </c>
+      <c r="D5" s="59">
+        <f>'Assumptions'!C40+-0.0075</f>
+        <v/>
+      </c>
+      <c r="E5" s="59">
+        <f>'Assumptions'!C40+0.0</f>
+        <v/>
+      </c>
+      <c r="F5" s="59">
+        <f>'Assumptions'!C40+0.0075</f>
+        <v/>
+      </c>
+      <c r="G5" s="59">
+        <f>'Assumptions'!C40+0.015</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="57">
-        <f>'Assumptions'!C39+0.02</f>
-        <v/>
-      </c>
-      <c r="C6" s="58">
+      <c r="B6" s="59">
+        <f>'Assumptions'!C42+0.02</f>
+        <v/>
+      </c>
+      <c r="C6" s="60">
         <f>(SUMPRODUCT('DCF Valuation'!$I$12:$O$12,(1+$B6)^(-'DCF Valuation'!$I$13:$O$13))+('DCF Valuation'!$O$12*(1+C$5)/($B6-C$5))*(1+$B6)^(-7)+'DCF Valuation'!$C$24)/'DCF Valuation'!$C$26</f>
         <v/>
       </c>
-      <c r="D6" s="58">
+      <c r="D6" s="60">
         <f>(SUMPRODUCT('DCF Valuation'!$I$12:$O$12,(1+$B6)^(-'DCF Valuation'!$I$13:$O$13))+('DCF Valuation'!$O$12*(1+D$5)/($B6-D$5))*(1+$B6)^(-7)+'DCF Valuation'!$C$24)/'DCF Valuation'!$C$26</f>
         <v/>
       </c>
-      <c r="E6" s="58">
+      <c r="E6" s="60">
         <f>(SUMPRODUCT('DCF Valuation'!$I$12:$O$12,(1+$B6)^(-'DCF Valuation'!$I$13:$O$13))+('DCF Valuation'!$O$12*(1+E$5)/($B6-E$5))*(1+$B6)^(-7)+'DCF Valuation'!$C$24)/'DCF Valuation'!$C$26</f>
         <v/>
       </c>
-      <c r="F6" s="58">
+      <c r="F6" s="60">
         <f>(SUMPRODUCT('DCF Valuation'!$I$12:$O$12,(1+$B6)^(-'DCF Valuation'!$I$13:$O$13))+('DCF Valuation'!$O$12*(1+F$5)/($B6-F$5))*(1+$B6)^(-7)+'DCF Valuation'!$C$24)/'DCF Valuation'!$C$26</f>
         <v/>
       </c>
-      <c r="G6" s="58">
+      <c r="G6" s="60">
         <f>(SUMPRODUCT('DCF Valuation'!$I$12:$O$12,(1+$B6)^(-'DCF Valuation'!$I$13:$O$13))+('DCF Valuation'!$O$12*(1+G$5)/($B6-G$5))*(1+$B6)^(-7)+'DCF Valuation'!$C$24)/'DCF Valuation'!$C$26</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="57">
-        <f>'Assumptions'!C39+0.01</f>
-        <v/>
-      </c>
-      <c r="C7" s="58">
+      <c r="B7" s="59">
+        <f>'Assumptions'!C42+0.01</f>
+        <v/>
+      </c>
+      <c r="C7" s="60">
         <f>(SUMPRODUCT('DCF Valuation'!$I$12:$O$12,(1+$B7)^(-'DCF Valuation'!$I$13:$O$13))+('DCF Valuation'!$O$12*(1+C$5)/($B7-C$5))*(1+$B7)^(-7)+'DCF Valuation'!$C$24)/'DCF Valuation'!$C$26</f>
         <v/>
       </c>
-      <c r="D7" s="58">
+      <c r="D7" s="60">
         <f>(SUMPRODUCT('DCF Valuation'!$I$12:$O$12,(1+$B7)^(-'DCF Valuation'!$I$13:$O$13))+('DCF Valuation'!$O$12*(1+D$5)/($B7-D$5))*(1+$B7)^(-7)+'DCF Valuation'!$C$24)/'DCF Valuation'!$C$26</f>
         <v/>
       </c>
-      <c r="E7" s="58">
+      <c r="E7" s="60">
         <f>(SUMPRODUCT('DCF Valuation'!$I$12:$O$12,(1+$B7)^(-'DCF Valuation'!$I$13:$O$13))+('DCF Valuation'!$O$12*(1+E$5)/($B7-E$5))*(1+$B7)^(-7)+'DCF Valuation'!$C$24)/'DCF Valuation'!$C$26</f>
         <v/>
       </c>
-      <c r="F7" s="58">
+      <c r="F7" s="60">
         <f>(SUMPRODUCT('DCF Valuation'!$I$12:$O$12,(1+$B7)^(-'DCF Valuation'!$I$13:$O$13))+('DCF Valuation'!$O$12*(1+F$5)/($B7-F$5))*(1+$B7)^(-7)+'DCF Valuation'!$C$24)/'DCF Valuation'!$C$26</f>
         <v/>
       </c>
-      <c r="G7" s="58">
+      <c r="G7" s="60">
         <f>(SUMPRODUCT('DCF Valuation'!$I$12:$O$12,(1+$B7)^(-'DCF Valuation'!$I$13:$O$13))+('DCF Valuation'!$O$12*(1+G$5)/($B7-G$5))*(1+$B7)^(-7)+'DCF Valuation'!$C$24)/'DCF Valuation'!$C$26</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="57">
-        <f>'Assumptions'!C39+0.0</f>
-        <v/>
-      </c>
-      <c r="C8" s="58">
+      <c r="B8" s="59">
+        <f>'Assumptions'!C42+0.0</f>
+        <v/>
+      </c>
+      <c r="C8" s="60">
         <f>(SUMPRODUCT('DCF Valuation'!$I$12:$O$12,(1+$B8)^(-'DCF Valuation'!$I$13:$O$13))+('DCF Valuation'!$O$12*(1+C$5)/($B8-C$5))*(1+$B8)^(-7)+'DCF Valuation'!$C$24)/'DCF Valuation'!$C$26</f>
         <v/>
       </c>
-      <c r="D8" s="58">
+      <c r="D8" s="60">
         <f>(SUMPRODUCT('DCF Valuation'!$I$12:$O$12,(1+$B8)^(-'DCF Valuation'!$I$13:$O$13))+('DCF Valuation'!$O$12*(1+D$5)/($B8-D$5))*(1+$B8)^(-7)+'DCF Valuation'!$C$24)/'DCF Valuation'!$C$26</f>
         <v/>
       </c>
-      <c r="E8" s="49">
+      <c r="E8" s="51">
         <f>(SUMPRODUCT('DCF Valuation'!$I$12:$O$12,(1+$B8)^(-'DCF Valuation'!$I$13:$O$13))+('DCF Valuation'!$O$12*(1+E$5)/($B8-E$5))*(1+$B8)^(-7)+'DCF Valuation'!$C$24)/'DCF Valuation'!$C$26</f>
         <v/>
       </c>
-      <c r="F8" s="58">
+      <c r="F8" s="60">
         <f>(SUMPRODUCT('DCF Valuation'!$I$12:$O$12,(1+$B8)^(-'DCF Valuation'!$I$13:$O$13))+('DCF Valuation'!$O$12*(1+F$5)/($B8-F$5))*(1+$B8)^(-7)+'DCF Valuation'!$C$24)/'DCF Valuation'!$C$26</f>
         <v/>
       </c>
-      <c r="G8" s="58">
+      <c r="G8" s="60">
         <f>(SUMPRODUCT('DCF Valuation'!$I$12:$O$12,(1+$B8)^(-'DCF Valuation'!$I$13:$O$13))+('DCF Valuation'!$O$12*(1+G$5)/($B8-G$5))*(1+$B8)^(-7)+'DCF Valuation'!$C$24)/'DCF Valuation'!$C$26</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="57">
-        <f>'Assumptions'!C39+-0.01</f>
-        <v/>
-      </c>
-      <c r="C9" s="58">
+      <c r="B9" s="59">
+        <f>'Assumptions'!C42+-0.01</f>
+        <v/>
+      </c>
+      <c r="C9" s="60">
         <f>(SUMPRODUCT('DCF Valuation'!$I$12:$O$12,(1+$B9)^(-'DCF Valuation'!$I$13:$O$13))+('DCF Valuation'!$O$12*(1+C$5)/($B9-C$5))*(1+$B9)^(-7)+'DCF Valuation'!$C$24)/'DCF Valuation'!$C$26</f>
         <v/>
       </c>
-      <c r="D9" s="58">
+      <c r="D9" s="60">
         <f>(SUMPRODUCT('DCF Valuation'!$I$12:$O$12,(1+$B9)^(-'DCF Valuation'!$I$13:$O$13))+('DCF Valuation'!$O$12*(1+D$5)/($B9-D$5))*(1+$B9)^(-7)+'DCF Valuation'!$C$24)/'DCF Valuation'!$C$26</f>
         <v/>
       </c>
-      <c r="E9" s="58">
+      <c r="E9" s="60">
         <f>(SUMPRODUCT('DCF Valuation'!$I$12:$O$12,(1+$B9)^(-'DCF Valuation'!$I$13:$O$13))+('DCF Valuation'!$O$12*(1+E$5)/($B9-E$5))*(1+$B9)^(-7)+'DCF Valuation'!$C$24)/'DCF Valuation'!$C$26</f>
         <v/>
       </c>
-      <c r="F9" s="58">
+      <c r="F9" s="60">
         <f>(SUMPRODUCT('DCF Valuation'!$I$12:$O$12,(1+$B9)^(-'DCF Valuation'!$I$13:$O$13))+('DCF Valuation'!$O$12*(1+F$5)/($B9-F$5))*(1+$B9)^(-7)+'DCF Valuation'!$C$24)/'DCF Valuation'!$C$26</f>
         <v/>
       </c>
-      <c r="G9" s="58">
+      <c r="G9" s="60">
         <f>(SUMPRODUCT('DCF Valuation'!$I$12:$O$12,(1+$B9)^(-'DCF Valuation'!$I$13:$O$13))+('DCF Valuation'!$O$12*(1+G$5)/($B9-G$5))*(1+$B9)^(-7)+'DCF Valuation'!$C$24)/'DCF Valuation'!$C$26</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="57">
-        <f>'Assumptions'!C39+-0.02</f>
-        <v/>
-      </c>
-      <c r="C10" s="58">
+      <c r="B10" s="59">
+        <f>'Assumptions'!C42+-0.02</f>
+        <v/>
+      </c>
+      <c r="C10" s="60">
         <f>(SUMPRODUCT('DCF Valuation'!$I$12:$O$12,(1+$B10)^(-'DCF Valuation'!$I$13:$O$13))+('DCF Valuation'!$O$12*(1+C$5)/($B10-C$5))*(1+$B10)^(-7)+'DCF Valuation'!$C$24)/'DCF Valuation'!$C$26</f>
         <v/>
       </c>
-      <c r="D10" s="58">
+      <c r="D10" s="60">
         <f>(SUMPRODUCT('DCF Valuation'!$I$12:$O$12,(1+$B10)^(-'DCF Valuation'!$I$13:$O$13))+('DCF Valuation'!$O$12*(1+D$5)/($B10-D$5))*(1+$B10)^(-7)+'DCF Valuation'!$C$24)/'DCF Valuation'!$C$26</f>
         <v/>
       </c>
-      <c r="E10" s="58">
+      <c r="E10" s="60">
         <f>(SUMPRODUCT('DCF Valuation'!$I$12:$O$12,(1+$B10)^(-'DCF Valuation'!$I$13:$O$13))+('DCF Valuation'!$O$12*(1+E$5)/($B10-E$5))*(1+$B10)^(-7)+'DCF Valuation'!$C$24)/'DCF Valuation'!$C$26</f>
         <v/>
       </c>
-      <c r="F10" s="58">
+      <c r="F10" s="60">
         <f>(SUMPRODUCT('DCF Valuation'!$I$12:$O$12,(1+$B10)^(-'DCF Valuation'!$I$13:$O$13))+('DCF Valuation'!$O$12*(1+F$5)/($B10-F$5))*(1+$B10)^(-7)+'DCF Valuation'!$C$24)/'DCF Valuation'!$C$26</f>
         <v/>
       </c>
-      <c r="G10" s="58">
+      <c r="G10" s="60">
         <f>(SUMPRODUCT('DCF Valuation'!$I$12:$O$12,(1+$B10)^(-'DCF Valuation'!$I$13:$O$13))+('DCF Valuation'!$O$12*(1+G$5)/($B10-G$5))*(1+$B10)^(-7)+'DCF Valuation'!$C$24)/'DCF Valuation'!$C$26</f>
         <v/>
       </c>
@@ -8535,7 +9510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O42"/>
+  <dimension ref="A1:O45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -9304,142 +10279,226 @@
         <v>0.08500000000000001</v>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>LT borrowings (% of total debt)</t>
+        </is>
+      </c>
+      <c r="I28" s="14" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="J28" s="14" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="K28" s="14" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="L28" s="14" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="M28" s="14" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="N28" s="14" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="O28" s="14" t="n">
+        <v>0.35</v>
+      </c>
+    </row>
     <row r="29">
-      <c r="A29" s="6" t="inlineStr">
-        <is>
-          <t>WACC &amp; valuation inputs</t>
-        </is>
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Other non-current assets (closing)</t>
+        </is>
+      </c>
+      <c r="I29" s="15" t="n">
+        <v>15500</v>
+      </c>
+      <c r="J29" s="15" t="n">
+        <v>16000</v>
+      </c>
+      <c r="K29" s="15" t="n">
+        <v>16500</v>
+      </c>
+      <c r="L29" s="15" t="n">
+        <v>17000</v>
+      </c>
+      <c r="M29" s="15" t="n">
+        <v>17500</v>
+      </c>
+      <c r="N29" s="15" t="n">
+        <v>18000</v>
+      </c>
+      <c r="O29" s="15" t="n">
+        <v>18500</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>Risk-free rate (10Y India G-Sec)</t>
-        </is>
-      </c>
-      <c r="C30" s="14" t="n">
-        <v>0.068</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="5" t="inlineStr">
-        <is>
-          <t>Levered beta</t>
-        </is>
-      </c>
-      <c r="C31" s="17" t="n">
-        <v>1.25</v>
+          <t>Other non-current liabilities (closing)</t>
+        </is>
+      </c>
+      <c r="I30" s="15" t="n">
+        <v>6200</v>
+      </c>
+      <c r="J30" s="15" t="n">
+        <v>6400</v>
+      </c>
+      <c r="K30" s="15" t="n">
+        <v>6600</v>
+      </c>
+      <c r="L30" s="15" t="n">
+        <v>6800</v>
+      </c>
+      <c r="M30" s="15" t="n">
+        <v>7000</v>
+      </c>
+      <c r="N30" s="15" t="n">
+        <v>7200</v>
+      </c>
+      <c r="O30" s="15" t="n">
+        <v>7400</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="5" t="inlineStr">
-        <is>
-          <t>Equity risk premium</t>
-        </is>
-      </c>
-      <c r="C32" s="14" t="n">
-        <v>0.065</v>
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>WACC &amp; valuation inputs</t>
+        </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>Pre-tax cost of debt</t>
+          <t>Risk-free rate (10Y India G-Sec)</t>
         </is>
       </c>
       <c r="C33" s="14" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.068</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>Marginal tax rate (WACC)</t>
-        </is>
-      </c>
-      <c r="C34" s="14" t="n">
-        <v>0.25</v>
+          <t>Levered beta</t>
+        </is>
+      </c>
+      <c r="C34" s="17" t="n">
+        <v>1.25</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>Target weight of debt</t>
+          <t>Equity risk premium</t>
         </is>
       </c>
       <c r="C35" s="14" t="n">
-        <v>0.15</v>
+        <v>0.065</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>Target weight of equity</t>
+          <t>Pre-tax cost of debt</t>
         </is>
       </c>
       <c r="C36" s="14" t="n">
-        <v>0.85</v>
+        <v>0.08500000000000001</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>Terminal growth rate</t>
+          <t>Marginal tax rate (WACC)</t>
         </is>
       </c>
       <c r="C37" s="14" t="n">
-        <v>0.045</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="4" t="inlineStr">
-        <is>
-          <t>Cost of equity (Ke = Rf + B x ERP)</t>
-        </is>
-      </c>
-      <c r="C38" s="18">
-        <f>'Assumptions'!C30+'Assumptions'!C31*'Assumptions'!C32</f>
-        <v/>
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Target weight of debt</t>
+        </is>
+      </c>
+      <c r="C38" s="14" t="n">
+        <v>0.15</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="4" t="inlineStr">
-        <is>
-          <t>WACC (We*Ke + Wd*Kd*(1-t))</t>
-        </is>
-      </c>
-      <c r="C39" s="19">
-        <f>'Assumptions'!C36*'Assumptions'!C38+'Assumptions'!C35*'Assumptions'!C33*(1-'Assumptions'!C34)</f>
-        <v/>
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>Target weight of equity</t>
+        </is>
+      </c>
+      <c r="C39" s="14" t="n">
+        <v>0.85</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
+          <t>Terminal growth rate</t>
+        </is>
+      </c>
+      <c r="C40" s="14" t="n">
+        <v>0.045</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Cost of equity (Ke = Rf + B x ERP)</t>
+        </is>
+      </c>
+      <c r="C41" s="18">
+        <f>'Assumptions'!C33+'Assumptions'!C34*'Assumptions'!C35</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>WACC (We*Ke + Wd*Kd*(1-t))</t>
+        </is>
+      </c>
+      <c r="C42" s="19">
+        <f>'Assumptions'!C39*'Assumptions'!C41+'Assumptions'!C38*'Assumptions'!C36*(1-'Assumptions'!C37)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
           <t>Shares outstanding (crore)</t>
         </is>
       </c>
-      <c r="C40" s="20" t="n">
+      <c r="C43" s="20" t="n">
         <v>348.05</v>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="5" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
         <is>
           <t>Current market price (INR)</t>
         </is>
       </c>
-      <c r="C41" s="17" t="n">
+      <c r="C44" s="17" t="n">
         <v>403</v>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="5" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
         <is>
           <t>Face value (INR)</t>
         </is>
       </c>
-      <c r="C42" s="17" t="n">
+      <c r="C45" s="17" t="n">
         <v>2</v>
       </c>
     </row>
@@ -9544,7 +10603,7 @@
       <c r="B5" s="15" t="n">
         <v>68000</v>
       </c>
-      <c r="C5" s="47">
+      <c r="C5" s="49">
         <f>'Forecast Financial Statements'!O5</f>
         <v/>
       </c>
@@ -9561,7 +10620,7 @@
       <c r="B6" s="14" t="n">
         <v>0.09</v>
       </c>
-      <c r="C6" s="45">
+      <c r="C6" s="47">
         <f>'Forecast Financial Statements'!O12/'Forecast Financial Statements'!O5</f>
         <v/>
       </c>
@@ -9575,13 +10634,13 @@
           <t>Exit EV/EBITDA multiple (x)</t>
         </is>
       </c>
-      <c r="B7" s="51" t="n">
+      <c r="B7" s="53" t="n">
         <v>14</v>
       </c>
-      <c r="C7" s="51" t="n">
+      <c r="C7" s="53" t="n">
         <v>18</v>
       </c>
-      <c r="D7" s="51" t="n">
+      <c r="D7" s="53" t="n">
         <v>24</v>
       </c>
     </row>
@@ -9594,8 +10653,8 @@
       <c r="B8" s="14" t="n">
         <v>0.155</v>
       </c>
-      <c r="C8" s="45">
-        <f>'Assumptions'!C39</f>
+      <c r="C8" s="47">
+        <f>'Assumptions'!C42</f>
         <v/>
       </c>
       <c r="D8" s="14" t="n">
@@ -9608,15 +10667,15 @@
           <t>FY2033E EBITDA (INR Cr)</t>
         </is>
       </c>
-      <c r="B9" s="44">
+      <c r="B9" s="46">
         <f>B5*B6</f>
         <v/>
       </c>
-      <c r="C9" s="44">
+      <c r="C9" s="46">
         <f>C5*C6</f>
         <v/>
       </c>
-      <c r="D9" s="44">
+      <c r="D9" s="46">
         <f>D5*D6</f>
         <v/>
       </c>
@@ -9627,15 +10686,15 @@
           <t>Terminal EV (INR Cr)</t>
         </is>
       </c>
-      <c r="B10" s="44">
+      <c r="B10" s="46">
         <f>B9*B7</f>
         <v/>
       </c>
-      <c r="C10" s="44">
+      <c r="C10" s="46">
         <f>C9*C7</f>
         <v/>
       </c>
-      <c r="D10" s="44">
+      <c r="D10" s="46">
         <f>D9*D7</f>
         <v/>
       </c>
@@ -9646,15 +10705,15 @@
           <t>PV of EV (discounted 7y)</t>
         </is>
       </c>
-      <c r="B11" s="44">
+      <c r="B11" s="46">
         <f>B10/(1+B8)^7</f>
         <v/>
       </c>
-      <c r="C11" s="44">
+      <c r="C11" s="46">
         <f>C10/(1+C8)^7</f>
         <v/>
       </c>
-      <c r="D11" s="44">
+      <c r="D11" s="46">
         <f>D10/(1+D8)^7</f>
         <v/>
       </c>
@@ -9665,16 +10724,16 @@
           <t>Less: net debt (FY26)</t>
         </is>
       </c>
-      <c r="B12" s="47">
-        <f>'Forecast Financial Statements'!H37-'Forecast Financial Statements'!H32</f>
-        <v/>
-      </c>
-      <c r="C12" s="47">
-        <f>'Forecast Financial Statements'!H37-'Forecast Financial Statements'!H32</f>
-        <v/>
-      </c>
-      <c r="D12" s="47">
-        <f>'Forecast Financial Statements'!H37-'Forecast Financial Statements'!H32</f>
+      <c r="B12" s="49">
+        <f>'Forecast Financial Statements'!H63-'Forecast Financial Statements'!H58</f>
+        <v/>
+      </c>
+      <c r="C12" s="49">
+        <f>'Forecast Financial Statements'!H63-'Forecast Financial Statements'!H58</f>
+        <v/>
+      </c>
+      <c r="D12" s="49">
+        <f>'Forecast Financial Statements'!H63-'Forecast Financial Statements'!H58</f>
         <v/>
       </c>
     </row>
@@ -9684,15 +10743,15 @@
           <t>Equity value (INR Cr)</t>
         </is>
       </c>
-      <c r="B13" s="44">
+      <c r="B13" s="46">
         <f>B11-B12</f>
         <v/>
       </c>
-      <c r="C13" s="44">
+      <c r="C13" s="46">
         <f>C11-C12</f>
         <v/>
       </c>
-      <c r="D13" s="44">
+      <c r="D13" s="46">
         <f>D11-D12</f>
         <v/>
       </c>
@@ -9703,16 +10762,16 @@
           <t>Target price (INR)</t>
         </is>
       </c>
-      <c r="B14" s="49">
-        <f>B13/'Assumptions'!C40</f>
-        <v/>
-      </c>
-      <c r="C14" s="49">
-        <f>C13/'Assumptions'!C40</f>
-        <v/>
-      </c>
-      <c r="D14" s="49">
-        <f>D13/'Assumptions'!C40</f>
+      <c r="B14" s="51">
+        <f>B13/'Assumptions'!C43</f>
+        <v/>
+      </c>
+      <c r="C14" s="51">
+        <f>C13/'Assumptions'!C43</f>
+        <v/>
+      </c>
+      <c r="D14" s="51">
+        <f>D13/'Assumptions'!C43</f>
         <v/>
       </c>
     </row>
@@ -9738,7 +10797,7 @@
           <t>Probability-weighted target price (INR)</t>
         </is>
       </c>
-      <c r="B17" s="56">
+      <c r="B17" s="58">
         <f>SUMPRODUCT(B14:D14,B15:D15)</f>
         <v/>
       </c>
@@ -9783,117 +10842,117 @@
       <c r="H1" s="1" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="59" t="inlineStr">
+      <c r="A3" s="61" t="inlineStr">
         <is>
           <t>DCF value / share (INR)</t>
         </is>
       </c>
-      <c r="B3" s="59" t="inlineStr">
+      <c r="B3" s="61" t="inlineStr">
         <is>
           <t>Current price (INR)</t>
         </is>
       </c>
-      <c r="D3" s="59" t="inlineStr">
+      <c r="D3" s="61" t="inlineStr">
         <is>
           <t>Upside / (downside)</t>
         </is>
       </c>
-      <c r="E3" s="59" t="inlineStr">
+      <c r="E3" s="61" t="inlineStr">
         <is>
           <t>Prob-weighted TP (INR)</t>
         </is>
       </c>
-      <c r="G3" s="59" t="inlineStr">
+      <c r="G3" s="61" t="inlineStr">
         <is>
           <t>Avg relative TP (INR)</t>
         </is>
       </c>
-      <c r="H3" s="59" t="inlineStr">
+      <c r="H3" s="61" t="inlineStr">
         <is>
           <t>WACC</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="60">
+      <c r="A4" s="62">
         <f>'DCF Valuation'!C27</f>
         <v/>
       </c>
-      <c r="B4" s="60">
+      <c r="B4" s="62">
         <f>'DCF Valuation'!C28</f>
         <v/>
       </c>
-      <c r="D4" s="61">
+      <c r="D4" s="63">
         <f>'DCF Valuation'!C29</f>
         <v/>
       </c>
-      <c r="E4" s="60">
+      <c r="E4" s="62">
         <f>'Scenario Analysis'!B17</f>
         <v/>
       </c>
-      <c r="G4" s="60">
+      <c r="G4" s="62">
         <f>'Relative Valuation'!C29</f>
         <v/>
       </c>
-      <c r="H4" s="61">
-        <f>'Assumptions'!C39</f>
+      <c r="H4" s="63">
+        <f>'Assumptions'!C42</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="59" t="inlineStr">
+      <c r="A6" s="61" t="inlineStr">
         <is>
           <t>FY27E revenue (INR Cr)</t>
         </is>
       </c>
-      <c r="B6" s="59" t="inlineStr">
+      <c r="B6" s="61" t="inlineStr">
         <is>
           <t>FY33E revenue (INR Cr)</t>
         </is>
       </c>
-      <c r="D6" s="59" t="inlineStr">
+      <c r="D6" s="61" t="inlineStr">
         <is>
           <t>FY27E EBITDA margin</t>
         </is>
       </c>
-      <c r="E6" s="59" t="inlineStr">
+      <c r="E6" s="61" t="inlineStr">
         <is>
           <t>FY33E EBITDA margin</t>
         </is>
       </c>
-      <c r="G6" s="59" t="inlineStr">
+      <c r="G6" s="61" t="inlineStr">
         <is>
           <t>FY26 order book (INR Cr)</t>
         </is>
       </c>
-      <c r="H6" s="59" t="inlineStr">
+      <c r="H6" s="61" t="inlineStr">
         <is>
           <t>FY33E PAT (INR Cr)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="62">
+      <c r="A7" s="64">
         <f>'Forecast Financial Statements'!I5</f>
         <v/>
       </c>
-      <c r="B7" s="62">
+      <c r="B7" s="64">
         <f>'Forecast Financial Statements'!O5</f>
         <v/>
       </c>
-      <c r="D7" s="61">
+      <c r="D7" s="63">
         <f>'Forecast Financial Statements'!I12/'Forecast Financial Statements'!I5</f>
         <v/>
       </c>
-      <c r="E7" s="61">
+      <c r="E7" s="63">
         <f>'Forecast Financial Statements'!O12/'Forecast Financial Statements'!O5</f>
         <v/>
       </c>
-      <c r="G7" s="62">
+      <c r="G7" s="64">
         <f>'Revenue Build-up'!H9</f>
         <v/>
       </c>
-      <c r="H7" s="62">
+      <c r="H7" s="64">
         <f>'Forecast Financial Statements'!O20</f>
         <v/>
       </c>
@@ -9906,56 +10965,56 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="63" t="inlineStr">
+      <c r="A10" s="65" t="inlineStr">
         <is>
           <t>PV of explicit FCFF</t>
         </is>
       </c>
-      <c r="B10" s="47">
+      <c r="B10" s="49">
         <f>'DCF Valuation'!C18</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="63" t="inlineStr">
+      <c r="A11" s="65" t="inlineStr">
         <is>
           <t>PV of terminal value</t>
         </is>
       </c>
-      <c r="B11" s="47">
+      <c r="B11" s="49">
         <f>'DCF Valuation'!C22</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="63" t="inlineStr">
+      <c r="A12" s="65" t="inlineStr">
         <is>
           <t>Enterprise value</t>
         </is>
       </c>
-      <c r="B12" s="47">
+      <c r="B12" s="49">
         <f>'DCF Valuation'!C23</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="63" t="inlineStr">
+      <c r="A13" s="65" t="inlineStr">
         <is>
           <t>Less: net debt</t>
         </is>
       </c>
-      <c r="B13" s="47">
+      <c r="B13" s="49">
         <f>'DCF Valuation'!C24</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="63" t="inlineStr">
+      <c r="A14" s="65" t="inlineStr">
         <is>
           <t>Equity value</t>
         </is>
       </c>
-      <c r="B14" s="47">
+      <c r="B14" s="49">
         <f>'DCF Valuation'!C25</f>
         <v/>
       </c>
@@ -10022,7 +11081,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="59" t="inlineStr">
+      <c r="A4" s="61" t="inlineStr">
         <is>
           <t>Check</t>
         </is>
@@ -10080,36 +11139,60 @@
           <t>Balance sheet balances (TA = TE&amp;L)</t>
         </is>
       </c>
-      <c r="H5" s="64">
-        <f>IF(ABS('Forecast Financial Statements'!H34-'Forecast Financial Statements'!H41)&lt;0.5,"OK","REVIEW")</f>
-        <v/>
-      </c>
-      <c r="I5" s="64">
-        <f>IF(ABS('Forecast Financial Statements'!I34-'Forecast Financial Statements'!I41)&lt;0.5,"OK","REVIEW")</f>
-        <v/>
-      </c>
-      <c r="J5" s="64">
-        <f>IF(ABS('Forecast Financial Statements'!J34-'Forecast Financial Statements'!J41)&lt;0.5,"OK","REVIEW")</f>
-        <v/>
-      </c>
-      <c r="K5" s="64">
-        <f>IF(ABS('Forecast Financial Statements'!K34-'Forecast Financial Statements'!K41)&lt;0.5,"OK","REVIEW")</f>
-        <v/>
-      </c>
-      <c r="L5" s="64">
-        <f>IF(ABS('Forecast Financial Statements'!L34-'Forecast Financial Statements'!L41)&lt;0.5,"OK","REVIEW")</f>
-        <v/>
-      </c>
-      <c r="M5" s="64">
-        <f>IF(ABS('Forecast Financial Statements'!M34-'Forecast Financial Statements'!M41)&lt;0.5,"OK","REVIEW")</f>
-        <v/>
-      </c>
-      <c r="N5" s="64">
-        <f>IF(ABS('Forecast Financial Statements'!N34-'Forecast Financial Statements'!N41)&lt;0.5,"OK","REVIEW")</f>
-        <v/>
-      </c>
-      <c r="O5" s="64">
-        <f>IF(ABS('Forecast Financial Statements'!O34-'Forecast Financial Statements'!O41)&lt;0.5,"OK","REVIEW")</f>
+      <c r="B5" s="66">
+        <f>IF(ABS('Forecast Financial Statements'!B61-'Forecast Financial Statements'!B42)&lt;0.5,"OK","REVIEW")</f>
+        <v/>
+      </c>
+      <c r="C5" s="66">
+        <f>IF(ABS('Forecast Financial Statements'!C61-'Forecast Financial Statements'!C42)&lt;0.5,"OK","REVIEW")</f>
+        <v/>
+      </c>
+      <c r="D5" s="66">
+        <f>IF(ABS('Forecast Financial Statements'!D61-'Forecast Financial Statements'!D42)&lt;0.5,"OK","REVIEW")</f>
+        <v/>
+      </c>
+      <c r="E5" s="66">
+        <f>IF(ABS('Forecast Financial Statements'!E61-'Forecast Financial Statements'!E42)&lt;0.5,"OK","REVIEW")</f>
+        <v/>
+      </c>
+      <c r="F5" s="66">
+        <f>IF(ABS('Forecast Financial Statements'!F61-'Forecast Financial Statements'!F42)&lt;0.5,"OK","REVIEW")</f>
+        <v/>
+      </c>
+      <c r="G5" s="66">
+        <f>IF(ABS('Forecast Financial Statements'!G61-'Forecast Financial Statements'!G42)&lt;0.5,"OK","REVIEW")</f>
+        <v/>
+      </c>
+      <c r="H5" s="66">
+        <f>IF(ABS('Forecast Financial Statements'!H61-'Forecast Financial Statements'!H42)&lt;0.5,"OK","REVIEW")</f>
+        <v/>
+      </c>
+      <c r="I5" s="66">
+        <f>IF(ABS('Forecast Financial Statements'!I61-'Forecast Financial Statements'!I42)&lt;0.5,"OK","REVIEW")</f>
+        <v/>
+      </c>
+      <c r="J5" s="66">
+        <f>IF(ABS('Forecast Financial Statements'!J61-'Forecast Financial Statements'!J42)&lt;0.5,"OK","REVIEW")</f>
+        <v/>
+      </c>
+      <c r="K5" s="66">
+        <f>IF(ABS('Forecast Financial Statements'!K61-'Forecast Financial Statements'!K42)&lt;0.5,"OK","REVIEW")</f>
+        <v/>
+      </c>
+      <c r="L5" s="66">
+        <f>IF(ABS('Forecast Financial Statements'!L61-'Forecast Financial Statements'!L42)&lt;0.5,"OK","REVIEW")</f>
+        <v/>
+      </c>
+      <c r="M5" s="66">
+        <f>IF(ABS('Forecast Financial Statements'!M61-'Forecast Financial Statements'!M42)&lt;0.5,"OK","REVIEW")</f>
+        <v/>
+      </c>
+      <c r="N5" s="66">
+        <f>IF(ABS('Forecast Financial Statements'!N61-'Forecast Financial Statements'!N42)&lt;0.5,"OK","REVIEW")</f>
+        <v/>
+      </c>
+      <c r="O5" s="66">
+        <f>IF(ABS('Forecast Financial Statements'!O61-'Forecast Financial Statements'!O42)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
     </row>
@@ -10119,32 +11202,32 @@
           <t>Cash: Balance sheet = Cash flow stmt</t>
         </is>
       </c>
-      <c r="I6" s="64">
-        <f>IF(ABS('Forecast Financial Statements'!I32-'Cash Flow Statement'!I25)&lt;0.5,"OK","REVIEW")</f>
-        <v/>
-      </c>
-      <c r="J6" s="64">
-        <f>IF(ABS('Forecast Financial Statements'!J32-'Cash Flow Statement'!J25)&lt;0.5,"OK","REVIEW")</f>
-        <v/>
-      </c>
-      <c r="K6" s="64">
-        <f>IF(ABS('Forecast Financial Statements'!K32-'Cash Flow Statement'!K25)&lt;0.5,"OK","REVIEW")</f>
-        <v/>
-      </c>
-      <c r="L6" s="64">
-        <f>IF(ABS('Forecast Financial Statements'!L32-'Cash Flow Statement'!L25)&lt;0.5,"OK","REVIEW")</f>
-        <v/>
-      </c>
-      <c r="M6" s="64">
-        <f>IF(ABS('Forecast Financial Statements'!M32-'Cash Flow Statement'!M25)&lt;0.5,"OK","REVIEW")</f>
-        <v/>
-      </c>
-      <c r="N6" s="64">
-        <f>IF(ABS('Forecast Financial Statements'!N32-'Cash Flow Statement'!N25)&lt;0.5,"OK","REVIEW")</f>
-        <v/>
-      </c>
-      <c r="O6" s="64">
-        <f>IF(ABS('Forecast Financial Statements'!O32-'Cash Flow Statement'!O25)&lt;0.5,"OK","REVIEW")</f>
+      <c r="I6" s="66">
+        <f>IF(ABS('Forecast Financial Statements'!I58-'Cash Flow Statement'!I25)&lt;0.5,"OK","REVIEW")</f>
+        <v/>
+      </c>
+      <c r="J6" s="66">
+        <f>IF(ABS('Forecast Financial Statements'!J58-'Cash Flow Statement'!J25)&lt;0.5,"OK","REVIEW")</f>
+        <v/>
+      </c>
+      <c r="K6" s="66">
+        <f>IF(ABS('Forecast Financial Statements'!K58-'Cash Flow Statement'!K25)&lt;0.5,"OK","REVIEW")</f>
+        <v/>
+      </c>
+      <c r="L6" s="66">
+        <f>IF(ABS('Forecast Financial Statements'!L58-'Cash Flow Statement'!L25)&lt;0.5,"OK","REVIEW")</f>
+        <v/>
+      </c>
+      <c r="M6" s="66">
+        <f>IF(ABS('Forecast Financial Statements'!M58-'Cash Flow Statement'!M25)&lt;0.5,"OK","REVIEW")</f>
+        <v/>
+      </c>
+      <c r="N6" s="66">
+        <f>IF(ABS('Forecast Financial Statements'!N58-'Cash Flow Statement'!N25)&lt;0.5,"OK","REVIEW")</f>
+        <v/>
+      </c>
+      <c r="O6" s="66">
+        <f>IF(ABS('Forecast Financial Statements'!O58-'Cash Flow Statement'!O25)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
     </row>
@@ -10154,32 +11237,32 @@
           <t>Retained earnings roll-forward ties</t>
         </is>
       </c>
-      <c r="I7" s="64">
-        <f>IF(ABS('Forecast Financial Statements'!I36-'Equity Schedule'!I10)&lt;0.5,"OK","REVIEW")</f>
-        <v/>
-      </c>
-      <c r="J7" s="64">
-        <f>IF(ABS('Forecast Financial Statements'!J36-'Equity Schedule'!J10)&lt;0.5,"OK","REVIEW")</f>
-        <v/>
-      </c>
-      <c r="K7" s="64">
-        <f>IF(ABS('Forecast Financial Statements'!K36-'Equity Schedule'!K10)&lt;0.5,"OK","REVIEW")</f>
-        <v/>
-      </c>
-      <c r="L7" s="64">
-        <f>IF(ABS('Forecast Financial Statements'!L36-'Equity Schedule'!L10)&lt;0.5,"OK","REVIEW")</f>
-        <v/>
-      </c>
-      <c r="M7" s="64">
-        <f>IF(ABS('Forecast Financial Statements'!M36-'Equity Schedule'!M10)&lt;0.5,"OK","REVIEW")</f>
-        <v/>
-      </c>
-      <c r="N7" s="64">
-        <f>IF(ABS('Forecast Financial Statements'!N36-'Equity Schedule'!N10)&lt;0.5,"OK","REVIEW")</f>
-        <v/>
-      </c>
-      <c r="O7" s="64">
-        <f>IF(ABS('Forecast Financial Statements'!O36-'Equity Schedule'!O10)&lt;0.5,"OK","REVIEW")</f>
+      <c r="I7" s="66">
+        <f>IF(ABS('Forecast Financial Statements'!I29-'Equity Schedule'!I10)&lt;0.5,"OK","REVIEW")</f>
+        <v/>
+      </c>
+      <c r="J7" s="66">
+        <f>IF(ABS('Forecast Financial Statements'!J29-'Equity Schedule'!J10)&lt;0.5,"OK","REVIEW")</f>
+        <v/>
+      </c>
+      <c r="K7" s="66">
+        <f>IF(ABS('Forecast Financial Statements'!K29-'Equity Schedule'!K10)&lt;0.5,"OK","REVIEW")</f>
+        <v/>
+      </c>
+      <c r="L7" s="66">
+        <f>IF(ABS('Forecast Financial Statements'!L29-'Equity Schedule'!L10)&lt;0.5,"OK","REVIEW")</f>
+        <v/>
+      </c>
+      <c r="M7" s="66">
+        <f>IF(ABS('Forecast Financial Statements'!M29-'Equity Schedule'!M10)&lt;0.5,"OK","REVIEW")</f>
+        <v/>
+      </c>
+      <c r="N7" s="66">
+        <f>IF(ABS('Forecast Financial Statements'!N29-'Equity Schedule'!N10)&lt;0.5,"OK","REVIEW")</f>
+        <v/>
+      </c>
+      <c r="O7" s="66">
+        <f>IF(ABS('Forecast Financial Statements'!O29-'Equity Schedule'!O10)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
     </row>
@@ -10189,32 +11272,32 @@
           <t>Debt roll-forward ties</t>
         </is>
       </c>
-      <c r="I8" s="64">
-        <f>IF(ABS('Forecast Financial Statements'!I37-'Debt Schedule'!I9)&lt;0.5,"OK","REVIEW")</f>
-        <v/>
-      </c>
-      <c r="J8" s="64">
-        <f>IF(ABS('Forecast Financial Statements'!J37-'Debt Schedule'!J9)&lt;0.5,"OK","REVIEW")</f>
-        <v/>
-      </c>
-      <c r="K8" s="64">
-        <f>IF(ABS('Forecast Financial Statements'!K37-'Debt Schedule'!K9)&lt;0.5,"OK","REVIEW")</f>
-        <v/>
-      </c>
-      <c r="L8" s="64">
-        <f>IF(ABS('Forecast Financial Statements'!L37-'Debt Schedule'!L9)&lt;0.5,"OK","REVIEW")</f>
-        <v/>
-      </c>
-      <c r="M8" s="64">
-        <f>IF(ABS('Forecast Financial Statements'!M37-'Debt Schedule'!M9)&lt;0.5,"OK","REVIEW")</f>
-        <v/>
-      </c>
-      <c r="N8" s="64">
-        <f>IF(ABS('Forecast Financial Statements'!N37-'Debt Schedule'!N9)&lt;0.5,"OK","REVIEW")</f>
-        <v/>
-      </c>
-      <c r="O8" s="64">
-        <f>IF(ABS('Forecast Financial Statements'!O37-'Debt Schedule'!O9)&lt;0.5,"OK","REVIEW")</f>
+      <c r="I8" s="66">
+        <f>IF(ABS('Forecast Financial Statements'!I63-'Debt Schedule'!I9)&lt;0.5,"OK","REVIEW")</f>
+        <v/>
+      </c>
+      <c r="J8" s="66">
+        <f>IF(ABS('Forecast Financial Statements'!J63-'Debt Schedule'!J9)&lt;0.5,"OK","REVIEW")</f>
+        <v/>
+      </c>
+      <c r="K8" s="66">
+        <f>IF(ABS('Forecast Financial Statements'!K63-'Debt Schedule'!K9)&lt;0.5,"OK","REVIEW")</f>
+        <v/>
+      </c>
+      <c r="L8" s="66">
+        <f>IF(ABS('Forecast Financial Statements'!L63-'Debt Schedule'!L9)&lt;0.5,"OK","REVIEW")</f>
+        <v/>
+      </c>
+      <c r="M8" s="66">
+        <f>IF(ABS('Forecast Financial Statements'!M63-'Debt Schedule'!M9)&lt;0.5,"OK","REVIEW")</f>
+        <v/>
+      </c>
+      <c r="N8" s="66">
+        <f>IF(ABS('Forecast Financial Statements'!N63-'Debt Schedule'!N9)&lt;0.5,"OK","REVIEW")</f>
+        <v/>
+      </c>
+      <c r="O8" s="66">
+        <f>IF(ABS('Forecast Financial Statements'!O63-'Debt Schedule'!O9)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
     </row>
@@ -10224,31 +11307,31 @@
           <t>Depreciation ties to P&amp;L</t>
         </is>
       </c>
-      <c r="I9" s="64">
+      <c r="I9" s="66">
         <f>IF(ABS('Forecast Financial Statements'!I13-'Depreciation Schedule'!I8)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="J9" s="64">
+      <c r="J9" s="66">
         <f>IF(ABS('Forecast Financial Statements'!J13-'Depreciation Schedule'!J8)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="K9" s="64">
+      <c r="K9" s="66">
         <f>IF(ABS('Forecast Financial Statements'!K13-'Depreciation Schedule'!K8)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="L9" s="64">
+      <c r="L9" s="66">
         <f>IF(ABS('Forecast Financial Statements'!L13-'Depreciation Schedule'!L8)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="M9" s="64">
+      <c r="M9" s="66">
         <f>IF(ABS('Forecast Financial Statements'!M13-'Depreciation Schedule'!M8)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="N9" s="64">
+      <c r="N9" s="66">
         <f>IF(ABS('Forecast Financial Statements'!N13-'Depreciation Schedule'!N8)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="O9" s="64">
+      <c r="O9" s="66">
         <f>IF(ABS('Forecast Financial Statements'!O13-'Depreciation Schedule'!O8)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
@@ -10259,31 +11342,31 @@
           <t>Revenue ties to Revenue Build-up</t>
         </is>
       </c>
-      <c r="I10" s="64">
+      <c r="I10" s="66">
         <f>IF(ABS('Forecast Financial Statements'!I5-'Revenue Build-up'!I11)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="J10" s="64">
+      <c r="J10" s="66">
         <f>IF(ABS('Forecast Financial Statements'!J5-'Revenue Build-up'!J11)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="K10" s="64">
+      <c r="K10" s="66">
         <f>IF(ABS('Forecast Financial Statements'!K5-'Revenue Build-up'!K11)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="L10" s="64">
+      <c r="L10" s="66">
         <f>IF(ABS('Forecast Financial Statements'!L5-'Revenue Build-up'!L11)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="M10" s="64">
+      <c r="M10" s="66">
         <f>IF(ABS('Forecast Financial Statements'!M5-'Revenue Build-up'!M11)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="N10" s="64">
+      <c r="N10" s="66">
         <f>IF(ABS('Forecast Financial Statements'!N5-'Revenue Build-up'!N11)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="O10" s="64">
+      <c r="O10" s="66">
         <f>IF(ABS('Forecast Financial Statements'!O5-'Revenue Build-up'!O11)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
@@ -10294,32 +11377,32 @@
           <t>Net fixed assets tie to FA schedule</t>
         </is>
       </c>
-      <c r="I11" s="64">
-        <f>IF(ABS('Forecast Financial Statements'!I26-'Fixed Asset Schedule'!I10)&lt;0.5,"OK","REVIEW")</f>
-        <v/>
-      </c>
-      <c r="J11" s="64">
-        <f>IF(ABS('Forecast Financial Statements'!J26-'Fixed Asset Schedule'!J10)&lt;0.5,"OK","REVIEW")</f>
-        <v/>
-      </c>
-      <c r="K11" s="64">
-        <f>IF(ABS('Forecast Financial Statements'!K26-'Fixed Asset Schedule'!K10)&lt;0.5,"OK","REVIEW")</f>
-        <v/>
-      </c>
-      <c r="L11" s="64">
-        <f>IF(ABS('Forecast Financial Statements'!L26-'Fixed Asset Schedule'!L10)&lt;0.5,"OK","REVIEW")</f>
-        <v/>
-      </c>
-      <c r="M11" s="64">
-        <f>IF(ABS('Forecast Financial Statements'!M26-'Fixed Asset Schedule'!M10)&lt;0.5,"OK","REVIEW")</f>
-        <v/>
-      </c>
-      <c r="N11" s="64">
-        <f>IF(ABS('Forecast Financial Statements'!N26-'Fixed Asset Schedule'!N10)&lt;0.5,"OK","REVIEW")</f>
-        <v/>
-      </c>
-      <c r="O11" s="64">
-        <f>IF(ABS('Forecast Financial Statements'!O26-'Fixed Asset Schedule'!O10)&lt;0.5,"OK","REVIEW")</f>
+      <c r="I11" s="66">
+        <f>IF(ABS('Forecast Financial Statements'!I47-'Fixed Asset Schedule'!I10)&lt;0.5,"OK","REVIEW")</f>
+        <v/>
+      </c>
+      <c r="J11" s="66">
+        <f>IF(ABS('Forecast Financial Statements'!J47-'Fixed Asset Schedule'!J10)&lt;0.5,"OK","REVIEW")</f>
+        <v/>
+      </c>
+      <c r="K11" s="66">
+        <f>IF(ABS('Forecast Financial Statements'!K47-'Fixed Asset Schedule'!K10)&lt;0.5,"OK","REVIEW")</f>
+        <v/>
+      </c>
+      <c r="L11" s="66">
+        <f>IF(ABS('Forecast Financial Statements'!L47-'Fixed Asset Schedule'!L10)&lt;0.5,"OK","REVIEW")</f>
+        <v/>
+      </c>
+      <c r="M11" s="66">
+        <f>IF(ABS('Forecast Financial Statements'!M47-'Fixed Asset Schedule'!M10)&lt;0.5,"OK","REVIEW")</f>
+        <v/>
+      </c>
+      <c r="N11" s="66">
+        <f>IF(ABS('Forecast Financial Statements'!N47-'Fixed Asset Schedule'!N10)&lt;0.5,"OK","REVIEW")</f>
+        <v/>
+      </c>
+      <c r="O11" s="66">
+        <f>IF(ABS('Forecast Financial Statements'!O47-'Fixed Asset Schedule'!O10)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
     </row>
@@ -10329,7 +11412,7 @@
           <t>Historical balance check max |diff| (FY20-26)</t>
         </is>
       </c>
-      <c r="C13" s="65">
+      <c r="C13" s="67">
         <f>MAX(ABS('Historical Financial Statements'!B38),ABS('Historical Financial Statements'!C38),ABS('Historical Financial Statements'!D38),ABS('Historical Financial Statements'!E38),ABS('Historical Financial Statements'!F38),ABS('Historical Financial Statements'!G38),ABS('Historical Financial Statements'!H38))</f>
         <v/>
       </c>
@@ -10340,8 +11423,8 @@
           <t>Forecast balance check max |diff|</t>
         </is>
       </c>
-      <c r="C14" s="65">
-        <f>MAX(ABS('Forecast Financial Statements'!I42),ABS('Forecast Financial Statements'!J42),ABS('Forecast Financial Statements'!K42),ABS('Forecast Financial Statements'!L42),ABS('Forecast Financial Statements'!M42),ABS('Forecast Financial Statements'!N42),ABS('Forecast Financial Statements'!O42))</f>
+      <c r="C14" s="67">
+        <f>MAX(ABS('Forecast Financial Statements'!I62),ABS('Forecast Financial Statements'!J62),ABS('Forecast Financial Statements'!K62),ABS('Forecast Financial Statements'!L62),ABS('Forecast Financial Statements'!M62),ABS('Forecast Financial Statements'!N62),ABS('Forecast Financial Statements'!O62))</f>
         <v/>
       </c>
     </row>
@@ -10363,7 +11446,7 @@
           <t>Overall model status</t>
         </is>
       </c>
-      <c r="C16" s="66">
+      <c r="C16" s="68">
         <f>IF(COUNTIF(B5:O11,"REVIEW")=0,"ALL CHECKS PASS","REVIEW REQUIRED")</f>
         <v/>
       </c>
@@ -11007,31 +12090,31 @@
         </is>
       </c>
       <c r="B21" s="26">
-        <f>B20/'Assumptions'!C40</f>
+        <f>B20/'Assumptions'!C43</f>
         <v/>
       </c>
       <c r="C21" s="26">
-        <f>C20/'Assumptions'!C40</f>
+        <f>C20/'Assumptions'!C43</f>
         <v/>
       </c>
       <c r="D21" s="26">
-        <f>D20/'Assumptions'!C40</f>
+        <f>D20/'Assumptions'!C43</f>
         <v/>
       </c>
       <c r="E21" s="26">
-        <f>E20/'Assumptions'!C40</f>
+        <f>E20/'Assumptions'!C43</f>
         <v/>
       </c>
       <c r="F21" s="26">
-        <f>F20/'Assumptions'!C40</f>
+        <f>F20/'Assumptions'!C43</f>
         <v/>
       </c>
       <c r="G21" s="26">
-        <f>G20/'Assumptions'!C40</f>
+        <f>G20/'Assumptions'!C43</f>
         <v/>
       </c>
       <c r="H21" s="26">
-        <f>H20/'Assumptions'!C40</f>
+        <f>H20/'Assumptions'!C43</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix standalone/consolidated inconsistency: roll order book on standalone revenue (both sheets) and bridge standalone->consolidated revenue for the P&L
</commit_message>
<xml_diff>
--- a/BHEL_Financial_Model.xlsx
+++ b/BHEL_Financial_Model.xlsx
@@ -1720,31 +1720,31 @@
         </is>
       </c>
       <c r="I7" s="33">
-        <f>'Assumptions'!I34</f>
+        <f>'Assumptions'!I35</f>
         <v/>
       </c>
       <c r="J7" s="33">
-        <f>'Assumptions'!J34</f>
+        <f>'Assumptions'!J35</f>
         <v/>
       </c>
       <c r="K7" s="33">
-        <f>'Assumptions'!K34</f>
+        <f>'Assumptions'!K35</f>
         <v/>
       </c>
       <c r="L7" s="33">
-        <f>'Assumptions'!L34</f>
+        <f>'Assumptions'!L35</f>
         <v/>
       </c>
       <c r="M7" s="33">
-        <f>'Assumptions'!M34</f>
+        <f>'Assumptions'!M35</f>
         <v/>
       </c>
       <c r="N7" s="33">
-        <f>'Assumptions'!N34</f>
+        <f>'Assumptions'!N35</f>
         <v/>
       </c>
       <c r="O7" s="33">
-        <f>'Assumptions'!O34</f>
+        <f>'Assumptions'!O35</f>
         <v/>
       </c>
     </row>
@@ -1755,31 +1755,31 @@
         </is>
       </c>
       <c r="I8" s="33">
-        <f>-'Assumptions'!I35*I6</f>
+        <f>-'Assumptions'!I36*I6</f>
         <v/>
       </c>
       <c r="J8" s="33">
-        <f>-'Assumptions'!J35*J6</f>
+        <f>-'Assumptions'!J36*J6</f>
         <v/>
       </c>
       <c r="K8" s="33">
-        <f>-'Assumptions'!K35*K6</f>
+        <f>-'Assumptions'!K36*K6</f>
         <v/>
       </c>
       <c r="L8" s="33">
-        <f>-'Assumptions'!L35*L6</f>
+        <f>-'Assumptions'!L36*L6</f>
         <v/>
       </c>
       <c r="M8" s="33">
-        <f>-'Assumptions'!M35*M6</f>
+        <f>-'Assumptions'!M36*M6</f>
         <v/>
       </c>
       <c r="N8" s="33">
-        <f>-'Assumptions'!N35*N6</f>
+        <f>-'Assumptions'!N36*N6</f>
         <v/>
       </c>
       <c r="O8" s="33">
-        <f>-'Assumptions'!O35*O6</f>
+        <f>-'Assumptions'!O36*O6</f>
         <v/>
       </c>
     </row>
@@ -2066,31 +2066,31 @@
         </is>
       </c>
       <c r="I7" s="40">
-        <f>'Assumptions'!I35</f>
+        <f>'Assumptions'!I36</f>
         <v/>
       </c>
       <c r="J7" s="40">
-        <f>'Assumptions'!J35</f>
+        <f>'Assumptions'!J36</f>
         <v/>
       </c>
       <c r="K7" s="40">
-        <f>'Assumptions'!K35</f>
+        <f>'Assumptions'!K36</f>
         <v/>
       </c>
       <c r="L7" s="40">
-        <f>'Assumptions'!L35</f>
+        <f>'Assumptions'!L36</f>
         <v/>
       </c>
       <c r="M7" s="40">
-        <f>'Assumptions'!M35</f>
+        <f>'Assumptions'!M36</f>
         <v/>
       </c>
       <c r="N7" s="40">
-        <f>'Assumptions'!N35</f>
+        <f>'Assumptions'!N36</f>
         <v/>
       </c>
       <c r="O7" s="40">
-        <f>'Assumptions'!O35</f>
+        <f>'Assumptions'!O36</f>
         <v/>
       </c>
     </row>
@@ -2384,31 +2384,31 @@
         </is>
       </c>
       <c r="I7" s="33">
-        <f>'Assumptions'!I47</f>
+        <f>'Assumptions'!I48</f>
         <v/>
       </c>
       <c r="J7" s="33">
-        <f>'Assumptions'!J47</f>
+        <f>'Assumptions'!J48</f>
         <v/>
       </c>
       <c r="K7" s="33">
-        <f>'Assumptions'!K47</f>
+        <f>'Assumptions'!K48</f>
         <v/>
       </c>
       <c r="L7" s="33">
-        <f>'Assumptions'!L47</f>
+        <f>'Assumptions'!L48</f>
         <v/>
       </c>
       <c r="M7" s="33">
-        <f>'Assumptions'!M47</f>
+        <f>'Assumptions'!M48</f>
         <v/>
       </c>
       <c r="N7" s="33">
-        <f>'Assumptions'!N47</f>
+        <f>'Assumptions'!N48</f>
         <v/>
       </c>
       <c r="O7" s="33">
-        <f>'Assumptions'!O47</f>
+        <f>'Assumptions'!O48</f>
         <v/>
       </c>
     </row>
@@ -2419,31 +2419,31 @@
         </is>
       </c>
       <c r="I8" s="33">
-        <f>-'Assumptions'!I48</f>
+        <f>-'Assumptions'!I49</f>
         <v/>
       </c>
       <c r="J8" s="33">
-        <f>-'Assumptions'!J48</f>
+        <f>-'Assumptions'!J49</f>
         <v/>
       </c>
       <c r="K8" s="33">
-        <f>-'Assumptions'!K48</f>
+        <f>-'Assumptions'!K49</f>
         <v/>
       </c>
       <c r="L8" s="33">
-        <f>-'Assumptions'!L48</f>
+        <f>-'Assumptions'!L49</f>
         <v/>
       </c>
       <c r="M8" s="33">
-        <f>-'Assumptions'!M48</f>
+        <f>-'Assumptions'!M49</f>
         <v/>
       </c>
       <c r="N8" s="33">
-        <f>-'Assumptions'!N48</f>
+        <f>-'Assumptions'!N49</f>
         <v/>
       </c>
       <c r="O8" s="33">
-        <f>-'Assumptions'!O48</f>
+        <f>-'Assumptions'!O49</f>
         <v/>
       </c>
     </row>
@@ -2580,31 +2580,31 @@
         <v/>
       </c>
       <c r="I11" s="33">
-        <f>'Assumptions'!I49*I6</f>
+        <f>'Assumptions'!I50*I6</f>
         <v/>
       </c>
       <c r="J11" s="33">
-        <f>'Assumptions'!J49*J6</f>
+        <f>'Assumptions'!J50*J6</f>
         <v/>
       </c>
       <c r="K11" s="33">
-        <f>'Assumptions'!K49*K6</f>
+        <f>'Assumptions'!K50*K6</f>
         <v/>
       </c>
       <c r="L11" s="33">
-        <f>'Assumptions'!L49*L6</f>
+        <f>'Assumptions'!L50*L6</f>
         <v/>
       </c>
       <c r="M11" s="33">
-        <f>'Assumptions'!M49*M6</f>
+        <f>'Assumptions'!M50*M6</f>
         <v/>
       </c>
       <c r="N11" s="33">
-        <f>'Assumptions'!N49*N6</f>
+        <f>'Assumptions'!N50*N6</f>
         <v/>
       </c>
       <c r="O11" s="33">
-        <f>'Assumptions'!O49*O6</f>
+        <f>'Assumptions'!O50*O6</f>
         <v/>
       </c>
     </row>
@@ -3174,31 +3174,31 @@
         <v/>
       </c>
       <c r="I6" s="33">
-        <f>'Assumptions'!I43</f>
+        <f>'Assumptions'!I44</f>
         <v/>
       </c>
       <c r="J6" s="33">
-        <f>'Assumptions'!J43</f>
+        <f>'Assumptions'!J44</f>
         <v/>
       </c>
       <c r="K6" s="33">
-        <f>'Assumptions'!K43</f>
+        <f>'Assumptions'!K44</f>
         <v/>
       </c>
       <c r="L6" s="33">
-        <f>'Assumptions'!L43</f>
+        <f>'Assumptions'!L44</f>
         <v/>
       </c>
       <c r="M6" s="33">
-        <f>'Assumptions'!M43</f>
+        <f>'Assumptions'!M44</f>
         <v/>
       </c>
       <c r="N6" s="33">
-        <f>'Assumptions'!N43</f>
+        <f>'Assumptions'!N44</f>
         <v/>
       </c>
       <c r="O6" s="33">
-        <f>'Assumptions'!O43</f>
+        <f>'Assumptions'!O44</f>
         <v/>
       </c>
     </row>
@@ -3237,31 +3237,31 @@
         <v/>
       </c>
       <c r="I7" s="33">
-        <f>'Assumptions'!I44</f>
+        <f>'Assumptions'!I45</f>
         <v/>
       </c>
       <c r="J7" s="33">
-        <f>'Assumptions'!J44</f>
+        <f>'Assumptions'!J45</f>
         <v/>
       </c>
       <c r="K7" s="33">
-        <f>'Assumptions'!K44</f>
+        <f>'Assumptions'!K45</f>
         <v/>
       </c>
       <c r="L7" s="33">
-        <f>'Assumptions'!L44</f>
+        <f>'Assumptions'!L45</f>
         <v/>
       </c>
       <c r="M7" s="33">
-        <f>'Assumptions'!M44</f>
+        <f>'Assumptions'!M45</f>
         <v/>
       </c>
       <c r="N7" s="33">
-        <f>'Assumptions'!N44</f>
+        <f>'Assumptions'!N45</f>
         <v/>
       </c>
       <c r="O7" s="33">
-        <f>'Assumptions'!O44</f>
+        <f>'Assumptions'!O45</f>
         <v/>
       </c>
     </row>
@@ -3758,31 +3758,31 @@
         </is>
       </c>
       <c r="I12" s="33">
-        <f>-'Assumptions'!I34</f>
+        <f>-'Assumptions'!I35</f>
         <v/>
       </c>
       <c r="J12" s="33">
-        <f>-'Assumptions'!J34</f>
+        <f>-'Assumptions'!J35</f>
         <v/>
       </c>
       <c r="K12" s="33">
-        <f>-'Assumptions'!K34</f>
+        <f>-'Assumptions'!K35</f>
         <v/>
       </c>
       <c r="L12" s="33">
-        <f>-'Assumptions'!L34</f>
+        <f>-'Assumptions'!L35</f>
         <v/>
       </c>
       <c r="M12" s="33">
-        <f>-'Assumptions'!M34</f>
+        <f>-'Assumptions'!M35</f>
         <v/>
       </c>
       <c r="N12" s="33">
-        <f>-'Assumptions'!N34</f>
+        <f>-'Assumptions'!N35</f>
         <v/>
       </c>
       <c r="O12" s="33">
-        <f>-'Assumptions'!O34</f>
+        <f>-'Assumptions'!O35</f>
         <v/>
       </c>
     </row>
@@ -3793,31 +3793,31 @@
         </is>
       </c>
       <c r="I13" s="33">
-        <f>-('Assumptions'!I43-'Historical Financial Statements'!H29)</f>
+        <f>-('Assumptions'!I44-'Historical Financial Statements'!H29)</f>
         <v/>
       </c>
       <c r="J13" s="33">
-        <f>-('Assumptions'!J43-'Assumptions'!I43)</f>
+        <f>-('Assumptions'!J44-'Assumptions'!I44)</f>
         <v/>
       </c>
       <c r="K13" s="33">
-        <f>-('Assumptions'!K43-'Assumptions'!J43)</f>
+        <f>-('Assumptions'!K44-'Assumptions'!J44)</f>
         <v/>
       </c>
       <c r="L13" s="33">
-        <f>-('Assumptions'!L43-'Assumptions'!K43)</f>
+        <f>-('Assumptions'!L44-'Assumptions'!K44)</f>
         <v/>
       </c>
       <c r="M13" s="33">
-        <f>-('Assumptions'!M43-'Assumptions'!L43)</f>
+        <f>-('Assumptions'!M44-'Assumptions'!L44)</f>
         <v/>
       </c>
       <c r="N13" s="33">
-        <f>-('Assumptions'!N43-'Assumptions'!M43)</f>
+        <f>-('Assumptions'!N44-'Assumptions'!M44)</f>
         <v/>
       </c>
       <c r="O13" s="33">
-        <f>-('Assumptions'!O43-'Assumptions'!N43)</f>
+        <f>-('Assumptions'!O44-'Assumptions'!N44)</f>
         <v/>
       </c>
     </row>
@@ -3828,31 +3828,31 @@
         </is>
       </c>
       <c r="I14" s="33">
-        <f>-('Assumptions'!I44-'Historical Financial Statements'!H30)</f>
+        <f>-('Assumptions'!I45-'Historical Financial Statements'!H30)</f>
         <v/>
       </c>
       <c r="J14" s="33">
-        <f>-('Assumptions'!J44-'Assumptions'!I44)</f>
+        <f>-('Assumptions'!J45-'Assumptions'!I45)</f>
         <v/>
       </c>
       <c r="K14" s="33">
-        <f>-('Assumptions'!K44-'Assumptions'!J44)</f>
+        <f>-('Assumptions'!K45-'Assumptions'!J45)</f>
         <v/>
       </c>
       <c r="L14" s="33">
-        <f>-('Assumptions'!L44-'Assumptions'!K44)</f>
+        <f>-('Assumptions'!L45-'Assumptions'!K45)</f>
         <v/>
       </c>
       <c r="M14" s="33">
-        <f>-('Assumptions'!M44-'Assumptions'!L44)</f>
+        <f>-('Assumptions'!M45-'Assumptions'!L45)</f>
         <v/>
       </c>
       <c r="N14" s="33">
-        <f>-('Assumptions'!N44-'Assumptions'!M44)</f>
+        <f>-('Assumptions'!N45-'Assumptions'!M45)</f>
         <v/>
       </c>
       <c r="O14" s="33">
-        <f>-('Assumptions'!O44-'Assumptions'!N44)</f>
+        <f>-('Assumptions'!O45-'Assumptions'!N45)</f>
         <v/>
       </c>
     </row>
@@ -4482,31 +4482,31 @@
         <v/>
       </c>
       <c r="I5" s="33">
-        <f>'Revenue Build-up'!I11</f>
+        <f>'Revenue Build-up'!I14</f>
         <v/>
       </c>
       <c r="J5" s="33">
-        <f>'Revenue Build-up'!J11</f>
+        <f>'Revenue Build-up'!J14</f>
         <v/>
       </c>
       <c r="K5" s="33">
-        <f>'Revenue Build-up'!K11</f>
+        <f>'Revenue Build-up'!K14</f>
         <v/>
       </c>
       <c r="L5" s="33">
-        <f>'Revenue Build-up'!L11</f>
+        <f>'Revenue Build-up'!L14</f>
         <v/>
       </c>
       <c r="M5" s="33">
-        <f>'Revenue Build-up'!M11</f>
+        <f>'Revenue Build-up'!M14</f>
         <v/>
       </c>
       <c r="N5" s="33">
-        <f>'Revenue Build-up'!N11</f>
+        <f>'Revenue Build-up'!N14</f>
         <v/>
       </c>
       <c r="O5" s="33">
-        <f>'Revenue Build-up'!O11</f>
+        <f>'Revenue Build-up'!O14</f>
         <v/>
       </c>
     </row>
@@ -5056,31 +5056,31 @@
         <v/>
       </c>
       <c r="I15" s="33">
-        <f>'Assumptions'!I22*I5</f>
+        <f>'Assumptions'!I23*I5</f>
         <v/>
       </c>
       <c r="J15" s="33">
-        <f>'Assumptions'!J22*J5</f>
+        <f>'Assumptions'!J23*J5</f>
         <v/>
       </c>
       <c r="K15" s="33">
-        <f>'Assumptions'!K22*K5</f>
+        <f>'Assumptions'!K23*K5</f>
         <v/>
       </c>
       <c r="L15" s="33">
-        <f>'Assumptions'!L22*L5</f>
+        <f>'Assumptions'!L23*L5</f>
         <v/>
       </c>
       <c r="M15" s="33">
-        <f>'Assumptions'!M22*M5</f>
+        <f>'Assumptions'!M23*M5</f>
         <v/>
       </c>
       <c r="N15" s="33">
-        <f>'Assumptions'!N22*N5</f>
+        <f>'Assumptions'!N23*N5</f>
         <v/>
       </c>
       <c r="O15" s="33">
-        <f>'Assumptions'!O22*O5</f>
+        <f>'Assumptions'!O23*O5</f>
         <v/>
       </c>
     </row>
@@ -5245,31 +5245,31 @@
         <v/>
       </c>
       <c r="I18" s="33">
-        <f>'Assumptions'!I45*I17</f>
+        <f>'Assumptions'!I46*I17</f>
         <v/>
       </c>
       <c r="J18" s="33">
-        <f>'Assumptions'!J45*J17</f>
+        <f>'Assumptions'!J46*J17</f>
         <v/>
       </c>
       <c r="K18" s="33">
-        <f>'Assumptions'!K45*K17</f>
+        <f>'Assumptions'!K46*K17</f>
         <v/>
       </c>
       <c r="L18" s="33">
-        <f>'Assumptions'!L45*L17</f>
+        <f>'Assumptions'!L46*L17</f>
         <v/>
       </c>
       <c r="M18" s="33">
-        <f>'Assumptions'!M45*M17</f>
+        <f>'Assumptions'!M46*M17</f>
         <v/>
       </c>
       <c r="N18" s="33">
-        <f>'Assumptions'!N45*N17</f>
+        <f>'Assumptions'!N46*N17</f>
         <v/>
       </c>
       <c r="O18" s="33">
-        <f>'Assumptions'!O45*O17</f>
+        <f>'Assumptions'!O46*O17</f>
         <v/>
       </c>
     </row>
@@ -5399,59 +5399,59 @@
         </is>
       </c>
       <c r="B21" s="35">
-        <f>B20/'Assumptions'!C65</f>
+        <f>B20/'Assumptions'!C66</f>
         <v/>
       </c>
       <c r="C21" s="35">
-        <f>C20/'Assumptions'!C65</f>
+        <f>C20/'Assumptions'!C66</f>
         <v/>
       </c>
       <c r="D21" s="35">
-        <f>D20/'Assumptions'!C65</f>
+        <f>D20/'Assumptions'!C66</f>
         <v/>
       </c>
       <c r="E21" s="35">
-        <f>E20/'Assumptions'!C65</f>
+        <f>E20/'Assumptions'!C66</f>
         <v/>
       </c>
       <c r="F21" s="35">
-        <f>F20/'Assumptions'!C65</f>
+        <f>F20/'Assumptions'!C66</f>
         <v/>
       </c>
       <c r="G21" s="35">
-        <f>G20/'Assumptions'!C65</f>
+        <f>G20/'Assumptions'!C66</f>
         <v/>
       </c>
       <c r="H21" s="35">
-        <f>H20/'Assumptions'!C65</f>
+        <f>H20/'Assumptions'!C66</f>
         <v/>
       </c>
       <c r="I21" s="35">
-        <f>I20/'Assumptions'!C65</f>
+        <f>I20/'Assumptions'!C66</f>
         <v/>
       </c>
       <c r="J21" s="35">
-        <f>J20/'Assumptions'!C65</f>
+        <f>J20/'Assumptions'!C66</f>
         <v/>
       </c>
       <c r="K21" s="35">
-        <f>K20/'Assumptions'!C65</f>
+        <f>K20/'Assumptions'!C66</f>
         <v/>
       </c>
       <c r="L21" s="35">
-        <f>L20/'Assumptions'!C65</f>
+        <f>L20/'Assumptions'!C66</f>
         <v/>
       </c>
       <c r="M21" s="35">
-        <f>M20/'Assumptions'!C65</f>
+        <f>M20/'Assumptions'!C66</f>
         <v/>
       </c>
       <c r="N21" s="35">
-        <f>N20/'Assumptions'!C65</f>
+        <f>N20/'Assumptions'!C66</f>
         <v/>
       </c>
       <c r="O21" s="35">
-        <f>O20/'Assumptions'!C65</f>
+        <f>O20/'Assumptions'!C66</f>
         <v/>
       </c>
     </row>
@@ -5490,31 +5490,31 @@
         <v/>
       </c>
       <c r="I22" s="33">
-        <f>'Assumptions'!I46*I20</f>
+        <f>'Assumptions'!I47*I20</f>
         <v/>
       </c>
       <c r="J22" s="33">
-        <f>'Assumptions'!J46*J20</f>
+        <f>'Assumptions'!J47*J20</f>
         <v/>
       </c>
       <c r="K22" s="33">
-        <f>'Assumptions'!K46*K20</f>
+        <f>'Assumptions'!K47*K20</f>
         <v/>
       </c>
       <c r="L22" s="33">
-        <f>'Assumptions'!L46*L20</f>
+        <f>'Assumptions'!L47*L20</f>
         <v/>
       </c>
       <c r="M22" s="33">
-        <f>'Assumptions'!M46*M20</f>
+        <f>'Assumptions'!M47*M20</f>
         <v/>
       </c>
       <c r="N22" s="33">
-        <f>'Assumptions'!N46*N20</f>
+        <f>'Assumptions'!N47*N20</f>
         <v/>
       </c>
       <c r="O22" s="33">
-        <f>'Assumptions'!O46*O20</f>
+        <f>'Assumptions'!O47*O20</f>
         <v/>
       </c>
     </row>
@@ -5861,31 +5861,31 @@
         <v>2865</v>
       </c>
       <c r="I34" s="43">
-        <f>'Assumptions'!I50*'Debt Schedule'!I9</f>
+        <f>'Assumptions'!I51*'Debt Schedule'!I9</f>
         <v/>
       </c>
       <c r="J34" s="43">
-        <f>'Assumptions'!J50*'Debt Schedule'!J9</f>
+        <f>'Assumptions'!J51*'Debt Schedule'!J9</f>
         <v/>
       </c>
       <c r="K34" s="43">
-        <f>'Assumptions'!K50*'Debt Schedule'!K9</f>
+        <f>'Assumptions'!K51*'Debt Schedule'!K9</f>
         <v/>
       </c>
       <c r="L34" s="43">
-        <f>'Assumptions'!L50*'Debt Schedule'!L9</f>
+        <f>'Assumptions'!L51*'Debt Schedule'!L9</f>
         <v/>
       </c>
       <c r="M34" s="43">
-        <f>'Assumptions'!M50*'Debt Schedule'!M9</f>
+        <f>'Assumptions'!M51*'Debt Schedule'!M9</f>
         <v/>
       </c>
       <c r="N34" s="43">
-        <f>'Assumptions'!N50*'Debt Schedule'!N9</f>
+        <f>'Assumptions'!N51*'Debt Schedule'!N9</f>
         <v/>
       </c>
       <c r="O34" s="43">
-        <f>'Assumptions'!O50*'Debt Schedule'!O9</f>
+        <f>'Assumptions'!O51*'Debt Schedule'!O9</f>
         <v/>
       </c>
     </row>
@@ -5917,31 +5917,31 @@
         <v>6000</v>
       </c>
       <c r="I35" s="43">
-        <f>'Assumptions'!I52</f>
+        <f>'Assumptions'!I53</f>
         <v/>
       </c>
       <c r="J35" s="43">
-        <f>'Assumptions'!J52</f>
+        <f>'Assumptions'!J53</f>
         <v/>
       </c>
       <c r="K35" s="43">
-        <f>'Assumptions'!K52</f>
+        <f>'Assumptions'!K53</f>
         <v/>
       </c>
       <c r="L35" s="43">
-        <f>'Assumptions'!L52</f>
+        <f>'Assumptions'!L53</f>
         <v/>
       </c>
       <c r="M35" s="43">
-        <f>'Assumptions'!M52</f>
+        <f>'Assumptions'!M53</f>
         <v/>
       </c>
       <c r="N35" s="43">
-        <f>'Assumptions'!N52</f>
+        <f>'Assumptions'!N53</f>
         <v/>
       </c>
       <c r="O35" s="43">
-        <f>'Assumptions'!O52</f>
+        <f>'Assumptions'!O53</f>
         <v/>
       </c>
     </row>
@@ -6421,31 +6421,31 @@
         <v>399</v>
       </c>
       <c r="I48" s="43">
-        <f>'Assumptions'!I43</f>
+        <f>'Assumptions'!I44</f>
         <v/>
       </c>
       <c r="J48" s="43">
-        <f>'Assumptions'!J43</f>
+        <f>'Assumptions'!J44</f>
         <v/>
       </c>
       <c r="K48" s="43">
-        <f>'Assumptions'!K43</f>
+        <f>'Assumptions'!K44</f>
         <v/>
       </c>
       <c r="L48" s="43">
-        <f>'Assumptions'!L43</f>
+        <f>'Assumptions'!L44</f>
         <v/>
       </c>
       <c r="M48" s="43">
-        <f>'Assumptions'!M43</f>
+        <f>'Assumptions'!M44</f>
         <v/>
       </c>
       <c r="N48" s="43">
-        <f>'Assumptions'!N43</f>
+        <f>'Assumptions'!N44</f>
         <v/>
       </c>
       <c r="O48" s="43">
-        <f>'Assumptions'!O43</f>
+        <f>'Assumptions'!O44</f>
         <v/>
       </c>
     </row>
@@ -6477,31 +6477,31 @@
         <v>302</v>
       </c>
       <c r="I49" s="43">
-        <f>'Assumptions'!I44</f>
+        <f>'Assumptions'!I45</f>
         <v/>
       </c>
       <c r="J49" s="43">
-        <f>'Assumptions'!J44</f>
+        <f>'Assumptions'!J45</f>
         <v/>
       </c>
       <c r="K49" s="43">
-        <f>'Assumptions'!K44</f>
+        <f>'Assumptions'!K45</f>
         <v/>
       </c>
       <c r="L49" s="43">
-        <f>'Assumptions'!L44</f>
+        <f>'Assumptions'!L45</f>
         <v/>
       </c>
       <c r="M49" s="43">
-        <f>'Assumptions'!M44</f>
+        <f>'Assumptions'!M45</f>
         <v/>
       </c>
       <c r="N49" s="43">
-        <f>'Assumptions'!N44</f>
+        <f>'Assumptions'!N45</f>
         <v/>
       </c>
       <c r="O49" s="43">
-        <f>'Assumptions'!O44</f>
+        <f>'Assumptions'!O45</f>
         <v/>
       </c>
     </row>
@@ -6596,31 +6596,31 @@
         <v>15000</v>
       </c>
       <c r="I51" s="43">
-        <f>'Assumptions'!I51</f>
+        <f>'Assumptions'!I52</f>
         <v/>
       </c>
       <c r="J51" s="43">
-        <f>'Assumptions'!J51</f>
+        <f>'Assumptions'!J52</f>
         <v/>
       </c>
       <c r="K51" s="43">
-        <f>'Assumptions'!K51</f>
+        <f>'Assumptions'!K52</f>
         <v/>
       </c>
       <c r="L51" s="43">
-        <f>'Assumptions'!L51</f>
+        <f>'Assumptions'!L52</f>
         <v/>
       </c>
       <c r="M51" s="43">
-        <f>'Assumptions'!M51</f>
+        <f>'Assumptions'!M52</f>
         <v/>
       </c>
       <c r="N51" s="43">
-        <f>'Assumptions'!N51</f>
+        <f>'Assumptions'!N52</f>
         <v/>
       </c>
       <c r="O51" s="43">
-        <f>'Assumptions'!O51</f>
+        <f>'Assumptions'!O52</f>
         <v/>
       </c>
     </row>
@@ -8590,59 +8590,59 @@
         </is>
       </c>
       <c r="B25" s="50">
-        <f>'Historical Financial Statements'!B22/'Assumptions'!C65</f>
+        <f>'Historical Financial Statements'!B22/'Assumptions'!C66</f>
         <v/>
       </c>
       <c r="C25" s="50">
-        <f>'Historical Financial Statements'!C22/'Assumptions'!C65</f>
+        <f>'Historical Financial Statements'!C22/'Assumptions'!C66</f>
         <v/>
       </c>
       <c r="D25" s="50">
-        <f>'Historical Financial Statements'!D22/'Assumptions'!C65</f>
+        <f>'Historical Financial Statements'!D22/'Assumptions'!C66</f>
         <v/>
       </c>
       <c r="E25" s="50">
-        <f>'Historical Financial Statements'!E22/'Assumptions'!C65</f>
+        <f>'Historical Financial Statements'!E22/'Assumptions'!C66</f>
         <v/>
       </c>
       <c r="F25" s="50">
-        <f>'Historical Financial Statements'!F22/'Assumptions'!C65</f>
+        <f>'Historical Financial Statements'!F22/'Assumptions'!C66</f>
         <v/>
       </c>
       <c r="G25" s="50">
-        <f>'Historical Financial Statements'!G22/'Assumptions'!C65</f>
+        <f>'Historical Financial Statements'!G22/'Assumptions'!C66</f>
         <v/>
       </c>
       <c r="H25" s="50">
-        <f>'Forecast Financial Statements'!H22/'Assumptions'!C65</f>
+        <f>'Forecast Financial Statements'!H22/'Assumptions'!C66</f>
         <v/>
       </c>
       <c r="I25" s="50">
-        <f>'Forecast Financial Statements'!I22/'Assumptions'!C65</f>
+        <f>'Forecast Financial Statements'!I22/'Assumptions'!C66</f>
         <v/>
       </c>
       <c r="J25" s="50">
-        <f>'Forecast Financial Statements'!J22/'Assumptions'!C65</f>
+        <f>'Forecast Financial Statements'!J22/'Assumptions'!C66</f>
         <v/>
       </c>
       <c r="K25" s="50">
-        <f>'Forecast Financial Statements'!K22/'Assumptions'!C65</f>
+        <f>'Forecast Financial Statements'!K22/'Assumptions'!C66</f>
         <v/>
       </c>
       <c r="L25" s="50">
-        <f>'Forecast Financial Statements'!L22/'Assumptions'!C65</f>
+        <f>'Forecast Financial Statements'!L22/'Assumptions'!C66</f>
         <v/>
       </c>
       <c r="M25" s="50">
-        <f>'Forecast Financial Statements'!M22/'Assumptions'!C65</f>
+        <f>'Forecast Financial Statements'!M22/'Assumptions'!C66</f>
         <v/>
       </c>
       <c r="N25" s="50">
-        <f>'Forecast Financial Statements'!N22/'Assumptions'!C65</f>
+        <f>'Forecast Financial Statements'!N22/'Assumptions'!C66</f>
         <v/>
       </c>
       <c r="O25" s="50">
-        <f>'Forecast Financial Statements'!O22/'Assumptions'!C65</f>
+        <f>'Forecast Financial Statements'!O22/'Assumptions'!C66</f>
         <v/>
       </c>
     </row>
@@ -8716,59 +8716,59 @@
         </is>
       </c>
       <c r="B27" s="50">
-        <f>('Historical Financial Statements'!B33+'Historical Financial Statements'!B34)/'Assumptions'!C65</f>
+        <f>('Historical Financial Statements'!B33+'Historical Financial Statements'!B34)/'Assumptions'!C66</f>
         <v/>
       </c>
       <c r="C27" s="50">
-        <f>('Historical Financial Statements'!C33+'Historical Financial Statements'!C34)/'Assumptions'!C65</f>
+        <f>('Historical Financial Statements'!C33+'Historical Financial Statements'!C34)/'Assumptions'!C66</f>
         <v/>
       </c>
       <c r="D27" s="50">
-        <f>('Historical Financial Statements'!D33+'Historical Financial Statements'!D34)/'Assumptions'!C65</f>
+        <f>('Historical Financial Statements'!D33+'Historical Financial Statements'!D34)/'Assumptions'!C66</f>
         <v/>
       </c>
       <c r="E27" s="50">
-        <f>('Historical Financial Statements'!E33+'Historical Financial Statements'!E34)/'Assumptions'!C65</f>
+        <f>('Historical Financial Statements'!E33+'Historical Financial Statements'!E34)/'Assumptions'!C66</f>
         <v/>
       </c>
       <c r="F27" s="50">
-        <f>('Historical Financial Statements'!F33+'Historical Financial Statements'!F34)/'Assumptions'!C65</f>
+        <f>('Historical Financial Statements'!F33+'Historical Financial Statements'!F34)/'Assumptions'!C66</f>
         <v/>
       </c>
       <c r="G27" s="50">
-        <f>('Historical Financial Statements'!G33+'Historical Financial Statements'!G34)/'Assumptions'!C65</f>
+        <f>('Historical Financial Statements'!G33+'Historical Financial Statements'!G34)/'Assumptions'!C66</f>
         <v/>
       </c>
       <c r="H27" s="50">
-        <f>('Forecast Financial Statements'!H28+'Forecast Financial Statements'!H29)/'Assumptions'!C65</f>
+        <f>('Forecast Financial Statements'!H28+'Forecast Financial Statements'!H29)/'Assumptions'!C66</f>
         <v/>
       </c>
       <c r="I27" s="50">
-        <f>('Forecast Financial Statements'!I28+'Forecast Financial Statements'!I29)/'Assumptions'!C65</f>
+        <f>('Forecast Financial Statements'!I28+'Forecast Financial Statements'!I29)/'Assumptions'!C66</f>
         <v/>
       </c>
       <c r="J27" s="50">
-        <f>('Forecast Financial Statements'!J28+'Forecast Financial Statements'!J29)/'Assumptions'!C65</f>
+        <f>('Forecast Financial Statements'!J28+'Forecast Financial Statements'!J29)/'Assumptions'!C66</f>
         <v/>
       </c>
       <c r="K27" s="50">
-        <f>('Forecast Financial Statements'!K28+'Forecast Financial Statements'!K29)/'Assumptions'!C65</f>
+        <f>('Forecast Financial Statements'!K28+'Forecast Financial Statements'!K29)/'Assumptions'!C66</f>
         <v/>
       </c>
       <c r="L27" s="50">
-        <f>('Forecast Financial Statements'!L28+'Forecast Financial Statements'!L29)/'Assumptions'!C65</f>
+        <f>('Forecast Financial Statements'!L28+'Forecast Financial Statements'!L29)/'Assumptions'!C66</f>
         <v/>
       </c>
       <c r="M27" s="50">
-        <f>('Forecast Financial Statements'!M28+'Forecast Financial Statements'!M29)/'Assumptions'!C65</f>
+        <f>('Forecast Financial Statements'!M28+'Forecast Financial Statements'!M29)/'Assumptions'!C66</f>
         <v/>
       </c>
       <c r="N27" s="50">
-        <f>('Forecast Financial Statements'!N28+'Forecast Financial Statements'!N29)/'Assumptions'!C65</f>
+        <f>('Forecast Financial Statements'!N28+'Forecast Financial Statements'!N29)/'Assumptions'!C66</f>
         <v/>
       </c>
       <c r="O27" s="50">
-        <f>('Forecast Financial Statements'!O28+'Forecast Financial Statements'!O29)/'Assumptions'!C65</f>
+        <f>('Forecast Financial Statements'!O28+'Forecast Financial Statements'!O29)/'Assumptions'!C66</f>
         <v/>
       </c>
     </row>
@@ -8944,31 +8944,31 @@
         </is>
       </c>
       <c r="I34" s="36">
-        <f>'Assumptions'!I34/'Forecast Financial Statements'!I5</f>
+        <f>'Assumptions'!I35/'Forecast Financial Statements'!I5</f>
         <v/>
       </c>
       <c r="J34" s="36">
-        <f>'Assumptions'!J34/'Forecast Financial Statements'!J5</f>
+        <f>'Assumptions'!J35/'Forecast Financial Statements'!J5</f>
         <v/>
       </c>
       <c r="K34" s="36">
-        <f>'Assumptions'!K34/'Forecast Financial Statements'!K5</f>
+        <f>'Assumptions'!K35/'Forecast Financial Statements'!K5</f>
         <v/>
       </c>
       <c r="L34" s="36">
-        <f>'Assumptions'!L34/'Forecast Financial Statements'!L5</f>
+        <f>'Assumptions'!L35/'Forecast Financial Statements'!L5</f>
         <v/>
       </c>
       <c r="M34" s="36">
-        <f>'Assumptions'!M34/'Forecast Financial Statements'!M5</f>
+        <f>'Assumptions'!M35/'Forecast Financial Statements'!M5</f>
         <v/>
       </c>
       <c r="N34" s="36">
-        <f>'Assumptions'!N34/'Forecast Financial Statements'!N5</f>
+        <f>'Assumptions'!N35/'Forecast Financial Statements'!N5</f>
         <v/>
       </c>
       <c r="O34" s="36">
-        <f>'Assumptions'!O34/'Forecast Financial Statements'!O5</f>
+        <f>'Assumptions'!O35/'Forecast Financial Statements'!O5</f>
         <v/>
       </c>
     </row>
@@ -8979,31 +8979,31 @@
         </is>
       </c>
       <c r="I35" s="43">
-        <f>'DCF Valuation'!I12-'Forecast Financial Statements'!I16*(1-'Assumptions'!I45)+'Debt Schedule'!I7+'Debt Schedule'!I8</f>
+        <f>'DCF Valuation'!I12-'Forecast Financial Statements'!I16*(1-'Assumptions'!I46)+'Debt Schedule'!I7+'Debt Schedule'!I8</f>
         <v/>
       </c>
       <c r="J35" s="43">
-        <f>'DCF Valuation'!J12-'Forecast Financial Statements'!J16*(1-'Assumptions'!J45)+'Debt Schedule'!J7+'Debt Schedule'!J8</f>
+        <f>'DCF Valuation'!J12-'Forecast Financial Statements'!J16*(1-'Assumptions'!J46)+'Debt Schedule'!J7+'Debt Schedule'!J8</f>
         <v/>
       </c>
       <c r="K35" s="43">
-        <f>'DCF Valuation'!K12-'Forecast Financial Statements'!K16*(1-'Assumptions'!K45)+'Debt Schedule'!K7+'Debt Schedule'!K8</f>
+        <f>'DCF Valuation'!K12-'Forecast Financial Statements'!K16*(1-'Assumptions'!K46)+'Debt Schedule'!K7+'Debt Schedule'!K8</f>
         <v/>
       </c>
       <c r="L35" s="43">
-        <f>'DCF Valuation'!L12-'Forecast Financial Statements'!L16*(1-'Assumptions'!L45)+'Debt Schedule'!L7+'Debt Schedule'!L8</f>
+        <f>'DCF Valuation'!L12-'Forecast Financial Statements'!L16*(1-'Assumptions'!L46)+'Debt Schedule'!L7+'Debt Schedule'!L8</f>
         <v/>
       </c>
       <c r="M35" s="43">
-        <f>'DCF Valuation'!M12-'Forecast Financial Statements'!M16*(1-'Assumptions'!M45)+'Debt Schedule'!M7+'Debt Schedule'!M8</f>
+        <f>'DCF Valuation'!M12-'Forecast Financial Statements'!M16*(1-'Assumptions'!M46)+'Debt Schedule'!M7+'Debt Schedule'!M8</f>
         <v/>
       </c>
       <c r="N35" s="43">
-        <f>'DCF Valuation'!N12-'Forecast Financial Statements'!N16*(1-'Assumptions'!N45)+'Debt Schedule'!N7+'Debt Schedule'!N8</f>
+        <f>'DCF Valuation'!N12-'Forecast Financial Statements'!N16*(1-'Assumptions'!N46)+'Debt Schedule'!N7+'Debt Schedule'!N8</f>
         <v/>
       </c>
       <c r="O35" s="43">
-        <f>'DCF Valuation'!O12-'Forecast Financial Statements'!O16*(1-'Assumptions'!O45)+'Debt Schedule'!O7+'Debt Schedule'!O8</f>
+        <f>'DCF Valuation'!O12-'Forecast Financial Statements'!O16*(1-'Assumptions'!O46)+'Debt Schedule'!O7+'Debt Schedule'!O8</f>
         <v/>
       </c>
     </row>
@@ -9172,31 +9172,31 @@
         </is>
       </c>
       <c r="I7" s="33">
-        <f>-I6*'Assumptions'!I45</f>
+        <f>-I6*'Assumptions'!I46</f>
         <v/>
       </c>
       <c r="J7" s="33">
-        <f>-J6*'Assumptions'!J45</f>
+        <f>-J6*'Assumptions'!J46</f>
         <v/>
       </c>
       <c r="K7" s="33">
-        <f>-K6*'Assumptions'!K45</f>
+        <f>-K6*'Assumptions'!K46</f>
         <v/>
       </c>
       <c r="L7" s="33">
-        <f>-L6*'Assumptions'!L45</f>
+        <f>-L6*'Assumptions'!L46</f>
         <v/>
       </c>
       <c r="M7" s="33">
-        <f>-M6*'Assumptions'!M45</f>
+        <f>-M6*'Assumptions'!M46</f>
         <v/>
       </c>
       <c r="N7" s="33">
-        <f>-N6*'Assumptions'!N45</f>
+        <f>-N6*'Assumptions'!N46</f>
         <v/>
       </c>
       <c r="O7" s="33">
-        <f>-O6*'Assumptions'!O45</f>
+        <f>-O6*'Assumptions'!O46</f>
         <v/>
       </c>
     </row>
@@ -9277,31 +9277,31 @@
         </is>
       </c>
       <c r="I10" s="43">
-        <f>-'Assumptions'!I34</f>
+        <f>-'Assumptions'!I35</f>
         <v/>
       </c>
       <c r="J10" s="43">
-        <f>-'Assumptions'!J34</f>
+        <f>-'Assumptions'!J35</f>
         <v/>
       </c>
       <c r="K10" s="43">
-        <f>-'Assumptions'!K34</f>
+        <f>-'Assumptions'!K35</f>
         <v/>
       </c>
       <c r="L10" s="43">
-        <f>-'Assumptions'!L34</f>
+        <f>-'Assumptions'!L35</f>
         <v/>
       </c>
       <c r="M10" s="43">
-        <f>-'Assumptions'!M34</f>
+        <f>-'Assumptions'!M35</f>
         <v/>
       </c>
       <c r="N10" s="43">
-        <f>-'Assumptions'!N34</f>
+        <f>-'Assumptions'!N35</f>
         <v/>
       </c>
       <c r="O10" s="43">
-        <f>-'Assumptions'!O34</f>
+        <f>-'Assumptions'!O35</f>
         <v/>
       </c>
     </row>
@@ -9410,31 +9410,31 @@
         </is>
       </c>
       <c r="I14" s="53">
-        <f>1/(1+'Assumptions'!C64)^I13</f>
+        <f>1/(1+'Assumptions'!C65)^I13</f>
         <v/>
       </c>
       <c r="J14" s="53">
-        <f>1/(1+'Assumptions'!C64)^J13</f>
+        <f>1/(1+'Assumptions'!C65)^J13</f>
         <v/>
       </c>
       <c r="K14" s="53">
-        <f>1/(1+'Assumptions'!C64)^K13</f>
+        <f>1/(1+'Assumptions'!C65)^K13</f>
         <v/>
       </c>
       <c r="L14" s="53">
-        <f>1/(1+'Assumptions'!C64)^L13</f>
+        <f>1/(1+'Assumptions'!C65)^L13</f>
         <v/>
       </c>
       <c r="M14" s="53">
-        <f>1/(1+'Assumptions'!C64)^M13</f>
+        <f>1/(1+'Assumptions'!C65)^M13</f>
         <v/>
       </c>
       <c r="N14" s="53">
-        <f>1/(1+'Assumptions'!C64)^N13</f>
+        <f>1/(1+'Assumptions'!C65)^N13</f>
         <v/>
       </c>
       <c r="O14" s="53">
-        <f>1/(1+'Assumptions'!C64)^O13</f>
+        <f>1/(1+'Assumptions'!C65)^O13</f>
         <v/>
       </c>
     </row>
@@ -9512,7 +9512,7 @@
         </is>
       </c>
       <c r="C19" s="55">
-        <f>'Assumptions'!C64</f>
+        <f>'Assumptions'!C65</f>
         <v/>
       </c>
     </row>
@@ -9523,7 +9523,7 @@
         </is>
       </c>
       <c r="C20" s="55">
-        <f>'Assumptions'!C62</f>
+        <f>'Assumptions'!C63</f>
         <v/>
       </c>
     </row>
@@ -9589,7 +9589,7 @@
         </is>
       </c>
       <c r="C26" s="57">
-        <f>'Assumptions'!C65</f>
+        <f>'Assumptions'!C66</f>
         <v/>
       </c>
     </row>
@@ -9611,7 +9611,7 @@
         </is>
       </c>
       <c r="C28" s="59">
-        <f>'Assumptions'!C66</f>
+        <f>'Assumptions'!C67</f>
         <v/>
       </c>
     </row>
@@ -10018,7 +10018,7 @@
         </is>
       </c>
       <c r="C24" s="58">
-        <f>C23/'Assumptions'!C65</f>
+        <f>C23/'Assumptions'!C66</f>
         <v/>
       </c>
     </row>
@@ -10051,7 +10051,7 @@
         </is>
       </c>
       <c r="C27" s="58">
-        <f>(C26-C20)/'Assumptions'!C65</f>
+        <f>(C26-C20)/'Assumptions'!C66</f>
         <v/>
       </c>
     </row>
@@ -10078,7 +10078,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P67"/>
+  <dimension ref="A1:P68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -10684,259 +10684,264 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>Other income (% revenue)</t>
+          <t>Consolidation uplift (consol vs standalone rev) %</t>
         </is>
       </c>
       <c r="I22" s="19" t="n">
-        <v>0.018</v>
+        <v>0.02</v>
       </c>
       <c r="J22" s="19" t="n">
-        <v>0.018</v>
+        <v>0.02</v>
       </c>
       <c r="K22" s="19" t="n">
-        <v>0.018</v>
+        <v>0.02</v>
       </c>
       <c r="L22" s="19" t="n">
-        <v>0.018</v>
+        <v>0.02</v>
       </c>
       <c r="M22" s="19" t="n">
-        <v>0.018</v>
+        <v>0.02</v>
       </c>
       <c r="N22" s="19" t="n">
-        <v>0.018</v>
+        <v>0.02</v>
       </c>
       <c r="O22" s="19" t="n">
-        <v>0.018</v>
+        <v>0.02</v>
+      </c>
+      <c r="P22" s="13" t="inlineStr">
+        <is>
+          <t>Subsidiary/JV contribution to revenue; historical 0-6% (FY26 ~0%).</t>
+        </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>Employee cost (% revenue)</t>
+          <t>Other income (% revenue)</t>
         </is>
       </c>
       <c r="I23" s="19" t="n">
-        <v>0.135</v>
+        <v>0.018</v>
       </c>
       <c r="J23" s="19" t="n">
-        <v>0.128</v>
+        <v>0.018</v>
       </c>
       <c r="K23" s="19" t="n">
-        <v>0.122</v>
+        <v>0.018</v>
       </c>
       <c r="L23" s="19" t="n">
-        <v>0.116</v>
+        <v>0.018</v>
       </c>
       <c r="M23" s="19" t="n">
-        <v>0.112</v>
+        <v>0.018</v>
       </c>
       <c r="N23" s="19" t="n">
-        <v>0.108</v>
+        <v>0.018</v>
       </c>
       <c r="O23" s="19" t="n">
-        <v>0.105</v>
+        <v>0.018</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>Subcontracting &amp; erection (% revenue, in COGS)</t>
+          <t>Employee cost (% revenue)</t>
         </is>
       </c>
       <c r="I24" s="19" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.135</v>
       </c>
       <c r="J24" s="19" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.128</v>
       </c>
       <c r="K24" s="19" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.122</v>
       </c>
       <c r="L24" s="19" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.116</v>
       </c>
       <c r="M24" s="19" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.112</v>
       </c>
       <c r="N24" s="19" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.108</v>
       </c>
       <c r="O24" s="19" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.105</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>Selling &amp; admin (% revenue)</t>
+          <t>Subcontracting &amp; erection (% revenue, in COGS)</t>
         </is>
       </c>
       <c r="I25" s="19" t="n">
-        <v>0.075</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="J25" s="19" t="n">
-        <v>0.075</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="K25" s="19" t="n">
-        <v>0.075</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="L25" s="19" t="n">
-        <v>0.075</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="M25" s="19" t="n">
-        <v>0.075</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="N25" s="19" t="n">
-        <v>0.075</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="O25" s="19" t="n">
-        <v>0.075</v>
+        <v>0.08500000000000001</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  COGS: Steel (% revenue)</t>
+          <t>Selling &amp; admin (% revenue)</t>
         </is>
       </c>
       <c r="I26" s="19" t="n">
-        <v>0.12</v>
+        <v>0.075</v>
       </c>
       <c r="J26" s="19" t="n">
-        <v>0.12</v>
+        <v>0.075</v>
       </c>
       <c r="K26" s="19" t="n">
-        <v>0.12</v>
+        <v>0.075</v>
       </c>
       <c r="L26" s="19" t="n">
-        <v>0.12</v>
+        <v>0.075</v>
       </c>
       <c r="M26" s="19" t="n">
-        <v>0.12</v>
+        <v>0.075</v>
       </c>
       <c r="N26" s="19" t="n">
-        <v>0.12</v>
+        <v>0.075</v>
       </c>
       <c r="O26" s="19" t="n">
-        <v>0.12</v>
+        <v>0.075</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  COGS: Copper (% revenue)</t>
+          <t xml:space="preserve">  COGS: Steel (% revenue)</t>
         </is>
       </c>
       <c r="I27" s="19" t="n">
-        <v>0.05</v>
+        <v>0.12</v>
       </c>
       <c r="J27" s="19" t="n">
-        <v>0.05</v>
+        <v>0.12</v>
       </c>
       <c r="K27" s="19" t="n">
-        <v>0.05</v>
+        <v>0.12</v>
       </c>
       <c r="L27" s="19" t="n">
-        <v>0.05</v>
+        <v>0.12</v>
       </c>
       <c r="M27" s="19" t="n">
-        <v>0.05</v>
+        <v>0.12</v>
       </c>
       <c r="N27" s="19" t="n">
-        <v>0.05</v>
+        <v>0.12</v>
       </c>
       <c r="O27" s="19" t="n">
-        <v>0.05</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  COGS: Electrical &amp; electronic components (% rev)</t>
+          <t xml:space="preserve">  COGS: Copper (% revenue)</t>
         </is>
       </c>
       <c r="I28" s="19" t="n">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="J28" s="19" t="n">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="K28" s="19" t="n">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="L28" s="19" t="n">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="M28" s="19" t="n">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="N28" s="19" t="n">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="O28" s="19" t="n">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  COGS: Imported components (% revenue)</t>
+          <t xml:space="preserve">  COGS: Electrical &amp; electronic components (% rev)</t>
         </is>
       </c>
       <c r="I29" s="19" t="n">
-        <v>0.08</v>
+        <v>0.1</v>
       </c>
       <c r="J29" s="19" t="n">
-        <v>0.08</v>
+        <v>0.1</v>
       </c>
       <c r="K29" s="19" t="n">
-        <v>0.08</v>
+        <v>0.1</v>
       </c>
       <c r="L29" s="19" t="n">
-        <v>0.08</v>
+        <v>0.1</v>
       </c>
       <c r="M29" s="19" t="n">
-        <v>0.08</v>
+        <v>0.1</v>
       </c>
       <c r="N29" s="19" t="n">
-        <v>0.08</v>
+        <v>0.1</v>
       </c>
       <c r="O29" s="19" t="n">
-        <v>0.08</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  OpEx: Selling &amp; distribution (% revenue)</t>
+          <t xml:space="preserve">  COGS: Imported components (% revenue)</t>
         </is>
       </c>
       <c r="I30" s="19" t="n">
-        <v>0.025</v>
+        <v>0.08</v>
       </c>
       <c r="J30" s="19" t="n">
-        <v>0.025</v>
+        <v>0.08</v>
       </c>
       <c r="K30" s="19" t="n">
-        <v>0.025</v>
+        <v>0.08</v>
       </c>
       <c r="L30" s="19" t="n">
-        <v>0.025</v>
+        <v>0.08</v>
       </c>
       <c r="M30" s="19" t="n">
-        <v>0.025</v>
+        <v>0.08</v>
       </c>
       <c r="N30" s="19" t="n">
-        <v>0.025</v>
+        <v>0.08</v>
       </c>
       <c r="O30" s="19" t="n">
-        <v>0.025</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  OpEx: Research &amp; development (% revenue)</t>
+          <t xml:space="preserve">  OpEx: Selling &amp; distribution (% revenue)</t>
         </is>
       </c>
       <c r="I31" s="19" t="n">
@@ -10964,287 +10969,287 @@
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>Revenue mix: Power segment %</t>
+          <t xml:space="preserve">  OpEx: Research &amp; development (% revenue)</t>
         </is>
       </c>
       <c r="I32" s="19" t="n">
-        <v>0.75</v>
+        <v>0.025</v>
       </c>
       <c r="J32" s="19" t="n">
-        <v>0.75</v>
+        <v>0.025</v>
       </c>
       <c r="K32" s="19" t="n">
-        <v>0.75</v>
+        <v>0.025</v>
       </c>
       <c r="L32" s="19" t="n">
-        <v>0.75</v>
+        <v>0.025</v>
       </c>
       <c r="M32" s="19" t="n">
-        <v>0.75</v>
+        <v>0.025</v>
       </c>
       <c r="N32" s="19" t="n">
-        <v>0.75</v>
+        <v>0.025</v>
       </c>
       <c r="O32" s="19" t="n">
-        <v>0.75</v>
+        <v>0.025</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>Revenue mix: Industry segment %</t>
+          <t>Revenue mix: Power segment %</t>
         </is>
       </c>
       <c r="I33" s="19" t="n">
-        <v>0.22</v>
+        <v>0.75</v>
       </c>
       <c r="J33" s="19" t="n">
-        <v>0.22</v>
+        <v>0.75</v>
       </c>
       <c r="K33" s="19" t="n">
-        <v>0.22</v>
+        <v>0.75</v>
       </c>
       <c r="L33" s="19" t="n">
-        <v>0.22</v>
+        <v>0.75</v>
       </c>
       <c r="M33" s="19" t="n">
-        <v>0.22</v>
+        <v>0.75</v>
       </c>
       <c r="N33" s="19" t="n">
-        <v>0.22</v>
+        <v>0.75</v>
       </c>
       <c r="O33" s="19" t="n">
-        <v>0.22</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>Capital expenditure</t>
-        </is>
-      </c>
-      <c r="I34" s="17" t="n">
-        <v>600</v>
-      </c>
-      <c r="J34" s="17" t="n">
-        <v>700</v>
-      </c>
-      <c r="K34" s="17" t="n">
-        <v>750</v>
-      </c>
-      <c r="L34" s="17" t="n">
-        <v>800</v>
-      </c>
-      <c r="M34" s="17" t="n">
-        <v>850</v>
-      </c>
-      <c r="N34" s="17" t="n">
-        <v>900</v>
-      </c>
-      <c r="O34" s="17" t="n">
-        <v>950</v>
+          <t>Revenue mix: Industry segment %</t>
+        </is>
+      </c>
+      <c r="I34" s="19" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="J34" s="19" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="K34" s="19" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="L34" s="19" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="M34" s="19" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="N34" s="19" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="O34" s="19" t="n">
+        <v>0.22</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>Depreciation rate (% opening net block)</t>
-        </is>
-      </c>
-      <c r="I35" s="19" t="n">
-        <v>0.095</v>
-      </c>
-      <c r="J35" s="19" t="n">
-        <v>0.095</v>
-      </c>
-      <c r="K35" s="19" t="n">
-        <v>0.095</v>
-      </c>
-      <c r="L35" s="19" t="n">
-        <v>0.095</v>
-      </c>
-      <c r="M35" s="19" t="n">
-        <v>0.095</v>
-      </c>
-      <c r="N35" s="19" t="n">
-        <v>0.095</v>
-      </c>
-      <c r="O35" s="19" t="n">
-        <v>0.095</v>
+          <t>Capital expenditure</t>
+        </is>
+      </c>
+      <c r="I35" s="17" t="n">
+        <v>600</v>
+      </c>
+      <c r="J35" s="17" t="n">
+        <v>700</v>
+      </c>
+      <c r="K35" s="17" t="n">
+        <v>750</v>
+      </c>
+      <c r="L35" s="17" t="n">
+        <v>800</v>
+      </c>
+      <c r="M35" s="17" t="n">
+        <v>850</v>
+      </c>
+      <c r="N35" s="17" t="n">
+        <v>900</v>
+      </c>
+      <c r="O35" s="17" t="n">
+        <v>950</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>Trade receivable days</t>
-        </is>
-      </c>
-      <c r="I36" s="20" t="n">
-        <v>75</v>
-      </c>
-      <c r="J36" s="20" t="n">
-        <v>75</v>
-      </c>
-      <c r="K36" s="20" t="n">
-        <v>75</v>
-      </c>
-      <c r="L36" s="20" t="n">
-        <v>75</v>
-      </c>
-      <c r="M36" s="20" t="n">
-        <v>75</v>
-      </c>
-      <c r="N36" s="20" t="n">
-        <v>75</v>
-      </c>
-      <c r="O36" s="20" t="n">
-        <v>75</v>
+          <t>Depreciation rate (% opening net block)</t>
+        </is>
+      </c>
+      <c r="I36" s="19" t="n">
+        <v>0.095</v>
+      </c>
+      <c r="J36" s="19" t="n">
+        <v>0.095</v>
+      </c>
+      <c r="K36" s="19" t="n">
+        <v>0.095</v>
+      </c>
+      <c r="L36" s="19" t="n">
+        <v>0.095</v>
+      </c>
+      <c r="M36" s="19" t="n">
+        <v>0.095</v>
+      </c>
+      <c r="N36" s="19" t="n">
+        <v>0.095</v>
+      </c>
+      <c r="O36" s="19" t="n">
+        <v>0.095</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>Inventory days</t>
+          <t>Trade receivable days</t>
         </is>
       </c>
       <c r="I37" s="20" t="n">
-        <v>210</v>
+        <v>75</v>
       </c>
       <c r="J37" s="20" t="n">
-        <v>205</v>
+        <v>75</v>
       </c>
       <c r="K37" s="20" t="n">
-        <v>200</v>
+        <v>75</v>
       </c>
       <c r="L37" s="20" t="n">
-        <v>200</v>
+        <v>75</v>
       </c>
       <c r="M37" s="20" t="n">
-        <v>195</v>
+        <v>75</v>
       </c>
       <c r="N37" s="20" t="n">
-        <v>195</v>
+        <v>75</v>
       </c>
       <c r="O37" s="20" t="n">
-        <v>190</v>
+        <v>75</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t>Trade payable days</t>
+          <t>Inventory days</t>
         </is>
       </c>
       <c r="I38" s="20" t="n">
-        <v>175</v>
+        <v>210</v>
       </c>
       <c r="J38" s="20" t="n">
-        <v>175</v>
+        <v>205</v>
       </c>
       <c r="K38" s="20" t="n">
-        <v>175</v>
+        <v>200</v>
       </c>
       <c r="L38" s="20" t="n">
-        <v>175</v>
+        <v>200</v>
       </c>
       <c r="M38" s="20" t="n">
-        <v>175</v>
+        <v>195</v>
       </c>
       <c r="N38" s="20" t="n">
-        <v>175</v>
+        <v>195</v>
       </c>
       <c r="O38" s="20" t="n">
-        <v>175</v>
+        <v>190</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>Contract assets (% revenue)</t>
-        </is>
-      </c>
-      <c r="I39" s="19" t="n">
-        <v>0.235</v>
-      </c>
-      <c r="J39" s="19" t="n">
-        <v>0.235</v>
-      </c>
-      <c r="K39" s="19" t="n">
-        <v>0.235</v>
-      </c>
-      <c r="L39" s="19" t="n">
-        <v>0.235</v>
-      </c>
-      <c r="M39" s="19" t="n">
-        <v>0.235</v>
-      </c>
-      <c r="N39" s="19" t="n">
-        <v>0.235</v>
-      </c>
-      <c r="O39" s="19" t="n">
-        <v>0.235</v>
+          <t>Trade payable days</t>
+        </is>
+      </c>
+      <c r="I39" s="20" t="n">
+        <v>175</v>
+      </c>
+      <c r="J39" s="20" t="n">
+        <v>175</v>
+      </c>
+      <c r="K39" s="20" t="n">
+        <v>175</v>
+      </c>
+      <c r="L39" s="20" t="n">
+        <v>175</v>
+      </c>
+      <c r="M39" s="20" t="n">
+        <v>175</v>
+      </c>
+      <c r="N39" s="20" t="n">
+        <v>175</v>
+      </c>
+      <c r="O39" s="20" t="n">
+        <v>175</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t>Contract liabilities / advances (% revenue)</t>
+          <t>Contract assets (% revenue)</t>
         </is>
       </c>
       <c r="I40" s="19" t="n">
-        <v>0.355</v>
+        <v>0.235</v>
       </c>
       <c r="J40" s="19" t="n">
-        <v>0.355</v>
+        <v>0.235</v>
       </c>
       <c r="K40" s="19" t="n">
-        <v>0.355</v>
+        <v>0.235</v>
       </c>
       <c r="L40" s="19" t="n">
-        <v>0.355</v>
+        <v>0.235</v>
       </c>
       <c r="M40" s="19" t="n">
-        <v>0.355</v>
+        <v>0.235</v>
       </c>
       <c r="N40" s="19" t="n">
-        <v>0.355</v>
+        <v>0.235</v>
       </c>
       <c r="O40" s="19" t="n">
-        <v>0.355</v>
+        <v>0.235</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>Other current/non-curr assets growth %</t>
+          <t>Contract liabilities / advances (% revenue)</t>
         </is>
       </c>
       <c r="I41" s="19" t="n">
-        <v>0.03</v>
+        <v>0.355</v>
       </c>
       <c r="J41" s="19" t="n">
-        <v>0.03</v>
+        <v>0.355</v>
       </c>
       <c r="K41" s="19" t="n">
-        <v>0.03</v>
+        <v>0.355</v>
       </c>
       <c r="L41" s="19" t="n">
-        <v>0.03</v>
+        <v>0.355</v>
       </c>
       <c r="M41" s="19" t="n">
-        <v>0.03</v>
+        <v>0.355</v>
       </c>
       <c r="N41" s="19" t="n">
-        <v>0.03</v>
+        <v>0.355</v>
       </c>
       <c r="O41" s="19" t="n">
-        <v>0.03</v>
+        <v>0.355</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t>Provisions &amp; other liabilities growth %</t>
+          <t>Other current/non-curr assets growth %</t>
         </is>
       </c>
       <c r="I42" s="19" t="n">
@@ -11272,419 +11277,447 @@
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
         <is>
-          <t>Capital work-in-progress (closing)</t>
-        </is>
-      </c>
-      <c r="I43" s="17" t="n">
-        <v>400</v>
-      </c>
-      <c r="J43" s="17" t="n">
-        <v>400</v>
-      </c>
-      <c r="K43" s="17" t="n">
-        <v>400</v>
-      </c>
-      <c r="L43" s="17" t="n">
-        <v>400</v>
-      </c>
-      <c r="M43" s="17" t="n">
-        <v>400</v>
-      </c>
-      <c r="N43" s="17" t="n">
-        <v>400</v>
-      </c>
-      <c r="O43" s="17" t="n">
-        <v>400</v>
+          <t>Provisions &amp; other liabilities growth %</t>
+        </is>
+      </c>
+      <c r="I43" s="19" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="J43" s="19" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="K43" s="19" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="L43" s="19" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="M43" s="19" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="N43" s="19" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="O43" s="19" t="n">
+        <v>0.03</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
         <is>
-          <t>Investments (closing)</t>
+          <t>Capital work-in-progress (closing)</t>
         </is>
       </c>
       <c r="I44" s="17" t="n">
-        <v>310</v>
+        <v>400</v>
       </c>
       <c r="J44" s="17" t="n">
-        <v>320</v>
+        <v>400</v>
       </c>
       <c r="K44" s="17" t="n">
-        <v>330</v>
+        <v>400</v>
       </c>
       <c r="L44" s="17" t="n">
-        <v>340</v>
+        <v>400</v>
       </c>
       <c r="M44" s="17" t="n">
-        <v>350</v>
+        <v>400</v>
       </c>
       <c r="N44" s="17" t="n">
-        <v>360</v>
+        <v>400</v>
       </c>
       <c r="O44" s="17" t="n">
-        <v>370</v>
+        <v>400</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
         <is>
-          <t>Effective tax rate</t>
-        </is>
-      </c>
-      <c r="I45" s="19" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="J45" s="19" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="K45" s="19" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="L45" s="19" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="M45" s="19" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="N45" s="19" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="O45" s="19" t="n">
-        <v>0.25</v>
+          <t>Investments (closing)</t>
+        </is>
+      </c>
+      <c r="I45" s="17" t="n">
+        <v>310</v>
+      </c>
+      <c r="J45" s="17" t="n">
+        <v>320</v>
+      </c>
+      <c r="K45" s="17" t="n">
+        <v>330</v>
+      </c>
+      <c r="L45" s="17" t="n">
+        <v>340</v>
+      </c>
+      <c r="M45" s="17" t="n">
+        <v>350</v>
+      </c>
+      <c r="N45" s="17" t="n">
+        <v>360</v>
+      </c>
+      <c r="O45" s="17" t="n">
+        <v>370</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t>Dividend payout (% PAT)</t>
+          <t>Effective tax rate</t>
         </is>
       </c>
       <c r="I46" s="19" t="n">
-        <v>0.3</v>
+        <v>0.25</v>
       </c>
       <c r="J46" s="19" t="n">
-        <v>0.3</v>
+        <v>0.25</v>
       </c>
       <c r="K46" s="19" t="n">
-        <v>0.3</v>
+        <v>0.25</v>
       </c>
       <c r="L46" s="19" t="n">
-        <v>0.3</v>
+        <v>0.25</v>
       </c>
       <c r="M46" s="19" t="n">
-        <v>0.3</v>
+        <v>0.25</v>
       </c>
       <c r="N46" s="19" t="n">
-        <v>0.3</v>
+        <v>0.25</v>
       </c>
       <c r="O46" s="19" t="n">
-        <v>0.3</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>New borrowings drawn</t>
-        </is>
-      </c>
-      <c r="I47" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="J47" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="K47" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="L47" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="M47" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="N47" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="O47" s="17" t="n">
-        <v>0</v>
+          <t>Dividend payout (% PAT)</t>
+        </is>
+      </c>
+      <c r="I47" s="19" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J47" s="19" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="K47" s="19" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="L47" s="19" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="M47" s="19" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="N47" s="19" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="O47" s="19" t="n">
+        <v>0.3</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t>Debt repayment</t>
+          <t>New borrowings drawn</t>
         </is>
       </c>
       <c r="I48" s="17" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="J48" s="17" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="K48" s="17" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="L48" s="17" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="M48" s="17" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="N48" s="17" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="O48" s="17" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>Interest rate on opening debt</t>
-        </is>
-      </c>
-      <c r="I49" s="19" t="n">
-        <v>0.08500000000000001</v>
-      </c>
-      <c r="J49" s="19" t="n">
-        <v>0.08500000000000001</v>
-      </c>
-      <c r="K49" s="19" t="n">
-        <v>0.08500000000000001</v>
-      </c>
-      <c r="L49" s="19" t="n">
-        <v>0.08500000000000001</v>
-      </c>
-      <c r="M49" s="19" t="n">
-        <v>0.08500000000000001</v>
-      </c>
-      <c r="N49" s="19" t="n">
-        <v>0.08500000000000001</v>
-      </c>
-      <c r="O49" s="19" t="n">
-        <v>0.08500000000000001</v>
+          <t>Debt repayment</t>
+        </is>
+      </c>
+      <c r="I49" s="17" t="n">
+        <v>1000</v>
+      </c>
+      <c r="J49" s="17" t="n">
+        <v>1000</v>
+      </c>
+      <c r="K49" s="17" t="n">
+        <v>1000</v>
+      </c>
+      <c r="L49" s="17" t="n">
+        <v>1000</v>
+      </c>
+      <c r="M49" s="17" t="n">
+        <v>1000</v>
+      </c>
+      <c r="N49" s="17" t="n">
+        <v>1000</v>
+      </c>
+      <c r="O49" s="17" t="n">
+        <v>1000</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t>LT borrowings (% of total debt)</t>
+          <t>Interest rate on opening debt</t>
         </is>
       </c>
       <c r="I50" s="19" t="n">
-        <v>0.35</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="J50" s="19" t="n">
-        <v>0.35</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="K50" s="19" t="n">
-        <v>0.35</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="L50" s="19" t="n">
-        <v>0.35</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="M50" s="19" t="n">
-        <v>0.35</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="N50" s="19" t="n">
-        <v>0.35</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="O50" s="19" t="n">
-        <v>0.35</v>
+        <v>0.08500000000000001</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>Other non-current assets (closing)</t>
-        </is>
-      </c>
-      <c r="I51" s="17" t="n">
-        <v>15500</v>
-      </c>
-      <c r="J51" s="17" t="n">
-        <v>16000</v>
-      </c>
-      <c r="K51" s="17" t="n">
-        <v>16500</v>
-      </c>
-      <c r="L51" s="17" t="n">
-        <v>17000</v>
-      </c>
-      <c r="M51" s="17" t="n">
-        <v>17500</v>
-      </c>
-      <c r="N51" s="17" t="n">
-        <v>18000</v>
-      </c>
-      <c r="O51" s="17" t="n">
-        <v>18500</v>
+          <t>LT borrowings (% of total debt)</t>
+        </is>
+      </c>
+      <c r="I51" s="19" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="J51" s="19" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="K51" s="19" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="L51" s="19" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="M51" s="19" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="N51" s="19" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="O51" s="19" t="n">
+        <v>0.35</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
         <is>
+          <t>Other non-current assets (closing)</t>
+        </is>
+      </c>
+      <c r="I52" s="17" t="n">
+        <v>15500</v>
+      </c>
+      <c r="J52" s="17" t="n">
+        <v>16000</v>
+      </c>
+      <c r="K52" s="17" t="n">
+        <v>16500</v>
+      </c>
+      <c r="L52" s="17" t="n">
+        <v>17000</v>
+      </c>
+      <c r="M52" s="17" t="n">
+        <v>17500</v>
+      </c>
+      <c r="N52" s="17" t="n">
+        <v>18000</v>
+      </c>
+      <c r="O52" s="17" t="n">
+        <v>18500</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
           <t>Other non-current liabilities (closing)</t>
         </is>
       </c>
-      <c r="I52" s="17" t="n">
+      <c r="I53" s="17" t="n">
         <v>6200</v>
       </c>
-      <c r="J52" s="17" t="n">
+      <c r="J53" s="17" t="n">
         <v>6400</v>
       </c>
-      <c r="K52" s="17" t="n">
+      <c r="K53" s="17" t="n">
         <v>6600</v>
       </c>
-      <c r="L52" s="17" t="n">
+      <c r="L53" s="17" t="n">
         <v>6800</v>
       </c>
-      <c r="M52" s="17" t="n">
+      <c r="M53" s="17" t="n">
         <v>7000</v>
       </c>
-      <c r="N52" s="17" t="n">
+      <c r="N53" s="17" t="n">
         <v>7200</v>
       </c>
-      <c r="O52" s="17" t="n">
+      <c r="O53" s="17" t="n">
         <v>7400</v>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="6" t="inlineStr">
+    <row r="55">
+      <c r="A55" s="6" t="inlineStr">
         <is>
           <t>WACC &amp; valuation inputs</t>
         </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="5" t="inlineStr">
-        <is>
-          <t>Risk-free rate (10Y India G-Sec)</t>
-        </is>
-      </c>
-      <c r="C55" s="19" t="n">
-        <v>0.068</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="5" t="inlineStr">
         <is>
-          <t>Levered beta</t>
-        </is>
-      </c>
-      <c r="C56" s="21" t="n">
-        <v>1.25</v>
+          <t>Risk-free rate (10Y India G-Sec)</t>
+        </is>
+      </c>
+      <c r="C56" s="19" t="n">
+        <v>0.068</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="5" t="inlineStr">
         <is>
-          <t>Equity risk premium</t>
-        </is>
-      </c>
-      <c r="C57" s="19" t="n">
-        <v>0.065</v>
+          <t>Levered beta</t>
+        </is>
+      </c>
+      <c r="C57" s="21" t="n">
+        <v>1.25</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="5" t="inlineStr">
         <is>
-          <t>Pre-tax cost of debt</t>
+          <t>Equity risk premium</t>
         </is>
       </c>
       <c r="C58" s="19" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.065</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="5" t="inlineStr">
         <is>
-          <t>Marginal tax rate (WACC)</t>
+          <t>Pre-tax cost of debt</t>
         </is>
       </c>
       <c r="C59" s="19" t="n">
-        <v>0.25</v>
+        <v>0.08500000000000001</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="5" t="inlineStr">
         <is>
-          <t>Target weight of debt</t>
+          <t>Marginal tax rate (WACC)</t>
         </is>
       </c>
       <c r="C60" s="19" t="n">
-        <v>0.15</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="5" t="inlineStr">
         <is>
-          <t>Target weight of equity</t>
+          <t>Target weight of debt</t>
         </is>
       </c>
       <c r="C61" s="19" t="n">
-        <v>0.85</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="5" t="inlineStr">
         <is>
+          <t>Target weight of equity</t>
+        </is>
+      </c>
+      <c r="C62" s="19" t="n">
+        <v>0.85</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="5" t="inlineStr">
+        <is>
           <t>Terminal growth rate</t>
         </is>
       </c>
-      <c r="C62" s="19" t="n">
+      <c r="C63" s="19" t="n">
         <v>0.045</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="4" t="inlineStr">
-        <is>
-          <t>Cost of equity (Ke = Rf + B x ERP)</t>
-        </is>
-      </c>
-      <c r="C63" s="22">
-        <f>'Assumptions'!C55+'Assumptions'!C56*'Assumptions'!C57</f>
-        <v/>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
         <is>
+          <t>Cost of equity (Ke = Rf + B x ERP)</t>
+        </is>
+      </c>
+      <c r="C64" s="22">
+        <f>'Assumptions'!C56+'Assumptions'!C57*'Assumptions'!C58</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="4" t="inlineStr">
+        <is>
           <t>WACC (We*Ke + Wd*Kd*(1-t))</t>
         </is>
       </c>
-      <c r="C64" s="18">
-        <f>'Assumptions'!C61*'Assumptions'!C63+'Assumptions'!C60*'Assumptions'!C58*(1-'Assumptions'!C59)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="5" t="inlineStr">
-        <is>
-          <t>Shares outstanding (crore)</t>
-        </is>
-      </c>
-      <c r="C65" s="23" t="n">
-        <v>348.05</v>
+      <c r="C65" s="18">
+        <f>'Assumptions'!C62*'Assumptions'!C64+'Assumptions'!C61*'Assumptions'!C59*(1-'Assumptions'!C60)</f>
+        <v/>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="5" t="inlineStr">
         <is>
-          <t>Current market price (INR)</t>
-        </is>
-      </c>
-      <c r="C66" s="21" t="n">
-        <v>403</v>
+          <t>Shares outstanding (crore)</t>
+        </is>
+      </c>
+      <c r="C66" s="23" t="n">
+        <v>348.05</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="5" t="inlineStr">
         <is>
+          <t>Current market price (INR)</t>
+        </is>
+      </c>
+      <c r="C67" s="21" t="n">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="5" t="inlineStr">
+        <is>
           <t>Face value (INR)</t>
         </is>
       </c>
-      <c r="C67" s="21" t="n">
+      <c r="C68" s="21" t="n">
         <v>2</v>
       </c>
     </row>
@@ -11766,29 +11799,29 @@
         </is>
       </c>
       <c r="C5" s="66">
-        <f>'Assumptions'!C62+-0.015</f>
+        <f>'Assumptions'!C63+-0.015</f>
         <v/>
       </c>
       <c r="D5" s="66">
-        <f>'Assumptions'!C62+-0.0075</f>
+        <f>'Assumptions'!C63+-0.0075</f>
         <v/>
       </c>
       <c r="E5" s="66">
-        <f>'Assumptions'!C62+0.0</f>
+        <f>'Assumptions'!C63+0.0</f>
         <v/>
       </c>
       <c r="F5" s="66">
-        <f>'Assumptions'!C62+0.0075</f>
+        <f>'Assumptions'!C63+0.0075</f>
         <v/>
       </c>
       <c r="G5" s="66">
-        <f>'Assumptions'!C62+0.015</f>
+        <f>'Assumptions'!C63+0.015</f>
         <v/>
       </c>
     </row>
     <row r="6">
       <c r="B6" s="66">
-        <f>'Assumptions'!C64+0.02</f>
+        <f>'Assumptions'!C65+0.02</f>
         <v/>
       </c>
       <c r="C6" s="67">
@@ -11814,7 +11847,7 @@
     </row>
     <row r="7">
       <c r="B7" s="66">
-        <f>'Assumptions'!C64+0.01</f>
+        <f>'Assumptions'!C65+0.01</f>
         <v/>
       </c>
       <c r="C7" s="67">
@@ -11840,7 +11873,7 @@
     </row>
     <row r="8">
       <c r="B8" s="66">
-        <f>'Assumptions'!C64+0.0</f>
+        <f>'Assumptions'!C65+0.0</f>
         <v/>
       </c>
       <c r="C8" s="67">
@@ -11866,7 +11899,7 @@
     </row>
     <row r="9">
       <c r="B9" s="66">
-        <f>'Assumptions'!C64+-0.01</f>
+        <f>'Assumptions'!C65+-0.01</f>
         <v/>
       </c>
       <c r="C9" s="67">
@@ -11892,7 +11925,7 @@
     </row>
     <row r="10">
       <c r="B10" s="66">
-        <f>'Assumptions'!C64+-0.02</f>
+        <f>'Assumptions'!C65+-0.02</f>
         <v/>
       </c>
       <c r="C10" s="67">
@@ -12075,7 +12108,7 @@
         <v>0.155</v>
       </c>
       <c r="C8" s="55">
-        <f>'Assumptions'!C64</f>
+        <f>'Assumptions'!C65</f>
         <v/>
       </c>
       <c r="D8" s="19" t="n">
@@ -12184,15 +12217,15 @@
         </is>
       </c>
       <c r="B14" s="58">
-        <f>B13/'Assumptions'!C65</f>
+        <f>B13/'Assumptions'!C66</f>
         <v/>
       </c>
       <c r="C14" s="58">
-        <f>C13/'Assumptions'!C65</f>
+        <f>C13/'Assumptions'!C66</f>
         <v/>
       </c>
       <c r="D14" s="58">
-        <f>D13/'Assumptions'!C65</f>
+        <f>D13/'Assumptions'!C66</f>
         <v/>
       </c>
     </row>
@@ -12316,7 +12349,7 @@
         <v/>
       </c>
       <c r="H4" s="69">
-        <f>'Assumptions'!C64</f>
+        <f>'Assumptions'!C65</f>
         <v/>
       </c>
     </row>
@@ -12764,31 +12797,31 @@
         </is>
       </c>
       <c r="I10" s="72">
-        <f>IF(ABS('Forecast Financial Statements'!I5-'Revenue Build-up'!I11)&lt;0.5,"OK","REVIEW")</f>
+        <f>IF(ABS('Forecast Financial Statements'!I5-'Revenue Build-up'!I14)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
       <c r="J10" s="72">
-        <f>IF(ABS('Forecast Financial Statements'!J5-'Revenue Build-up'!J11)&lt;0.5,"OK","REVIEW")</f>
+        <f>IF(ABS('Forecast Financial Statements'!J5-'Revenue Build-up'!J14)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
       <c r="K10" s="72">
-        <f>IF(ABS('Forecast Financial Statements'!K5-'Revenue Build-up'!K11)&lt;0.5,"OK","REVIEW")</f>
+        <f>IF(ABS('Forecast Financial Statements'!K5-'Revenue Build-up'!K14)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
       <c r="L10" s="72">
-        <f>IF(ABS('Forecast Financial Statements'!L5-'Revenue Build-up'!L11)&lt;0.5,"OK","REVIEW")</f>
+        <f>IF(ABS('Forecast Financial Statements'!L5-'Revenue Build-up'!L14)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
       <c r="M10" s="72">
-        <f>IF(ABS('Forecast Financial Statements'!M5-'Revenue Build-up'!M11)&lt;0.5,"OK","REVIEW")</f>
+        <f>IF(ABS('Forecast Financial Statements'!M5-'Revenue Build-up'!M14)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
       <c r="N10" s="72">
-        <f>IF(ABS('Forecast Financial Statements'!N5-'Revenue Build-up'!N11)&lt;0.5,"OK","REVIEW")</f>
+        <f>IF(ABS('Forecast Financial Statements'!N5-'Revenue Build-up'!N14)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
       <c r="O10" s="72">
-        <f>IF(ABS('Forecast Financial Statements'!O5-'Revenue Build-up'!O11)&lt;0.5,"OK","REVIEW")</f>
+        <f>IF(ABS('Forecast Financial Statements'!O5-'Revenue Build-up'!O14)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
     </row>
@@ -14237,31 +14270,31 @@
         </is>
       </c>
       <c r="B21" s="35">
-        <f>B20/'Assumptions'!C65</f>
+        <f>B20/'Assumptions'!C66</f>
         <v/>
       </c>
       <c r="C21" s="35">
-        <f>C20/'Assumptions'!C65</f>
+        <f>C20/'Assumptions'!C66</f>
         <v/>
       </c>
       <c r="D21" s="35">
-        <f>D20/'Assumptions'!C65</f>
+        <f>D20/'Assumptions'!C66</f>
         <v/>
       </c>
       <c r="E21" s="35">
-        <f>E20/'Assumptions'!C65</f>
+        <f>E20/'Assumptions'!C66</f>
         <v/>
       </c>
       <c r="F21" s="35">
-        <f>F20/'Assumptions'!C65</f>
+        <f>F20/'Assumptions'!C66</f>
         <v/>
       </c>
       <c r="G21" s="35">
-        <f>G20/'Assumptions'!C65</f>
+        <f>G20/'Assumptions'!C66</f>
         <v/>
       </c>
       <c r="H21" s="35">
-        <f>H20/'Assumptions'!C65</f>
+        <f>H20/'Assumptions'!C66</f>
         <v/>
       </c>
     </row>
@@ -15911,16 +15944,16 @@
         </is>
       </c>
       <c r="B8" s="30" t="n">
-        <v>-21000</v>
+        <v>-20495</v>
       </c>
       <c r="C8" s="30" t="n">
-        <v>-17000</v>
+        <v>-16296</v>
       </c>
       <c r="D8" s="30" t="n">
-        <v>-20800</v>
+        <v>-20153</v>
       </c>
       <c r="E8" s="30" t="n">
-        <v>-22921</v>
+        <v>-22136</v>
       </c>
       <c r="F8" s="30" t="n">
         <v>-22921</v>
@@ -15929,7 +15962,12 @@
         <v>-27355</v>
       </c>
       <c r="H8" s="30" t="n">
-        <v>-33800</v>
+        <v>-33782</v>
+      </c>
+      <c r="P8" s="13" t="inlineStr">
+        <is>
+          <t>standalone rev from operations</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -16371,7 +16409,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O20"/>
+  <dimension ref="A1:O23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -16415,7 +16453,7 @@
     <row r="2">
       <c r="A2" s="13" t="inlineStr">
         <is>
-          <t>Order-book-driven: Revenue = Execution rate x Opening order book. Closing OB = Opening + Inflow - Revenue.</t>
+          <t>Order book is rolled on a STANDALONE basis (as BHEL discloses it): Standalone revenue = Execution rate x Opening order book; Closing OB = Opening + Inflow - Standalone revenue. Consolidated revenue (used in the P&amp;L) is then bridged from standalone via a consolidation uplift.</t>
         </is>
       </c>
     </row>
@@ -16499,7 +16537,7 @@
     <row r="5">
       <c r="A5" s="11" t="inlineStr">
         <is>
-          <t>Order book roll-forward &amp; revenue recognition</t>
+          <t>A.  Order book roll-forward  (standalone basis, as disclosed)</t>
         </is>
       </c>
       <c r="B5" s="1" t="n"/>
@@ -16520,7 +16558,7 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Opening order book</t>
+          <t>Opening order book (standalone)</t>
         </is>
       </c>
       <c r="B6" s="43">
@@ -16646,35 +16684,35 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Less: revenue executed</t>
+          <t>Less: standalone revenue executed</t>
         </is>
       </c>
       <c r="B8" s="43">
-        <f>-'Historical Financial Statements'!B5</f>
+        <f>'Operational Drivers'!B8</f>
         <v/>
       </c>
       <c r="C8" s="43">
-        <f>-'Historical Financial Statements'!C5</f>
+        <f>'Operational Drivers'!C8</f>
         <v/>
       </c>
       <c r="D8" s="43">
-        <f>-'Historical Financial Statements'!D5</f>
+        <f>'Operational Drivers'!D8</f>
         <v/>
       </c>
       <c r="E8" s="43">
-        <f>-'Historical Financial Statements'!E5</f>
+        <f>'Operational Drivers'!E8</f>
         <v/>
       </c>
       <c r="F8" s="43">
-        <f>-'Historical Financial Statements'!F5</f>
+        <f>'Operational Drivers'!F8</f>
         <v/>
       </c>
       <c r="G8" s="43">
-        <f>-'Historical Financial Statements'!G5</f>
+        <f>'Operational Drivers'!G8</f>
         <v/>
       </c>
       <c r="H8" s="43">
-        <f>-'Historical Financial Statements'!H5</f>
+        <f>'Operational Drivers'!H8</f>
         <v/>
       </c>
       <c r="I8" s="33">
@@ -16709,7 +16747,7 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Closing order book</t>
+          <t>Closing order book (standalone)</t>
         </is>
       </c>
       <c r="B9" s="44">
@@ -16770,523 +16808,670 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>Revenue from operations</t>
-        </is>
-      </c>
-      <c r="B11" s="44">
-        <f>'Historical Financial Statements'!B5</f>
-        <v/>
-      </c>
-      <c r="C11" s="44">
-        <f>'Historical Financial Statements'!C5</f>
-        <v/>
-      </c>
-      <c r="D11" s="44">
-        <f>'Historical Financial Statements'!D5</f>
-        <v/>
-      </c>
-      <c r="E11" s="44">
-        <f>'Historical Financial Statements'!E5</f>
-        <v/>
-      </c>
-      <c r="F11" s="44">
-        <f>'Historical Financial Statements'!F5</f>
-        <v/>
-      </c>
-      <c r="G11" s="44">
-        <f>'Historical Financial Statements'!G5</f>
-        <v/>
-      </c>
-      <c r="H11" s="44">
-        <f>'Historical Financial Statements'!H5</f>
-        <v/>
-      </c>
-      <c r="I11" s="45">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>B.  Standalone -&gt; consolidated revenue bridge</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="n"/>
+      <c r="C11" s="1" t="n"/>
+      <c r="D11" s="1" t="n"/>
+      <c r="E11" s="1" t="n"/>
+      <c r="F11" s="1" t="n"/>
+      <c r="G11" s="1" t="n"/>
+      <c r="H11" s="1" t="n"/>
+      <c r="I11" s="1" t="n"/>
+      <c r="J11" s="1" t="n"/>
+      <c r="K11" s="1" t="n"/>
+      <c r="L11" s="1" t="n"/>
+      <c r="M11" s="1" t="n"/>
+      <c r="N11" s="1" t="n"/>
+      <c r="O11" s="1" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Standalone revenue from operations</t>
+        </is>
+      </c>
+      <c r="B12" s="43">
+        <f>-B8</f>
+        <v/>
+      </c>
+      <c r="C12" s="43">
+        <f>-C8</f>
+        <v/>
+      </c>
+      <c r="D12" s="43">
+        <f>-D8</f>
+        <v/>
+      </c>
+      <c r="E12" s="43">
+        <f>-E8</f>
+        <v/>
+      </c>
+      <c r="F12" s="43">
+        <f>-F8</f>
+        <v/>
+      </c>
+      <c r="G12" s="43">
+        <f>-G8</f>
+        <v/>
+      </c>
+      <c r="H12" s="43">
+        <f>-H8</f>
+        <v/>
+      </c>
+      <c r="I12" s="33">
         <f>-I8</f>
         <v/>
       </c>
-      <c r="J11" s="45">
+      <c r="J12" s="33">
         <f>-J8</f>
         <v/>
       </c>
-      <c r="K11" s="45">
+      <c r="K12" s="33">
         <f>-K8</f>
         <v/>
       </c>
-      <c r="L11" s="45">
+      <c r="L12" s="33">
         <f>-L8</f>
         <v/>
       </c>
-      <c r="M11" s="45">
+      <c r="M12" s="33">
         <f>-M8</f>
         <v/>
       </c>
-      <c r="N11" s="45">
+      <c r="N12" s="33">
         <f>-N8</f>
         <v/>
       </c>
-      <c r="O11" s="45">
+      <c r="O12" s="33">
         <f>-O8</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>Revenue growth %</t>
-        </is>
-      </c>
-      <c r="C12" s="40">
-        <f>C11/B11-1</f>
-        <v/>
-      </c>
-      <c r="D12" s="40">
-        <f>D11/C11-1</f>
-        <v/>
-      </c>
-      <c r="E12" s="40">
-        <f>E11/D11-1</f>
-        <v/>
-      </c>
-      <c r="F12" s="40">
-        <f>F11/E11-1</f>
-        <v/>
-      </c>
-      <c r="G12" s="40">
-        <f>G11/F11-1</f>
-        <v/>
-      </c>
-      <c r="H12" s="40">
-        <f>H11/G11-1</f>
-        <v/>
-      </c>
-      <c r="I12" s="40">
-        <f>I11/H11-1</f>
-        <v/>
-      </c>
-      <c r="J12" s="40">
-        <f>J11/I11-1</f>
-        <v/>
-      </c>
-      <c r="K12" s="40">
-        <f>K11/J11-1</f>
-        <v/>
-      </c>
-      <c r="L12" s="40">
-        <f>L11/K11-1</f>
-        <v/>
-      </c>
-      <c r="M12" s="40">
-        <f>M11/L11-1</f>
-        <v/>
-      </c>
-      <c r="N12" s="40">
-        <f>N11/M11-1</f>
-        <v/>
-      </c>
-      <c r="O12" s="40">
-        <f>O11/N11-1</f>
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Execution rate %</t>
-        </is>
-      </c>
-      <c r="B13" s="40">
-        <f>B11/B6</f>
-        <v/>
-      </c>
-      <c r="C13" s="40">
-        <f>C11/C6</f>
-        <v/>
-      </c>
-      <c r="D13" s="40">
-        <f>D11/D6</f>
-        <v/>
-      </c>
-      <c r="E13" s="40">
-        <f>E11/E6</f>
-        <v/>
-      </c>
-      <c r="F13" s="40">
-        <f>F11/F6</f>
-        <v/>
-      </c>
-      <c r="G13" s="40">
-        <f>G11/G6</f>
-        <v/>
-      </c>
-      <c r="H13" s="40">
-        <f>H11/H6</f>
+          <t>Consolidation uplift % (consol/standalone - 1)</t>
+        </is>
+      </c>
+      <c r="B13" s="36">
+        <f>'Historical Financial Statements'!B5/B12-1</f>
+        <v/>
+      </c>
+      <c r="C13" s="36">
+        <f>'Historical Financial Statements'!C5/C12-1</f>
+        <v/>
+      </c>
+      <c r="D13" s="36">
+        <f>'Historical Financial Statements'!D5/D12-1</f>
+        <v/>
+      </c>
+      <c r="E13" s="36">
+        <f>'Historical Financial Statements'!E5/E12-1</f>
+        <v/>
+      </c>
+      <c r="F13" s="36">
+        <f>'Historical Financial Statements'!F5/F12-1</f>
+        <v/>
+      </c>
+      <c r="G13" s="36">
+        <f>'Historical Financial Statements'!G5/G12-1</f>
+        <v/>
+      </c>
+      <c r="H13" s="36">
+        <f>'Historical Financial Statements'!H5/H12-1</f>
         <v/>
       </c>
       <c r="I13" s="40">
-        <f>I11/I6</f>
+        <f>'Assumptions'!I22</f>
         <v/>
       </c>
       <c r="J13" s="40">
-        <f>J11/J6</f>
+        <f>'Assumptions'!J22</f>
         <v/>
       </c>
       <c r="K13" s="40">
-        <f>K11/K6</f>
+        <f>'Assumptions'!K22</f>
         <v/>
       </c>
       <c r="L13" s="40">
-        <f>L11/L6</f>
+        <f>'Assumptions'!L22</f>
         <v/>
       </c>
       <c r="M13" s="40">
-        <f>M11/M6</f>
+        <f>'Assumptions'!M22</f>
         <v/>
       </c>
       <c r="N13" s="40">
-        <f>N11/N6</f>
+        <f>'Assumptions'!N22</f>
         <v/>
       </c>
       <c r="O13" s="40">
-        <f>O11/O6</f>
+        <f>'Assumptions'!O22</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>Book-to-bill (x)</t>
-        </is>
-      </c>
-      <c r="B14" s="39">
-        <f>B9/B11</f>
-        <v/>
-      </c>
-      <c r="C14" s="39">
-        <f>C9/C11</f>
-        <v/>
-      </c>
-      <c r="D14" s="39">
-        <f>D9/D11</f>
-        <v/>
-      </c>
-      <c r="E14" s="39">
-        <f>E9/E11</f>
-        <v/>
-      </c>
-      <c r="F14" s="39">
-        <f>F9/F11</f>
-        <v/>
-      </c>
-      <c r="G14" s="39">
-        <f>G9/G11</f>
-        <v/>
-      </c>
-      <c r="H14" s="39">
-        <f>H9/H11</f>
-        <v/>
-      </c>
-      <c r="I14" s="39">
-        <f>I9/I11</f>
-        <v/>
-      </c>
-      <c r="J14" s="39">
-        <f>J9/J11</f>
-        <v/>
-      </c>
-      <c r="K14" s="39">
-        <f>K9/K11</f>
-        <v/>
-      </c>
-      <c r="L14" s="39">
-        <f>L9/L11</f>
-        <v/>
-      </c>
-      <c r="M14" s="39">
-        <f>M9/M11</f>
-        <v/>
-      </c>
-      <c r="N14" s="39">
-        <f>N9/N11</f>
-        <v/>
-      </c>
-      <c r="O14" s="39">
-        <f>O9/O11</f>
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Consolidated revenue from operations  -&gt;  P&amp;L</t>
+        </is>
+      </c>
+      <c r="B14" s="32">
+        <f>B12*(1+B13)</f>
+        <v/>
+      </c>
+      <c r="C14" s="32">
+        <f>C12*(1+C13)</f>
+        <v/>
+      </c>
+      <c r="D14" s="32">
+        <f>D12*(1+D13)</f>
+        <v/>
+      </c>
+      <c r="E14" s="32">
+        <f>E12*(1+E13)</f>
+        <v/>
+      </c>
+      <c r="F14" s="32">
+        <f>F12*(1+F13)</f>
+        <v/>
+      </c>
+      <c r="G14" s="32">
+        <f>G12*(1+G13)</f>
+        <v/>
+      </c>
+      <c r="H14" s="32">
+        <f>H12*(1+H13)</f>
+        <v/>
+      </c>
+      <c r="I14" s="32">
+        <f>I12*(1+I13)</f>
+        <v/>
+      </c>
+      <c r="J14" s="32">
+        <f>J12*(1+J13)</f>
+        <v/>
+      </c>
+      <c r="K14" s="32">
+        <f>K12*(1+K13)</f>
+        <v/>
+      </c>
+      <c r="L14" s="32">
+        <f>L12*(1+L13)</f>
+        <v/>
+      </c>
+      <c r="M14" s="32">
+        <f>M12*(1+M13)</f>
+        <v/>
+      </c>
+      <c r="N14" s="32">
+        <f>N12*(1+N13)</f>
+        <v/>
+      </c>
+      <c r="O14" s="32">
+        <f>O12*(1+O13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Revenue growth % (consolidated)</t>
+        </is>
+      </c>
+      <c r="C15" s="40">
+        <f>C14/B14-1</f>
+        <v/>
+      </c>
+      <c r="D15" s="40">
+        <f>D14/C14-1</f>
+        <v/>
+      </c>
+      <c r="E15" s="40">
+        <f>E14/D14-1</f>
+        <v/>
+      </c>
+      <c r="F15" s="40">
+        <f>F14/E14-1</f>
+        <v/>
+      </c>
+      <c r="G15" s="40">
+        <f>G14/F14-1</f>
+        <v/>
+      </c>
+      <c r="H15" s="40">
+        <f>H14/G14-1</f>
+        <v/>
+      </c>
+      <c r="I15" s="40">
+        <f>I14/H14-1</f>
+        <v/>
+      </c>
+      <c r="J15" s="40">
+        <f>J14/I14-1</f>
+        <v/>
+      </c>
+      <c r="K15" s="40">
+        <f>K14/J14-1</f>
+        <v/>
+      </c>
+      <c r="L15" s="40">
+        <f>L14/K14-1</f>
+        <v/>
+      </c>
+      <c r="M15" s="40">
+        <f>M14/L14-1</f>
+        <v/>
+      </c>
+      <c r="N15" s="40">
+        <f>N14/M14-1</f>
+        <v/>
+      </c>
+      <c r="O15" s="40">
+        <f>O14/N14-1</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="11" t="inlineStr">
-        <is>
-          <t>Segment revenue breakup</t>
-        </is>
-      </c>
-      <c r="B16" s="1" t="n"/>
-      <c r="C16" s="1" t="n"/>
-      <c r="D16" s="1" t="n"/>
-      <c r="E16" s="1" t="n"/>
-      <c r="F16" s="1" t="n"/>
-      <c r="G16" s="1" t="n"/>
-      <c r="H16" s="1" t="n"/>
-      <c r="I16" s="1" t="n"/>
-      <c r="J16" s="1" t="n"/>
-      <c r="K16" s="1" t="n"/>
-      <c r="L16" s="1" t="n"/>
-      <c r="M16" s="1" t="n"/>
-      <c r="N16" s="1" t="n"/>
-      <c r="O16" s="1" t="n"/>
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Execution rate % (standalone rev / opening OB)</t>
+        </is>
+      </c>
+      <c r="B16" s="40">
+        <f>B12/B6</f>
+        <v/>
+      </c>
+      <c r="C16" s="40">
+        <f>C12/C6</f>
+        <v/>
+      </c>
+      <c r="D16" s="40">
+        <f>D12/D6</f>
+        <v/>
+      </c>
+      <c r="E16" s="40">
+        <f>E12/E6</f>
+        <v/>
+      </c>
+      <c r="F16" s="40">
+        <f>F12/F6</f>
+        <v/>
+      </c>
+      <c r="G16" s="40">
+        <f>G12/G6</f>
+        <v/>
+      </c>
+      <c r="H16" s="40">
+        <f>H12/H6</f>
+        <v/>
+      </c>
+      <c r="I16" s="40">
+        <f>I12/I6</f>
+        <v/>
+      </c>
+      <c r="J16" s="40">
+        <f>J12/J6</f>
+        <v/>
+      </c>
+      <c r="K16" s="40">
+        <f>K12/K6</f>
+        <v/>
+      </c>
+      <c r="L16" s="40">
+        <f>L12/L6</f>
+        <v/>
+      </c>
+      <c r="M16" s="40">
+        <f>M12/M6</f>
+        <v/>
+      </c>
+      <c r="N16" s="40">
+        <f>N12/N6</f>
+        <v/>
+      </c>
+      <c r="O16" s="40">
+        <f>O12/O6</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
+          <t>Book-to-bill (closing OB / standalone rev, x)</t>
+        </is>
+      </c>
+      <c r="B17" s="39">
+        <f>B9/B12</f>
+        <v/>
+      </c>
+      <c r="C17" s="39">
+        <f>C9/C12</f>
+        <v/>
+      </c>
+      <c r="D17" s="39">
+        <f>D9/D12</f>
+        <v/>
+      </c>
+      <c r="E17" s="39">
+        <f>E9/E12</f>
+        <v/>
+      </c>
+      <c r="F17" s="39">
+        <f>F9/F12</f>
+        <v/>
+      </c>
+      <c r="G17" s="39">
+        <f>G9/G12</f>
+        <v/>
+      </c>
+      <c r="H17" s="39">
+        <f>H9/H12</f>
+        <v/>
+      </c>
+      <c r="I17" s="39">
+        <f>I9/I12</f>
+        <v/>
+      </c>
+      <c r="J17" s="39">
+        <f>J9/J12</f>
+        <v/>
+      </c>
+      <c r="K17" s="39">
+        <f>K9/K12</f>
+        <v/>
+      </c>
+      <c r="L17" s="39">
+        <f>L9/L12</f>
+        <v/>
+      </c>
+      <c r="M17" s="39">
+        <f>M9/M12</f>
+        <v/>
+      </c>
+      <c r="N17" s="39">
+        <f>N9/N12</f>
+        <v/>
+      </c>
+      <c r="O17" s="39">
+        <f>O9/O12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="11" t="inlineStr">
+        <is>
+          <t>C.  Segment revenue breakup (consolidated)</t>
+        </is>
+      </c>
+      <c r="B19" s="1" t="n"/>
+      <c r="C19" s="1" t="n"/>
+      <c r="D19" s="1" t="n"/>
+      <c r="E19" s="1" t="n"/>
+      <c r="F19" s="1" t="n"/>
+      <c r="G19" s="1" t="n"/>
+      <c r="H19" s="1" t="n"/>
+      <c r="I19" s="1" t="n"/>
+      <c r="J19" s="1" t="n"/>
+      <c r="K19" s="1" t="n"/>
+      <c r="L19" s="1" t="n"/>
+      <c r="M19" s="1" t="n"/>
+      <c r="N19" s="1" t="n"/>
+      <c r="O19" s="1" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
           <t>Power segment</t>
         </is>
       </c>
-      <c r="B17" s="43">
+      <c r="B20" s="43">
         <f>'Operational Drivers'!B14</f>
         <v/>
       </c>
-      <c r="C17" s="43">
+      <c r="C20" s="43">
         <f>'Operational Drivers'!C14</f>
         <v/>
       </c>
-      <c r="D17" s="43">
+      <c r="D20" s="43">
         <f>'Operational Drivers'!D14</f>
         <v/>
       </c>
-      <c r="E17" s="43">
+      <c r="E20" s="43">
         <f>'Operational Drivers'!E14</f>
         <v/>
       </c>
-      <c r="F17" s="43">
+      <c r="F20" s="43">
         <f>'Operational Drivers'!F14</f>
         <v/>
       </c>
-      <c r="G17" s="43">
+      <c r="G20" s="43">
         <f>'Operational Drivers'!G14</f>
         <v/>
       </c>
-      <c r="H17" s="43">
+      <c r="H20" s="43">
         <f>'Operational Drivers'!H14</f>
         <v/>
       </c>
-      <c r="I17" s="33">
-        <f>I11*'Assumptions'!I32</f>
-        <v/>
-      </c>
-      <c r="J17" s="33">
-        <f>J11*'Assumptions'!J32</f>
-        <v/>
-      </c>
-      <c r="K17" s="33">
-        <f>K11*'Assumptions'!K32</f>
-        <v/>
-      </c>
-      <c r="L17" s="33">
-        <f>L11*'Assumptions'!L32</f>
-        <v/>
-      </c>
-      <c r="M17" s="33">
-        <f>M11*'Assumptions'!M32</f>
-        <v/>
-      </c>
-      <c r="N17" s="33">
-        <f>N11*'Assumptions'!N32</f>
-        <v/>
-      </c>
-      <c r="O17" s="33">
-        <f>O11*'Assumptions'!O32</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="5" t="inlineStr">
+      <c r="I20" s="33">
+        <f>I14*'Assumptions'!I33</f>
+        <v/>
+      </c>
+      <c r="J20" s="33">
+        <f>J14*'Assumptions'!J33</f>
+        <v/>
+      </c>
+      <c r="K20" s="33">
+        <f>K14*'Assumptions'!K33</f>
+        <v/>
+      </c>
+      <c r="L20" s="33">
+        <f>L14*'Assumptions'!L33</f>
+        <v/>
+      </c>
+      <c r="M20" s="33">
+        <f>M14*'Assumptions'!M33</f>
+        <v/>
+      </c>
+      <c r="N20" s="33">
+        <f>N14*'Assumptions'!N33</f>
+        <v/>
+      </c>
+      <c r="O20" s="33">
+        <f>O14*'Assumptions'!O33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
         <is>
           <t>Industry segment</t>
         </is>
       </c>
-      <c r="B18" s="43">
+      <c r="B21" s="43">
         <f>'Operational Drivers'!B15</f>
         <v/>
       </c>
-      <c r="C18" s="43">
+      <c r="C21" s="43">
         <f>'Operational Drivers'!C15</f>
         <v/>
       </c>
-      <c r="D18" s="43">
+      <c r="D21" s="43">
         <f>'Operational Drivers'!D15</f>
         <v/>
       </c>
-      <c r="E18" s="43">
+      <c r="E21" s="43">
         <f>'Operational Drivers'!E15</f>
         <v/>
       </c>
-      <c r="F18" s="43">
+      <c r="F21" s="43">
         <f>'Operational Drivers'!F15</f>
         <v/>
       </c>
-      <c r="G18" s="43">
+      <c r="G21" s="43">
         <f>'Operational Drivers'!G15</f>
         <v/>
       </c>
-      <c r="H18" s="43">
+      <c r="H21" s="43">
         <f>'Operational Drivers'!H15</f>
         <v/>
       </c>
-      <c r="I18" s="33">
-        <f>I11*'Assumptions'!I33</f>
-        <v/>
-      </c>
-      <c r="J18" s="33">
-        <f>J11*'Assumptions'!J33</f>
-        <v/>
-      </c>
-      <c r="K18" s="33">
-        <f>K11*'Assumptions'!K33</f>
-        <v/>
-      </c>
-      <c r="L18" s="33">
-        <f>L11*'Assumptions'!L33</f>
-        <v/>
-      </c>
-      <c r="M18" s="33">
-        <f>M11*'Assumptions'!M33</f>
-        <v/>
-      </c>
-      <c r="N18" s="33">
-        <f>N11*'Assumptions'!N33</f>
-        <v/>
-      </c>
-      <c r="O18" s="33">
-        <f>O11*'Assumptions'!O33</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="5" t="inlineStr">
+      <c r="I21" s="33">
+        <f>I14*'Assumptions'!I34</f>
+        <v/>
+      </c>
+      <c r="J21" s="33">
+        <f>J14*'Assumptions'!J34</f>
+        <v/>
+      </c>
+      <c r="K21" s="33">
+        <f>K14*'Assumptions'!K34</f>
+        <v/>
+      </c>
+      <c r="L21" s="33">
+        <f>L14*'Assumptions'!L34</f>
+        <v/>
+      </c>
+      <c r="M21" s="33">
+        <f>M14*'Assumptions'!M34</f>
+        <v/>
+      </c>
+      <c r="N21" s="33">
+        <f>N14*'Assumptions'!N34</f>
+        <v/>
+      </c>
+      <c r="O21" s="33">
+        <f>O14*'Assumptions'!O34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>Others / exports / renewables</t>
         </is>
       </c>
-      <c r="B19" s="43">
+      <c r="B22" s="43">
         <f>'Operational Drivers'!B16</f>
         <v/>
       </c>
-      <c r="C19" s="43">
+      <c r="C22" s="43">
         <f>'Operational Drivers'!C16</f>
         <v/>
       </c>
-      <c r="D19" s="43">
+      <c r="D22" s="43">
         <f>'Operational Drivers'!D16</f>
         <v/>
       </c>
-      <c r="E19" s="43">
+      <c r="E22" s="43">
         <f>'Operational Drivers'!E16</f>
         <v/>
       </c>
-      <c r="F19" s="43">
+      <c r="F22" s="43">
         <f>'Operational Drivers'!F16</f>
         <v/>
       </c>
-      <c r="G19" s="43">
+      <c r="G22" s="43">
         <f>'Operational Drivers'!G16</f>
         <v/>
       </c>
-      <c r="H19" s="43">
+      <c r="H22" s="43">
         <f>'Operational Drivers'!H16</f>
         <v/>
       </c>
-      <c r="I19" s="33">
-        <f>I11*(1-'Assumptions'!I32-'Assumptions'!I33)</f>
-        <v/>
-      </c>
-      <c r="J19" s="33">
-        <f>J11*(1-'Assumptions'!J32-'Assumptions'!J33)</f>
-        <v/>
-      </c>
-      <c r="K19" s="33">
-        <f>K11*(1-'Assumptions'!K32-'Assumptions'!K33)</f>
-        <v/>
-      </c>
-      <c r="L19" s="33">
-        <f>L11*(1-'Assumptions'!L32-'Assumptions'!L33)</f>
-        <v/>
-      </c>
-      <c r="M19" s="33">
-        <f>M11*(1-'Assumptions'!M32-'Assumptions'!M33)</f>
-        <v/>
-      </c>
-      <c r="N19" s="33">
-        <f>N11*(1-'Assumptions'!N32-'Assumptions'!N33)</f>
-        <v/>
-      </c>
-      <c r="O19" s="33">
-        <f>O11*(1-'Assumptions'!O32-'Assumptions'!O33)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>Total segment revenue (check vs total)</t>
-        </is>
-      </c>
-      <c r="B20" s="45">
-        <f>SUM(B17:B19)</f>
-        <v/>
-      </c>
-      <c r="C20" s="45">
-        <f>SUM(C17:C19)</f>
-        <v/>
-      </c>
-      <c r="D20" s="45">
-        <f>SUM(D17:D19)</f>
-        <v/>
-      </c>
-      <c r="E20" s="45">
-        <f>SUM(E17:E19)</f>
-        <v/>
-      </c>
-      <c r="F20" s="45">
-        <f>SUM(F17:F19)</f>
-        <v/>
-      </c>
-      <c r="G20" s="45">
-        <f>SUM(G17:G19)</f>
-        <v/>
-      </c>
-      <c r="H20" s="45">
-        <f>SUM(H17:H19)</f>
-        <v/>
-      </c>
-      <c r="I20" s="45">
-        <f>SUM(I17:I19)</f>
-        <v/>
-      </c>
-      <c r="J20" s="45">
-        <f>SUM(J17:J19)</f>
-        <v/>
-      </c>
-      <c r="K20" s="45">
-        <f>SUM(K17:K19)</f>
-        <v/>
-      </c>
-      <c r="L20" s="45">
-        <f>SUM(L17:L19)</f>
-        <v/>
-      </c>
-      <c r="M20" s="45">
-        <f>SUM(M17:M19)</f>
-        <v/>
-      </c>
-      <c r="N20" s="45">
-        <f>SUM(N17:N19)</f>
-        <v/>
-      </c>
-      <c r="O20" s="45">
-        <f>SUM(O17:O19)</f>
+      <c r="I22" s="33">
+        <f>I14*(1-'Assumptions'!I33-'Assumptions'!I34)</f>
+        <v/>
+      </c>
+      <c r="J22" s="33">
+        <f>J14*(1-'Assumptions'!J33-'Assumptions'!J34)</f>
+        <v/>
+      </c>
+      <c r="K22" s="33">
+        <f>K14*(1-'Assumptions'!K33-'Assumptions'!K34)</f>
+        <v/>
+      </c>
+      <c r="L22" s="33">
+        <f>L14*(1-'Assumptions'!L33-'Assumptions'!L34)</f>
+        <v/>
+      </c>
+      <c r="M22" s="33">
+        <f>M14*(1-'Assumptions'!M33-'Assumptions'!M34)</f>
+        <v/>
+      </c>
+      <c r="N22" s="33">
+        <f>N14*(1-'Assumptions'!N33-'Assumptions'!N34)</f>
+        <v/>
+      </c>
+      <c r="O22" s="33">
+        <f>O14*(1-'Assumptions'!O33-'Assumptions'!O34)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Total segment revenue (check vs consolidated)</t>
+        </is>
+      </c>
+      <c r="B23" s="45">
+        <f>SUM(B20:B22)</f>
+        <v/>
+      </c>
+      <c r="C23" s="45">
+        <f>SUM(C20:C22)</f>
+        <v/>
+      </c>
+      <c r="D23" s="45">
+        <f>SUM(D20:D22)</f>
+        <v/>
+      </c>
+      <c r="E23" s="45">
+        <f>SUM(E20:E22)</f>
+        <v/>
+      </c>
+      <c r="F23" s="45">
+        <f>SUM(F20:F22)</f>
+        <v/>
+      </c>
+      <c r="G23" s="45">
+        <f>SUM(G20:G22)</f>
+        <v/>
+      </c>
+      <c r="H23" s="45">
+        <f>SUM(H20:H22)</f>
+        <v/>
+      </c>
+      <c r="I23" s="45">
+        <f>SUM(I20:I22)</f>
+        <v/>
+      </c>
+      <c r="J23" s="45">
+        <f>SUM(J20:J22)</f>
+        <v/>
+      </c>
+      <c r="K23" s="45">
+        <f>SUM(K20:K22)</f>
+        <v/>
+      </c>
+      <c r="L23" s="45">
+        <f>SUM(L20:L22)</f>
+        <v/>
+      </c>
+      <c r="M23" s="45">
+        <f>SUM(M20:M22)</f>
+        <v/>
+      </c>
+      <c r="N23" s="45">
+        <f>SUM(N20:N22)</f>
+        <v/>
+      </c>
+      <c r="O23" s="45">
+        <f>SUM(O20:O22)</f>
         <v/>
       </c>
     </row>
@@ -17482,31 +17667,31 @@
         <v/>
       </c>
       <c r="I6" s="33">
-        <f>'Revenue Build-up'!I11</f>
+        <f>'Revenue Build-up'!I14</f>
         <v/>
       </c>
       <c r="J6" s="33">
-        <f>'Revenue Build-up'!J11</f>
+        <f>'Revenue Build-up'!J14</f>
         <v/>
       </c>
       <c r="K6" s="33">
-        <f>'Revenue Build-up'!K11</f>
+        <f>'Revenue Build-up'!K14</f>
         <v/>
       </c>
       <c r="L6" s="33">
-        <f>'Revenue Build-up'!L11</f>
+        <f>'Revenue Build-up'!L14</f>
         <v/>
       </c>
       <c r="M6" s="33">
-        <f>'Revenue Build-up'!M11</f>
+        <f>'Revenue Build-up'!M14</f>
         <v/>
       </c>
       <c r="N6" s="33">
-        <f>'Revenue Build-up'!N11</f>
+        <f>'Revenue Build-up'!N14</f>
         <v/>
       </c>
       <c r="O6" s="33">
-        <f>'Revenue Build-up'!O11</f>
+        <f>'Revenue Build-up'!O14</f>
         <v/>
       </c>
     </row>
@@ -17517,31 +17702,31 @@
         </is>
       </c>
       <c r="I7" s="33">
-        <f>I6*'Assumptions'!I26</f>
+        <f>I6*'Assumptions'!I27</f>
         <v/>
       </c>
       <c r="J7" s="33">
-        <f>J6*'Assumptions'!J26</f>
+        <f>J6*'Assumptions'!J27</f>
         <v/>
       </c>
       <c r="K7" s="33">
-        <f>K6*'Assumptions'!K26</f>
+        <f>K6*'Assumptions'!K27</f>
         <v/>
       </c>
       <c r="L7" s="33">
-        <f>L6*'Assumptions'!L26</f>
+        <f>L6*'Assumptions'!L27</f>
         <v/>
       </c>
       <c r="M7" s="33">
-        <f>M6*'Assumptions'!M26</f>
+        <f>M6*'Assumptions'!M27</f>
         <v/>
       </c>
       <c r="N7" s="33">
-        <f>N6*'Assumptions'!N26</f>
+        <f>N6*'Assumptions'!N27</f>
         <v/>
       </c>
       <c r="O7" s="33">
-        <f>O6*'Assumptions'!O26</f>
+        <f>O6*'Assumptions'!O27</f>
         <v/>
       </c>
     </row>
@@ -17552,31 +17737,31 @@
         </is>
       </c>
       <c r="I8" s="33">
-        <f>I6*'Assumptions'!I27</f>
+        <f>I6*'Assumptions'!I28</f>
         <v/>
       </c>
       <c r="J8" s="33">
-        <f>J6*'Assumptions'!J27</f>
+        <f>J6*'Assumptions'!J28</f>
         <v/>
       </c>
       <c r="K8" s="33">
-        <f>K6*'Assumptions'!K27</f>
+        <f>K6*'Assumptions'!K28</f>
         <v/>
       </c>
       <c r="L8" s="33">
-        <f>L6*'Assumptions'!L27</f>
+        <f>L6*'Assumptions'!L28</f>
         <v/>
       </c>
       <c r="M8" s="33">
-        <f>M6*'Assumptions'!M27</f>
+        <f>M6*'Assumptions'!M28</f>
         <v/>
       </c>
       <c r="N8" s="33">
-        <f>N6*'Assumptions'!N27</f>
+        <f>N6*'Assumptions'!N28</f>
         <v/>
       </c>
       <c r="O8" s="33">
-        <f>O6*'Assumptions'!O27</f>
+        <f>O6*'Assumptions'!O28</f>
         <v/>
       </c>
     </row>
@@ -17587,31 +17772,31 @@
         </is>
       </c>
       <c r="I9" s="33">
-        <f>I6*'Assumptions'!I28</f>
+        <f>I6*'Assumptions'!I29</f>
         <v/>
       </c>
       <c r="J9" s="33">
-        <f>J6*'Assumptions'!J28</f>
+        <f>J6*'Assumptions'!J29</f>
         <v/>
       </c>
       <c r="K9" s="33">
-        <f>K6*'Assumptions'!K28</f>
+        <f>K6*'Assumptions'!K29</f>
         <v/>
       </c>
       <c r="L9" s="33">
-        <f>L6*'Assumptions'!L28</f>
+        <f>L6*'Assumptions'!L29</f>
         <v/>
       </c>
       <c r="M9" s="33">
-        <f>M6*'Assumptions'!M28</f>
+        <f>M6*'Assumptions'!M29</f>
         <v/>
       </c>
       <c r="N9" s="33">
-        <f>N6*'Assumptions'!N28</f>
+        <f>N6*'Assumptions'!N29</f>
         <v/>
       </c>
       <c r="O9" s="33">
-        <f>O6*'Assumptions'!O28</f>
+        <f>O6*'Assumptions'!O29</f>
         <v/>
       </c>
     </row>
@@ -17622,31 +17807,31 @@
         </is>
       </c>
       <c r="I10" s="33">
-        <f>I6*'Assumptions'!I29</f>
+        <f>I6*'Assumptions'!I30</f>
         <v/>
       </c>
       <c r="J10" s="33">
-        <f>J6*'Assumptions'!J29</f>
+        <f>J6*'Assumptions'!J30</f>
         <v/>
       </c>
       <c r="K10" s="33">
-        <f>K6*'Assumptions'!K29</f>
+        <f>K6*'Assumptions'!K30</f>
         <v/>
       </c>
       <c r="L10" s="33">
-        <f>L6*'Assumptions'!L29</f>
+        <f>L6*'Assumptions'!L30</f>
         <v/>
       </c>
       <c r="M10" s="33">
-        <f>M6*'Assumptions'!M29</f>
+        <f>M6*'Assumptions'!M30</f>
         <v/>
       </c>
       <c r="N10" s="33">
-        <f>N6*'Assumptions'!N29</f>
+        <f>N6*'Assumptions'!N30</f>
         <v/>
       </c>
       <c r="O10" s="33">
-        <f>O6*'Assumptions'!O29</f>
+        <f>O6*'Assumptions'!O30</f>
         <v/>
       </c>
     </row>
@@ -17657,31 +17842,31 @@
         </is>
       </c>
       <c r="I11" s="33">
-        <f>I6*(1-'Assumptions'!I15-'Assumptions'!I23-'Assumptions'!I24-'Assumptions'!I25-'Assumptions'!I26-'Assumptions'!I27-'Assumptions'!I28-'Assumptions'!I29)</f>
+        <f>I6*(1-'Assumptions'!I15-'Assumptions'!I24-'Assumptions'!I25-'Assumptions'!I26-'Assumptions'!I27-'Assumptions'!I28-'Assumptions'!I29-'Assumptions'!I30)</f>
         <v/>
       </c>
       <c r="J11" s="33">
-        <f>J6*(1-'Assumptions'!J15-'Assumptions'!J23-'Assumptions'!J24-'Assumptions'!J25-'Assumptions'!J26-'Assumptions'!J27-'Assumptions'!J28-'Assumptions'!J29)</f>
+        <f>J6*(1-'Assumptions'!J15-'Assumptions'!J24-'Assumptions'!J25-'Assumptions'!J26-'Assumptions'!J27-'Assumptions'!J28-'Assumptions'!J29-'Assumptions'!J30)</f>
         <v/>
       </c>
       <c r="K11" s="33">
-        <f>K6*(1-'Assumptions'!K15-'Assumptions'!K23-'Assumptions'!K24-'Assumptions'!K25-'Assumptions'!K26-'Assumptions'!K27-'Assumptions'!K28-'Assumptions'!K29)</f>
+        <f>K6*(1-'Assumptions'!K15-'Assumptions'!K24-'Assumptions'!K25-'Assumptions'!K26-'Assumptions'!K27-'Assumptions'!K28-'Assumptions'!K29-'Assumptions'!K30)</f>
         <v/>
       </c>
       <c r="L11" s="33">
-        <f>L6*(1-'Assumptions'!L15-'Assumptions'!L23-'Assumptions'!L24-'Assumptions'!L25-'Assumptions'!L26-'Assumptions'!L27-'Assumptions'!L28-'Assumptions'!L29)</f>
+        <f>L6*(1-'Assumptions'!L15-'Assumptions'!L24-'Assumptions'!L25-'Assumptions'!L26-'Assumptions'!L27-'Assumptions'!L28-'Assumptions'!L29-'Assumptions'!L30)</f>
         <v/>
       </c>
       <c r="M11" s="33">
-        <f>M6*(1-'Assumptions'!M15-'Assumptions'!M23-'Assumptions'!M24-'Assumptions'!M25-'Assumptions'!M26-'Assumptions'!M27-'Assumptions'!M28-'Assumptions'!M29)</f>
+        <f>M6*(1-'Assumptions'!M15-'Assumptions'!M24-'Assumptions'!M25-'Assumptions'!M26-'Assumptions'!M27-'Assumptions'!M28-'Assumptions'!M29-'Assumptions'!M30)</f>
         <v/>
       </c>
       <c r="N11" s="33">
-        <f>N6*(1-'Assumptions'!N15-'Assumptions'!N23-'Assumptions'!N24-'Assumptions'!N25-'Assumptions'!N26-'Assumptions'!N27-'Assumptions'!N28-'Assumptions'!N29)</f>
+        <f>N6*(1-'Assumptions'!N15-'Assumptions'!N24-'Assumptions'!N25-'Assumptions'!N26-'Assumptions'!N27-'Assumptions'!N28-'Assumptions'!N29-'Assumptions'!N30)</f>
         <v/>
       </c>
       <c r="O11" s="33">
-        <f>O6*(1-'Assumptions'!O15-'Assumptions'!O23-'Assumptions'!O24-'Assumptions'!O25-'Assumptions'!O26-'Assumptions'!O27-'Assumptions'!O28-'Assumptions'!O29)</f>
+        <f>O6*(1-'Assumptions'!O15-'Assumptions'!O24-'Assumptions'!O25-'Assumptions'!O26-'Assumptions'!O27-'Assumptions'!O28-'Assumptions'!O29-'Assumptions'!O30)</f>
         <v/>
       </c>
     </row>
@@ -17692,31 +17877,31 @@
         </is>
       </c>
       <c r="I12" s="33">
-        <f>I6*'Assumptions'!I24</f>
+        <f>I6*'Assumptions'!I25</f>
         <v/>
       </c>
       <c r="J12" s="33">
-        <f>J6*'Assumptions'!J24</f>
+        <f>J6*'Assumptions'!J25</f>
         <v/>
       </c>
       <c r="K12" s="33">
-        <f>K6*'Assumptions'!K24</f>
+        <f>K6*'Assumptions'!K25</f>
         <v/>
       </c>
       <c r="L12" s="33">
-        <f>L6*'Assumptions'!L24</f>
+        <f>L6*'Assumptions'!L25</f>
         <v/>
       </c>
       <c r="M12" s="33">
-        <f>M6*'Assumptions'!M24</f>
+        <f>M6*'Assumptions'!M25</f>
         <v/>
       </c>
       <c r="N12" s="33">
-        <f>N6*'Assumptions'!N24</f>
+        <f>N6*'Assumptions'!N25</f>
         <v/>
       </c>
       <c r="O12" s="33">
-        <f>O6*'Assumptions'!O24</f>
+        <f>O6*'Assumptions'!O25</f>
         <v/>
       </c>
     </row>
@@ -17902,31 +18087,31 @@
         <v/>
       </c>
       <c r="I16" s="33">
-        <f>I6*'Assumptions'!I23</f>
+        <f>I6*'Assumptions'!I24</f>
         <v/>
       </c>
       <c r="J16" s="33">
-        <f>J6*'Assumptions'!J23</f>
+        <f>J6*'Assumptions'!J24</f>
         <v/>
       </c>
       <c r="K16" s="33">
-        <f>K6*'Assumptions'!K23</f>
+        <f>K6*'Assumptions'!K24</f>
         <v/>
       </c>
       <c r="L16" s="33">
-        <f>L6*'Assumptions'!L23</f>
+        <f>L6*'Assumptions'!L24</f>
         <v/>
       </c>
       <c r="M16" s="33">
-        <f>M6*'Assumptions'!M23</f>
+        <f>M6*'Assumptions'!M24</f>
         <v/>
       </c>
       <c r="N16" s="33">
-        <f>N6*'Assumptions'!N23</f>
+        <f>N6*'Assumptions'!N24</f>
         <v/>
       </c>
       <c r="O16" s="33">
-        <f>O6*'Assumptions'!O23</f>
+        <f>O6*'Assumptions'!O24</f>
         <v/>
       </c>
     </row>
@@ -17937,31 +18122,31 @@
         </is>
       </c>
       <c r="I17" s="33">
-        <f>I6*'Assumptions'!I30</f>
+        <f>I6*'Assumptions'!I31</f>
         <v/>
       </c>
       <c r="J17" s="33">
-        <f>J6*'Assumptions'!J30</f>
+        <f>J6*'Assumptions'!J31</f>
         <v/>
       </c>
       <c r="K17" s="33">
-        <f>K6*'Assumptions'!K30</f>
+        <f>K6*'Assumptions'!K31</f>
         <v/>
       </c>
       <c r="L17" s="33">
-        <f>L6*'Assumptions'!L30</f>
+        <f>L6*'Assumptions'!L31</f>
         <v/>
       </c>
       <c r="M17" s="33">
-        <f>M6*'Assumptions'!M30</f>
+        <f>M6*'Assumptions'!M31</f>
         <v/>
       </c>
       <c r="N17" s="33">
-        <f>N6*'Assumptions'!N30</f>
+        <f>N6*'Assumptions'!N31</f>
         <v/>
       </c>
       <c r="O17" s="33">
-        <f>O6*'Assumptions'!O30</f>
+        <f>O6*'Assumptions'!O31</f>
         <v/>
       </c>
     </row>
@@ -17972,31 +18157,31 @@
         </is>
       </c>
       <c r="I18" s="33">
-        <f>I6*('Assumptions'!I25-'Assumptions'!I30-'Assumptions'!I31)</f>
+        <f>I6*('Assumptions'!I26-'Assumptions'!I31-'Assumptions'!I32)</f>
         <v/>
       </c>
       <c r="J18" s="33">
-        <f>J6*('Assumptions'!J25-'Assumptions'!J30-'Assumptions'!J31)</f>
+        <f>J6*('Assumptions'!J26-'Assumptions'!J31-'Assumptions'!J32)</f>
         <v/>
       </c>
       <c r="K18" s="33">
-        <f>K6*('Assumptions'!K25-'Assumptions'!K30-'Assumptions'!K31)</f>
+        <f>K6*('Assumptions'!K26-'Assumptions'!K31-'Assumptions'!K32)</f>
         <v/>
       </c>
       <c r="L18" s="33">
-        <f>L6*('Assumptions'!L25-'Assumptions'!L30-'Assumptions'!L31)</f>
+        <f>L6*('Assumptions'!L26-'Assumptions'!L31-'Assumptions'!L32)</f>
         <v/>
       </c>
       <c r="M18" s="33">
-        <f>M6*('Assumptions'!M25-'Assumptions'!M30-'Assumptions'!M31)</f>
+        <f>M6*('Assumptions'!M26-'Assumptions'!M31-'Assumptions'!M32)</f>
         <v/>
       </c>
       <c r="N18" s="33">
-        <f>N6*('Assumptions'!N25-'Assumptions'!N30-'Assumptions'!N31)</f>
+        <f>N6*('Assumptions'!N26-'Assumptions'!N31-'Assumptions'!N32)</f>
         <v/>
       </c>
       <c r="O18" s="33">
-        <f>O6*('Assumptions'!O25-'Assumptions'!O30-'Assumptions'!O31)</f>
+        <f>O6*('Assumptions'!O26-'Assumptions'!O31-'Assumptions'!O32)</f>
         <v/>
       </c>
     </row>
@@ -18007,31 +18192,31 @@
         </is>
       </c>
       <c r="I19" s="33">
-        <f>I6*'Assumptions'!I31</f>
+        <f>I6*'Assumptions'!I32</f>
         <v/>
       </c>
       <c r="J19" s="33">
-        <f>J6*'Assumptions'!J31</f>
+        <f>J6*'Assumptions'!J32</f>
         <v/>
       </c>
       <c r="K19" s="33">
-        <f>K6*'Assumptions'!K31</f>
+        <f>K6*'Assumptions'!K32</f>
         <v/>
       </c>
       <c r="L19" s="33">
-        <f>L6*'Assumptions'!L31</f>
+        <f>L6*'Assumptions'!L32</f>
         <v/>
       </c>
       <c r="M19" s="33">
-        <f>M6*'Assumptions'!M31</f>
+        <f>M6*'Assumptions'!M32</f>
         <v/>
       </c>
       <c r="N19" s="33">
-        <f>N6*'Assumptions'!N31</f>
+        <f>N6*'Assumptions'!N32</f>
         <v/>
       </c>
       <c r="O19" s="33">
-        <f>O6*'Assumptions'!O31</f>
+        <f>O6*'Assumptions'!O32</f>
         <v/>
       </c>
     </row>
@@ -18643,31 +18828,31 @@
         <v>6757</v>
       </c>
       <c r="I8" s="33">
-        <f>'Assumptions'!I36/365*I6</f>
+        <f>'Assumptions'!I37/365*I6</f>
         <v/>
       </c>
       <c r="J8" s="33">
-        <f>'Assumptions'!J36/365*J6</f>
+        <f>'Assumptions'!J37/365*J6</f>
         <v/>
       </c>
       <c r="K8" s="33">
-        <f>'Assumptions'!K36/365*K6</f>
+        <f>'Assumptions'!K37/365*K6</f>
         <v/>
       </c>
       <c r="L8" s="33">
-        <f>'Assumptions'!L36/365*L6</f>
+        <f>'Assumptions'!L37/365*L6</f>
         <v/>
       </c>
       <c r="M8" s="33">
-        <f>'Assumptions'!M36/365*M6</f>
+        <f>'Assumptions'!M37/365*M6</f>
         <v/>
       </c>
       <c r="N8" s="33">
-        <f>'Assumptions'!N36/365*N6</f>
+        <f>'Assumptions'!N37/365*N6</f>
         <v/>
       </c>
       <c r="O8" s="33">
-        <f>'Assumptions'!O36/365*O6</f>
+        <f>'Assumptions'!O37/365*O6</f>
         <v/>
       </c>
     </row>
@@ -18681,31 +18866,31 @@
         <v>18260</v>
       </c>
       <c r="I9" s="33">
-        <f>'Assumptions'!I37/365*I7</f>
+        <f>'Assumptions'!I38/365*I7</f>
         <v/>
       </c>
       <c r="J9" s="33">
-        <f>'Assumptions'!J37/365*J7</f>
+        <f>'Assumptions'!J38/365*J7</f>
         <v/>
       </c>
       <c r="K9" s="33">
-        <f>'Assumptions'!K37/365*K7</f>
+        <f>'Assumptions'!K38/365*K7</f>
         <v/>
       </c>
       <c r="L9" s="33">
-        <f>'Assumptions'!L37/365*L7</f>
+        <f>'Assumptions'!L38/365*L7</f>
         <v/>
       </c>
       <c r="M9" s="33">
-        <f>'Assumptions'!M37/365*M7</f>
+        <f>'Assumptions'!M38/365*M7</f>
         <v/>
       </c>
       <c r="N9" s="33">
-        <f>'Assumptions'!N37/365*N7</f>
+        <f>'Assumptions'!N38/365*N7</f>
         <v/>
       </c>
       <c r="O9" s="33">
-        <f>'Assumptions'!O37/365*O7</f>
+        <f>'Assumptions'!O38/365*O7</f>
         <v/>
       </c>
     </row>
@@ -18719,31 +18904,31 @@
         <v>8000</v>
       </c>
       <c r="I10" s="33">
-        <f>'Assumptions'!I39*I6</f>
+        <f>'Assumptions'!I40*I6</f>
         <v/>
       </c>
       <c r="J10" s="33">
-        <f>'Assumptions'!J39*J6</f>
+        <f>'Assumptions'!J40*J6</f>
         <v/>
       </c>
       <c r="K10" s="33">
-        <f>'Assumptions'!K39*K6</f>
+        <f>'Assumptions'!K40*K6</f>
         <v/>
       </c>
       <c r="L10" s="33">
-        <f>'Assumptions'!L39*L6</f>
+        <f>'Assumptions'!L40*L6</f>
         <v/>
       </c>
       <c r="M10" s="33">
-        <f>'Assumptions'!M39*M6</f>
+        <f>'Assumptions'!M40*M6</f>
         <v/>
       </c>
       <c r="N10" s="33">
-        <f>'Assumptions'!N39*N6</f>
+        <f>'Assumptions'!N40*N6</f>
         <v/>
       </c>
       <c r="O10" s="33">
-        <f>'Assumptions'!O39*O6</f>
+        <f>'Assumptions'!O40*O6</f>
         <v/>
       </c>
     </row>
@@ -18757,31 +18942,31 @@
         <v>32373</v>
       </c>
       <c r="I11" s="33">
-        <f>H11*(1+'Assumptions'!I41)</f>
+        <f>H11*(1+'Assumptions'!I42)</f>
         <v/>
       </c>
       <c r="J11" s="33">
-        <f>I11*(1+'Assumptions'!J41)</f>
+        <f>I11*(1+'Assumptions'!J42)</f>
         <v/>
       </c>
       <c r="K11" s="33">
-        <f>J11*(1+'Assumptions'!K41)</f>
+        <f>J11*(1+'Assumptions'!K42)</f>
         <v/>
       </c>
       <c r="L11" s="33">
-        <f>K11*(1+'Assumptions'!L41)</f>
+        <f>K11*(1+'Assumptions'!L42)</f>
         <v/>
       </c>
       <c r="M11" s="33">
-        <f>L11*(1+'Assumptions'!M41)</f>
+        <f>L11*(1+'Assumptions'!M42)</f>
         <v/>
       </c>
       <c r="N11" s="33">
-        <f>M11*(1+'Assumptions'!N41)</f>
+        <f>M11*(1+'Assumptions'!N42)</f>
         <v/>
       </c>
       <c r="O11" s="33">
-        <f>N11*(1+'Assumptions'!O41)</f>
+        <f>N11*(1+'Assumptions'!O42)</f>
         <v/>
       </c>
     </row>
@@ -18834,31 +19019,31 @@
         <v>14386</v>
       </c>
       <c r="I13" s="33">
-        <f>'Assumptions'!I38/365*I7</f>
+        <f>'Assumptions'!I39/365*I7</f>
         <v/>
       </c>
       <c r="J13" s="33">
-        <f>'Assumptions'!J38/365*J7</f>
+        <f>'Assumptions'!J39/365*J7</f>
         <v/>
       </c>
       <c r="K13" s="33">
-        <f>'Assumptions'!K38/365*K7</f>
+        <f>'Assumptions'!K39/365*K7</f>
         <v/>
       </c>
       <c r="L13" s="33">
-        <f>'Assumptions'!L38/365*L7</f>
+        <f>'Assumptions'!L39/365*L7</f>
         <v/>
       </c>
       <c r="M13" s="33">
-        <f>'Assumptions'!M38/365*M7</f>
+        <f>'Assumptions'!M39/365*M7</f>
         <v/>
       </c>
       <c r="N13" s="33">
-        <f>'Assumptions'!N38/365*N7</f>
+        <f>'Assumptions'!N39/365*N7</f>
         <v/>
       </c>
       <c r="O13" s="33">
-        <f>'Assumptions'!O38/365*O7</f>
+        <f>'Assumptions'!O39/365*O7</f>
         <v/>
       </c>
     </row>
@@ -18872,31 +19057,31 @@
         <v>12000</v>
       </c>
       <c r="I14" s="33">
-        <f>'Assumptions'!I40*I6</f>
+        <f>'Assumptions'!I41*I6</f>
         <v/>
       </c>
       <c r="J14" s="33">
-        <f>'Assumptions'!J40*J6</f>
+        <f>'Assumptions'!J41*J6</f>
         <v/>
       </c>
       <c r="K14" s="33">
-        <f>'Assumptions'!K40*K6</f>
+        <f>'Assumptions'!K41*K6</f>
         <v/>
       </c>
       <c r="L14" s="33">
-        <f>'Assumptions'!L40*L6</f>
+        <f>'Assumptions'!L41*L6</f>
         <v/>
       </c>
       <c r="M14" s="33">
-        <f>'Assumptions'!M40*M6</f>
+        <f>'Assumptions'!M41*M6</f>
         <v/>
       </c>
       <c r="N14" s="33">
-        <f>'Assumptions'!N40*N6</f>
+        <f>'Assumptions'!N41*N6</f>
         <v/>
       </c>
       <c r="O14" s="33">
-        <f>'Assumptions'!O40*O6</f>
+        <f>'Assumptions'!O41*O6</f>
         <v/>
       </c>
     </row>
@@ -18910,31 +19095,31 @@
         <v>15466</v>
       </c>
       <c r="I15" s="33">
-        <f>H15*(1+'Assumptions'!I42)</f>
+        <f>H15*(1+'Assumptions'!I43)</f>
         <v/>
       </c>
       <c r="J15" s="33">
-        <f>I15*(1+'Assumptions'!J42)</f>
+        <f>I15*(1+'Assumptions'!J43)</f>
         <v/>
       </c>
       <c r="K15" s="33">
-        <f>J15*(1+'Assumptions'!K42)</f>
+        <f>J15*(1+'Assumptions'!K43)</f>
         <v/>
       </c>
       <c r="L15" s="33">
-        <f>K15*(1+'Assumptions'!L42)</f>
+        <f>K15*(1+'Assumptions'!L43)</f>
         <v/>
       </c>
       <c r="M15" s="33">
-        <f>L15*(1+'Assumptions'!M42)</f>
+        <f>L15*(1+'Assumptions'!M43)</f>
         <v/>
       </c>
       <c r="N15" s="33">
-        <f>M15*(1+'Assumptions'!N42)</f>
+        <f>M15*(1+'Assumptions'!N43)</f>
         <v/>
       </c>
       <c r="O15" s="33">
-        <f>N15*(1+'Assumptions'!O42)</f>
+        <f>N15*(1+'Assumptions'!O43)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Add order-book Adjustments line (cancellations/FX/scope/taxes) so historical roll ties to reported closing OB in both sheets
</commit_message>
<xml_diff>
--- a/BHEL_Financial_Model.xlsx
+++ b/BHEL_Financial_Model.xlsx
@@ -297,10 +297,10 @@
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -708,7 +708,7 @@
           </cat>
           <val>
             <numRef>
-              <f>'Revenue Build-up'!$B$9:$O$9</f>
+              <f>'Revenue Build-up'!$B$10:$O$10</f>
             </numRef>
           </val>
         </ser>
@@ -1817,59 +1817,59 @@
           <t>Closing net block</t>
         </is>
       </c>
-      <c r="B10" s="44">
+      <c r="B10" s="45">
         <f>'Historical Financial Statements'!B28</f>
         <v/>
       </c>
-      <c r="C10" s="44">
+      <c r="C10" s="45">
         <f>'Historical Financial Statements'!C28</f>
         <v/>
       </c>
-      <c r="D10" s="44">
+      <c r="D10" s="45">
         <f>'Historical Financial Statements'!D28</f>
         <v/>
       </c>
-      <c r="E10" s="44">
+      <c r="E10" s="45">
         <f>'Historical Financial Statements'!E28</f>
         <v/>
       </c>
-      <c r="F10" s="44">
+      <c r="F10" s="45">
         <f>'Historical Financial Statements'!F28</f>
         <v/>
       </c>
-      <c r="G10" s="44">
+      <c r="G10" s="45">
         <f>'Historical Financial Statements'!G28</f>
         <v/>
       </c>
-      <c r="H10" s="44">
+      <c r="H10" s="45">
         <f>'Historical Financial Statements'!H28</f>
         <v/>
       </c>
-      <c r="I10" s="45">
+      <c r="I10" s="44">
         <f>I6+I7+I8-I9</f>
         <v/>
       </c>
-      <c r="J10" s="45">
+      <c r="J10" s="44">
         <f>J6+J7+J8-J9</f>
         <v/>
       </c>
-      <c r="K10" s="45">
+      <c r="K10" s="44">
         <f>K6+K7+K8-K9</f>
         <v/>
       </c>
-      <c r="L10" s="45">
+      <c r="L10" s="44">
         <f>L6+L7+L8-L9</f>
         <v/>
       </c>
-      <c r="M10" s="45">
+      <c r="M10" s="44">
         <f>M6+M7+M8-M9</f>
         <v/>
       </c>
-      <c r="N10" s="45">
+      <c r="N10" s="44">
         <f>N6+N7+N8-N9</f>
         <v/>
       </c>
-      <c r="O10" s="45">
+      <c r="O10" s="44">
         <f>O6+O7+O8-O9</f>
         <v/>
       </c>
@@ -2100,59 +2100,59 @@
           <t>Depreciation expense</t>
         </is>
       </c>
-      <c r="B8" s="44">
+      <c r="B8" s="45">
         <f>'Historical Financial Statements'!B13</f>
         <v/>
       </c>
-      <c r="C8" s="44">
+      <c r="C8" s="45">
         <f>'Historical Financial Statements'!C13</f>
         <v/>
       </c>
-      <c r="D8" s="44">
+      <c r="D8" s="45">
         <f>'Historical Financial Statements'!D13</f>
         <v/>
       </c>
-      <c r="E8" s="44">
+      <c r="E8" s="45">
         <f>'Historical Financial Statements'!E13</f>
         <v/>
       </c>
-      <c r="F8" s="44">
+      <c r="F8" s="45">
         <f>'Historical Financial Statements'!F13</f>
         <v/>
       </c>
-      <c r="G8" s="44">
+      <c r="G8" s="45">
         <f>'Historical Financial Statements'!G13</f>
         <v/>
       </c>
-      <c r="H8" s="44">
+      <c r="H8" s="45">
         <f>'Historical Financial Statements'!H13</f>
         <v/>
       </c>
-      <c r="I8" s="45">
+      <c r="I8" s="44">
         <f>I6*I7</f>
         <v/>
       </c>
-      <c r="J8" s="45">
+      <c r="J8" s="44">
         <f>J6*J7</f>
         <v/>
       </c>
-      <c r="K8" s="45">
+      <c r="K8" s="44">
         <f>K6*K7</f>
         <v/>
       </c>
-      <c r="L8" s="45">
+      <c r="L8" s="44">
         <f>L6*L7</f>
         <v/>
       </c>
-      <c r="M8" s="45">
+      <c r="M8" s="44">
         <f>M6*M7</f>
         <v/>
       </c>
-      <c r="N8" s="45">
+      <c r="N8" s="44">
         <f>N6*N7</f>
         <v/>
       </c>
-      <c r="O8" s="45">
+      <c r="O8" s="44">
         <f>O6*O7</f>
         <v/>
       </c>
@@ -2453,59 +2453,59 @@
           <t>Closing debt</t>
         </is>
       </c>
-      <c r="B9" s="44">
+      <c r="B9" s="45">
         <f>'Historical Financial Statements'!B35</f>
         <v/>
       </c>
-      <c r="C9" s="44">
+      <c r="C9" s="45">
         <f>'Historical Financial Statements'!C35</f>
         <v/>
       </c>
-      <c r="D9" s="44">
+      <c r="D9" s="45">
         <f>'Historical Financial Statements'!D35</f>
         <v/>
       </c>
-      <c r="E9" s="44">
+      <c r="E9" s="45">
         <f>'Historical Financial Statements'!E35</f>
         <v/>
       </c>
-      <c r="F9" s="44">
+      <c r="F9" s="45">
         <f>'Historical Financial Statements'!F35</f>
         <v/>
       </c>
-      <c r="G9" s="44">
+      <c r="G9" s="45">
         <f>'Historical Financial Statements'!G35</f>
         <v/>
       </c>
-      <c r="H9" s="44">
+      <c r="H9" s="45">
         <f>'Historical Financial Statements'!H35</f>
         <v/>
       </c>
-      <c r="I9" s="45">
+      <c r="I9" s="44">
         <f>I6+I7+I8</f>
         <v/>
       </c>
-      <c r="J9" s="45">
+      <c r="J9" s="44">
         <f>J6+J7+J8</f>
         <v/>
       </c>
-      <c r="K9" s="45">
+      <c r="K9" s="44">
         <f>K6+K7+K8</f>
         <v/>
       </c>
-      <c r="L9" s="45">
+      <c r="L9" s="44">
         <f>L6+L7+L8</f>
         <v/>
       </c>
-      <c r="M9" s="45">
+      <c r="M9" s="44">
         <f>M6+M7+M8</f>
         <v/>
       </c>
-      <c r="N9" s="45">
+      <c r="N9" s="44">
         <f>N6+N7+N8</f>
         <v/>
       </c>
-      <c r="O9" s="45">
+      <c r="O9" s="44">
         <f>O6+O7+O8</f>
         <v/>
       </c>
@@ -2897,31 +2897,31 @@
           <t>Closing other equity</t>
         </is>
       </c>
-      <c r="I10" s="45">
+      <c r="I10" s="44">
         <f>SUM(I6:I9)</f>
         <v/>
       </c>
-      <c r="J10" s="45">
+      <c r="J10" s="44">
         <f>SUM(J6:J9)</f>
         <v/>
       </c>
-      <c r="K10" s="45">
+      <c r="K10" s="44">
         <f>SUM(K6:K9)</f>
         <v/>
       </c>
-      <c r="L10" s="45">
+      <c r="L10" s="44">
         <f>SUM(L6:L9)</f>
         <v/>
       </c>
-      <c r="M10" s="45">
+      <c r="M10" s="44">
         <f>SUM(M6:M9)</f>
         <v/>
       </c>
-      <c r="N10" s="45">
+      <c r="N10" s="44">
         <f>SUM(N6:N9)</f>
         <v/>
       </c>
-      <c r="O10" s="45">
+      <c r="O10" s="44">
         <f>SUM(O6:O9)</f>
         <v/>
       </c>
@@ -3673,59 +3673,59 @@
           <t>Cash flow from operating activities</t>
         </is>
       </c>
-      <c r="B9" s="44">
+      <c r="B9" s="45">
         <f>'Historical Financial Statements'!B42</f>
         <v/>
       </c>
-      <c r="C9" s="44">
+      <c r="C9" s="45">
         <f>'Historical Financial Statements'!C42</f>
         <v/>
       </c>
-      <c r="D9" s="44">
+      <c r="D9" s="45">
         <f>'Historical Financial Statements'!D42</f>
         <v/>
       </c>
-      <c r="E9" s="44">
+      <c r="E9" s="45">
         <f>'Historical Financial Statements'!E42</f>
         <v/>
       </c>
-      <c r="F9" s="44">
+      <c r="F9" s="45">
         <f>'Historical Financial Statements'!F42</f>
         <v/>
       </c>
-      <c r="G9" s="44">
+      <c r="G9" s="45">
         <f>'Historical Financial Statements'!G42</f>
         <v/>
       </c>
-      <c r="H9" s="44">
+      <c r="H9" s="45">
         <f>'Historical Financial Statements'!H42</f>
         <v/>
       </c>
-      <c r="I9" s="45">
+      <c r="I9" s="44">
         <f>SUM(I6:I8)</f>
         <v/>
       </c>
-      <c r="J9" s="45">
+      <c r="J9" s="44">
         <f>SUM(J6:J8)</f>
         <v/>
       </c>
-      <c r="K9" s="45">
+      <c r="K9" s="44">
         <f>SUM(K6:K8)</f>
         <v/>
       </c>
-      <c r="L9" s="45">
+      <c r="L9" s="44">
         <f>SUM(L6:L8)</f>
         <v/>
       </c>
-      <c r="M9" s="45">
+      <c r="M9" s="44">
         <f>SUM(M6:M8)</f>
         <v/>
       </c>
-      <c r="N9" s="45">
+      <c r="N9" s="44">
         <f>SUM(N6:N8)</f>
         <v/>
       </c>
-      <c r="O9" s="45">
+      <c r="O9" s="44">
         <f>SUM(O6:O8)</f>
         <v/>
       </c>
@@ -3862,59 +3862,59 @@
           <t>Cash flow from investing activities</t>
         </is>
       </c>
-      <c r="B15" s="44">
+      <c r="B15" s="45">
         <f>'Historical Financial Statements'!B43</f>
         <v/>
       </c>
-      <c r="C15" s="44">
+      <c r="C15" s="45">
         <f>'Historical Financial Statements'!C43</f>
         <v/>
       </c>
-      <c r="D15" s="44">
+      <c r="D15" s="45">
         <f>'Historical Financial Statements'!D43</f>
         <v/>
       </c>
-      <c r="E15" s="44">
+      <c r="E15" s="45">
         <f>'Historical Financial Statements'!E43</f>
         <v/>
       </c>
-      <c r="F15" s="44">
+      <c r="F15" s="45">
         <f>'Historical Financial Statements'!F43</f>
         <v/>
       </c>
-      <c r="G15" s="44">
+      <c r="G15" s="45">
         <f>'Historical Financial Statements'!G43</f>
         <v/>
       </c>
-      <c r="H15" s="44">
+      <c r="H15" s="45">
         <f>'Historical Financial Statements'!H43</f>
         <v/>
       </c>
-      <c r="I15" s="45">
+      <c r="I15" s="44">
         <f>SUM(I12:I14)</f>
         <v/>
       </c>
-      <c r="J15" s="45">
+      <c r="J15" s="44">
         <f>SUM(J12:J14)</f>
         <v/>
       </c>
-      <c r="K15" s="45">
+      <c r="K15" s="44">
         <f>SUM(K12:K14)</f>
         <v/>
       </c>
-      <c r="L15" s="45">
+      <c r="L15" s="44">
         <f>SUM(L12:L14)</f>
         <v/>
       </c>
-      <c r="M15" s="45">
+      <c r="M15" s="44">
         <f>SUM(M12:M14)</f>
         <v/>
       </c>
-      <c r="N15" s="45">
+      <c r="N15" s="44">
         <f>SUM(N12:N14)</f>
         <v/>
       </c>
-      <c r="O15" s="45">
+      <c r="O15" s="44">
         <f>SUM(O12:O14)</f>
         <v/>
       </c>
@@ -4051,59 +4051,59 @@
           <t>Cash flow from financing activities</t>
         </is>
       </c>
-      <c r="B21" s="44">
+      <c r="B21" s="45">
         <f>'Historical Financial Statements'!B44</f>
         <v/>
       </c>
-      <c r="C21" s="44">
+      <c r="C21" s="45">
         <f>'Historical Financial Statements'!C44</f>
         <v/>
       </c>
-      <c r="D21" s="44">
+      <c r="D21" s="45">
         <f>'Historical Financial Statements'!D44</f>
         <v/>
       </c>
-      <c r="E21" s="44">
+      <c r="E21" s="45">
         <f>'Historical Financial Statements'!E44</f>
         <v/>
       </c>
-      <c r="F21" s="44">
+      <c r="F21" s="45">
         <f>'Historical Financial Statements'!F44</f>
         <v/>
       </c>
-      <c r="G21" s="44">
+      <c r="G21" s="45">
         <f>'Historical Financial Statements'!G44</f>
         <v/>
       </c>
-      <c r="H21" s="44">
+      <c r="H21" s="45">
         <f>'Historical Financial Statements'!H44</f>
         <v/>
       </c>
-      <c r="I21" s="45">
+      <c r="I21" s="44">
         <f>SUM(I18:I20)</f>
         <v/>
       </c>
-      <c r="J21" s="45">
+      <c r="J21" s="44">
         <f>SUM(J18:J20)</f>
         <v/>
       </c>
-      <c r="K21" s="45">
+      <c r="K21" s="44">
         <f>SUM(K18:K20)</f>
         <v/>
       </c>
-      <c r="L21" s="45">
+      <c r="L21" s="44">
         <f>SUM(L18:L20)</f>
         <v/>
       </c>
-      <c r="M21" s="45">
+      <c r="M21" s="44">
         <f>SUM(M18:M20)</f>
         <v/>
       </c>
-      <c r="N21" s="45">
+      <c r="N21" s="44">
         <f>SUM(N18:N20)</f>
         <v/>
       </c>
-      <c r="O21" s="45">
+      <c r="O21" s="44">
         <f>SUM(O18:O20)</f>
         <v/>
       </c>
@@ -4142,31 +4142,31 @@
         <f>'Historical Financial Statements'!H45</f>
         <v/>
       </c>
-      <c r="I23" s="45">
+      <c r="I23" s="44">
         <f>I9+I15+I21</f>
         <v/>
       </c>
-      <c r="J23" s="45">
+      <c r="J23" s="44">
         <f>J9+J15+J21</f>
         <v/>
       </c>
-      <c r="K23" s="45">
+      <c r="K23" s="44">
         <f>K9+K15+K21</f>
         <v/>
       </c>
-      <c r="L23" s="45">
+      <c r="L23" s="44">
         <f>L9+L15+L21</f>
         <v/>
       </c>
-      <c r="M23" s="45">
+      <c r="M23" s="44">
         <f>M9+M15+M21</f>
         <v/>
       </c>
-      <c r="N23" s="45">
+      <c r="N23" s="44">
         <f>N9+N15+N21</f>
         <v/>
       </c>
-      <c r="O23" s="45">
+      <c r="O23" s="44">
         <f>O9+O15+O21</f>
         <v/>
       </c>
@@ -4254,31 +4254,31 @@
       <c r="H25" s="47" t="n">
         <v>7000</v>
       </c>
-      <c r="I25" s="45">
+      <c r="I25" s="44">
         <f>I24+I23</f>
         <v/>
       </c>
-      <c r="J25" s="45">
+      <c r="J25" s="44">
         <f>J24+J23</f>
         <v/>
       </c>
-      <c r="K25" s="45">
+      <c r="K25" s="44">
         <f>K24+K23</f>
         <v/>
       </c>
-      <c r="L25" s="45">
+      <c r="L25" s="44">
         <f>L24+L23</f>
         <v/>
       </c>
-      <c r="M25" s="45">
+      <c r="M25" s="44">
         <f>M24+M23</f>
         <v/>
       </c>
-      <c r="N25" s="45">
+      <c r="N25" s="44">
         <f>N24+N23</f>
         <v/>
       </c>
-      <c r="O25" s="45">
+      <c r="O25" s="44">
         <f>O24+O23</f>
         <v/>
       </c>
@@ -4482,31 +4482,31 @@
         <v/>
       </c>
       <c r="I5" s="33">
-        <f>'Revenue Build-up'!I14</f>
+        <f>'Revenue Build-up'!I15</f>
         <v/>
       </c>
       <c r="J5" s="33">
-        <f>'Revenue Build-up'!J14</f>
+        <f>'Revenue Build-up'!J15</f>
         <v/>
       </c>
       <c r="K5" s="33">
-        <f>'Revenue Build-up'!K14</f>
+        <f>'Revenue Build-up'!K15</f>
         <v/>
       </c>
       <c r="L5" s="33">
-        <f>'Revenue Build-up'!L14</f>
+        <f>'Revenue Build-up'!L15</f>
         <v/>
       </c>
       <c r="M5" s="33">
-        <f>'Revenue Build-up'!M14</f>
+        <f>'Revenue Build-up'!M15</f>
         <v/>
       </c>
       <c r="N5" s="33">
-        <f>'Revenue Build-up'!N14</f>
+        <f>'Revenue Build-up'!N15</f>
         <v/>
       </c>
       <c r="O5" s="33">
-        <f>'Revenue Build-up'!O14</f>
+        <f>'Revenue Build-up'!O15</f>
         <v/>
       </c>
     </row>
@@ -9346,31 +9346,31 @@
           <t>Free cash flow to firm (FCFF)</t>
         </is>
       </c>
-      <c r="I12" s="45">
+      <c r="I12" s="44">
         <f>I8+I9+I10+I11</f>
         <v/>
       </c>
-      <c r="J12" s="45">
+      <c r="J12" s="44">
         <f>J8+J9+J10+J11</f>
         <v/>
       </c>
-      <c r="K12" s="45">
+      <c r="K12" s="44">
         <f>K8+K9+K10+K11</f>
         <v/>
       </c>
-      <c r="L12" s="45">
+      <c r="L12" s="44">
         <f>L8+L9+L10+L11</f>
         <v/>
       </c>
-      <c r="M12" s="45">
+      <c r="M12" s="44">
         <f>M8+M9+M10+M11</f>
         <v/>
       </c>
-      <c r="N12" s="45">
+      <c r="N12" s="44">
         <f>N8+N9+N10+N11</f>
         <v/>
       </c>
-      <c r="O12" s="45">
+      <c r="O12" s="44">
         <f>O8+O9+O10+O11</f>
         <v/>
       </c>
@@ -9444,31 +9444,31 @@
           <t>PV of FCFF</t>
         </is>
       </c>
-      <c r="I15" s="45">
+      <c r="I15" s="44">
         <f>I12*I14</f>
         <v/>
       </c>
-      <c r="J15" s="45">
+      <c r="J15" s="44">
         <f>J12*J14</f>
         <v/>
       </c>
-      <c r="K15" s="45">
+      <c r="K15" s="44">
         <f>K12*K14</f>
         <v/>
       </c>
-      <c r="L15" s="45">
+      <c r="L15" s="44">
         <f>L12*L14</f>
         <v/>
       </c>
-      <c r="M15" s="45">
+      <c r="M15" s="44">
         <f>M12*M14</f>
         <v/>
       </c>
-      <c r="N15" s="45">
+      <c r="N15" s="44">
         <f>N12*N14</f>
         <v/>
       </c>
-      <c r="O15" s="45">
+      <c r="O15" s="44">
         <f>O12*O14</f>
         <v/>
       </c>
@@ -12403,7 +12403,7 @@
         <v/>
       </c>
       <c r="G7" s="70">
-        <f>'Revenue Build-up'!H9</f>
+        <f>'Revenue Build-up'!H10</f>
         <v/>
       </c>
       <c r="H7" s="70">
@@ -12797,31 +12797,31 @@
         </is>
       </c>
       <c r="I10" s="72">
-        <f>IF(ABS('Forecast Financial Statements'!I5-'Revenue Build-up'!I14)&lt;0.5,"OK","REVIEW")</f>
+        <f>IF(ABS('Forecast Financial Statements'!I5-'Revenue Build-up'!I15)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
       <c r="J10" s="72">
-        <f>IF(ABS('Forecast Financial Statements'!J5-'Revenue Build-up'!J14)&lt;0.5,"OK","REVIEW")</f>
+        <f>IF(ABS('Forecast Financial Statements'!J5-'Revenue Build-up'!J15)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
       <c r="K10" s="72">
-        <f>IF(ABS('Forecast Financial Statements'!K5-'Revenue Build-up'!K14)&lt;0.5,"OK","REVIEW")</f>
+        <f>IF(ABS('Forecast Financial Statements'!K5-'Revenue Build-up'!K15)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
       <c r="L10" s="72">
-        <f>IF(ABS('Forecast Financial Statements'!L5-'Revenue Build-up'!L14)&lt;0.5,"OK","REVIEW")</f>
+        <f>IF(ABS('Forecast Financial Statements'!L5-'Revenue Build-up'!L15)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
       <c r="M10" s="72">
-        <f>IF(ABS('Forecast Financial Statements'!M5-'Revenue Build-up'!M14)&lt;0.5,"OK","REVIEW")</f>
+        <f>IF(ABS('Forecast Financial Statements'!M5-'Revenue Build-up'!M15)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
       <c r="N10" s="72">
-        <f>IF(ABS('Forecast Financial Statements'!N5-'Revenue Build-up'!N14)&lt;0.5,"OK","REVIEW")</f>
+        <f>IF(ABS('Forecast Financial Statements'!N5-'Revenue Build-up'!N15)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
       <c r="O10" s="72">
-        <f>IF(ABS('Forecast Financial Statements'!O5-'Revenue Build-up'!O14)&lt;0.5,"OK","REVIEW")</f>
+        <f>IF(ABS('Forecast Financial Statements'!O5-'Revenue Build-up'!O15)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
     </row>
@@ -15725,7 +15725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P24"/>
+  <dimension ref="A1:P26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -15769,7 +15769,7 @@
     <row r="2">
       <c r="A2" s="13" t="inlineStr">
         <is>
-          <t>Order data on standalone basis; FY20-FY22 order book are estimates (flagged).</t>
+          <t>Order data on standalone basis. FY20-22 figures are estimates (flagged). The "Adjustments" line captures order cancellations, de-scoping, FX revaluation, price/scope revisions and tax-basis differences so the roll ties to the reported closing order book.</t>
         </is>
       </c>
     </row>
@@ -15853,7 +15853,7 @@
     <row r="5">
       <c r="A5" s="11" t="inlineStr">
         <is>
-          <t>Order book dynamics (INR Crore)</t>
+          <t>Order book dynamics (INR Crore, standalone)</t>
         </is>
       </c>
       <c r="B5" s="1" t="n"/>
@@ -15966,433 +15966,503 @@
       </c>
       <c r="P8" s="13" t="inlineStr">
         <is>
-          <t>standalone rev from operations</t>
+          <t>standalone rev</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Closing order book</t>
-        </is>
-      </c>
-      <c r="B9" s="30" t="n">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>+/- Adjustments (cancellations, FX, scope, taxes)</t>
+        </is>
+      </c>
+      <c r="B9" s="33">
+        <f>B10-B6-B7-B8</f>
+        <v/>
+      </c>
+      <c r="C9" s="33">
+        <f>C10-C6-C7-C8</f>
+        <v/>
+      </c>
+      <c r="D9" s="33">
+        <f>D10-D6-D7-D8</f>
+        <v/>
+      </c>
+      <c r="E9" s="33">
+        <f>E10-E6-E7-E8</f>
+        <v/>
+      </c>
+      <c r="F9" s="33">
+        <f>F10-F6-F7-F8</f>
+        <v/>
+      </c>
+      <c r="G9" s="33">
+        <f>G10-G6-G7-G8</f>
+        <v/>
+      </c>
+      <c r="H9" s="33">
+        <f>H10-H6-H7-H8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Closing order book (reported)</t>
+        </is>
+      </c>
+      <c r="B10" s="30" t="n">
         <v>110000</v>
       </c>
-      <c r="C9" s="30" t="n">
+      <c r="C10" s="30" t="n">
         <v>102000</v>
       </c>
-      <c r="D9" s="30" t="n">
+      <c r="D10" s="30" t="n">
         <v>98000</v>
       </c>
-      <c r="E9" s="30" t="n">
+      <c r="E10" s="30" t="n">
         <v>91336</v>
       </c>
-      <c r="F9" s="30" t="n">
+      <c r="F10" s="30" t="n">
         <v>131598</v>
       </c>
-      <c r="G9" s="30" t="n">
+      <c r="G10" s="30" t="n">
         <v>196328</v>
       </c>
-      <c r="H9" s="30" t="n">
+      <c r="H10" s="30" t="n">
         <v>240000</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>Book-to-bill (closing OB/revenue, x)</t>
-        </is>
-      </c>
-      <c r="B10" s="39">
-        <f>B9/-B8</f>
-        <v/>
-      </c>
-      <c r="C10" s="39">
-        <f>C9/-C8</f>
-        <v/>
-      </c>
-      <c r="D10" s="39">
-        <f>D9/-D8</f>
-        <v/>
-      </c>
-      <c r="E10" s="39">
-        <f>E9/-E8</f>
-        <v/>
-      </c>
-      <c r="F10" s="39">
-        <f>F9/-F8</f>
-        <v/>
-      </c>
-      <c r="G10" s="39">
-        <f>G9/-G8</f>
-        <v/>
-      </c>
-      <c r="H10" s="39">
-        <f>H9/-H8</f>
-        <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>Execution rate (revenue/opening OB)</t>
-        </is>
-      </c>
-      <c r="B11" s="40">
+          <t xml:space="preserve">  Roll check (open+inflow-rev+adj-close)</t>
+        </is>
+      </c>
+      <c r="B11" s="33">
+        <f>B6+B7+B8+B9-B10</f>
+        <v/>
+      </c>
+      <c r="C11" s="33">
+        <f>C6+C7+C8+C9-C10</f>
+        <v/>
+      </c>
+      <c r="D11" s="33">
+        <f>D6+D7+D8+D9-D10</f>
+        <v/>
+      </c>
+      <c r="E11" s="33">
+        <f>E6+E7+E8+E9-E10</f>
+        <v/>
+      </c>
+      <c r="F11" s="33">
+        <f>F6+F7+F8+F9-F10</f>
+        <v/>
+      </c>
+      <c r="G11" s="33">
+        <f>G6+G7+G8+G9-G10</f>
+        <v/>
+      </c>
+      <c r="H11" s="33">
+        <f>H6+H7+H8+H9-H10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Book-to-bill (closing OB / revenue, x)</t>
+        </is>
+      </c>
+      <c r="B12" s="39">
+        <f>B10/-B8</f>
+        <v/>
+      </c>
+      <c r="C12" s="39">
+        <f>C10/-C8</f>
+        <v/>
+      </c>
+      <c r="D12" s="39">
+        <f>D10/-D8</f>
+        <v/>
+      </c>
+      <c r="E12" s="39">
+        <f>E10/-E8</f>
+        <v/>
+      </c>
+      <c r="F12" s="39">
+        <f>F10/-F8</f>
+        <v/>
+      </c>
+      <c r="G12" s="39">
+        <f>G10/-G8</f>
+        <v/>
+      </c>
+      <c r="H12" s="39">
+        <f>H10/-H8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Execution rate (revenue / opening OB)</t>
+        </is>
+      </c>
+      <c r="B13" s="40">
         <f>-B8/B6</f>
         <v/>
       </c>
-      <c r="C11" s="40">
+      <c r="C13" s="40">
         <f>-C8/C6</f>
         <v/>
       </c>
-      <c r="D11" s="40">
+      <c r="D13" s="40">
         <f>-D8/D6</f>
         <v/>
       </c>
-      <c r="E11" s="40">
+      <c r="E13" s="40">
         <f>-E8/E6</f>
         <v/>
       </c>
-      <c r="F11" s="40">
+      <c r="F13" s="40">
         <f>-F8/F6</f>
         <v/>
       </c>
-      <c r="G11" s="40">
+      <c r="G13" s="40">
         <f>-G8/G6</f>
         <v/>
       </c>
-      <c r="H11" s="40">
+      <c r="H13" s="40">
         <f>-H8/H6</f>
         <v/>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="11" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="11" t="inlineStr">
         <is>
           <t>Segment revenue mix (INR Crore, est.)</t>
         </is>
       </c>
-      <c r="B13" s="1" t="n"/>
-      <c r="C13" s="1" t="n"/>
-      <c r="D13" s="1" t="n"/>
-      <c r="E13" s="1" t="n"/>
-      <c r="F13" s="1" t="n"/>
-      <c r="G13" s="1" t="n"/>
-      <c r="H13" s="1" t="n"/>
-      <c r="I13" s="1" t="n"/>
-      <c r="J13" s="1" t="n"/>
-      <c r="K13" s="1" t="n"/>
-      <c r="L13" s="1" t="n"/>
-      <c r="M13" s="1" t="n"/>
-      <c r="N13" s="1" t="n"/>
-      <c r="O13" s="1" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>Power segment</t>
-        </is>
-      </c>
-      <c r="B14" s="30" t="n">
-        <v>16800</v>
-      </c>
-      <c r="C14" s="30" t="n">
-        <v>13500</v>
-      </c>
-      <c r="D14" s="30" t="n">
-        <v>16500</v>
-      </c>
-      <c r="E14" s="30" t="n">
-        <v>18100</v>
-      </c>
-      <c r="F14" s="30" t="n">
-        <v>18600</v>
-      </c>
-      <c r="G14" s="30" t="n">
-        <v>20937</v>
-      </c>
-      <c r="H14" s="30" t="n">
-        <v>25407</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>Industry segment</t>
-        </is>
-      </c>
-      <c r="B15" s="30" t="n">
-        <v>3900</v>
-      </c>
-      <c r="C15" s="30" t="n">
-        <v>3200</v>
-      </c>
-      <c r="D15" s="30" t="n">
-        <v>4000</v>
-      </c>
-      <c r="E15" s="30" t="n">
-        <v>4600</v>
-      </c>
-      <c r="F15" s="30" t="n">
-        <v>4700</v>
-      </c>
-      <c r="G15" s="30" t="n">
-        <v>6400</v>
-      </c>
-      <c r="H15" s="30" t="n">
-        <v>7400</v>
-      </c>
+      <c r="B15" s="1" t="n"/>
+      <c r="C15" s="1" t="n"/>
+      <c r="D15" s="1" t="n"/>
+      <c r="E15" s="1" t="n"/>
+      <c r="F15" s="1" t="n"/>
+      <c r="G15" s="1" t="n"/>
+      <c r="H15" s="1" t="n"/>
+      <c r="I15" s="1" t="n"/>
+      <c r="J15" s="1" t="n"/>
+      <c r="K15" s="1" t="n"/>
+      <c r="L15" s="1" t="n"/>
+      <c r="M15" s="1" t="n"/>
+      <c r="N15" s="1" t="n"/>
+      <c r="O15" s="1" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Others / exports / renewables</t>
+          <t>Power segment</t>
         </is>
       </c>
       <c r="B16" s="30" t="n">
-        <v>763</v>
+        <v>16800</v>
       </c>
       <c r="C16" s="30" t="n">
-        <v>609</v>
+        <v>13500</v>
       </c>
       <c r="D16" s="30" t="n">
-        <v>711</v>
+        <v>16500</v>
       </c>
       <c r="E16" s="30" t="n">
-        <v>665</v>
+        <v>18100</v>
       </c>
       <c r="F16" s="30" t="n">
-        <v>593</v>
+        <v>18600</v>
       </c>
       <c r="G16" s="30" t="n">
-        <v>1002</v>
+        <v>20937</v>
       </c>
       <c r="H16" s="30" t="n">
-        <v>975</v>
+        <v>25407</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>Total (check vs revenue)</t>
-        </is>
-      </c>
-      <c r="B17" s="33">
-        <f>SUM(B14:B16)</f>
-        <v/>
-      </c>
-      <c r="C17" s="33">
-        <f>SUM(C14:C16)</f>
-        <v/>
-      </c>
-      <c r="D17" s="33">
-        <f>SUM(D14:D16)</f>
-        <v/>
-      </c>
-      <c r="E17" s="33">
-        <f>SUM(E14:E16)</f>
-        <v/>
-      </c>
-      <c r="F17" s="33">
-        <f>SUM(F14:F16)</f>
-        <v/>
-      </c>
-      <c r="G17" s="33">
-        <f>SUM(G14:G16)</f>
-        <v/>
-      </c>
-      <c r="H17" s="33">
-        <f>SUM(H14:H16)</f>
-        <v/>
+          <t>Industry segment</t>
+        </is>
+      </c>
+      <c r="B17" s="30" t="n">
+        <v>3900</v>
+      </c>
+      <c r="C17" s="30" t="n">
+        <v>3200</v>
+      </c>
+      <c r="D17" s="30" t="n">
+        <v>4000</v>
+      </c>
+      <c r="E17" s="30" t="n">
+        <v>4600</v>
+      </c>
+      <c r="F17" s="30" t="n">
+        <v>4700</v>
+      </c>
+      <c r="G17" s="30" t="n">
+        <v>6400</v>
+      </c>
+      <c r="H17" s="30" t="n">
+        <v>7400</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
+          <t>Others / exports / renewables</t>
+        </is>
+      </c>
+      <c r="B18" s="30" t="n">
+        <v>763</v>
+      </c>
+      <c r="C18" s="30" t="n">
+        <v>609</v>
+      </c>
+      <c r="D18" s="30" t="n">
+        <v>711</v>
+      </c>
+      <c r="E18" s="30" t="n">
+        <v>665</v>
+      </c>
+      <c r="F18" s="30" t="n">
+        <v>593</v>
+      </c>
+      <c r="G18" s="30" t="n">
+        <v>1002</v>
+      </c>
+      <c r="H18" s="30" t="n">
+        <v>975</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Total (check vs revenue)</t>
+        </is>
+      </c>
+      <c r="B19" s="33">
+        <f>SUM(B16:B18)</f>
+        <v/>
+      </c>
+      <c r="C19" s="33">
+        <f>SUM(C16:C18)</f>
+        <v/>
+      </c>
+      <c r="D19" s="33">
+        <f>SUM(D16:D18)</f>
+        <v/>
+      </c>
+      <c r="E19" s="33">
+        <f>SUM(E16:E18)</f>
+        <v/>
+      </c>
+      <c r="F19" s="33">
+        <f>SUM(F16:F18)</f>
+        <v/>
+      </c>
+      <c r="G19" s="33">
+        <f>SUM(G16:G18)</f>
+        <v/>
+      </c>
+      <c r="H19" s="33">
+        <f>SUM(H16:H18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
           <t>Power as % of revenue</t>
         </is>
       </c>
-      <c r="B18" s="40">
-        <f>B14/'Historical Financial Statements'!B5</f>
-        <v/>
-      </c>
-      <c r="C18" s="40">
-        <f>C14/'Historical Financial Statements'!C5</f>
-        <v/>
-      </c>
-      <c r="D18" s="40">
-        <f>D14/'Historical Financial Statements'!D5</f>
-        <v/>
-      </c>
-      <c r="E18" s="40">
-        <f>E14/'Historical Financial Statements'!E5</f>
-        <v/>
-      </c>
-      <c r="F18" s="40">
-        <f>F14/'Historical Financial Statements'!F5</f>
-        <v/>
-      </c>
-      <c r="G18" s="40">
-        <f>G14/'Historical Financial Statements'!G5</f>
-        <v/>
-      </c>
-      <c r="H18" s="40">
-        <f>H14/'Historical Financial Statements'!H5</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="11" t="inlineStr">
+      <c r="B20" s="40">
+        <f>B16/'Historical Financial Statements'!B5</f>
+        <v/>
+      </c>
+      <c r="C20" s="40">
+        <f>C16/'Historical Financial Statements'!C5</f>
+        <v/>
+      </c>
+      <c r="D20" s="40">
+        <f>D16/'Historical Financial Statements'!D5</f>
+        <v/>
+      </c>
+      <c r="E20" s="40">
+        <f>E16/'Historical Financial Statements'!E5</f>
+        <v/>
+      </c>
+      <c r="F20" s="40">
+        <f>F16/'Historical Financial Statements'!F5</f>
+        <v/>
+      </c>
+      <c r="G20" s="40">
+        <f>G16/'Historical Financial Statements'!G5</f>
+        <v/>
+      </c>
+      <c r="H20" s="40">
+        <f>H16/'Historical Financial Statements'!H5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="11" t="inlineStr">
         <is>
           <t>Other KPIs</t>
         </is>
       </c>
-      <c r="B20" s="1" t="n"/>
-      <c r="C20" s="1" t="n"/>
-      <c r="D20" s="1" t="n"/>
-      <c r="E20" s="1" t="n"/>
-      <c r="F20" s="1" t="n"/>
-      <c r="G20" s="1" t="n"/>
-      <c r="H20" s="1" t="n"/>
-      <c r="I20" s="1" t="n"/>
-      <c r="J20" s="1" t="n"/>
-      <c r="K20" s="1" t="n"/>
-      <c r="L20" s="1" t="n"/>
-      <c r="M20" s="1" t="n"/>
-      <c r="N20" s="1" t="n"/>
-      <c r="O20" s="1" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="5" t="inlineStr">
-        <is>
-          <t>Approx. workforce (number)</t>
-        </is>
-      </c>
-      <c r="B21" s="41" t="n">
-        <v>33500</v>
-      </c>
-      <c r="C21" s="41" t="n">
-        <v>31500</v>
-      </c>
-      <c r="D21" s="41" t="n">
-        <v>29800</v>
-      </c>
-      <c r="E21" s="41" t="n">
-        <v>28500</v>
-      </c>
-      <c r="F21" s="41" t="n">
-        <v>27000</v>
-      </c>
-      <c r="G21" s="41" t="n">
-        <v>26000</v>
-      </c>
-      <c r="H21" s="41" t="n">
-        <v>25500</v>
-      </c>
-      <c r="P21" s="13" t="inlineStr">
-        <is>
-          <t>approx.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="5" t="inlineStr">
-        <is>
-          <t>R&amp;D expenditure</t>
-        </is>
-      </c>
-      <c r="B22" s="30" t="n">
-        <v>1180</v>
-      </c>
-      <c r="C22" s="30" t="n">
-        <v>1090</v>
-      </c>
-      <c r="D22" s="30" t="n">
-        <v>1050</v>
-      </c>
-      <c r="E22" s="30" t="n">
-        <v>1100</v>
-      </c>
-      <c r="F22" s="30" t="n">
-        <v>1150</v>
-      </c>
-      <c r="G22" s="30" t="n">
-        <v>1300</v>
-      </c>
-      <c r="H22" s="30" t="n">
-        <v>1500</v>
-      </c>
-      <c r="P22" s="13" t="inlineStr">
-        <is>
-          <t>approx.</t>
-        </is>
-      </c>
+      <c r="B22" s="1" t="n"/>
+      <c r="C22" s="1" t="n"/>
+      <c r="D22" s="1" t="n"/>
+      <c r="E22" s="1" t="n"/>
+      <c r="F22" s="1" t="n"/>
+      <c r="G22" s="1" t="n"/>
+      <c r="H22" s="1" t="n"/>
+      <c r="I22" s="1" t="n"/>
+      <c r="J22" s="1" t="n"/>
+      <c r="K22" s="1" t="n"/>
+      <c r="L22" s="1" t="n"/>
+      <c r="M22" s="1" t="n"/>
+      <c r="N22" s="1" t="n"/>
+      <c r="O22" s="1" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>R&amp;D as % of revenue</t>
-        </is>
-      </c>
-      <c r="B23" s="40">
-        <f>B22/'Historical Financial Statements'!B5</f>
-        <v/>
-      </c>
-      <c r="C23" s="40">
-        <f>C22/'Historical Financial Statements'!C5</f>
-        <v/>
-      </c>
-      <c r="D23" s="40">
-        <f>D22/'Historical Financial Statements'!D5</f>
-        <v/>
-      </c>
-      <c r="E23" s="40">
-        <f>E22/'Historical Financial Statements'!E5</f>
-        <v/>
-      </c>
-      <c r="F23" s="40">
-        <f>F22/'Historical Financial Statements'!F5</f>
-        <v/>
-      </c>
-      <c r="G23" s="40">
-        <f>G22/'Historical Financial Statements'!G5</f>
-        <v/>
-      </c>
-      <c r="H23" s="40">
-        <f>H22/'Historical Financial Statements'!H5</f>
-        <v/>
+          <t>Approx. workforce (number)</t>
+        </is>
+      </c>
+      <c r="B23" s="41" t="n">
+        <v>33500</v>
+      </c>
+      <c r="C23" s="41" t="n">
+        <v>31500</v>
+      </c>
+      <c r="D23" s="41" t="n">
+        <v>29800</v>
+      </c>
+      <c r="E23" s="41" t="n">
+        <v>28500</v>
+      </c>
+      <c r="F23" s="41" t="n">
+        <v>27000</v>
+      </c>
+      <c r="G23" s="41" t="n">
+        <v>26000</v>
+      </c>
+      <c r="H23" s="41" t="n">
+        <v>25500</v>
+      </c>
+      <c r="P23" s="13" t="inlineStr">
+        <is>
+          <t>approx.</t>
+        </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
+          <t>R&amp;D expenditure</t>
+        </is>
+      </c>
+      <c r="B24" s="30" t="n">
+        <v>1180</v>
+      </c>
+      <c r="C24" s="30" t="n">
+        <v>1090</v>
+      </c>
+      <c r="D24" s="30" t="n">
+        <v>1050</v>
+      </c>
+      <c r="E24" s="30" t="n">
+        <v>1100</v>
+      </c>
+      <c r="F24" s="30" t="n">
+        <v>1150</v>
+      </c>
+      <c r="G24" s="30" t="n">
+        <v>1300</v>
+      </c>
+      <c r="H24" s="30" t="n">
+        <v>1500</v>
+      </c>
+      <c r="P24" s="13" t="inlineStr">
+        <is>
+          <t>approx.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>R&amp;D as % of revenue</t>
+        </is>
+      </c>
+      <c r="B25" s="40">
+        <f>B24/'Historical Financial Statements'!B5</f>
+        <v/>
+      </c>
+      <c r="C25" s="40">
+        <f>C24/'Historical Financial Statements'!C5</f>
+        <v/>
+      </c>
+      <c r="D25" s="40">
+        <f>D24/'Historical Financial Statements'!D5</f>
+        <v/>
+      </c>
+      <c r="E25" s="40">
+        <f>E24/'Historical Financial Statements'!E5</f>
+        <v/>
+      </c>
+      <c r="F25" s="40">
+        <f>F24/'Historical Financial Statements'!F5</f>
+        <v/>
+      </c>
+      <c r="G25" s="40">
+        <f>G24/'Historical Financial Statements'!G5</f>
+        <v/>
+      </c>
+      <c r="H25" s="40">
+        <f>H24/'Historical Financial Statements'!H5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
           <t>Capacity utilisation (mfg.)</t>
         </is>
       </c>
-      <c r="B24" s="42" t="n">
+      <c r="B26" s="42" t="n">
         <v>0.55</v>
       </c>
-      <c r="C24" s="42" t="n">
+      <c r="C26" s="42" t="n">
         <v>0.42</v>
       </c>
-      <c r="D24" s="42" t="n">
+      <c r="D26" s="42" t="n">
         <v>0.5</v>
       </c>
-      <c r="E24" s="42" t="n">
+      <c r="E26" s="42" t="n">
         <v>0.55</v>
       </c>
-      <c r="F24" s="42" t="n">
+      <c r="F26" s="42" t="n">
         <v>0.58</v>
       </c>
-      <c r="G24" s="42" t="n">
+      <c r="G26" s="42" t="n">
         <v>0.65</v>
       </c>
-      <c r="H24" s="42" t="n">
+      <c r="H26" s="42" t="n">
         <v>0.72</v>
       </c>
-      <c r="P24" s="13" t="inlineStr">
+      <c r="P26" s="13" t="inlineStr">
         <is>
           <t>approx.</t>
         </is>
@@ -16409,7 +16479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O23"/>
+  <dimension ref="A1:O24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -16453,7 +16523,7 @@
     <row r="2">
       <c r="A2" s="13" t="inlineStr">
         <is>
-          <t>Order book is rolled on a STANDALONE basis (as BHEL discloses it): Standalone revenue = Execution rate x Opening order book; Closing OB = Opening + Inflow - Standalone revenue. Consolidated revenue (used in the P&amp;L) is then bridged from standalone via a consolidation uplift.</t>
+          <t>Order book rolled on STANDALONE basis: Closing OB = Opening + Inflow - Standalone revenue + Adjustments (cancellations/FX/scope/taxes). Consolidated revenue (P&amp;L) is bridged from standalone via a consolidation uplift.</t>
         </is>
       </c>
     </row>
@@ -16590,31 +16660,31 @@
         <v/>
       </c>
       <c r="I6" s="33">
-        <f>'Operational Drivers'!H9</f>
+        <f>'Operational Drivers'!H10</f>
         <v/>
       </c>
       <c r="J6" s="33">
-        <f>I9</f>
+        <f>I10</f>
         <v/>
       </c>
       <c r="K6" s="33">
-        <f>J9</f>
+        <f>J10</f>
         <v/>
       </c>
       <c r="L6" s="33">
-        <f>K9</f>
+        <f>K10</f>
         <v/>
       </c>
       <c r="M6" s="33">
-        <f>L9</f>
+        <f>L10</f>
         <v/>
       </c>
       <c r="N6" s="33">
-        <f>M9</f>
+        <f>M10</f>
         <v/>
       </c>
       <c r="O6" s="33">
-        <f>N9</f>
+        <f>N10</f>
         <v/>
       </c>
     </row>
@@ -16745,733 +16815,789 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>+/- Adjustments (cancellations/FX/scope/taxes)</t>
+        </is>
+      </c>
+      <c r="B9" s="43">
+        <f>'Operational Drivers'!B9</f>
+        <v/>
+      </c>
+      <c r="C9" s="43">
+        <f>'Operational Drivers'!C9</f>
+        <v/>
+      </c>
+      <c r="D9" s="43">
+        <f>'Operational Drivers'!D9</f>
+        <v/>
+      </c>
+      <c r="E9" s="43">
+        <f>'Operational Drivers'!E9</f>
+        <v/>
+      </c>
+      <c r="F9" s="43">
+        <f>'Operational Drivers'!F9</f>
+        <v/>
+      </c>
+      <c r="G9" s="43">
+        <f>'Operational Drivers'!G9</f>
+        <v/>
+      </c>
+      <c r="H9" s="43">
+        <f>'Operational Drivers'!H9</f>
+        <v/>
+      </c>
+      <c r="I9" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" s="33" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Closing order book (standalone)</t>
         </is>
       </c>
-      <c r="B9" s="44">
-        <f>'Operational Drivers'!B9</f>
-        <v/>
-      </c>
-      <c r="C9" s="44">
-        <f>'Operational Drivers'!C9</f>
-        <v/>
-      </c>
-      <c r="D9" s="44">
-        <f>'Operational Drivers'!D9</f>
-        <v/>
-      </c>
-      <c r="E9" s="44">
-        <f>'Operational Drivers'!E9</f>
-        <v/>
-      </c>
-      <c r="F9" s="44">
-        <f>'Operational Drivers'!F9</f>
-        <v/>
-      </c>
-      <c r="G9" s="44">
-        <f>'Operational Drivers'!G9</f>
-        <v/>
-      </c>
-      <c r="H9" s="44">
-        <f>'Operational Drivers'!H9</f>
-        <v/>
-      </c>
-      <c r="I9" s="45">
-        <f>I6+I7+I8</f>
-        <v/>
-      </c>
-      <c r="J9" s="45">
-        <f>J6+J7+J8</f>
-        <v/>
-      </c>
-      <c r="K9" s="45">
-        <f>K6+K7+K8</f>
-        <v/>
-      </c>
-      <c r="L9" s="45">
-        <f>L6+L7+L8</f>
-        <v/>
-      </c>
-      <c r="M9" s="45">
-        <f>M6+M7+M8</f>
-        <v/>
-      </c>
-      <c r="N9" s="45">
-        <f>N6+N7+N8</f>
-        <v/>
-      </c>
-      <c r="O9" s="45">
-        <f>O6+O7+O8</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="11" t="inlineStr">
+      <c r="B10" s="44">
+        <f>B6+B7+B8+B9</f>
+        <v/>
+      </c>
+      <c r="C10" s="44">
+        <f>C6+C7+C8+C9</f>
+        <v/>
+      </c>
+      <c r="D10" s="44">
+        <f>D6+D7+D8+D9</f>
+        <v/>
+      </c>
+      <c r="E10" s="44">
+        <f>E6+E7+E8+E9</f>
+        <v/>
+      </c>
+      <c r="F10" s="44">
+        <f>F6+F7+F8+F9</f>
+        <v/>
+      </c>
+      <c r="G10" s="44">
+        <f>G6+G7+G8+G9</f>
+        <v/>
+      </c>
+      <c r="H10" s="44">
+        <f>H6+H7+H8+H9</f>
+        <v/>
+      </c>
+      <c r="I10" s="44">
+        <f>I6+I7+I8+I9</f>
+        <v/>
+      </c>
+      <c r="J10" s="44">
+        <f>J6+J7+J8+J9</f>
+        <v/>
+      </c>
+      <c r="K10" s="44">
+        <f>K6+K7+K8+K9</f>
+        <v/>
+      </c>
+      <c r="L10" s="44">
+        <f>L6+L7+L8+L9</f>
+        <v/>
+      </c>
+      <c r="M10" s="44">
+        <f>M6+M7+M8+M9</f>
+        <v/>
+      </c>
+      <c r="N10" s="44">
+        <f>N6+N7+N8+N9</f>
+        <v/>
+      </c>
+      <c r="O10" s="44">
+        <f>O6+O7+O8+O9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="inlineStr">
         <is>
           <t>B.  Standalone -&gt; consolidated revenue bridge</t>
         </is>
       </c>
-      <c r="B11" s="1" t="n"/>
-      <c r="C11" s="1" t="n"/>
-      <c r="D11" s="1" t="n"/>
-      <c r="E11" s="1" t="n"/>
-      <c r="F11" s="1" t="n"/>
-      <c r="G11" s="1" t="n"/>
-      <c r="H11" s="1" t="n"/>
-      <c r="I11" s="1" t="n"/>
-      <c r="J11" s="1" t="n"/>
-      <c r="K11" s="1" t="n"/>
-      <c r="L11" s="1" t="n"/>
-      <c r="M11" s="1" t="n"/>
-      <c r="N11" s="1" t="n"/>
-      <c r="O11" s="1" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="B12" s="1" t="n"/>
+      <c r="C12" s="1" t="n"/>
+      <c r="D12" s="1" t="n"/>
+      <c r="E12" s="1" t="n"/>
+      <c r="F12" s="1" t="n"/>
+      <c r="G12" s="1" t="n"/>
+      <c r="H12" s="1" t="n"/>
+      <c r="I12" s="1" t="n"/>
+      <c r="J12" s="1" t="n"/>
+      <c r="K12" s="1" t="n"/>
+      <c r="L12" s="1" t="n"/>
+      <c r="M12" s="1" t="n"/>
+      <c r="N12" s="1" t="n"/>
+      <c r="O12" s="1" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>Standalone revenue from operations</t>
         </is>
       </c>
-      <c r="B12" s="43">
+      <c r="B13" s="43">
         <f>-B8</f>
         <v/>
       </c>
-      <c r="C12" s="43">
+      <c r="C13" s="43">
         <f>-C8</f>
         <v/>
       </c>
-      <c r="D12" s="43">
+      <c r="D13" s="43">
         <f>-D8</f>
         <v/>
       </c>
-      <c r="E12" s="43">
+      <c r="E13" s="43">
         <f>-E8</f>
         <v/>
       </c>
-      <c r="F12" s="43">
+      <c r="F13" s="43">
         <f>-F8</f>
         <v/>
       </c>
-      <c r="G12" s="43">
+      <c r="G13" s="43">
         <f>-G8</f>
         <v/>
       </c>
-      <c r="H12" s="43">
+      <c r="H13" s="43">
         <f>-H8</f>
         <v/>
       </c>
-      <c r="I12" s="33">
+      <c r="I13" s="33">
         <f>-I8</f>
         <v/>
       </c>
-      <c r="J12" s="33">
+      <c r="J13" s="33">
         <f>-J8</f>
         <v/>
       </c>
-      <c r="K12" s="33">
+      <c r="K13" s="33">
         <f>-K8</f>
         <v/>
       </c>
-      <c r="L12" s="33">
+      <c r="L13" s="33">
         <f>-L8</f>
         <v/>
       </c>
-      <c r="M12" s="33">
+      <c r="M13" s="33">
         <f>-M8</f>
         <v/>
       </c>
-      <c r="N12" s="33">
+      <c r="N13" s="33">
         <f>-N8</f>
         <v/>
       </c>
-      <c r="O12" s="33">
+      <c r="O13" s="33">
         <f>-O8</f>
         <v/>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>Consolidation uplift % (consol/standalone - 1)</t>
         </is>
       </c>
-      <c r="B13" s="36">
-        <f>'Historical Financial Statements'!B5/B12-1</f>
-        <v/>
-      </c>
-      <c r="C13" s="36">
-        <f>'Historical Financial Statements'!C5/C12-1</f>
-        <v/>
-      </c>
-      <c r="D13" s="36">
-        <f>'Historical Financial Statements'!D5/D12-1</f>
-        <v/>
-      </c>
-      <c r="E13" s="36">
-        <f>'Historical Financial Statements'!E5/E12-1</f>
-        <v/>
-      </c>
-      <c r="F13" s="36">
-        <f>'Historical Financial Statements'!F5/F12-1</f>
-        <v/>
-      </c>
-      <c r="G13" s="36">
-        <f>'Historical Financial Statements'!G5/G12-1</f>
-        <v/>
-      </c>
-      <c r="H13" s="36">
-        <f>'Historical Financial Statements'!H5/H12-1</f>
-        <v/>
-      </c>
-      <c r="I13" s="40">
+      <c r="B14" s="36">
+        <f>'Historical Financial Statements'!B5/B13-1</f>
+        <v/>
+      </c>
+      <c r="C14" s="36">
+        <f>'Historical Financial Statements'!C5/C13-1</f>
+        <v/>
+      </c>
+      <c r="D14" s="36">
+        <f>'Historical Financial Statements'!D5/D13-1</f>
+        <v/>
+      </c>
+      <c r="E14" s="36">
+        <f>'Historical Financial Statements'!E5/E13-1</f>
+        <v/>
+      </c>
+      <c r="F14" s="36">
+        <f>'Historical Financial Statements'!F5/F13-1</f>
+        <v/>
+      </c>
+      <c r="G14" s="36">
+        <f>'Historical Financial Statements'!G5/G13-1</f>
+        <v/>
+      </c>
+      <c r="H14" s="36">
+        <f>'Historical Financial Statements'!H5/H13-1</f>
+        <v/>
+      </c>
+      <c r="I14" s="40">
         <f>'Assumptions'!I22</f>
         <v/>
       </c>
-      <c r="J13" s="40">
+      <c r="J14" s="40">
         <f>'Assumptions'!J22</f>
         <v/>
       </c>
-      <c r="K13" s="40">
+      <c r="K14" s="40">
         <f>'Assumptions'!K22</f>
         <v/>
       </c>
-      <c r="L13" s="40">
+      <c r="L14" s="40">
         <f>'Assumptions'!L22</f>
         <v/>
       </c>
-      <c r="M13" s="40">
+      <c r="M14" s="40">
         <f>'Assumptions'!M22</f>
         <v/>
       </c>
-      <c r="N13" s="40">
+      <c r="N14" s="40">
         <f>'Assumptions'!N22</f>
         <v/>
       </c>
-      <c r="O13" s="40">
+      <c r="O14" s="40">
         <f>'Assumptions'!O22</f>
         <v/>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>Consolidated revenue from operations  -&gt;  P&amp;L</t>
         </is>
       </c>
-      <c r="B14" s="32">
-        <f>B12*(1+B13)</f>
-        <v/>
-      </c>
-      <c r="C14" s="32">
-        <f>C12*(1+C13)</f>
-        <v/>
-      </c>
-      <c r="D14" s="32">
-        <f>D12*(1+D13)</f>
-        <v/>
-      </c>
-      <c r="E14" s="32">
-        <f>E12*(1+E13)</f>
-        <v/>
-      </c>
-      <c r="F14" s="32">
-        <f>F12*(1+F13)</f>
-        <v/>
-      </c>
-      <c r="G14" s="32">
-        <f>G12*(1+G13)</f>
-        <v/>
-      </c>
-      <c r="H14" s="32">
-        <f>H12*(1+H13)</f>
-        <v/>
-      </c>
-      <c r="I14" s="32">
-        <f>I12*(1+I13)</f>
-        <v/>
-      </c>
-      <c r="J14" s="32">
-        <f>J12*(1+J13)</f>
-        <v/>
-      </c>
-      <c r="K14" s="32">
-        <f>K12*(1+K13)</f>
-        <v/>
-      </c>
-      <c r="L14" s="32">
-        <f>L12*(1+L13)</f>
-        <v/>
-      </c>
-      <c r="M14" s="32">
-        <f>M12*(1+M13)</f>
-        <v/>
-      </c>
-      <c r="N14" s="32">
-        <f>N12*(1+N13)</f>
-        <v/>
-      </c>
-      <c r="O14" s="32">
-        <f>O12*(1+O13)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>Revenue growth % (consolidated)</t>
-        </is>
-      </c>
-      <c r="C15" s="40">
-        <f>C14/B14-1</f>
-        <v/>
-      </c>
-      <c r="D15" s="40">
-        <f>D14/C14-1</f>
-        <v/>
-      </c>
-      <c r="E15" s="40">
-        <f>E14/D14-1</f>
-        <v/>
-      </c>
-      <c r="F15" s="40">
-        <f>F14/E14-1</f>
-        <v/>
-      </c>
-      <c r="G15" s="40">
-        <f>G14/F14-1</f>
-        <v/>
-      </c>
-      <c r="H15" s="40">
-        <f>H14/G14-1</f>
-        <v/>
-      </c>
-      <c r="I15" s="40">
-        <f>I14/H14-1</f>
-        <v/>
-      </c>
-      <c r="J15" s="40">
-        <f>J14/I14-1</f>
-        <v/>
-      </c>
-      <c r="K15" s="40">
-        <f>K14/J14-1</f>
-        <v/>
-      </c>
-      <c r="L15" s="40">
-        <f>L14/K14-1</f>
-        <v/>
-      </c>
-      <c r="M15" s="40">
-        <f>M14/L14-1</f>
-        <v/>
-      </c>
-      <c r="N15" s="40">
-        <f>N14/M14-1</f>
-        <v/>
-      </c>
-      <c r="O15" s="40">
-        <f>O14/N14-1</f>
+      <c r="B15" s="32">
+        <f>B13*(1+B14)</f>
+        <v/>
+      </c>
+      <c r="C15" s="32">
+        <f>C13*(1+C14)</f>
+        <v/>
+      </c>
+      <c r="D15" s="32">
+        <f>D13*(1+D14)</f>
+        <v/>
+      </c>
+      <c r="E15" s="32">
+        <f>E13*(1+E14)</f>
+        <v/>
+      </c>
+      <c r="F15" s="32">
+        <f>F13*(1+F14)</f>
+        <v/>
+      </c>
+      <c r="G15" s="32">
+        <f>G13*(1+G14)</f>
+        <v/>
+      </c>
+      <c r="H15" s="32">
+        <f>H13*(1+H14)</f>
+        <v/>
+      </c>
+      <c r="I15" s="32">
+        <f>I13*(1+I14)</f>
+        <v/>
+      </c>
+      <c r="J15" s="32">
+        <f>J13*(1+J14)</f>
+        <v/>
+      </c>
+      <c r="K15" s="32">
+        <f>K13*(1+K14)</f>
+        <v/>
+      </c>
+      <c r="L15" s="32">
+        <f>L13*(1+L14)</f>
+        <v/>
+      </c>
+      <c r="M15" s="32">
+        <f>M13*(1+M14)</f>
+        <v/>
+      </c>
+      <c r="N15" s="32">
+        <f>N13*(1+N14)</f>
+        <v/>
+      </c>
+      <c r="O15" s="32">
+        <f>O13*(1+O14)</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Execution rate % (standalone rev / opening OB)</t>
-        </is>
-      </c>
-      <c r="B16" s="40">
-        <f>B12/B6</f>
-        <v/>
+          <t>Revenue growth % (consolidated)</t>
+        </is>
       </c>
       <c r="C16" s="40">
-        <f>C12/C6</f>
+        <f>C15/B15-1</f>
         <v/>
       </c>
       <c r="D16" s="40">
-        <f>D12/D6</f>
+        <f>D15/C15-1</f>
         <v/>
       </c>
       <c r="E16" s="40">
-        <f>E12/E6</f>
+        <f>E15/D15-1</f>
         <v/>
       </c>
       <c r="F16" s="40">
-        <f>F12/F6</f>
+        <f>F15/E15-1</f>
         <v/>
       </c>
       <c r="G16" s="40">
-        <f>G12/G6</f>
+        <f>G15/F15-1</f>
         <v/>
       </c>
       <c r="H16" s="40">
-        <f>H12/H6</f>
+        <f>H15/G15-1</f>
         <v/>
       </c>
       <c r="I16" s="40">
-        <f>I12/I6</f>
+        <f>I15/H15-1</f>
         <v/>
       </c>
       <c r="J16" s="40">
-        <f>J12/J6</f>
+        <f>J15/I15-1</f>
         <v/>
       </c>
       <c r="K16" s="40">
-        <f>K12/K6</f>
+        <f>K15/J15-1</f>
         <v/>
       </c>
       <c r="L16" s="40">
-        <f>L12/L6</f>
+        <f>L15/K15-1</f>
         <v/>
       </c>
       <c r="M16" s="40">
-        <f>M12/M6</f>
+        <f>M15/L15-1</f>
         <v/>
       </c>
       <c r="N16" s="40">
-        <f>N12/N6</f>
+        <f>N15/M15-1</f>
         <v/>
       </c>
       <c r="O16" s="40">
-        <f>O12/O6</f>
+        <f>O15/N15-1</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
+          <t>Execution rate % (standalone rev / opening OB)</t>
+        </is>
+      </c>
+      <c r="B17" s="40">
+        <f>B13/B6</f>
+        <v/>
+      </c>
+      <c r="C17" s="40">
+        <f>C13/C6</f>
+        <v/>
+      </c>
+      <c r="D17" s="40">
+        <f>D13/D6</f>
+        <v/>
+      </c>
+      <c r="E17" s="40">
+        <f>E13/E6</f>
+        <v/>
+      </c>
+      <c r="F17" s="40">
+        <f>F13/F6</f>
+        <v/>
+      </c>
+      <c r="G17" s="40">
+        <f>G13/G6</f>
+        <v/>
+      </c>
+      <c r="H17" s="40">
+        <f>H13/H6</f>
+        <v/>
+      </c>
+      <c r="I17" s="40">
+        <f>I13/I6</f>
+        <v/>
+      </c>
+      <c r="J17" s="40">
+        <f>J13/J6</f>
+        <v/>
+      </c>
+      <c r="K17" s="40">
+        <f>K13/K6</f>
+        <v/>
+      </c>
+      <c r="L17" s="40">
+        <f>L13/L6</f>
+        <v/>
+      </c>
+      <c r="M17" s="40">
+        <f>M13/M6</f>
+        <v/>
+      </c>
+      <c r="N17" s="40">
+        <f>N13/N6</f>
+        <v/>
+      </c>
+      <c r="O17" s="40">
+        <f>O13/O6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
           <t>Book-to-bill (closing OB / standalone rev, x)</t>
         </is>
       </c>
-      <c r="B17" s="39">
-        <f>B9/B12</f>
-        <v/>
-      </c>
-      <c r="C17" s="39">
-        <f>C9/C12</f>
-        <v/>
-      </c>
-      <c r="D17" s="39">
-        <f>D9/D12</f>
-        <v/>
-      </c>
-      <c r="E17" s="39">
-        <f>E9/E12</f>
-        <v/>
-      </c>
-      <c r="F17" s="39">
-        <f>F9/F12</f>
-        <v/>
-      </c>
-      <c r="G17" s="39">
-        <f>G9/G12</f>
-        <v/>
-      </c>
-      <c r="H17" s="39">
-        <f>H9/H12</f>
-        <v/>
-      </c>
-      <c r="I17" s="39">
-        <f>I9/I12</f>
-        <v/>
-      </c>
-      <c r="J17" s="39">
-        <f>J9/J12</f>
-        <v/>
-      </c>
-      <c r="K17" s="39">
-        <f>K9/K12</f>
-        <v/>
-      </c>
-      <c r="L17" s="39">
-        <f>L9/L12</f>
-        <v/>
-      </c>
-      <c r="M17" s="39">
-        <f>M9/M12</f>
-        <v/>
-      </c>
-      <c r="N17" s="39">
-        <f>N9/N12</f>
-        <v/>
-      </c>
-      <c r="O17" s="39">
-        <f>O9/O12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="11" t="inlineStr">
+      <c r="B18" s="39">
+        <f>B10/B13</f>
+        <v/>
+      </c>
+      <c r="C18" s="39">
+        <f>C10/C13</f>
+        <v/>
+      </c>
+      <c r="D18" s="39">
+        <f>D10/D13</f>
+        <v/>
+      </c>
+      <c r="E18" s="39">
+        <f>E10/E13</f>
+        <v/>
+      </c>
+      <c r="F18" s="39">
+        <f>F10/F13</f>
+        <v/>
+      </c>
+      <c r="G18" s="39">
+        <f>G10/G13</f>
+        <v/>
+      </c>
+      <c r="H18" s="39">
+        <f>H10/H13</f>
+        <v/>
+      </c>
+      <c r="I18" s="39">
+        <f>I10/I13</f>
+        <v/>
+      </c>
+      <c r="J18" s="39">
+        <f>J10/J13</f>
+        <v/>
+      </c>
+      <c r="K18" s="39">
+        <f>K10/K13</f>
+        <v/>
+      </c>
+      <c r="L18" s="39">
+        <f>L10/L13</f>
+        <v/>
+      </c>
+      <c r="M18" s="39">
+        <f>M10/M13</f>
+        <v/>
+      </c>
+      <c r="N18" s="39">
+        <f>N10/N13</f>
+        <v/>
+      </c>
+      <c r="O18" s="39">
+        <f>O10/O13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="11" t="inlineStr">
         <is>
           <t>C.  Segment revenue breakup (consolidated)</t>
         </is>
       </c>
-      <c r="B19" s="1" t="n"/>
-      <c r="C19" s="1" t="n"/>
-      <c r="D19" s="1" t="n"/>
-      <c r="E19" s="1" t="n"/>
-      <c r="F19" s="1" t="n"/>
-      <c r="G19" s="1" t="n"/>
-      <c r="H19" s="1" t="n"/>
-      <c r="I19" s="1" t="n"/>
-      <c r="J19" s="1" t="n"/>
-      <c r="K19" s="1" t="n"/>
-      <c r="L19" s="1" t="n"/>
-      <c r="M19" s="1" t="n"/>
-      <c r="N19" s="1" t="n"/>
-      <c r="O19" s="1" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>Power segment</t>
-        </is>
-      </c>
-      <c r="B20" s="43">
-        <f>'Operational Drivers'!B14</f>
-        <v/>
-      </c>
-      <c r="C20" s="43">
-        <f>'Operational Drivers'!C14</f>
-        <v/>
-      </c>
-      <c r="D20" s="43">
-        <f>'Operational Drivers'!D14</f>
-        <v/>
-      </c>
-      <c r="E20" s="43">
-        <f>'Operational Drivers'!E14</f>
-        <v/>
-      </c>
-      <c r="F20" s="43">
-        <f>'Operational Drivers'!F14</f>
-        <v/>
-      </c>
-      <c r="G20" s="43">
-        <f>'Operational Drivers'!G14</f>
-        <v/>
-      </c>
-      <c r="H20" s="43">
-        <f>'Operational Drivers'!H14</f>
-        <v/>
-      </c>
-      <c r="I20" s="33">
-        <f>I14*'Assumptions'!I33</f>
-        <v/>
-      </c>
-      <c r="J20" s="33">
-        <f>J14*'Assumptions'!J33</f>
-        <v/>
-      </c>
-      <c r="K20" s="33">
-        <f>K14*'Assumptions'!K33</f>
-        <v/>
-      </c>
-      <c r="L20" s="33">
-        <f>L14*'Assumptions'!L33</f>
-        <v/>
-      </c>
-      <c r="M20" s="33">
-        <f>M14*'Assumptions'!M33</f>
-        <v/>
-      </c>
-      <c r="N20" s="33">
-        <f>N14*'Assumptions'!N33</f>
-        <v/>
-      </c>
-      <c r="O20" s="33">
-        <f>O14*'Assumptions'!O33</f>
-        <v/>
-      </c>
+      <c r="B20" s="1" t="n"/>
+      <c r="C20" s="1" t="n"/>
+      <c r="D20" s="1" t="n"/>
+      <c r="E20" s="1" t="n"/>
+      <c r="F20" s="1" t="n"/>
+      <c r="G20" s="1" t="n"/>
+      <c r="H20" s="1" t="n"/>
+      <c r="I20" s="1" t="n"/>
+      <c r="J20" s="1" t="n"/>
+      <c r="K20" s="1" t="n"/>
+      <c r="L20" s="1" t="n"/>
+      <c r="M20" s="1" t="n"/>
+      <c r="N20" s="1" t="n"/>
+      <c r="O20" s="1" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>Industry segment</t>
+          <t>Power segment</t>
         </is>
       </c>
       <c r="B21" s="43">
-        <f>'Operational Drivers'!B15</f>
+        <f>'Operational Drivers'!B16</f>
         <v/>
       </c>
       <c r="C21" s="43">
-        <f>'Operational Drivers'!C15</f>
+        <f>'Operational Drivers'!C16</f>
         <v/>
       </c>
       <c r="D21" s="43">
-        <f>'Operational Drivers'!D15</f>
+        <f>'Operational Drivers'!D16</f>
         <v/>
       </c>
       <c r="E21" s="43">
-        <f>'Operational Drivers'!E15</f>
+        <f>'Operational Drivers'!E16</f>
         <v/>
       </c>
       <c r="F21" s="43">
-        <f>'Operational Drivers'!F15</f>
+        <f>'Operational Drivers'!F16</f>
         <v/>
       </c>
       <c r="G21" s="43">
-        <f>'Operational Drivers'!G15</f>
+        <f>'Operational Drivers'!G16</f>
         <v/>
       </c>
       <c r="H21" s="43">
-        <f>'Operational Drivers'!H15</f>
+        <f>'Operational Drivers'!H16</f>
         <v/>
       </c>
       <c r="I21" s="33">
-        <f>I14*'Assumptions'!I34</f>
+        <f>I15*'Assumptions'!I33</f>
         <v/>
       </c>
       <c r="J21" s="33">
-        <f>J14*'Assumptions'!J34</f>
+        <f>J15*'Assumptions'!J33</f>
         <v/>
       </c>
       <c r="K21" s="33">
-        <f>K14*'Assumptions'!K34</f>
+        <f>K15*'Assumptions'!K33</f>
         <v/>
       </c>
       <c r="L21" s="33">
-        <f>L14*'Assumptions'!L34</f>
+        <f>L15*'Assumptions'!L33</f>
         <v/>
       </c>
       <c r="M21" s="33">
-        <f>M14*'Assumptions'!M34</f>
+        <f>M15*'Assumptions'!M33</f>
         <v/>
       </c>
       <c r="N21" s="33">
-        <f>N14*'Assumptions'!N34</f>
+        <f>N15*'Assumptions'!N33</f>
         <v/>
       </c>
       <c r="O21" s="33">
-        <f>O14*'Assumptions'!O34</f>
+        <f>O15*'Assumptions'!O33</f>
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
+          <t>Industry segment</t>
+        </is>
+      </c>
+      <c r="B22" s="43">
+        <f>'Operational Drivers'!B17</f>
+        <v/>
+      </c>
+      <c r="C22" s="43">
+        <f>'Operational Drivers'!C17</f>
+        <v/>
+      </c>
+      <c r="D22" s="43">
+        <f>'Operational Drivers'!D17</f>
+        <v/>
+      </c>
+      <c r="E22" s="43">
+        <f>'Operational Drivers'!E17</f>
+        <v/>
+      </c>
+      <c r="F22" s="43">
+        <f>'Operational Drivers'!F17</f>
+        <v/>
+      </c>
+      <c r="G22" s="43">
+        <f>'Operational Drivers'!G17</f>
+        <v/>
+      </c>
+      <c r="H22" s="43">
+        <f>'Operational Drivers'!H17</f>
+        <v/>
+      </c>
+      <c r="I22" s="33">
+        <f>I15*'Assumptions'!I34</f>
+        <v/>
+      </c>
+      <c r="J22" s="33">
+        <f>J15*'Assumptions'!J34</f>
+        <v/>
+      </c>
+      <c r="K22" s="33">
+        <f>K15*'Assumptions'!K34</f>
+        <v/>
+      </c>
+      <c r="L22" s="33">
+        <f>L15*'Assumptions'!L34</f>
+        <v/>
+      </c>
+      <c r="M22" s="33">
+        <f>M15*'Assumptions'!M34</f>
+        <v/>
+      </c>
+      <c r="N22" s="33">
+        <f>N15*'Assumptions'!N34</f>
+        <v/>
+      </c>
+      <c r="O22" s="33">
+        <f>O15*'Assumptions'!O34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
           <t>Others / exports / renewables</t>
         </is>
       </c>
-      <c r="B22" s="43">
-        <f>'Operational Drivers'!B16</f>
-        <v/>
-      </c>
-      <c r="C22" s="43">
-        <f>'Operational Drivers'!C16</f>
-        <v/>
-      </c>
-      <c r="D22" s="43">
-        <f>'Operational Drivers'!D16</f>
-        <v/>
-      </c>
-      <c r="E22" s="43">
-        <f>'Operational Drivers'!E16</f>
-        <v/>
-      </c>
-      <c r="F22" s="43">
-        <f>'Operational Drivers'!F16</f>
-        <v/>
-      </c>
-      <c r="G22" s="43">
-        <f>'Operational Drivers'!G16</f>
-        <v/>
-      </c>
-      <c r="H22" s="43">
-        <f>'Operational Drivers'!H16</f>
-        <v/>
-      </c>
-      <c r="I22" s="33">
-        <f>I14*(1-'Assumptions'!I33-'Assumptions'!I34)</f>
-        <v/>
-      </c>
-      <c r="J22" s="33">
-        <f>J14*(1-'Assumptions'!J33-'Assumptions'!J34)</f>
-        <v/>
-      </c>
-      <c r="K22" s="33">
-        <f>K14*(1-'Assumptions'!K33-'Assumptions'!K34)</f>
-        <v/>
-      </c>
-      <c r="L22" s="33">
-        <f>L14*(1-'Assumptions'!L33-'Assumptions'!L34)</f>
-        <v/>
-      </c>
-      <c r="M22" s="33">
-        <f>M14*(1-'Assumptions'!M33-'Assumptions'!M34)</f>
-        <v/>
-      </c>
-      <c r="N22" s="33">
-        <f>N14*(1-'Assumptions'!N33-'Assumptions'!N34)</f>
-        <v/>
-      </c>
-      <c r="O22" s="33">
-        <f>O14*(1-'Assumptions'!O33-'Assumptions'!O34)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
+      <c r="B23" s="43">
+        <f>'Operational Drivers'!B18</f>
+        <v/>
+      </c>
+      <c r="C23" s="43">
+        <f>'Operational Drivers'!C18</f>
+        <v/>
+      </c>
+      <c r="D23" s="43">
+        <f>'Operational Drivers'!D18</f>
+        <v/>
+      </c>
+      <c r="E23" s="43">
+        <f>'Operational Drivers'!E18</f>
+        <v/>
+      </c>
+      <c r="F23" s="43">
+        <f>'Operational Drivers'!F18</f>
+        <v/>
+      </c>
+      <c r="G23" s="43">
+        <f>'Operational Drivers'!G18</f>
+        <v/>
+      </c>
+      <c r="H23" s="43">
+        <f>'Operational Drivers'!H18</f>
+        <v/>
+      </c>
+      <c r="I23" s="33">
+        <f>I15*(1-'Assumptions'!I33-'Assumptions'!I34)</f>
+        <v/>
+      </c>
+      <c r="J23" s="33">
+        <f>J15*(1-'Assumptions'!J33-'Assumptions'!J34)</f>
+        <v/>
+      </c>
+      <c r="K23" s="33">
+        <f>K15*(1-'Assumptions'!K33-'Assumptions'!K34)</f>
+        <v/>
+      </c>
+      <c r="L23" s="33">
+        <f>L15*(1-'Assumptions'!L33-'Assumptions'!L34)</f>
+        <v/>
+      </c>
+      <c r="M23" s="33">
+        <f>M15*(1-'Assumptions'!M33-'Assumptions'!M34)</f>
+        <v/>
+      </c>
+      <c r="N23" s="33">
+        <f>N15*(1-'Assumptions'!N33-'Assumptions'!N34)</f>
+        <v/>
+      </c>
+      <c r="O23" s="33">
+        <f>O15*(1-'Assumptions'!O33-'Assumptions'!O34)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>Total segment revenue (check vs consolidated)</t>
         </is>
       </c>
-      <c r="B23" s="45">
-        <f>SUM(B20:B22)</f>
-        <v/>
-      </c>
-      <c r="C23" s="45">
-        <f>SUM(C20:C22)</f>
-        <v/>
-      </c>
-      <c r="D23" s="45">
-        <f>SUM(D20:D22)</f>
-        <v/>
-      </c>
-      <c r="E23" s="45">
-        <f>SUM(E20:E22)</f>
-        <v/>
-      </c>
-      <c r="F23" s="45">
-        <f>SUM(F20:F22)</f>
-        <v/>
-      </c>
-      <c r="G23" s="45">
-        <f>SUM(G20:G22)</f>
-        <v/>
-      </c>
-      <c r="H23" s="45">
-        <f>SUM(H20:H22)</f>
-        <v/>
-      </c>
-      <c r="I23" s="45">
-        <f>SUM(I20:I22)</f>
-        <v/>
-      </c>
-      <c r="J23" s="45">
-        <f>SUM(J20:J22)</f>
-        <v/>
-      </c>
-      <c r="K23" s="45">
-        <f>SUM(K20:K22)</f>
-        <v/>
-      </c>
-      <c r="L23" s="45">
-        <f>SUM(L20:L22)</f>
-        <v/>
-      </c>
-      <c r="M23" s="45">
-        <f>SUM(M20:M22)</f>
-        <v/>
-      </c>
-      <c r="N23" s="45">
-        <f>SUM(N20:N22)</f>
-        <v/>
-      </c>
-      <c r="O23" s="45">
-        <f>SUM(O20:O22)</f>
+      <c r="B24" s="44">
+        <f>SUM(B21:B23)</f>
+        <v/>
+      </c>
+      <c r="C24" s="44">
+        <f>SUM(C21:C23)</f>
+        <v/>
+      </c>
+      <c r="D24" s="44">
+        <f>SUM(D21:D23)</f>
+        <v/>
+      </c>
+      <c r="E24" s="44">
+        <f>SUM(E21:E23)</f>
+        <v/>
+      </c>
+      <c r="F24" s="44">
+        <f>SUM(F21:F23)</f>
+        <v/>
+      </c>
+      <c r="G24" s="44">
+        <f>SUM(G21:G23)</f>
+        <v/>
+      </c>
+      <c r="H24" s="44">
+        <f>SUM(H21:H23)</f>
+        <v/>
+      </c>
+      <c r="I24" s="44">
+        <f>SUM(I21:I23)</f>
+        <v/>
+      </c>
+      <c r="J24" s="44">
+        <f>SUM(J21:J23)</f>
+        <v/>
+      </c>
+      <c r="K24" s="44">
+        <f>SUM(K21:K23)</f>
+        <v/>
+      </c>
+      <c r="L24" s="44">
+        <f>SUM(L21:L23)</f>
+        <v/>
+      </c>
+      <c r="M24" s="44">
+        <f>SUM(M21:M23)</f>
+        <v/>
+      </c>
+      <c r="N24" s="44">
+        <f>SUM(N21:N23)</f>
+        <v/>
+      </c>
+      <c r="O24" s="44">
+        <f>SUM(O21:O23)</f>
         <v/>
       </c>
     </row>
@@ -17667,31 +17793,31 @@
         <v/>
       </c>
       <c r="I6" s="33">
-        <f>'Revenue Build-up'!I14</f>
+        <f>'Revenue Build-up'!I15</f>
         <v/>
       </c>
       <c r="J6" s="33">
-        <f>'Revenue Build-up'!J14</f>
+        <f>'Revenue Build-up'!J15</f>
         <v/>
       </c>
       <c r="K6" s="33">
-        <f>'Revenue Build-up'!K14</f>
+        <f>'Revenue Build-up'!K15</f>
         <v/>
       </c>
       <c r="L6" s="33">
-        <f>'Revenue Build-up'!L14</f>
+        <f>'Revenue Build-up'!L15</f>
         <v/>
       </c>
       <c r="M6" s="33">
-        <f>'Revenue Build-up'!M14</f>
+        <f>'Revenue Build-up'!M15</f>
         <v/>
       </c>
       <c r="N6" s="33">
-        <f>'Revenue Build-up'!N14</f>
+        <f>'Revenue Build-up'!N15</f>
         <v/>
       </c>
       <c r="O6" s="33">
-        <f>'Revenue Build-up'!O14</f>
+        <f>'Revenue Build-up'!O15</f>
         <v/>
       </c>
     </row>
@@ -17911,59 +18037,59 @@
           <t>Total COGS</t>
         </is>
       </c>
-      <c r="B13" s="44">
+      <c r="B13" s="45">
         <f>'Historical Financial Statements'!B6</f>
         <v/>
       </c>
-      <c r="C13" s="44">
+      <c r="C13" s="45">
         <f>'Historical Financial Statements'!C6</f>
         <v/>
       </c>
-      <c r="D13" s="44">
+      <c r="D13" s="45">
         <f>'Historical Financial Statements'!D6</f>
         <v/>
       </c>
-      <c r="E13" s="44">
+      <c r="E13" s="45">
         <f>'Historical Financial Statements'!E6</f>
         <v/>
       </c>
-      <c r="F13" s="44">
+      <c r="F13" s="45">
         <f>'Historical Financial Statements'!F6</f>
         <v/>
       </c>
-      <c r="G13" s="44">
+      <c r="G13" s="45">
         <f>'Historical Financial Statements'!G6</f>
         <v/>
       </c>
-      <c r="H13" s="44">
+      <c r="H13" s="45">
         <f>'Historical Financial Statements'!H6</f>
         <v/>
       </c>
-      <c r="I13" s="45">
+      <c r="I13" s="44">
         <f>SUM(I7:I12)</f>
         <v/>
       </c>
-      <c r="J13" s="45">
+      <c r="J13" s="44">
         <f>SUM(J7:J12)</f>
         <v/>
       </c>
-      <c r="K13" s="45">
+      <c r="K13" s="44">
         <f>SUM(K7:K12)</f>
         <v/>
       </c>
-      <c r="L13" s="45">
+      <c r="L13" s="44">
         <f>SUM(L7:L12)</f>
         <v/>
       </c>
-      <c r="M13" s="45">
+      <c r="M13" s="44">
         <f>SUM(M7:M12)</f>
         <v/>
       </c>
-      <c r="N13" s="45">
+      <c r="N13" s="44">
         <f>SUM(N7:N12)</f>
         <v/>
       </c>
-      <c r="O13" s="45">
+      <c r="O13" s="44">
         <f>SUM(O7:O12)</f>
         <v/>
       </c>
@@ -18289,59 +18415,59 @@
           <t>Total operating expenses</t>
         </is>
       </c>
-      <c r="B21" s="44">
+      <c r="B21" s="45">
         <f>'Historical Financial Statements'!B11</f>
         <v/>
       </c>
-      <c r="C21" s="44">
+      <c r="C21" s="45">
         <f>'Historical Financial Statements'!C11</f>
         <v/>
       </c>
-      <c r="D21" s="44">
+      <c r="D21" s="45">
         <f>'Historical Financial Statements'!D11</f>
         <v/>
       </c>
-      <c r="E21" s="44">
+      <c r="E21" s="45">
         <f>'Historical Financial Statements'!E11</f>
         <v/>
       </c>
-      <c r="F21" s="44">
+      <c r="F21" s="45">
         <f>'Historical Financial Statements'!F11</f>
         <v/>
       </c>
-      <c r="G21" s="44">
+      <c r="G21" s="45">
         <f>'Historical Financial Statements'!G11</f>
         <v/>
       </c>
-      <c r="H21" s="44">
+      <c r="H21" s="45">
         <f>'Historical Financial Statements'!H11</f>
         <v/>
       </c>
-      <c r="I21" s="45">
+      <c r="I21" s="44">
         <f>I16+I20</f>
         <v/>
       </c>
-      <c r="J21" s="45">
+      <c r="J21" s="44">
         <f>J16+J20</f>
         <v/>
       </c>
-      <c r="K21" s="45">
+      <c r="K21" s="44">
         <f>K16+K20</f>
         <v/>
       </c>
-      <c r="L21" s="45">
+      <c r="L21" s="44">
         <f>L16+L20</f>
         <v/>
       </c>
-      <c r="M21" s="45">
+      <c r="M21" s="44">
         <f>M16+M20</f>
         <v/>
       </c>
-      <c r="N21" s="45">
+      <c r="N21" s="44">
         <f>N16+N20</f>
         <v/>
       </c>
-      <c r="O21" s="45">
+      <c r="O21" s="44">
         <f>O16+O20</f>
         <v/>
       </c>
@@ -18352,59 +18478,59 @@
           <t>EBITDA</t>
         </is>
       </c>
-      <c r="B22" s="44">
+      <c r="B22" s="45">
         <f>'Historical Financial Statements'!B12</f>
         <v/>
       </c>
-      <c r="C22" s="44">
+      <c r="C22" s="45">
         <f>'Historical Financial Statements'!C12</f>
         <v/>
       </c>
-      <c r="D22" s="44">
+      <c r="D22" s="45">
         <f>'Historical Financial Statements'!D12</f>
         <v/>
       </c>
-      <c r="E22" s="44">
+      <c r="E22" s="45">
         <f>'Historical Financial Statements'!E12</f>
         <v/>
       </c>
-      <c r="F22" s="44">
+      <c r="F22" s="45">
         <f>'Historical Financial Statements'!F12</f>
         <v/>
       </c>
-      <c r="G22" s="44">
+      <c r="G22" s="45">
         <f>'Historical Financial Statements'!G12</f>
         <v/>
       </c>
-      <c r="H22" s="44">
+      <c r="H22" s="45">
         <f>'Historical Financial Statements'!H12</f>
         <v/>
       </c>
-      <c r="I22" s="45">
+      <c r="I22" s="44">
         <f>I14-I21</f>
         <v/>
       </c>
-      <c r="J22" s="45">
+      <c r="J22" s="44">
         <f>J14-J21</f>
         <v/>
       </c>
-      <c r="K22" s="45">
+      <c r="K22" s="44">
         <f>K14-K21</f>
         <v/>
       </c>
-      <c r="L22" s="45">
+      <c r="L22" s="44">
         <f>L14-L21</f>
         <v/>
       </c>
-      <c r="M22" s="45">
+      <c r="M22" s="44">
         <f>M14-M21</f>
         <v/>
       </c>
-      <c r="N22" s="45">
+      <c r="N22" s="44">
         <f>N14-N21</f>
         <v/>
       </c>
-      <c r="O22" s="45">
+      <c r="O22" s="44">
         <f>O14-O21</f>
         <v/>
       </c>
@@ -18976,35 +19102,35 @@
           <t>Total operating assets</t>
         </is>
       </c>
-      <c r="H12" s="45">
+      <c r="H12" s="44">
         <f>SUM(H8:H11)</f>
         <v/>
       </c>
-      <c r="I12" s="45">
+      <c r="I12" s="44">
         <f>SUM(I8:I11)</f>
         <v/>
       </c>
-      <c r="J12" s="45">
+      <c r="J12" s="44">
         <f>SUM(J8:J11)</f>
         <v/>
       </c>
-      <c r="K12" s="45">
+      <c r="K12" s="44">
         <f>SUM(K8:K11)</f>
         <v/>
       </c>
-      <c r="L12" s="45">
+      <c r="L12" s="44">
         <f>SUM(L8:L11)</f>
         <v/>
       </c>
-      <c r="M12" s="45">
+      <c r="M12" s="44">
         <f>SUM(M8:M11)</f>
         <v/>
       </c>
-      <c r="N12" s="45">
+      <c r="N12" s="44">
         <f>SUM(N8:N11)</f>
         <v/>
       </c>
-      <c r="O12" s="45">
+      <c r="O12" s="44">
         <f>SUM(O8:O11)</f>
         <v/>
       </c>
@@ -19129,35 +19255,35 @@
           <t>Total operating liabilities</t>
         </is>
       </c>
-      <c r="H16" s="45">
+      <c r="H16" s="44">
         <f>SUM(H13:H15)</f>
         <v/>
       </c>
-      <c r="I16" s="45">
+      <c r="I16" s="44">
         <f>SUM(I13:I15)</f>
         <v/>
       </c>
-      <c r="J16" s="45">
+      <c r="J16" s="44">
         <f>SUM(J13:J15)</f>
         <v/>
       </c>
-      <c r="K16" s="45">
+      <c r="K16" s="44">
         <f>SUM(K13:K15)</f>
         <v/>
       </c>
-      <c r="L16" s="45">
+      <c r="L16" s="44">
         <f>SUM(L13:L15)</f>
         <v/>
       </c>
-      <c r="M16" s="45">
+      <c r="M16" s="44">
         <f>SUM(M13:M15)</f>
         <v/>
       </c>
-      <c r="N16" s="45">
+      <c r="N16" s="44">
         <f>SUM(N13:N15)</f>
         <v/>
       </c>
-      <c r="O16" s="45">
+      <c r="O16" s="44">
         <f>SUM(O13:O15)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Fix long-term borrowings split: 35% -> audited ~2% (lease liabilities only)
BHEL's borrowings are ~98% short-term working-capital lines; the only long-term
piece is lease liabilities (~2% of total, FY26). The prior 35% forecast split was
an arbitrary legacy placeholder inconsistent with the audited data (and with its
own rationale note). Re-anchored lt_debt_pct to 2% and corrected the rationale.
</commit_message>
<xml_diff>
--- a/BHEL_Financial_Model.xlsx
+++ b/BHEL_Financial_Model.xlsx
@@ -11789,25 +11789,25 @@
         </is>
       </c>
       <c r="I51" s="19" t="n">
-        <v>0.35</v>
+        <v>0.02</v>
       </c>
       <c r="J51" s="19" t="n">
-        <v>0.35</v>
+        <v>0.02</v>
       </c>
       <c r="K51" s="19" t="n">
-        <v>0.35</v>
+        <v>0.02</v>
       </c>
       <c r="L51" s="19" t="n">
-        <v>0.35</v>
+        <v>0.02</v>
       </c>
       <c r="M51" s="19" t="n">
-        <v>0.35</v>
+        <v>0.02</v>
       </c>
       <c r="N51" s="19" t="n">
-        <v>0.35</v>
+        <v>0.02</v>
       </c>
       <c r="O51" s="19" t="n">
-        <v>0.35</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="52">
@@ -13740,12 +13740,12 @@
       </c>
       <c r="B34" s="28" t="inlineStr">
         <is>
-          <t>35% LT / 65% ST</t>
+          <t>~2% LT / 98% ST</t>
         </is>
       </c>
       <c r="C34" s="29" t="inlineStr">
         <is>
-          <t>BHEL borrowings are largely short-term working-capital lines; ~35% assumed long-term/leases. Editable split.</t>
+          <t>Audited: BHEL borrowings are almost entirely short-term working-capital lines. The only "long-term" borrowing is lease liabilities (~Rs170 cr in FY26 = 2.05% of total; FY20-26 range 0.3-2.1%). Re-anchored from the prior arbitrary 35% split to the audited actual ~2%.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix debt-repayment placeholder, normalize terminal WC, re-anchor other income
- debt_repay: Rs1,000 cr/yr placeholder -> 0 (BHEL debt is short-term working-
  capital lines, not a term loan; no fixed repayment schedule; funded by cash)
- Terminal value: normalize terminal working-capital investment to the perpetuity
  growth rate g (steady state) instead of the FY33 high-growth WC drain -
  corrects a methodology flaw that understated the terminal value (DCF 68.8 -> 82.5)
- Other income % re-anchored to FY26 audited actual (1.8% -> 2.4%)
- Updated rationale for debt and terminal growth
All balance checks pass
</commit_message>
<xml_diff>
--- a/BHEL_Financial_Model.xlsx
+++ b/BHEL_Financial_Model.xlsx
@@ -9814,11 +9814,11 @@
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>Terminal value (Gordon growth)</t>
+          <t>Terminal value (Gordon growth, normalized WC)</t>
         </is>
       </c>
       <c r="C21" s="53">
-        <f>O12*(1+C20)/(C19-C20)</f>
+        <f>(O8+O9+O10-C20*'Working Capital Schedule'!O17)*(1+C20)/(C19-C20)</f>
         <v/>
       </c>
     </row>
@@ -11005,25 +11005,25 @@
         </is>
       </c>
       <c r="I23" s="19" t="n">
-        <v>0.018</v>
+        <v>0.024</v>
       </c>
       <c r="J23" s="19" t="n">
-        <v>0.018</v>
+        <v>0.024</v>
       </c>
       <c r="K23" s="19" t="n">
-        <v>0.018</v>
+        <v>0.024</v>
       </c>
       <c r="L23" s="19" t="n">
-        <v>0.018</v>
+        <v>0.024</v>
       </c>
       <c r="M23" s="19" t="n">
-        <v>0.018</v>
+        <v>0.024</v>
       </c>
       <c r="N23" s="19" t="n">
-        <v>0.018</v>
+        <v>0.024</v>
       </c>
       <c r="O23" s="19" t="n">
-        <v>0.018</v>
+        <v>0.024</v>
       </c>
     </row>
     <row r="24">
@@ -11733,25 +11733,25 @@
         </is>
       </c>
       <c r="I49" s="17" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="J49" s="17" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="K49" s="17" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="L49" s="17" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="M49" s="17" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="N49" s="17" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="O49" s="17" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50">
@@ -13757,12 +13757,12 @@
       </c>
       <c r="B35" s="28" t="inlineStr">
         <is>
-          <t>0 / Rs1,000 cr p.a.</t>
+          <t>held flat</t>
         </is>
       </c>
       <c r="C35" s="29" t="inlineStr">
         <is>
-          <t>Strong forecast FCF and large cash allow steady deleveraging; gross debt declines over the horizon.</t>
+          <t>BHEL borrowings are short-term working-capital lines (not a term loan) - no fixed repayment schedule. Held flat: the large cash balance (net cash ~Rs3,700 cr) funds working-capital growth. The prior Rs1,000 cr/yr repayment was an unsupported placeholder. Financing choices do not affect FCFF/EV (pre-financing).</t>
         </is>
       </c>
     </row>
@@ -13907,7 +13907,7 @@
       </c>
       <c r="C44" s="29" t="inlineStr">
         <is>
-          <t>Below long-run nominal GDP (~10-11%); conservative perpetuity for a mature franchise (~inflation + modest real growth).</t>
+          <t>Below long-run nominal GDP (~10-11%); conservative perpetuity. Terminal FCFF is NORMALIZED so working capital grows at g (steady state), not at the FY33 high-growth rate - otherwise the terminal value understates value because the last explicit year still carries a large growth-driven WC investment.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Incorporate management guidance from Q4FY24 concall into the forecast
- Revenue growth (~13.5% CAGR) confirmed within management's guided 12-15% CAGR
- Working capital: build in the guided WC-efficiency improvement (legacy NTPC
  projects clearing, faster milestone billing, better advance/payment terms) -
  NWC tapers ~54% -> ~38% of revenue over FY27-33 instead of holding flat at ~50%
  (contract assets 45%->39%, receivable days 74->68, inventory 210->192 vs COGS,
  advances 27%->30%). Moderate/defensible - not the aggressive move to peer levels
- FCFF turns positive from FY28; DCF value/share 82.5 -> 102.4
- Rationale entries cite the concall (21-May-2024)
All balance checks pass
</commit_message>
<xml_diff>
--- a/BHEL_Financial_Model.xlsx
+++ b/BHEL_Financial_Model.xlsx
@@ -11400,22 +11400,22 @@
         <v>74</v>
       </c>
       <c r="J37" s="20" t="n">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="K37" s="20" t="n">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="L37" s="20" t="n">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="M37" s="20" t="n">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="N37" s="20" t="n">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="O37" s="20" t="n">
-        <v>74</v>
+        <v>68</v>
       </c>
     </row>
     <row r="38">
@@ -11428,22 +11428,22 @@
         <v>210</v>
       </c>
       <c r="J38" s="20" t="n">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="K38" s="20" t="n">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="L38" s="20" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="M38" s="20" t="n">
         <v>198</v>
       </c>
       <c r="N38" s="20" t="n">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="O38" s="20" t="n">
-        <v>195</v>
+        <v>192</v>
       </c>
     </row>
     <row r="39">
@@ -11484,22 +11484,22 @@
         <v>0.45</v>
       </c>
       <c r="J40" s="19" t="n">
-        <v>0.45</v>
+        <v>0.44</v>
       </c>
       <c r="K40" s="19" t="n">
-        <v>0.45</v>
+        <v>0.43</v>
       </c>
       <c r="L40" s="19" t="n">
-        <v>0.45</v>
+        <v>0.42</v>
       </c>
       <c r="M40" s="19" t="n">
-        <v>0.45</v>
+        <v>0.41</v>
       </c>
       <c r="N40" s="19" t="n">
-        <v>0.45</v>
+        <v>0.4</v>
       </c>
       <c r="O40" s="19" t="n">
-        <v>0.45</v>
+        <v>0.39</v>
       </c>
     </row>
     <row r="41">
@@ -11512,22 +11512,22 @@
         <v>0.27</v>
       </c>
       <c r="J41" s="19" t="n">
-        <v>0.27</v>
+        <v>0.28</v>
       </c>
       <c r="K41" s="19" t="n">
-        <v>0.27</v>
+        <v>0.28</v>
       </c>
       <c r="L41" s="19" t="n">
-        <v>0.27</v>
+        <v>0.29</v>
       </c>
       <c r="M41" s="19" t="n">
-        <v>0.27</v>
+        <v>0.29</v>
       </c>
       <c r="N41" s="19" t="n">
-        <v>0.27</v>
+        <v>0.3</v>
       </c>
       <c r="O41" s="19" t="n">
-        <v>0.27</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="42">
@@ -13276,7 +13276,7 @@
       </c>
       <c r="C5" s="29" t="inlineStr">
         <is>
-          <t>Revenue recognised as a % of opening order book. Historically BHEL executed ~15-17% of opening OB p.a.; order book is ~7x revenue. Ramp reflects rising capacity utilisation (~65%-&gt;80%) and faster thermal execution as supply chains normalise. Sensitivity: +/-1pp ~ +/-Rs2,400-4,000 cr revenue.</t>
+          <t>Revenue = execution rate x opening order book. Implies ~13.5% revenue CAGR - within management guidance of 12-15% CAGR (Q4FY24 concall). BHEL has ~10 GW/yr execution capacity (demonstrated 12 GW); 80+ GW thermal to be ordered by 2032. Historically executed ~15-17% of opening OB.</t>
         </is>
       </c>
     </row>
@@ -13578,12 +13578,12 @@
       </c>
       <c r="B24" s="28" t="inlineStr">
         <is>
-          <t>74</t>
+          <t>74 -&gt; 68</t>
         </is>
       </c>
       <c r="C24" s="29" t="inlineStr">
         <is>
-          <t>Audited history 49-121 days; recent FY24-26 ~73-76. Large PSU/SEB customers; collections steady. Anchored to the recent ~74-day level.</t>
+          <t>Audited history 49-121 (FY26 73). Tapered down per management WC-improvement focus (Q4FY24 concall): legacy dues clearing within a quarter of milestone completion.</t>
         </is>
       </c>
     </row>
@@ -13595,12 +13595,12 @@
       </c>
       <c r="B25" s="28" t="inlineStr">
         <is>
-          <t>210-&gt;195</t>
+          <t>210 -&gt; 192</t>
         </is>
       </c>
       <c r="C25" s="29" t="inlineStr">
         <is>
-          <t>Audited history 151-232 days (FY26 212); long manufacturing/project cycle. Computed on COGS (consistent with the historical ratio sheet). Gradual improvement assumed.</t>
+          <t>Audited history 151-232 (FY26 212); long project cycle. Tapered per management guidance on better execution &amp; supply-chain/vendor normalisation (Q4FY24 concall).</t>
         </is>
       </c>
     </row>
@@ -13629,12 +13629,12 @@
       </c>
       <c r="B27" s="28" t="inlineStr">
         <is>
-          <t>45%</t>
+          <t>45% -&gt; 39%</t>
         </is>
       </c>
       <c r="C27" s="29" t="inlineStr">
         <is>
-          <t>Unbilled revenue on long-cycle EPC projects (percentage-of-completion). Audited FY26 current contract assets Rs15,193 cr = 45% of revenue (total incl non-current Rs29,390 cr ~ 87%). Re-anchored from the prior 23.5% estimate to the audited actual.</t>
+          <t>Unbilled revenue on long-cycle EPC (percentage-of-completion). Audited FY26 current contract assets = 45% of revenue. Tapered down per management guidance (Q4FY24 concall, 21-May-24): legacy NTPC projects clearing, faster milestone billing and improved payment terms -&gt; working capital "getting better".</t>
         </is>
       </c>
     </row>
@@ -13646,12 +13646,12 @@
       </c>
       <c r="B28" s="28" t="inlineStr">
         <is>
-          <t>27%</t>
+          <t>27% -&gt; 30%</t>
         </is>
       </c>
       <c r="C28" s="29" t="inlineStr">
         <is>
-          <t>Customer advances &amp; billing-in-excess - a key working-capital funding source. Audited FY26 current contract liabilities Rs9,110 cr = 27% of revenue (total incl non-current Rs22,524 cr ~ 67%). Re-anchored from the prior 35.5% estimate to the audited actual.</t>
+          <t>Customer advances &amp; billing-in-excess - key WC funding. Audited FY26 = 27% of revenue. Rising modestly per management (Q4FY24 concall): improved advance / milestone payment terms on new orders (e.g. NTPC bulk orders).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cite FY26 supplementary evidence in assumptions rationale (order book, contract assets flat YoY)
</commit_message>
<xml_diff>
--- a/BHEL_Financial_Model.xlsx
+++ b/BHEL_Financial_Model.xlsx
@@ -13293,7 +13293,7 @@
       </c>
       <c r="C6" s="29" t="inlineStr">
         <is>
-          <t>FY25 record inflow Rs92,535 cr; FY26 ~Rs75,000 cr. Driven by ~80 GW thermal pipeline (NTPC/NLC/state gencos) to FY32, plus T&amp;D, railways and defence diversification. Set conservatively below the FY25 peak; macro driver = power capex super-cycle.</t>
+          <t>FY25 record inflow Rs92,535 cr; FY26 actual Rs75,916 cr (Q4FY26 supplementary); FY26 closing order book Rs2,40,000 cr - highest ever (Power 81% / Industry 18% / Export 1%), CONFIRMING the model driver. ~80 GW thermal to be ordered by 2032 (~10-12 GW/yr) plus T&amp;D, railways, defence, nuclear.</t>
         </is>
       </c>
     </row>
@@ -13634,7 +13634,7 @@
       </c>
       <c r="C27" s="29" t="inlineStr">
         <is>
-          <t>Unbilled revenue on long-cycle EPC (percentage-of-completion). Audited FY26 current contract assets = 45% of revenue. Tapered down per management guidance (Q4FY24 concall, 21-May-24): legacy NTPC projects clearing, faster milestone billing and improved payment terms -&gt; working capital "getting better".</t>
+          <t>Unbilled revenue on long-cycle EPC (percentage-of-completion). Audited FY26 current contract assets = 45% of revenue. VALIDATION: per Q4FY26 supplementary, TOTAL contract assets were ~flat YoY (Rs29,444-&gt;29,390 cr) despite +19% revenue, so contract-assets/revenue fell ~104%-&gt;~87% - the taper is thus conservative. Consistent with Q4FY24 concall guidance (legacy NTPC clearing, faster billing, better payment terms) -&gt; working capital "getting better".</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Price Targets sheet + rework Relative Valuation (blended valuation, 3/6/12M scenarios)
- Relative Valuation: dropped the invalid EV/Revenue method (mismatched margins);
  updated to current (2025-26) peer multiples; added a quality-discount block
  (BHEL vs premium MNC peers) with bear/base/bull EV/EBITDA (15/20/28x) and P/E
  (25/35/45x); implied prices and a relative fair value
- New Price Targets sheet: fundamental fair value (50% DCF + 50% relative, bear/
  base/bull ~Rs117/154/198) and 3/6/12-month scenario price targets wired to live
  forward EBITDA + net cash (Bull ~402/411/529, Base ~385/359/435, Bear ~341/289/317)
- All balance checks pass
</commit_message>
<xml_diff>
--- a/BHEL_Financial_Model.xlsx
+++ b/BHEL_Financial_Model.xlsx
@@ -4,7 +4,7 @@
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="21" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="22" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Cover Page" sheetId="1" state="visible" r:id="rId1"/>
@@ -28,8 +28,9 @@
     <sheet name="Relative Valuation" sheetId="19" state="visible" r:id="rId19"/>
     <sheet name="Sensitivity Analysis" sheetId="20" state="visible" r:id="rId20"/>
     <sheet name="Scenario Analysis" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="Dashboard" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="Error Checks" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="Price Targets" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="Dashboard" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="Error Checks" sheetId="24" state="visible" r:id="rId24"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -200,7 +201,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -351,14 +352,17 @@
     <xf numFmtId="169" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="2" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="165" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="2" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="12" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -9922,15 +9926,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O29"/>
+  <dimension ref="A1:O30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
     <col width="11.5" customWidth="1" min="7" max="7"/>
     <col width="11.5" customWidth="1" min="8" max="8"/>
     <col width="11.5" customWidth="1" min="9" max="9"/>
@@ -9966,14 +9970,14 @@
     <row r="2">
       <c r="A2" s="13" t="inlineStr">
         <is>
-          <t>Peer trading multiples are INDICATIVE; refresh with live market data before use.</t>
+          <t>Peer multiples reflect current (2025-26) market levels. BHEL is valued at a QUALITY DISCOUNT to premium MNC peers (Siemens/ABB ~50x P/E) given its lower margins (~8% vs 15-18%), low ROE (~2-8% vs 15-30%) and PSU profile; the closest large comp is L&amp;T (~20x EV/EBITDA, ~33x P/E). EV/Revenue is intentionally EXCLUDED - it is invalid across such different margin profiles. Refresh peer data before use.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>A.  Peer trading multiples (indicative)</t>
+          <t>A.  Peer trading multiples (current, indicative)</t>
         </is>
       </c>
       <c r="B4" s="1" t="n"/>
@@ -9990,27 +9994,27 @@
       </c>
       <c r="B5" s="15" t="inlineStr">
         <is>
-          <t>EV/Revenue (x)</t>
+          <t>EV/EBITDA (x)</t>
         </is>
       </c>
       <c r="C5" s="15" t="inlineStr">
         <is>
-          <t>EV/EBITDA (x)</t>
+          <t>P/E (x)</t>
         </is>
       </c>
       <c r="D5" s="15" t="inlineStr">
         <is>
-          <t>P/E (x)</t>
+          <t>P/B (x)</t>
         </is>
       </c>
       <c r="E5" s="15" t="inlineStr">
         <is>
-          <t>P/B (x)</t>
+          <t>ROE %</t>
         </is>
       </c>
       <c r="F5" s="15" t="inlineStr">
         <is>
-          <t>Div yield %</t>
+          <t>Div yld %</t>
         </is>
       </c>
     </row>
@@ -10021,16 +10025,16 @@
         </is>
       </c>
       <c r="B6" s="59" t="n">
-        <v>5.5</v>
+        <v>42</v>
       </c>
       <c r="C6" s="59" t="n">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="D6" s="59" t="n">
-        <v>60</v>
-      </c>
-      <c r="E6" s="59" t="n">
         <v>9</v>
+      </c>
+      <c r="E6" s="60" t="n">
+        <v>16</v>
       </c>
       <c r="F6" s="60" t="n">
         <v>0.4</v>
@@ -10043,16 +10047,16 @@
         </is>
       </c>
       <c r="B7" s="59" t="n">
-        <v>7</v>
+        <v>48</v>
       </c>
       <c r="C7" s="59" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D7" s="59" t="n">
-        <v>68</v>
-      </c>
-      <c r="E7" s="59" t="n">
         <v>14</v>
+      </c>
+      <c r="E7" s="60" t="n">
+        <v>20</v>
       </c>
       <c r="F7" s="60" t="n">
         <v>0.4</v>
@@ -10065,16 +10069,16 @@
         </is>
       </c>
       <c r="B8" s="59" t="n">
-        <v>6.5</v>
+        <v>45</v>
       </c>
       <c r="C8" s="59" t="n">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="D8" s="59" t="n">
-        <v>62</v>
-      </c>
-      <c r="E8" s="59" t="n">
         <v>18</v>
+      </c>
+      <c r="E8" s="60" t="n">
+        <v>22</v>
       </c>
       <c r="F8" s="60" t="n">
         <v>0.2</v>
@@ -10083,270 +10087,321 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>GE Vernova T&amp;D India</t>
+          <t>Thermax</t>
         </is>
       </c>
       <c r="B9" s="59" t="n">
-        <v>8</v>
+        <v>34</v>
       </c>
       <c r="C9" s="59" t="n">
         <v>48</v>
       </c>
       <c r="D9" s="59" t="n">
-        <v>65</v>
-      </c>
-      <c r="E9" s="59" t="n">
-        <v>20</v>
+        <v>8</v>
+      </c>
+      <c r="E9" s="60" t="n">
+        <v>14</v>
       </c>
       <c r="F9" s="60" t="n">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Thermax</t>
+          <t>Triveni Turbine</t>
         </is>
       </c>
       <c r="B10" s="59" t="n">
-        <v>4</v>
+        <v>38</v>
       </c>
       <c r="C10" s="59" t="n">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D10" s="59" t="n">
-        <v>55</v>
-      </c>
-      <c r="E10" s="59" t="n">
-        <v>8</v>
+        <v>16</v>
+      </c>
+      <c r="E10" s="60" t="n">
+        <v>30</v>
       </c>
       <c r="F10" s="60" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>Triveni Turbine</t>
+          <t>Larsen &amp; Toubro</t>
         </is>
       </c>
       <c r="B11" s="59" t="n">
-        <v>7.5</v>
+        <v>20</v>
       </c>
       <c r="C11" s="59" t="n">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="D11" s="59" t="n">
-        <v>52</v>
-      </c>
-      <c r="E11" s="59" t="n">
-        <v>16</v>
+        <v>5</v>
+      </c>
+      <c r="E11" s="60" t="n">
+        <v>15</v>
       </c>
       <c r="F11" s="60" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>Larsen &amp; Toubro</t>
+          <t>Kalpataru Projects</t>
         </is>
       </c>
       <c r="B12" s="59" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="C12" s="59" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D12" s="59" t="n">
-        <v>32</v>
-      </c>
-      <c r="E12" s="59" t="n">
-        <v>5</v>
+        <v>3</v>
+      </c>
+      <c r="E12" s="60" t="n">
+        <v>11</v>
       </c>
       <c r="F12" s="60" t="n">
-        <v>0.7</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>Kalpataru Projects</t>
-        </is>
-      </c>
-      <c r="B13" s="59" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="C13" s="59" t="n">
-        <v>12</v>
-      </c>
-      <c r="D13" s="59" t="n">
-        <v>22</v>
-      </c>
-      <c r="E13" s="59" t="n">
-        <v>3</v>
-      </c>
-      <c r="F13" s="60" t="n">
-        <v>0.4</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="61" t="inlineStr">
-        <is>
-          <t>Median</t>
-        </is>
-      </c>
-      <c r="B14" s="62">
-        <f>MEDIAN(B6:B13)</f>
-        <v/>
-      </c>
-      <c r="C14" s="62">
-        <f>MEDIAN(C6:C13)</f>
-        <v/>
-      </c>
-      <c r="D14" s="62">
-        <f>MEDIAN(D6:D13)</f>
-        <v/>
-      </c>
-      <c r="E14" s="62">
-        <f>MEDIAN(E6:E13)</f>
-        <v/>
-      </c>
-      <c r="F14" s="63">
-        <f>MEDIAN(F6:F13)</f>
-        <v/>
-      </c>
+      <c r="A13" s="61" t="inlineStr">
+        <is>
+          <t>Peer median</t>
+        </is>
+      </c>
+      <c r="B13" s="62">
+        <f>MEDIAN(B6:B12)</f>
+        <v/>
+      </c>
+      <c r="C13" s="62">
+        <f>MEDIAN(C6:C12)</f>
+        <v/>
+      </c>
+      <c r="D13" s="62">
+        <f>MEDIAN(D6:D12)</f>
+        <v/>
+      </c>
+      <c r="E13" s="63">
+        <f>MEDIAN(E6:E12)</f>
+        <v/>
+      </c>
+      <c r="F13" s="63">
+        <f>MEDIAN(F6:F12)</f>
+        <v/>
+      </c>
+      <c r="G13" s="13" t="inlineStr">
+        <is>
+          <t>BHEL ROE ~2-8% -&gt; discount to peers</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>B.  BHEL target multiples (quality-discounted)</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="n"/>
+      <c r="C15" s="1" t="n"/>
+      <c r="D15" s="1" t="n"/>
+      <c r="E15" s="1" t="n"/>
+      <c r="F15" s="1" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="11" t="inlineStr">
-        <is>
-          <t>B.  Implied valuation for BHEL (on FY2027E)</t>
-        </is>
-      </c>
-      <c r="B16" s="1" t="n"/>
-      <c r="C16" s="1" t="n"/>
-      <c r="D16" s="1" t="n"/>
-      <c r="E16" s="1" t="n"/>
-      <c r="F16" s="1" t="n"/>
+      <c r="A16" s="15" t="inlineStr">
+        <is>
+          <t>Multiple</t>
+        </is>
+      </c>
+      <c r="B16" s="15" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="C16" s="15" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="D16" s="15" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>BHEL FY2027E revenue</t>
-        </is>
-      </c>
-      <c r="C17" s="55">
-        <f>'Forecast Financial Statements'!I5</f>
-        <v/>
+          <t>EV/EBITDA (x)  [L&amp;T ~20x]</t>
+        </is>
+      </c>
+      <c r="B17" s="59" t="n">
+        <v>15</v>
+      </c>
+      <c r="C17" s="59" t="n">
+        <v>20</v>
+      </c>
+      <c r="D17" s="59" t="n">
+        <v>28</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
+          <t>P/E (x)  [L&amp;T ~33x]</t>
+        </is>
+      </c>
+      <c r="B18" s="59" t="n">
+        <v>25</v>
+      </c>
+      <c r="C18" s="59" t="n">
+        <v>35</v>
+      </c>
+      <c r="D18" s="59" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="11" t="inlineStr">
+        <is>
+          <t>C.  Implied value for BHEL (FY2027E)</t>
+        </is>
+      </c>
+      <c r="B20" s="1" t="n"/>
+      <c r="C20" s="1" t="n"/>
+      <c r="D20" s="1" t="n"/>
+      <c r="E20" s="1" t="n"/>
+      <c r="F20" s="1" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
           <t>BHEL FY2027E EBITDA</t>
         </is>
       </c>
-      <c r="C18" s="55">
+      <c r="C21" s="55">
         <f>'Forecast Financial Statements'!I12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>BHEL FY2027E EPS (INR)</t>
-        </is>
-      </c>
-      <c r="C19" s="58">
-        <f>'Forecast Financial Statements'!I21</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>Net debt (FY26)</t>
-        </is>
-      </c>
-      <c r="C20" s="55">
-        <f>'Forecast Financial Statements'!H63-'Forecast Financial Statements'!H58</f>
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>Implied EV (EV/EBITDA method)</t>
-        </is>
-      </c>
-      <c r="C22" s="53">
-        <f>C18*C14</f>
+          <t>BHEL FY2027E EPS (INR)</t>
+        </is>
+      </c>
+      <c r="C22" s="58">
+        <f>'Forecast Financial Statements'!I21</f>
         <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>Implied equity value (EV/EBITDA)</t>
-        </is>
-      </c>
-      <c r="C23" s="53">
-        <f>C22-C20</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>Implied price - EV/EBITDA (INR)</t>
-        </is>
-      </c>
-      <c r="C24" s="57">
-        <f>C23/'Assumptions'!C66</f>
+          <t>Net cash (FY26)</t>
+        </is>
+      </c>
+      <c r="C23" s="55">
+        <f>'Forecast Financial Statements'!H58-'Forecast Financial Statements'!H63</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t>Implied price - P/E method (INR)</t>
-        </is>
-      </c>
-      <c r="C25" s="57">
-        <f>C19*D14</f>
-        <v/>
+      <c r="A25" s="15" t="inlineStr">
+        <is>
+          <t>Implied price (INR)</t>
+        </is>
+      </c>
+      <c r="B25" s="15" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="C25" s="15" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="D25" s="15" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>Implied EV (EV/Revenue method)</t>
-        </is>
-      </c>
-      <c r="C26" s="53">
-        <f>C17*B14</f>
+          <t>EV/EBITDA method</t>
+        </is>
+      </c>
+      <c r="B26" s="64">
+        <f>(B17*$C$21+$C$23)/'Assumptions'!C66</f>
+        <v/>
+      </c>
+      <c r="C26" s="64">
+        <f>(C17*$C$21+$C$23)/'Assumptions'!C66</f>
+        <v/>
+      </c>
+      <c r="D26" s="64">
+        <f>(D17*$C$21+$C$23)/'Assumptions'!C66</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>Implied price - EV/Revenue (INR)</t>
-        </is>
-      </c>
-      <c r="C27" s="57">
-        <f>(C26-C20)/'Assumptions'!C66</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t>Average implied target price (INR)</t>
-        </is>
-      </c>
-      <c r="C29" s="64">
-        <f>AVERAGE(C24,C25,C27)</f>
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>P/E method</t>
+        </is>
+      </c>
+      <c r="B27" s="64">
+        <f>B18*$C$22</f>
+        <v/>
+      </c>
+      <c r="C27" s="64">
+        <f>C18*$C$22</f>
+        <v/>
+      </c>
+      <c r="D27" s="64">
+        <f>D18*$C$22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Relative fair value (avg of methods)</t>
+        </is>
+      </c>
+      <c r="B28" s="57">
+        <f>AVERAGE(B26,B27)</f>
+        <v/>
+      </c>
+      <c r="C28" s="57">
+        <f>AVERAGE(C26,C27)</f>
+        <v/>
+      </c>
+      <c r="D28" s="57">
+        <f>AVERAGE(D26,D27)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>Memo: sector-parity (peer median EV/EBITDA, no discount)</t>
+        </is>
+      </c>
+      <c r="C30" s="64">
+        <f>(C13*$C$21+$C$23)/'Assumptions'!C66</f>
         <v/>
       </c>
     </row>
@@ -12108,23 +12163,23 @@
         <f>'Assumptions'!C65+0.02</f>
         <v/>
       </c>
-      <c r="C6" s="66">
+      <c r="C6" s="64">
         <f>(SUMPRODUCT('DCF Valuation'!$I$12:$O$12,(1+$B6)^(-'DCF Valuation'!$I$13:$O$13))+('DCF Valuation'!$O$12*(1+C$5)/($B6-C$5))*(1+$B6)^(-7)+'DCF Valuation'!$C$24)/'DCF Valuation'!$C$26</f>
         <v/>
       </c>
-      <c r="D6" s="66">
+      <c r="D6" s="64">
         <f>(SUMPRODUCT('DCF Valuation'!$I$12:$O$12,(1+$B6)^(-'DCF Valuation'!$I$13:$O$13))+('DCF Valuation'!$O$12*(1+D$5)/($B6-D$5))*(1+$B6)^(-7)+'DCF Valuation'!$C$24)/'DCF Valuation'!$C$26</f>
         <v/>
       </c>
-      <c r="E6" s="66">
+      <c r="E6" s="64">
         <f>(SUMPRODUCT('DCF Valuation'!$I$12:$O$12,(1+$B6)^(-'DCF Valuation'!$I$13:$O$13))+('DCF Valuation'!$O$12*(1+E$5)/($B6-E$5))*(1+$B6)^(-7)+'DCF Valuation'!$C$24)/'DCF Valuation'!$C$26</f>
         <v/>
       </c>
-      <c r="F6" s="66">
+      <c r="F6" s="64">
         <f>(SUMPRODUCT('DCF Valuation'!$I$12:$O$12,(1+$B6)^(-'DCF Valuation'!$I$13:$O$13))+('DCF Valuation'!$O$12*(1+F$5)/($B6-F$5))*(1+$B6)^(-7)+'DCF Valuation'!$C$24)/'DCF Valuation'!$C$26</f>
         <v/>
       </c>
-      <c r="G6" s="66">
+      <c r="G6" s="64">
         <f>(SUMPRODUCT('DCF Valuation'!$I$12:$O$12,(1+$B6)^(-'DCF Valuation'!$I$13:$O$13))+('DCF Valuation'!$O$12*(1+G$5)/($B6-G$5))*(1+$B6)^(-7)+'DCF Valuation'!$C$24)/'DCF Valuation'!$C$26</f>
         <v/>
       </c>
@@ -12134,23 +12189,23 @@
         <f>'Assumptions'!C65+0.01</f>
         <v/>
       </c>
-      <c r="C7" s="66">
+      <c r="C7" s="64">
         <f>(SUMPRODUCT('DCF Valuation'!$I$12:$O$12,(1+$B7)^(-'DCF Valuation'!$I$13:$O$13))+('DCF Valuation'!$O$12*(1+C$5)/($B7-C$5))*(1+$B7)^(-7)+'DCF Valuation'!$C$24)/'DCF Valuation'!$C$26</f>
         <v/>
       </c>
-      <c r="D7" s="66">
+      <c r="D7" s="64">
         <f>(SUMPRODUCT('DCF Valuation'!$I$12:$O$12,(1+$B7)^(-'DCF Valuation'!$I$13:$O$13))+('DCF Valuation'!$O$12*(1+D$5)/($B7-D$5))*(1+$B7)^(-7)+'DCF Valuation'!$C$24)/'DCF Valuation'!$C$26</f>
         <v/>
       </c>
-      <c r="E7" s="66">
+      <c r="E7" s="64">
         <f>(SUMPRODUCT('DCF Valuation'!$I$12:$O$12,(1+$B7)^(-'DCF Valuation'!$I$13:$O$13))+('DCF Valuation'!$O$12*(1+E$5)/($B7-E$5))*(1+$B7)^(-7)+'DCF Valuation'!$C$24)/'DCF Valuation'!$C$26</f>
         <v/>
       </c>
-      <c r="F7" s="66">
+      <c r="F7" s="64">
         <f>(SUMPRODUCT('DCF Valuation'!$I$12:$O$12,(1+$B7)^(-'DCF Valuation'!$I$13:$O$13))+('DCF Valuation'!$O$12*(1+F$5)/($B7-F$5))*(1+$B7)^(-7)+'DCF Valuation'!$C$24)/'DCF Valuation'!$C$26</f>
         <v/>
       </c>
-      <c r="G7" s="66">
+      <c r="G7" s="64">
         <f>(SUMPRODUCT('DCF Valuation'!$I$12:$O$12,(1+$B7)^(-'DCF Valuation'!$I$13:$O$13))+('DCF Valuation'!$O$12*(1+G$5)/($B7-G$5))*(1+$B7)^(-7)+'DCF Valuation'!$C$24)/'DCF Valuation'!$C$26</f>
         <v/>
       </c>
@@ -12160,11 +12215,11 @@
         <f>'Assumptions'!C65+0.0</f>
         <v/>
       </c>
-      <c r="C8" s="66">
+      <c r="C8" s="64">
         <f>(SUMPRODUCT('DCF Valuation'!$I$12:$O$12,(1+$B8)^(-'DCF Valuation'!$I$13:$O$13))+('DCF Valuation'!$O$12*(1+C$5)/($B8-C$5))*(1+$B8)^(-7)+'DCF Valuation'!$C$24)/'DCF Valuation'!$C$26</f>
         <v/>
       </c>
-      <c r="D8" s="66">
+      <c r="D8" s="64">
         <f>(SUMPRODUCT('DCF Valuation'!$I$12:$O$12,(1+$B8)^(-'DCF Valuation'!$I$13:$O$13))+('DCF Valuation'!$O$12*(1+D$5)/($B8-D$5))*(1+$B8)^(-7)+'DCF Valuation'!$C$24)/'DCF Valuation'!$C$26</f>
         <v/>
       </c>
@@ -12172,11 +12227,11 @@
         <f>(SUMPRODUCT('DCF Valuation'!$I$12:$O$12,(1+$B8)^(-'DCF Valuation'!$I$13:$O$13))+('DCF Valuation'!$O$12*(1+E$5)/($B8-E$5))*(1+$B8)^(-7)+'DCF Valuation'!$C$24)/'DCF Valuation'!$C$26</f>
         <v/>
       </c>
-      <c r="F8" s="66">
+      <c r="F8" s="64">
         <f>(SUMPRODUCT('DCF Valuation'!$I$12:$O$12,(1+$B8)^(-'DCF Valuation'!$I$13:$O$13))+('DCF Valuation'!$O$12*(1+F$5)/($B8-F$5))*(1+$B8)^(-7)+'DCF Valuation'!$C$24)/'DCF Valuation'!$C$26</f>
         <v/>
       </c>
-      <c r="G8" s="66">
+      <c r="G8" s="64">
         <f>(SUMPRODUCT('DCF Valuation'!$I$12:$O$12,(1+$B8)^(-'DCF Valuation'!$I$13:$O$13))+('DCF Valuation'!$O$12*(1+G$5)/($B8-G$5))*(1+$B8)^(-7)+'DCF Valuation'!$C$24)/'DCF Valuation'!$C$26</f>
         <v/>
       </c>
@@ -12186,23 +12241,23 @@
         <f>'Assumptions'!C65+-0.01</f>
         <v/>
       </c>
-      <c r="C9" s="66">
+      <c r="C9" s="64">
         <f>(SUMPRODUCT('DCF Valuation'!$I$12:$O$12,(1+$B9)^(-'DCF Valuation'!$I$13:$O$13))+('DCF Valuation'!$O$12*(1+C$5)/($B9-C$5))*(1+$B9)^(-7)+'DCF Valuation'!$C$24)/'DCF Valuation'!$C$26</f>
         <v/>
       </c>
-      <c r="D9" s="66">
+      <c r="D9" s="64">
         <f>(SUMPRODUCT('DCF Valuation'!$I$12:$O$12,(1+$B9)^(-'DCF Valuation'!$I$13:$O$13))+('DCF Valuation'!$O$12*(1+D$5)/($B9-D$5))*(1+$B9)^(-7)+'DCF Valuation'!$C$24)/'DCF Valuation'!$C$26</f>
         <v/>
       </c>
-      <c r="E9" s="66">
+      <c r="E9" s="64">
         <f>(SUMPRODUCT('DCF Valuation'!$I$12:$O$12,(1+$B9)^(-'DCF Valuation'!$I$13:$O$13))+('DCF Valuation'!$O$12*(1+E$5)/($B9-E$5))*(1+$B9)^(-7)+'DCF Valuation'!$C$24)/'DCF Valuation'!$C$26</f>
         <v/>
       </c>
-      <c r="F9" s="66">
+      <c r="F9" s="64">
         <f>(SUMPRODUCT('DCF Valuation'!$I$12:$O$12,(1+$B9)^(-'DCF Valuation'!$I$13:$O$13))+('DCF Valuation'!$O$12*(1+F$5)/($B9-F$5))*(1+$B9)^(-7)+'DCF Valuation'!$C$24)/'DCF Valuation'!$C$26</f>
         <v/>
       </c>
-      <c r="G9" s="66">
+      <c r="G9" s="64">
         <f>(SUMPRODUCT('DCF Valuation'!$I$12:$O$12,(1+$B9)^(-'DCF Valuation'!$I$13:$O$13))+('DCF Valuation'!$O$12*(1+G$5)/($B9-G$5))*(1+$B9)^(-7)+'DCF Valuation'!$C$24)/'DCF Valuation'!$C$26</f>
         <v/>
       </c>
@@ -12212,23 +12267,23 @@
         <f>'Assumptions'!C65+-0.02</f>
         <v/>
       </c>
-      <c r="C10" s="66">
+      <c r="C10" s="64">
         <f>(SUMPRODUCT('DCF Valuation'!$I$12:$O$12,(1+$B10)^(-'DCF Valuation'!$I$13:$O$13))+('DCF Valuation'!$O$12*(1+C$5)/($B10-C$5))*(1+$B10)^(-7)+'DCF Valuation'!$C$24)/'DCF Valuation'!$C$26</f>
         <v/>
       </c>
-      <c r="D10" s="66">
+      <c r="D10" s="64">
         <f>(SUMPRODUCT('DCF Valuation'!$I$12:$O$12,(1+$B10)^(-'DCF Valuation'!$I$13:$O$13))+('DCF Valuation'!$O$12*(1+D$5)/($B10-D$5))*(1+$B10)^(-7)+'DCF Valuation'!$C$24)/'DCF Valuation'!$C$26</f>
         <v/>
       </c>
-      <c r="E10" s="66">
+      <c r="E10" s="64">
         <f>(SUMPRODUCT('DCF Valuation'!$I$12:$O$12,(1+$B10)^(-'DCF Valuation'!$I$13:$O$13))+('DCF Valuation'!$O$12*(1+E$5)/($B10-E$5))*(1+$B10)^(-7)+'DCF Valuation'!$C$24)/'DCF Valuation'!$C$26</f>
         <v/>
       </c>
-      <c r="F10" s="66">
+      <c r="F10" s="64">
         <f>(SUMPRODUCT('DCF Valuation'!$I$12:$O$12,(1+$B10)^(-'DCF Valuation'!$I$13:$O$13))+('DCF Valuation'!$O$12*(1+F$5)/($B10-F$5))*(1+$B10)^(-7)+'DCF Valuation'!$C$24)/'DCF Valuation'!$C$26</f>
         <v/>
       </c>
-      <c r="G10" s="66">
+      <c r="G10" s="64">
         <f>(SUMPRODUCT('DCF Valuation'!$I$12:$O$12,(1+$B10)^(-'DCF Valuation'!$I$13:$O$13))+('DCF Valuation'!$O$12*(1+G$5)/($B10-G$5))*(1+$B10)^(-7)+'DCF Valuation'!$C$24)/'DCF Valuation'!$C$26</f>
         <v/>
       </c>
@@ -12535,7 +12590,7 @@
           <t>Probability-weighted target price (INR)</t>
         </is>
       </c>
-      <c r="B17" s="64">
+      <c r="B17" s="66">
         <f>SUMPRODUCT(B14:D14,B15:D15)</f>
         <v/>
       </c>
@@ -12546,6 +12601,552 @@
 </file>
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00548235"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:O39"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="11.5" customWidth="1" min="5" max="5"/>
+    <col width="11.5" customWidth="1" min="6" max="6"/>
+    <col width="11.5" customWidth="1" min="7" max="7"/>
+    <col width="11.5" customWidth="1" min="8" max="8"/>
+    <col width="11.5" customWidth="1" min="9" max="9"/>
+    <col width="11.5" customWidth="1" min="10" max="10"/>
+    <col width="11.5" customWidth="1" min="11" max="11"/>
+    <col width="11.5" customWidth="1" min="12" max="12"/>
+    <col width="11.5" customWidth="1" min="13" max="13"/>
+    <col width="11.5" customWidth="1" min="14" max="14"/>
+    <col width="11.5" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>PRICE TARGETS</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="n"/>
+      <c r="C1" s="1" t="n"/>
+      <c r="D1" s="1" t="n"/>
+      <c r="E1" s="1" t="n"/>
+      <c r="F1" s="1" t="n"/>
+      <c r="G1" s="1" t="n"/>
+      <c r="H1" s="1" t="n"/>
+      <c r="I1" s="1" t="n"/>
+      <c r="J1" s="1" t="n"/>
+      <c r="K1" s="1" t="n"/>
+      <c r="L1" s="1" t="n"/>
+      <c r="M1" s="1" t="n"/>
+      <c r="N1" s="1" t="n"/>
+      <c r="O1" s="1" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="13" t="inlineStr">
+        <is>
+          <t>Blended valuation &amp; scenario price targets. Fundamental fair value = 50% DCF + 50% quality-adjusted relative. Horizon targets apply scenario EV/EBITDA multiples to forward EBITDA (3M/6M on FY2027E, 12M rolled to FY2028E) plus net cash, per share. Multiples (gold) are editable. Model output, not investment advice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>A.  Inputs (live links)</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="n"/>
+      <c r="C4" s="1" t="n"/>
+      <c r="D4" s="1" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>FY2027E EBITDA (INR Cr)</t>
+        </is>
+      </c>
+      <c r="C5" s="55">
+        <f>'Forecast Financial Statements'!I12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>FY2028E EBITDA (INR Cr)</t>
+        </is>
+      </c>
+      <c r="C6" s="55">
+        <f>'Forecast Financial Statements'!J12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Net cash - FY26 (INR Cr)</t>
+        </is>
+      </c>
+      <c r="C7" s="55">
+        <f>'Forecast Financial Statements'!H58-'Forecast Financial Statements'!H63</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Shares outstanding (crore)</t>
+        </is>
+      </c>
+      <c r="C8" s="56">
+        <f>'Assumptions'!C66</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Current market price (INR)</t>
+        </is>
+      </c>
+      <c r="C9" s="58">
+        <f>'Assumptions'!C67</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>DCF value/share - base (INR)</t>
+        </is>
+      </c>
+      <c r="C10" s="58">
+        <f>'DCF Valuation'!C27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Relative fair value - Bear/Base/Bull (INR)</t>
+        </is>
+      </c>
+      <c r="B11" s="58">
+        <f>'Relative Valuation'!B28</f>
+        <v/>
+      </c>
+      <c r="C11" s="58">
+        <f>'Relative Valuation'!C28</f>
+        <v/>
+      </c>
+      <c r="D11" s="58">
+        <f>'Relative Valuation'!D28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>B.  Fundamental fair value (12-month)</t>
+        </is>
+      </c>
+      <c r="B13" s="1" t="n"/>
+      <c r="C13" s="1" t="n"/>
+      <c r="D13" s="1" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="15" t="inlineStr"/>
+      <c r="B14" s="15" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="C14" s="15" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="D14" s="15" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>DCF (INR/share)</t>
+        </is>
+      </c>
+      <c r="B15" s="64">
+        <f>$C$10*0.81</f>
+        <v/>
+      </c>
+      <c r="C15" s="64">
+        <f>$C$10</f>
+        <v/>
+      </c>
+      <c r="D15" s="64">
+        <f>$C$10*1.20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Relative (INR/share)</t>
+        </is>
+      </c>
+      <c r="B16" s="64">
+        <f>B11</f>
+        <v/>
+      </c>
+      <c r="C16" s="64">
+        <f>C11</f>
+        <v/>
+      </c>
+      <c r="D16" s="64">
+        <f>D11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Blended fair value (50/50)</t>
+        </is>
+      </c>
+      <c r="B17" s="57">
+        <f>AVERAGE(B15,B16)</f>
+        <v/>
+      </c>
+      <c r="C17" s="57">
+        <f>AVERAGE(C15,C16)</f>
+        <v/>
+      </c>
+      <c r="D17" s="57">
+        <f>AVERAGE(D15,D16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Upside/(downside) vs current price</t>
+        </is>
+      </c>
+      <c r="B18" s="22">
+        <f>B17/$C$9-1</f>
+        <v/>
+      </c>
+      <c r="C18" s="22">
+        <f>C17/$C$9-1</f>
+        <v/>
+      </c>
+      <c r="D18" s="22">
+        <f>D17/$C$9-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="11" t="inlineStr">
+        <is>
+          <t>C.  Scenario EV/EBITDA multiple (x) - editable</t>
+        </is>
+      </c>
+      <c r="B20" s="1" t="n"/>
+      <c r="C20" s="1" t="n"/>
+      <c r="D20" s="1" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="15" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="B21" s="15" t="inlineStr">
+        <is>
+          <t>3-month</t>
+        </is>
+      </c>
+      <c r="C21" s="15" t="inlineStr">
+        <is>
+          <t>6-month</t>
+        </is>
+      </c>
+      <c r="D21" s="15" t="inlineStr">
+        <is>
+          <t>12-month</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="B22" s="59" t="n">
+        <v>45</v>
+      </c>
+      <c r="C22" s="59" t="n">
+        <v>46</v>
+      </c>
+      <c r="D22" s="59" t="n">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="B23" s="59" t="n">
+        <v>43</v>
+      </c>
+      <c r="C23" s="59" t="n">
+        <v>40</v>
+      </c>
+      <c r="D23" s="59" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="B24" s="59" t="n">
+        <v>38</v>
+      </c>
+      <c r="C24" s="59" t="n">
+        <v>32</v>
+      </c>
+      <c r="D24" s="59" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>EBITDA basis</t>
+        </is>
+      </c>
+      <c r="B25" s="67" t="inlineStr">
+        <is>
+          <t>FY2027E</t>
+        </is>
+      </c>
+      <c r="C25" s="67" t="inlineStr">
+        <is>
+          <t>FY2027E</t>
+        </is>
+      </c>
+      <c r="D25" s="67" t="inlineStr">
+        <is>
+          <t>FY2028E</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="11" t="inlineStr">
+        <is>
+          <t>D.  Scenario price target (INR/share)</t>
+        </is>
+      </c>
+      <c r="B27" s="1" t="n"/>
+      <c r="C27" s="1" t="n"/>
+      <c r="D27" s="1" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="15" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="B28" s="15" t="inlineStr">
+        <is>
+          <t>3-month</t>
+        </is>
+      </c>
+      <c r="C28" s="15" t="inlineStr">
+        <is>
+          <t>6-month</t>
+        </is>
+      </c>
+      <c r="D28" s="15" t="inlineStr">
+        <is>
+          <t>12-month</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="B29" s="64">
+        <f>(B22*$C$5+$C$7)/$C$8</f>
+        <v/>
+      </c>
+      <c r="C29" s="64">
+        <f>(C22*$C$5+$C$7)/$C$8</f>
+        <v/>
+      </c>
+      <c r="D29" s="64">
+        <f>(D22*$C$6+$C$7)/$C$8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="B30" s="57">
+        <f>(B23*$C$5+$C$7)/$C$8</f>
+        <v/>
+      </c>
+      <c r="C30" s="57">
+        <f>(C23*$C$5+$C$7)/$C$8</f>
+        <v/>
+      </c>
+      <c r="D30" s="57">
+        <f>(D23*$C$6+$C$7)/$C$8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="B31" s="64">
+        <f>(B24*$C$5+$C$7)/$C$8</f>
+        <v/>
+      </c>
+      <c r="C31" s="64">
+        <f>(C24*$C$5+$C$7)/$C$8</f>
+        <v/>
+      </c>
+      <c r="D31" s="64">
+        <f>(D24*$C$6+$C$7)/$C$8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="11" t="inlineStr">
+        <is>
+          <t>E.  Upside/(downside) vs current price</t>
+        </is>
+      </c>
+      <c r="B33" s="1" t="n"/>
+      <c r="C33" s="1" t="n"/>
+      <c r="D33" s="1" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="15" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="B34" s="15" t="inlineStr">
+        <is>
+          <t>3-month</t>
+        </is>
+      </c>
+      <c r="C34" s="15" t="inlineStr">
+        <is>
+          <t>6-month</t>
+        </is>
+      </c>
+      <c r="D34" s="15" t="inlineStr">
+        <is>
+          <t>12-month</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="B35" s="22">
+        <f>B29/$C$9-1</f>
+        <v/>
+      </c>
+      <c r="C35" s="22">
+        <f>C29/$C$9-1</f>
+        <v/>
+      </c>
+      <c r="D35" s="22">
+        <f>D29/$C$9-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="B36" s="22">
+        <f>B30/$C$9-1</f>
+        <v/>
+      </c>
+      <c r="C36" s="22">
+        <f>C30/$C$9-1</f>
+        <v/>
+      </c>
+      <c r="D36" s="22">
+        <f>D30/$C$9-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="B37" s="22">
+        <f>B31/$C$9-1</f>
+        <v/>
+      </c>
+      <c r="C37" s="22">
+        <f>C31/$C$9-1</f>
+        <v/>
+      </c>
+      <c r="D37" s="22">
+        <f>D31/$C$9-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="13" t="inlineStr">
+        <is>
+          <t>Verdict: fundamental fair value ~Rs110-190 (base ~Rs145) implies BHEL is expensive vs the market price; the price is sustained by sector-premium multiples. Bull requires strong growth to materialise AND premium multiples to persist; Bear reflects de-rating toward fundamentals.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="001F3864"/>
@@ -12612,27 +13213,27 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="67">
+      <c r="A4" s="68">
         <f>'DCF Valuation'!C27</f>
         <v/>
       </c>
-      <c r="B4" s="67">
+      <c r="B4" s="68">
         <f>'DCF Valuation'!C28</f>
         <v/>
       </c>
-      <c r="D4" s="68">
+      <c r="D4" s="69">
         <f>'DCF Valuation'!C29</f>
         <v/>
       </c>
-      <c r="E4" s="67">
+      <c r="E4" s="68">
         <f>'Scenario Analysis'!B17</f>
         <v/>
       </c>
-      <c r="G4" s="67">
-        <f>'Relative Valuation'!C29</f>
-        <v/>
-      </c>
-      <c r="H4" s="68">
+      <c r="G4" s="68">
+        <f>'Relative Valuation'!C28</f>
+        <v/>
+      </c>
+      <c r="H4" s="69">
         <f>'Assumptions'!C65</f>
         <v/>
       </c>
@@ -12670,27 +13271,27 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="69">
+      <c r="A7" s="70">
         <f>'Forecast Financial Statements'!I5</f>
         <v/>
       </c>
-      <c r="B7" s="69">
+      <c r="B7" s="70">
         <f>'Forecast Financial Statements'!O5</f>
         <v/>
       </c>
-      <c r="D7" s="68">
+      <c r="D7" s="69">
         <f>'Forecast Financial Statements'!I12/'Forecast Financial Statements'!I5</f>
         <v/>
       </c>
-      <c r="E7" s="68">
+      <c r="E7" s="69">
         <f>'Forecast Financial Statements'!O12/'Forecast Financial Statements'!O5</f>
         <v/>
       </c>
-      <c r="G7" s="69">
+      <c r="G7" s="70">
         <f>'Revenue Build-up'!H10</f>
         <v/>
       </c>
-      <c r="H7" s="69">
+      <c r="H7" s="70">
         <f>'Forecast Financial Statements'!O20</f>
         <v/>
       </c>
@@ -12703,7 +13304,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="70" t="inlineStr">
+      <c r="A10" s="71" t="inlineStr">
         <is>
           <t>PV of explicit FCFF</t>
         </is>
@@ -12714,7 +13315,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="70" t="inlineStr">
+      <c r="A11" s="71" t="inlineStr">
         <is>
           <t>PV of terminal value</t>
         </is>
@@ -12725,7 +13326,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="70" t="inlineStr">
+      <c r="A12" s="71" t="inlineStr">
         <is>
           <t>Enterprise value</t>
         </is>
@@ -12736,7 +13337,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="70" t="inlineStr">
+      <c r="A13" s="71" t="inlineStr">
         <is>
           <t>Less: net debt</t>
         </is>
@@ -12747,7 +13348,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="70" t="inlineStr">
+      <c r="A14" s="71" t="inlineStr">
         <is>
           <t>Equity value</t>
         </is>
@@ -12763,7 +13364,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00C00000"/>
@@ -12877,59 +13478,59 @@
           <t>Balance sheet balances (TA = TE&amp;L)</t>
         </is>
       </c>
-      <c r="B5" s="71">
+      <c r="B5" s="72">
         <f>IF(ABS('Forecast Financial Statements'!B61-'Forecast Financial Statements'!B42)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="C5" s="71">
+      <c r="C5" s="72">
         <f>IF(ABS('Forecast Financial Statements'!C61-'Forecast Financial Statements'!C42)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="D5" s="71">
+      <c r="D5" s="72">
         <f>IF(ABS('Forecast Financial Statements'!D61-'Forecast Financial Statements'!D42)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="E5" s="71">
+      <c r="E5" s="72">
         <f>IF(ABS('Forecast Financial Statements'!E61-'Forecast Financial Statements'!E42)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="F5" s="71">
+      <c r="F5" s="72">
         <f>IF(ABS('Forecast Financial Statements'!F61-'Forecast Financial Statements'!F42)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="G5" s="71">
+      <c r="G5" s="72">
         <f>IF(ABS('Forecast Financial Statements'!G61-'Forecast Financial Statements'!G42)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="H5" s="71">
+      <c r="H5" s="72">
         <f>IF(ABS('Forecast Financial Statements'!H61-'Forecast Financial Statements'!H42)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="I5" s="71">
+      <c r="I5" s="72">
         <f>IF(ABS('Forecast Financial Statements'!I61-'Forecast Financial Statements'!I42)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="J5" s="71">
+      <c r="J5" s="72">
         <f>IF(ABS('Forecast Financial Statements'!J61-'Forecast Financial Statements'!J42)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="K5" s="71">
+      <c r="K5" s="72">
         <f>IF(ABS('Forecast Financial Statements'!K61-'Forecast Financial Statements'!K42)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="L5" s="71">
+      <c r="L5" s="72">
         <f>IF(ABS('Forecast Financial Statements'!L61-'Forecast Financial Statements'!L42)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="M5" s="71">
+      <c r="M5" s="72">
         <f>IF(ABS('Forecast Financial Statements'!M61-'Forecast Financial Statements'!M42)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="N5" s="71">
+      <c r="N5" s="72">
         <f>IF(ABS('Forecast Financial Statements'!N61-'Forecast Financial Statements'!N42)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="O5" s="71">
+      <c r="O5" s="72">
         <f>IF(ABS('Forecast Financial Statements'!O61-'Forecast Financial Statements'!O42)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
@@ -12940,31 +13541,31 @@
           <t>Cash: Balance sheet = Cash flow stmt</t>
         </is>
       </c>
-      <c r="I6" s="71">
+      <c r="I6" s="72">
         <f>IF(ABS('Forecast Financial Statements'!I58-'Cash Flow Statement'!I25)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="J6" s="71">
+      <c r="J6" s="72">
         <f>IF(ABS('Forecast Financial Statements'!J58-'Cash Flow Statement'!J25)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="K6" s="71">
+      <c r="K6" s="72">
         <f>IF(ABS('Forecast Financial Statements'!K58-'Cash Flow Statement'!K25)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="L6" s="71">
+      <c r="L6" s="72">
         <f>IF(ABS('Forecast Financial Statements'!L58-'Cash Flow Statement'!L25)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="M6" s="71">
+      <c r="M6" s="72">
         <f>IF(ABS('Forecast Financial Statements'!M58-'Cash Flow Statement'!M25)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="N6" s="71">
+      <c r="N6" s="72">
         <f>IF(ABS('Forecast Financial Statements'!N58-'Cash Flow Statement'!N25)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="O6" s="71">
+      <c r="O6" s="72">
         <f>IF(ABS('Forecast Financial Statements'!O58-'Cash Flow Statement'!O25)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
@@ -12975,31 +13576,31 @@
           <t>Retained earnings roll-forward ties</t>
         </is>
       </c>
-      <c r="I7" s="71">
+      <c r="I7" s="72">
         <f>IF(ABS('Forecast Financial Statements'!I29-'Equity Schedule'!I10)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="J7" s="71">
+      <c r="J7" s="72">
         <f>IF(ABS('Forecast Financial Statements'!J29-'Equity Schedule'!J10)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="K7" s="71">
+      <c r="K7" s="72">
         <f>IF(ABS('Forecast Financial Statements'!K29-'Equity Schedule'!K10)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="L7" s="71">
+      <c r="L7" s="72">
         <f>IF(ABS('Forecast Financial Statements'!L29-'Equity Schedule'!L10)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="M7" s="71">
+      <c r="M7" s="72">
         <f>IF(ABS('Forecast Financial Statements'!M29-'Equity Schedule'!M10)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="N7" s="71">
+      <c r="N7" s="72">
         <f>IF(ABS('Forecast Financial Statements'!N29-'Equity Schedule'!N10)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="O7" s="71">
+      <c r="O7" s="72">
         <f>IF(ABS('Forecast Financial Statements'!O29-'Equity Schedule'!O10)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
@@ -13010,31 +13611,31 @@
           <t>Debt roll-forward ties</t>
         </is>
       </c>
-      <c r="I8" s="71">
+      <c r="I8" s="72">
         <f>IF(ABS('Forecast Financial Statements'!I63-'Debt Schedule'!I9)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="J8" s="71">
+      <c r="J8" s="72">
         <f>IF(ABS('Forecast Financial Statements'!J63-'Debt Schedule'!J9)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="K8" s="71">
+      <c r="K8" s="72">
         <f>IF(ABS('Forecast Financial Statements'!K63-'Debt Schedule'!K9)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="L8" s="71">
+      <c r="L8" s="72">
         <f>IF(ABS('Forecast Financial Statements'!L63-'Debt Schedule'!L9)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="M8" s="71">
+      <c r="M8" s="72">
         <f>IF(ABS('Forecast Financial Statements'!M63-'Debt Schedule'!M9)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="N8" s="71">
+      <c r="N8" s="72">
         <f>IF(ABS('Forecast Financial Statements'!N63-'Debt Schedule'!N9)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="O8" s="71">
+      <c r="O8" s="72">
         <f>IF(ABS('Forecast Financial Statements'!O63-'Debt Schedule'!O9)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
@@ -13045,31 +13646,31 @@
           <t>Depreciation ties to P&amp;L</t>
         </is>
       </c>
-      <c r="I9" s="71">
+      <c r="I9" s="72">
         <f>IF(ABS('Forecast Financial Statements'!I13-'Depreciation Schedule'!I8)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="J9" s="71">
+      <c r="J9" s="72">
         <f>IF(ABS('Forecast Financial Statements'!J13-'Depreciation Schedule'!J8)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="K9" s="71">
+      <c r="K9" s="72">
         <f>IF(ABS('Forecast Financial Statements'!K13-'Depreciation Schedule'!K8)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="L9" s="71">
+      <c r="L9" s="72">
         <f>IF(ABS('Forecast Financial Statements'!L13-'Depreciation Schedule'!L8)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="M9" s="71">
+      <c r="M9" s="72">
         <f>IF(ABS('Forecast Financial Statements'!M13-'Depreciation Schedule'!M8)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="N9" s="71">
+      <c r="N9" s="72">
         <f>IF(ABS('Forecast Financial Statements'!N13-'Depreciation Schedule'!N8)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="O9" s="71">
+      <c r="O9" s="72">
         <f>IF(ABS('Forecast Financial Statements'!O13-'Depreciation Schedule'!O8)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
@@ -13080,31 +13681,31 @@
           <t>Revenue ties to Revenue Build-up</t>
         </is>
       </c>
-      <c r="I10" s="71">
+      <c r="I10" s="72">
         <f>IF(ABS('Forecast Financial Statements'!I5-'Revenue Build-up'!I15)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="J10" s="71">
+      <c r="J10" s="72">
         <f>IF(ABS('Forecast Financial Statements'!J5-'Revenue Build-up'!J15)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="K10" s="71">
+      <c r="K10" s="72">
         <f>IF(ABS('Forecast Financial Statements'!K5-'Revenue Build-up'!K15)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="L10" s="71">
+      <c r="L10" s="72">
         <f>IF(ABS('Forecast Financial Statements'!L5-'Revenue Build-up'!L15)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="M10" s="71">
+      <c r="M10" s="72">
         <f>IF(ABS('Forecast Financial Statements'!M5-'Revenue Build-up'!M15)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="N10" s="71">
+      <c r="N10" s="72">
         <f>IF(ABS('Forecast Financial Statements'!N5-'Revenue Build-up'!N15)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="O10" s="71">
+      <c r="O10" s="72">
         <f>IF(ABS('Forecast Financial Statements'!O5-'Revenue Build-up'!O15)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
@@ -13115,31 +13716,31 @@
           <t>Net fixed assets tie to FA schedule</t>
         </is>
       </c>
-      <c r="I11" s="71">
+      <c r="I11" s="72">
         <f>IF(ABS('Forecast Financial Statements'!I47-'Fixed Asset Schedule'!I10)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="J11" s="71">
+      <c r="J11" s="72">
         <f>IF(ABS('Forecast Financial Statements'!J47-'Fixed Asset Schedule'!J10)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="K11" s="71">
+      <c r="K11" s="72">
         <f>IF(ABS('Forecast Financial Statements'!K47-'Fixed Asset Schedule'!K10)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="L11" s="71">
+      <c r="L11" s="72">
         <f>IF(ABS('Forecast Financial Statements'!L47-'Fixed Asset Schedule'!L10)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="M11" s="71">
+      <c r="M11" s="72">
         <f>IF(ABS('Forecast Financial Statements'!M47-'Fixed Asset Schedule'!M10)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="N11" s="71">
+      <c r="N11" s="72">
         <f>IF(ABS('Forecast Financial Statements'!N47-'Fixed Asset Schedule'!N10)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
-      <c r="O11" s="71">
+      <c r="O11" s="72">
         <f>IF(ABS('Forecast Financial Statements'!O47-'Fixed Asset Schedule'!O10)&lt;0.5,"OK","REVIEW")</f>
         <v/>
       </c>
@@ -13150,7 +13751,7 @@
           <t>Historical balance check max |diff| (FY20-26)</t>
         </is>
       </c>
-      <c r="C13" s="72">
+      <c r="C13" s="73">
         <f>MAX(ABS('Historical Financial Statements'!B38),ABS('Historical Financial Statements'!C38),ABS('Historical Financial Statements'!D38),ABS('Historical Financial Statements'!E38),ABS('Historical Financial Statements'!F38),ABS('Historical Financial Statements'!G38),ABS('Historical Financial Statements'!H38))</f>
         <v/>
       </c>
@@ -13161,7 +13762,7 @@
           <t>Forecast balance check max |diff|</t>
         </is>
       </c>
-      <c r="C14" s="72">
+      <c r="C14" s="73">
         <f>MAX(ABS('Forecast Financial Statements'!I62),ABS('Forecast Financial Statements'!J62),ABS('Forecast Financial Statements'!K62),ABS('Forecast Financial Statements'!L62),ABS('Forecast Financial Statements'!M62),ABS('Forecast Financial Statements'!N62),ABS('Forecast Financial Statements'!O62))</f>
         <v/>
       </c>
@@ -13184,7 +13785,7 @@
           <t>Overall model status</t>
         </is>
       </c>
-      <c r="C16" s="73">
+      <c r="C16" s="74">
         <f>IF(COUNTIF(B5:O11,"REVIEW")=0,"ALL CHECKS PASS","REVIEW REQUIRED")</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Refresh Dashboard with price-target tiles + football-field valuation chart
- Dashboard tiles now surface DCF base, blended fair value, current price, and
  3M/6M/12M Base price targets plus 12M Bull/Bear (replacing the old prob-weighted
  and avg-relative TP tiles)
- Added a football-field chart: horizontal floating bars for DCF (83-123),
  Relative (152-273), Blended fair value (117-198) and the 12M target range
  (317-529), compared against the current price (~403), via a stacked bar with
  an invisible base series
- All balance checks pass
</commit_message>
<xml_diff>
--- a/BHEL_Financial_Model.xlsx
+++ b/BHEL_Financial_Model.xlsx
@@ -826,6 +826,102 @@
 </chartSpace>
 </file>
 
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Valuation football field (INR/share)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="bar"/>
+        <grouping val="stacked"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Dashboard'!$J$51:$J$55</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Dashboard'!$K$51:$K$55</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Dashboard'!$J$51:$J$55</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Dashboard'!$L$51:$L$55</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <overlap val="100"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
@@ -911,6 +1007,28 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart r:id="rId4"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>49</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6120000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="5" name="Chart 5"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId5"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -13153,7 +13271,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:M55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -13183,32 +13301,32 @@
     <row r="3">
       <c r="A3" s="24" t="inlineStr">
         <is>
-          <t>DCF value / share (INR)</t>
+          <t>DCF value/share - base</t>
         </is>
       </c>
       <c r="B3" s="24" t="inlineStr">
         <is>
+          <t>Blended fair value - base</t>
+        </is>
+      </c>
+      <c r="D3" s="24" t="inlineStr">
+        <is>
           <t>Current price (INR)</t>
         </is>
       </c>
-      <c r="D3" s="24" t="inlineStr">
-        <is>
-          <t>Upside / (downside)</t>
-        </is>
-      </c>
       <c r="E3" s="24" t="inlineStr">
         <is>
-          <t>Prob-weighted TP (INR)</t>
+          <t>12M target - Base</t>
         </is>
       </c>
       <c r="G3" s="24" t="inlineStr">
         <is>
-          <t>Avg relative TP (INR)</t>
+          <t>12M target - Bull</t>
         </is>
       </c>
       <c r="H3" s="24" t="inlineStr">
         <is>
-          <t>WACC</t>
+          <t>12M target - Bear</t>
         </is>
       </c>
     </row>
@@ -13218,35 +13336,35 @@
         <v/>
       </c>
       <c r="B4" s="68">
-        <f>'DCF Valuation'!C28</f>
-        <v/>
-      </c>
-      <c r="D4" s="69">
-        <f>'DCF Valuation'!C29</f>
+        <f>'Price Targets'!C17</f>
+        <v/>
+      </c>
+      <c r="D4" s="68">
+        <f>'Price Targets'!C9</f>
         <v/>
       </c>
       <c r="E4" s="68">
-        <f>'Scenario Analysis'!B17</f>
+        <f>'Price Targets'!D30</f>
         <v/>
       </c>
       <c r="G4" s="68">
-        <f>'Relative Valuation'!C28</f>
-        <v/>
-      </c>
-      <c r="H4" s="69">
-        <f>'Assumptions'!C65</f>
+        <f>'Price Targets'!D29</f>
+        <v/>
+      </c>
+      <c r="H4" s="68">
+        <f>'Price Targets'!D31</f>
         <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="24" t="inlineStr">
         <is>
-          <t>FY27E revenue (INR Cr)</t>
+          <t>3M target - Base</t>
         </is>
       </c>
       <c r="B6" s="24" t="inlineStr">
         <is>
-          <t>FY33E revenue (INR Cr)</t>
+          <t>6M target - Base</t>
         </is>
       </c>
       <c r="D6" s="24" t="inlineStr">
@@ -13266,17 +13384,17 @@
       </c>
       <c r="H6" s="24" t="inlineStr">
         <is>
-          <t>FY33E PAT (INR Cr)</t>
+          <t>WACC</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="70">
-        <f>'Forecast Financial Statements'!I5</f>
-        <v/>
-      </c>
-      <c r="B7" s="70">
-        <f>'Forecast Financial Statements'!O5</f>
+      <c r="A7" s="68">
+        <f>'Price Targets'!B30</f>
+        <v/>
+      </c>
+      <c r="B7" s="68">
+        <f>'Price Targets'!C30</f>
         <v/>
       </c>
       <c r="D7" s="69">
@@ -13291,8 +13409,8 @@
         <f>'Revenue Build-up'!H10</f>
         <v/>
       </c>
-      <c r="H7" s="70">
-        <f>'Forecast Financial Statements'!O20</f>
+      <c r="H7" s="69">
+        <f>'Assumptions'!C65</f>
         <v/>
       </c>
     </row>
@@ -13355,6 +13473,129 @@
       </c>
       <c r="B14" s="55">
         <f>'DCF Valuation'!C25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="6" t="inlineStr">
+        <is>
+          <t>Valuation football field (INR/share)  -  bars = value range by method; compare to current price</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="J50" s="4" t="inlineStr">
+        <is>
+          <t>Method</t>
+        </is>
+      </c>
+      <c r="K50" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L50" s="4" t="inlineStr">
+        <is>
+          <t>Range</t>
+        </is>
+      </c>
+      <c r="M50" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="J51" s="5" t="inlineStr">
+        <is>
+          <t>DCF (bear-bull)</t>
+        </is>
+      </c>
+      <c r="K51" s="49">
+        <f>'Price Targets'!B15</f>
+        <v/>
+      </c>
+      <c r="L51" s="35">
+        <f>M51-K51</f>
+        <v/>
+      </c>
+      <c r="M51" s="49">
+        <f>'Price Targets'!D15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="J52" s="5" t="inlineStr">
+        <is>
+          <t>Relative (bear-bull)</t>
+        </is>
+      </c>
+      <c r="K52" s="49">
+        <f>'Price Targets'!B16</f>
+        <v/>
+      </c>
+      <c r="L52" s="35">
+        <f>M52-K52</f>
+        <v/>
+      </c>
+      <c r="M52" s="49">
+        <f>'Price Targets'!D16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="J53" s="5" t="inlineStr">
+        <is>
+          <t>Blended fair value</t>
+        </is>
+      </c>
+      <c r="K53" s="49">
+        <f>'Price Targets'!B17</f>
+        <v/>
+      </c>
+      <c r="L53" s="35">
+        <f>M53-K53</f>
+        <v/>
+      </c>
+      <c r="M53" s="49">
+        <f>'Price Targets'!D17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="J54" s="5" t="inlineStr">
+        <is>
+          <t>12M target (bear-bull)</t>
+        </is>
+      </c>
+      <c r="K54" s="49">
+        <f>'Price Targets'!D31</f>
+        <v/>
+      </c>
+      <c r="L54" s="35">
+        <f>M54-K54</f>
+        <v/>
+      </c>
+      <c r="M54" s="49">
+        <f>'Price Targets'!D29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="J55" s="5" t="inlineStr">
+        <is>
+          <t>Current price</t>
+        </is>
+      </c>
+      <c r="K55" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="L55" s="35">
+        <f>M55-K55</f>
+        <v/>
+      </c>
+      <c r="M55" s="49">
+        <f>'Price Targets'!C9</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Restructure working capital: exclude non-current & non-operating items
- Working Capital Schedule now holds ONLY current operating items (receivables,
  inventory, current contract assets, other current operating assets; payables,
  current contract liabilities, other current operating liabilities). Operating
  NWC runs ~45%->33% of revenue.
- Non-current & non-operating items (deferred tax assets, non-current contract
  assets/liabilities, long-term provisions) moved to a separate block, clearly
  EXCLUDED from operating NWC and from the DCF free cash flow.
- FCFF now uses operating change-in-NWC only (removes the ~Rs100 cr/yr non-current
  drag); DCF value/share 102 -> 106.
- Balance sheet still ties: the non-current change flows to cash via a 'total
  change in NWC' line, so cash and the BS are unchanged. ALL CHECKS PASS.
- Also confirms LT-borrowings split already at audited ~2% (lease liabilities).
</commit_message>
<xml_diff>
--- a/BHEL_Financial_Model.xlsx
+++ b/BHEL_Financial_Model.xlsx
@@ -3422,7 +3422,7 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Other operating assets (memo, from WC)</t>
+          <t>Other current operating assets (memo, from WC)</t>
         </is>
       </c>
       <c r="I9" s="33">
@@ -3492,7 +3492,7 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>Provisions &amp; other liabilities (memo, from WC)</t>
+          <t>Other current operating liabilities (memo, from WC)</t>
         </is>
       </c>
       <c r="I11" s="33">
@@ -3842,31 +3842,31 @@
         <v/>
       </c>
       <c r="I8" s="33">
-        <f>'Working Capital Schedule'!I18</f>
+        <f>'Working Capital Schedule'!I25</f>
         <v/>
       </c>
       <c r="J8" s="33">
-        <f>'Working Capital Schedule'!J18</f>
+        <f>'Working Capital Schedule'!J25</f>
         <v/>
       </c>
       <c r="K8" s="33">
-        <f>'Working Capital Schedule'!K18</f>
+        <f>'Working Capital Schedule'!K25</f>
         <v/>
       </c>
       <c r="L8" s="33">
-        <f>'Working Capital Schedule'!L18</f>
+        <f>'Working Capital Schedule'!L25</f>
         <v/>
       </c>
       <c r="M8" s="33">
-        <f>'Working Capital Schedule'!M18</f>
+        <f>'Working Capital Schedule'!M25</f>
         <v/>
       </c>
       <c r="N8" s="33">
-        <f>'Working Capital Schedule'!N18</f>
+        <f>'Working Capital Schedule'!N25</f>
         <v/>
       </c>
       <c r="O8" s="33">
-        <f>'Working Capital Schedule'!O18</f>
+        <f>'Working Capital Schedule'!O25</f>
         <v/>
       </c>
     </row>
@@ -4535,7 +4535,7 @@
         <v>439.21</v>
       </c>
       <c r="I24" s="33">
-        <f>'Working Capital Schedule'!H19</f>
+        <f>'Working Capital Schedule'!H27</f>
         <v/>
       </c>
       <c r="J24" s="33">
@@ -6554,31 +6554,31 @@
         <v>13791.81</v>
       </c>
       <c r="I39" s="43">
-        <f>'Working Capital Schedule'!I14+'Working Capital Schedule'!I15-I35</f>
+        <f>'Working Capital Schedule'!I14+'Working Capital Schedule'!I15</f>
         <v/>
       </c>
       <c r="J39" s="43">
-        <f>'Working Capital Schedule'!J14+'Working Capital Schedule'!J15-J35</f>
+        <f>'Working Capital Schedule'!J14+'Working Capital Schedule'!J15</f>
         <v/>
       </c>
       <c r="K39" s="43">
-        <f>'Working Capital Schedule'!K14+'Working Capital Schedule'!K15-K35</f>
+        <f>'Working Capital Schedule'!K14+'Working Capital Schedule'!K15</f>
         <v/>
       </c>
       <c r="L39" s="43">
-        <f>'Working Capital Schedule'!L14+'Working Capital Schedule'!L15-L35</f>
+        <f>'Working Capital Schedule'!L14+'Working Capital Schedule'!L15</f>
         <v/>
       </c>
       <c r="M39" s="43">
-        <f>'Working Capital Schedule'!M14+'Working Capital Schedule'!M15-M35</f>
+        <f>'Working Capital Schedule'!M14+'Working Capital Schedule'!M15</f>
         <v/>
       </c>
       <c r="N39" s="43">
-        <f>'Working Capital Schedule'!N14+'Working Capital Schedule'!N15-N35</f>
+        <f>'Working Capital Schedule'!N14+'Working Capital Schedule'!N15</f>
         <v/>
       </c>
       <c r="O39" s="43">
-        <f>'Working Capital Schedule'!O14+'Working Capital Schedule'!O15-O35</f>
+        <f>'Working Capital Schedule'!O14+'Working Capital Schedule'!O15</f>
         <v/>
       </c>
     </row>
@@ -7240,31 +7240,31 @@
         <v>19457.88</v>
       </c>
       <c r="I57" s="43">
-        <f>'Working Capital Schedule'!I10+'Working Capital Schedule'!I11-I51</f>
+        <f>'Working Capital Schedule'!I10+'Working Capital Schedule'!I11</f>
         <v/>
       </c>
       <c r="J57" s="43">
-        <f>'Working Capital Schedule'!J10+'Working Capital Schedule'!J11-J51</f>
+        <f>'Working Capital Schedule'!J10+'Working Capital Schedule'!J11</f>
         <v/>
       </c>
       <c r="K57" s="43">
-        <f>'Working Capital Schedule'!K10+'Working Capital Schedule'!K11-K51</f>
+        <f>'Working Capital Schedule'!K10+'Working Capital Schedule'!K11</f>
         <v/>
       </c>
       <c r="L57" s="43">
-        <f>'Working Capital Schedule'!L10+'Working Capital Schedule'!L11-L51</f>
+        <f>'Working Capital Schedule'!L10+'Working Capital Schedule'!L11</f>
         <v/>
       </c>
       <c r="M57" s="43">
-        <f>'Working Capital Schedule'!M10+'Working Capital Schedule'!M11-M51</f>
+        <f>'Working Capital Schedule'!M10+'Working Capital Schedule'!M11</f>
         <v/>
       </c>
       <c r="N57" s="43">
-        <f>'Working Capital Schedule'!N10+'Working Capital Schedule'!N11-N51</f>
+        <f>'Working Capital Schedule'!N10+'Working Capital Schedule'!N11</f>
         <v/>
       </c>
       <c r="O57" s="43">
-        <f>'Working Capital Schedule'!O10+'Working Capital Schedule'!O11-O51</f>
+        <f>'Working Capital Schedule'!O10+'Working Capital Schedule'!O11</f>
         <v/>
       </c>
     </row>
@@ -9714,7 +9714,7 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Add/(less): change in working capital</t>
+          <t xml:space="preserve">   Add/(less): change in operating working capital</t>
         </is>
       </c>
       <c r="I11" s="43">
@@ -19798,7 +19798,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O26"/>
+  <dimension ref="A1:P34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -19842,7 +19842,7 @@
     <row r="2">
       <c r="A2" s="13" t="inlineStr">
         <is>
-          <t>FY2026 seeds are AUDITED actuals (BHEL FY26 BSE filing); used to anchor the forecast. Contract assets/liabilities shown at their current portion; the non-current portion sits in the "other" catch-alls and is carved out on the balance sheet.</t>
+          <t>Working capital = CURRENT operating items only. Non-current &amp; non-operating items (deferred tax, non-current contract assets/liabilities, long-term provisions) are shown in a separate block and EXCLUDED from operating NWC and from the DCF free cash flow; their change flows to cash via the total line so the balance sheet still ties. FY2026 seeds are audited actuals.</t>
         </is>
       </c>
     </row>
@@ -20187,11 +20187,11 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Other current &amp; non-current assets</t>
+          <t xml:space="preserve">   Other current operating assets</t>
         </is>
       </c>
       <c r="H11" s="46" t="n">
-        <v>25199.61</v>
+        <v>4264.99</v>
       </c>
       <c r="I11" s="33">
         <f>H11*(1+'Assumptions'!I42)</f>
@@ -20225,7 +20225,7 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Total operating assets</t>
+          <t>Total current operating assets</t>
         </is>
       </c>
       <c r="H12" s="44">
@@ -20340,11 +20340,11 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Provisions &amp; other liabilities</t>
+          <t xml:space="preserve">   Other current operating liabilities</t>
         </is>
       </c>
       <c r="H15" s="46" t="n">
-        <v>22250.07</v>
+        <v>4681.42</v>
       </c>
       <c r="I15" s="33">
         <f>H15*(1+'Assumptions'!I43)</f>
@@ -20378,7 +20378,7 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Total operating liabilities</t>
+          <t>Total current operating liabilities</t>
         </is>
       </c>
       <c r="H16" s="44">
@@ -20417,7 +20417,7 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Net working capital</t>
+          <t>Operating net working capital (current only)</t>
         </is>
       </c>
       <c r="H17" s="32">
@@ -20456,7 +20456,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>(Increase)/decrease in NWC</t>
+          <t>(Increase)/decrease in operating NWC  -&gt;  FCFF</t>
         </is>
       </c>
       <c r="I18" s="33">
@@ -20488,208 +20488,419 @@
         <v/>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>Memo: cash &amp; bank (FY26 seed, audited)</t>
-        </is>
-      </c>
-      <c r="H19" s="46" t="n">
-        <v>11866.62</v>
+    <row r="20">
+      <c r="A20" s="11" t="inlineStr">
+        <is>
+          <t>Non-current &amp; non-operating items (on balance sheet; EXCLUDED from working capital)</t>
+        </is>
+      </c>
+      <c r="B20" s="1" t="n"/>
+      <c r="C20" s="1" t="n"/>
+      <c r="D20" s="1" t="n"/>
+      <c r="E20" s="1" t="n"/>
+      <c r="F20" s="1" t="n"/>
+      <c r="G20" s="1" t="n"/>
+      <c r="H20" s="1" t="n"/>
+      <c r="I20" s="1" t="n"/>
+      <c r="J20" s="1" t="n"/>
+      <c r="K20" s="1" t="n"/>
+      <c r="L20" s="1" t="n"/>
+      <c r="M20" s="1" t="n"/>
+      <c r="N20" s="1" t="n"/>
+      <c r="O20" s="1" t="n"/>
+      <c r="P20" s="13" t="inlineStr">
+        <is>
+          <t>incl deferred tax (non-operating) &amp; long-dated contract balances</t>
+        </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="11" t="inlineStr">
-        <is>
-          <t>Memo: current-asset composition (indicative, forecast)</t>
-        </is>
-      </c>
-      <c r="B21" s="1" t="n"/>
-      <c r="C21" s="1" t="n"/>
-      <c r="D21" s="1" t="n"/>
-      <c r="E21" s="1" t="n"/>
-      <c r="F21" s="1" t="n"/>
-      <c r="G21" s="1" t="n"/>
-      <c r="H21" s="1" t="n"/>
-      <c r="I21" s="1" t="n"/>
-      <c r="J21" s="1" t="n"/>
-      <c r="K21" s="1" t="n"/>
-      <c r="L21" s="1" t="n"/>
-      <c r="M21" s="1" t="n"/>
-      <c r="N21" s="1" t="n"/>
-      <c r="O21" s="1" t="n"/>
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Other non-current assets (incl deferred tax, NC contract assets)</t>
+        </is>
+      </c>
+      <c r="H21" s="46" t="n">
+        <v>20934.62</v>
+      </c>
+      <c r="I21" s="33">
+        <f>'Assumptions'!I52</f>
+        <v/>
+      </c>
+      <c r="J21" s="33">
+        <f>'Assumptions'!J52</f>
+        <v/>
+      </c>
+      <c r="K21" s="33">
+        <f>'Assumptions'!K52</f>
+        <v/>
+      </c>
+      <c r="L21" s="33">
+        <f>'Assumptions'!L52</f>
+        <v/>
+      </c>
+      <c r="M21" s="33">
+        <f>'Assumptions'!M52</f>
+        <v/>
+      </c>
+      <c r="N21" s="33">
+        <f>'Assumptions'!N52</f>
+        <v/>
+      </c>
+      <c r="O21" s="33">
+        <f>'Assumptions'!O52</f>
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Inventory: raw materials &amp; components (~45%)</t>
-        </is>
+          <t xml:space="preserve">   Other non-current liabilities (incl NC contract liab, LT provisions)</t>
+        </is>
+      </c>
+      <c r="H22" s="46" t="n">
+        <v>17568.65</v>
       </c>
       <c r="I22" s="33">
-        <f>I9*0.45</f>
+        <f>'Assumptions'!I53</f>
         <v/>
       </c>
       <c r="J22" s="33">
-        <f>J9*0.45</f>
+        <f>'Assumptions'!J53</f>
         <v/>
       </c>
       <c r="K22" s="33">
-        <f>K9*0.45</f>
+        <f>'Assumptions'!K53</f>
         <v/>
       </c>
       <c r="L22" s="33">
-        <f>L9*0.45</f>
+        <f>'Assumptions'!L53</f>
         <v/>
       </c>
       <c r="M22" s="33">
-        <f>M9*0.45</f>
+        <f>'Assumptions'!M53</f>
         <v/>
       </c>
       <c r="N22" s="33">
-        <f>N9*0.45</f>
+        <f>'Assumptions'!N53</f>
         <v/>
       </c>
       <c r="O22" s="33">
-        <f>O9*0.45</f>
+        <f>'Assumptions'!O53</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Inventory: work-in-progress (~35%)</t>
-        </is>
-      </c>
-      <c r="I23" s="33">
-        <f>I9*0.35</f>
-        <v/>
-      </c>
-      <c r="J23" s="33">
-        <f>J9*0.35</f>
-        <v/>
-      </c>
-      <c r="K23" s="33">
-        <f>K9*0.35</f>
-        <v/>
-      </c>
-      <c r="L23" s="33">
-        <f>L9*0.35</f>
-        <v/>
-      </c>
-      <c r="M23" s="33">
-        <f>M9*0.35</f>
-        <v/>
-      </c>
-      <c r="N23" s="33">
-        <f>N9*0.35</f>
-        <v/>
-      </c>
-      <c r="O23" s="33">
-        <f>O9*0.35</f>
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Net non-current items (assets - liabilities)</t>
+        </is>
+      </c>
+      <c r="H23" s="32">
+        <f>H21-H22</f>
+        <v/>
+      </c>
+      <c r="I23" s="32">
+        <f>I21-I22</f>
+        <v/>
+      </c>
+      <c r="J23" s="32">
+        <f>J21-J22</f>
+        <v/>
+      </c>
+      <c r="K23" s="32">
+        <f>K21-K22</f>
+        <v/>
+      </c>
+      <c r="L23" s="32">
+        <f>L21-L22</f>
+        <v/>
+      </c>
+      <c r="M23" s="32">
+        <f>M21-M22</f>
+        <v/>
+      </c>
+      <c r="N23" s="32">
+        <f>N21-N22</f>
+        <v/>
+      </c>
+      <c r="O23" s="32">
+        <f>O21-O22</f>
         <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
+          <t>(Increase)/decrease in net non-current items</t>
+        </is>
+      </c>
+      <c r="I24" s="33">
+        <f>-(I23-H23)</f>
+        <v/>
+      </c>
+      <c r="J24" s="33">
+        <f>-(J23-I23)</f>
+        <v/>
+      </c>
+      <c r="K24" s="33">
+        <f>-(K23-J23)</f>
+        <v/>
+      </c>
+      <c r="L24" s="33">
+        <f>-(L23-K23)</f>
+        <v/>
+      </c>
+      <c r="M24" s="33">
+        <f>-(M23-L23)</f>
+        <v/>
+      </c>
+      <c r="N24" s="33">
+        <f>-(N23-M23)</f>
+        <v/>
+      </c>
+      <c r="O24" s="33">
+        <f>-(O23-N23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Total (increase)/decrease in NWC incl non-current  -&gt;  cash flow</t>
+        </is>
+      </c>
+      <c r="I25" s="44">
+        <f>I18+I24</f>
+        <v/>
+      </c>
+      <c r="J25" s="44">
+        <f>J18+J24</f>
+        <v/>
+      </c>
+      <c r="K25" s="44">
+        <f>K18+K24</f>
+        <v/>
+      </c>
+      <c r="L25" s="44">
+        <f>L18+L24</f>
+        <v/>
+      </c>
+      <c r="M25" s="44">
+        <f>M18+M24</f>
+        <v/>
+      </c>
+      <c r="N25" s="44">
+        <f>N18+N24</f>
+        <v/>
+      </c>
+      <c r="O25" s="44">
+        <f>O18+O24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Memo: cash &amp; bank (FY26 seed, audited)</t>
+        </is>
+      </c>
+      <c r="H27" s="46" t="n">
+        <v>11866.62</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="11" t="inlineStr">
+        <is>
+          <t>Memo: current-asset composition (indicative, forecast)</t>
+        </is>
+      </c>
+      <c r="B29" s="1" t="n"/>
+      <c r="C29" s="1" t="n"/>
+      <c r="D29" s="1" t="n"/>
+      <c r="E29" s="1" t="n"/>
+      <c r="F29" s="1" t="n"/>
+      <c r="G29" s="1" t="n"/>
+      <c r="H29" s="1" t="n"/>
+      <c r="I29" s="1" t="n"/>
+      <c r="J29" s="1" t="n"/>
+      <c r="K29" s="1" t="n"/>
+      <c r="L29" s="1" t="n"/>
+      <c r="M29" s="1" t="n"/>
+      <c r="N29" s="1" t="n"/>
+      <c r="O29" s="1" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Inventory: raw materials &amp; components (~45%)</t>
+        </is>
+      </c>
+      <c r="I30" s="33">
+        <f>I9*0.45</f>
+        <v/>
+      </c>
+      <c r="J30" s="33">
+        <f>J9*0.45</f>
+        <v/>
+      </c>
+      <c r="K30" s="33">
+        <f>K9*0.45</f>
+        <v/>
+      </c>
+      <c r="L30" s="33">
+        <f>L9*0.45</f>
+        <v/>
+      </c>
+      <c r="M30" s="33">
+        <f>M9*0.45</f>
+        <v/>
+      </c>
+      <c r="N30" s="33">
+        <f>N9*0.45</f>
+        <v/>
+      </c>
+      <c r="O30" s="33">
+        <f>O9*0.45</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Inventory: work-in-progress (~35%)</t>
+        </is>
+      </c>
+      <c r="I31" s="33">
+        <f>I9*0.35</f>
+        <v/>
+      </c>
+      <c r="J31" s="33">
+        <f>J9*0.35</f>
+        <v/>
+      </c>
+      <c r="K31" s="33">
+        <f>K9*0.35</f>
+        <v/>
+      </c>
+      <c r="L31" s="33">
+        <f>L9*0.35</f>
+        <v/>
+      </c>
+      <c r="M31" s="33">
+        <f>M9*0.35</f>
+        <v/>
+      </c>
+      <c r="N31" s="33">
+        <f>N9*0.35</f>
+        <v/>
+      </c>
+      <c r="O31" s="33">
+        <f>O9*0.35</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">   Inventory: finished goods &amp; stores (~20%)</t>
         </is>
       </c>
-      <c r="I24" s="33">
+      <c r="I32" s="33">
         <f>I9*0.20</f>
         <v/>
       </c>
-      <c r="J24" s="33">
+      <c r="J32" s="33">
         <f>J9*0.20</f>
         <v/>
       </c>
-      <c r="K24" s="33">
+      <c r="K32" s="33">
         <f>K9*0.20</f>
         <v/>
       </c>
-      <c r="L24" s="33">
+      <c r="L32" s="33">
         <f>L9*0.20</f>
         <v/>
       </c>
-      <c r="M24" s="33">
+      <c r="M32" s="33">
         <f>M9*0.20</f>
         <v/>
       </c>
-      <c r="N24" s="33">
+      <c r="N32" s="33">
         <f>N9*0.20</f>
         <v/>
       </c>
-      <c r="O24" s="33">
+      <c r="O32" s="33">
         <f>O9*0.20</f>
         <v/>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="5" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">   Receivables: billed / trade (~70%)</t>
         </is>
       </c>
-      <c r="I25" s="33">
+      <c r="I33" s="33">
         <f>I8*0.70</f>
         <v/>
       </c>
-      <c r="J25" s="33">
+      <c r="J33" s="33">
         <f>J8*0.70</f>
         <v/>
       </c>
-      <c r="K25" s="33">
+      <c r="K33" s="33">
         <f>K8*0.70</f>
         <v/>
       </c>
-      <c r="L25" s="33">
+      <c r="L33" s="33">
         <f>L8*0.70</f>
         <v/>
       </c>
-      <c r="M25" s="33">
+      <c r="M33" s="33">
         <f>M8*0.70</f>
         <v/>
       </c>
-      <c r="N25" s="33">
+      <c r="N33" s="33">
         <f>N8*0.70</f>
         <v/>
       </c>
-      <c r="O25" s="33">
+      <c r="O33" s="33">
         <f>O8*0.70</f>
         <v/>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="5" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">   Receivables: unbilled / retention (~30%)</t>
         </is>
       </c>
-      <c r="I26" s="33">
+      <c r="I34" s="33">
         <f>I8*0.30</f>
         <v/>
       </c>
-      <c r="J26" s="33">
+      <c r="J34" s="33">
         <f>J8*0.30</f>
         <v/>
       </c>
-      <c r="K26" s="33">
+      <c r="K34" s="33">
         <f>K8*0.30</f>
         <v/>
       </c>
-      <c r="L26" s="33">
+      <c r="L34" s="33">
         <f>L8*0.30</f>
         <v/>
       </c>
-      <c r="M26" s="33">
+      <c r="M34" s="33">
         <f>M8*0.30</f>
         <v/>
       </c>
-      <c r="N26" s="33">
+      <c r="N34" s="33">
         <f>N8*0.30</f>
         <v/>
       </c>
-      <c r="O26" s="33">
+      <c r="O34" s="33">
         <f>O8*0.30</f>
         <v/>
       </c>

</xml_diff>